<commit_message>
chore: actualizar reporte FT buffer [2026-06-30]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:33 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:33 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:33 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:33 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:33 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:33 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:33 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:33 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/29/2026 at 12:34 PM ET)</t>
+          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>291 days</t>
+          <t>290 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>53 days</t>
+          <t>52 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>172 days</t>
+          <t>171 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>235 days</t>
+          <t>234 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>200 days</t>
+          <t>199 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>18 days</t>
+          <t>17 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>353 days</t>
+          <t>352 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>263 days</t>
+          <t>262 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>326 days</t>
+          <t>325 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>144 days</t>
+          <t>143 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>109 days</t>
+          <t>108 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>81 days</t>
+          <t>80 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>291 days</t>
+          <t>290 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>53 days</t>
+          <t>52 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>172 days</t>
+          <t>171 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>235 days</t>
+          <t>234 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>200 days</t>
+          <t>199 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>18 days</t>
+          <t>17 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>353 days</t>
+          <t>352 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>263 days</t>
+          <t>262 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>326 days</t>
+          <t>325 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>144 days</t>
+          <t>143 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>109 days</t>
+          <t>108 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>81 days</t>
+          <t>80 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.48 / 2.67%</t>
+          <t>$46.67 / 3.10%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.25 / 10.98%</t>
+          <t>$56.42 / 11.30%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.18 / 6.21%</t>
+          <t>$54.38 / 6.61%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$60.70 / 4.80%</t>
+          <t>$60.96 / 5.26%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$54.85 / 4.93%</t>
+          <t>$55.10 / 5.41%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.40 / 12.93%</t>
+          <t>$59.54 / 13.19%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.53 / -0.57%</t>
+          <t>$59.86 / -0.03%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.08 / 7.79%</t>
+          <t>$52.24 / 8.12%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$55.81 / 0.44%</t>
+          <t>$56.15 / 1.05%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.14 / 9.19%</t>
+          <t>$58.39 / 9.65%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.02 / 8.67%</t>
+          <t>$52.26 / 9.17%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$54.81 / 8.72%</t>
+          <t>$55.06 / 9.23%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.51 / 2.12%</t>
+          <t>$41.63 / 2.43%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.27 / 9.14%</t>
+          <t>$41.40 / 9.48%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.64 / 5.17%</t>
+          <t>$39.77 / 5.51%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$43.87 / 3.91%</t>
+          <t>$43.98 / 4.16%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$44.82 / 4.10%</t>
+          <t>$44.98 / 4.48%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.42 / 10.68%</t>
+          <t>$43.49 / 10.86%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$40.95 / -0.48%</t>
+          <t>$41.13 / -0.05%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.11 / 6.20%</t>
+          <t>$44.21 / 6.44%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$42.84 / 0.46%</t>
+          <t>$43.03 / 0.92%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.62 / 7.49%</t>
+          <t>$41.76 / 7.85%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.37 / 7.26%</t>
+          <t>$41.49 / 7.58%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$40.81 / 7.46%</t>
+          <t>$40.93 / 7.78%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$738.18 / 3.95%</t>
+          <t>$745.88 / 5.03%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$738.18 / 14.72%</t>
+          <t>$745.88 / 15.92%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$738.07 / 8.45%</t>
+          <t>$745.88 / 9.59%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$738.18 / 7.07%</t>
+          <t>$745.88 / 8.19%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$738.18 / 6.73%</t>
+          <t>$745.88 / 7.84%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$738.18 / 17.62%</t>
+          <t>$745.88 / 18.85%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$738.18 / -1.15%</t>
+          <t>$745.88 / -0.12%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$738.18 / 13.82%</t>
+          <t>$745.88 / 15.00%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$738.18 / -0.13%</t>
+          <t>$745.88 / 0.91%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$738.07 / 11.99%</t>
+          <t>$745.88 / 13.18%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$738.07 / 11.09%</t>
+          <t>$745.88 / 12.26%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$738.07 / 11.21%</t>
+          <t>$745.88 / 12.38%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$738.07 / 3.93%</t>
+          <t>$745.88 / 5.03%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$738.07 / 14.71%</t>
+          <t>$745.88 / 15.92%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$738.07 / 8.45%</t>
+          <t>$745.88 / 9.59%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$738.07 / 7.06%</t>
+          <t>$745.88 / 8.19%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$738.07 / 6.71%</t>
+          <t>$745.88 / 7.84%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$738.07 / 17.61%</t>
+          <t>$745.88 / 18.85%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$738.07 / -1.16%</t>
+          <t>$745.88 / -0.12%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$738.07 / 13.80%</t>
+          <t>$745.88 / 15.00%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$738.07 / -0.15%</t>
+          <t>$745.88 / 0.91%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$738.07 / 11.99%</t>
+          <t>$745.88 / 13.18%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$738.07 / 11.09%</t>
+          <t>$745.88 / 12.26%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$738.07 / 11.21%</t>
+          <t>$745.88 / 12.38%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>12.00% (11.34%)</t>
+          <t>11.53% (10.88%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2.32% (2.21%)</t>
+          <t>2.02% (1.91%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.62% (7.24%)</t>
+          <t>7.21% (6.84%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>9.45% (8.93%)</t>
+          <t>8.98% (8.46%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.78% (8.34%)</t>
+          <t>8.29% (7.85%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.72% (0.68%)</t>
+          <t>0.48% (0.45%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>17.09% (16.27%)</t>
+          <t>16.45% (15.63%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.48% (7.91%)</t>
+          <t>8.15% (7.58%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>16.47% (15.71%)</t>
+          <t>15.77% (15.02%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>6.34% (6.03%)</t>
+          <t>5.88% (5.58%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5.36% (5.13%)</t>
+          <t>4.87% (4.64%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>4.25% (4.07%)</t>
+          <t>3.76% (3.59%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.84% (9.18%)</t>
+          <t>9.51% (8.85%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.85% (1.74%)</t>
+          <t>1.53% (1.42%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>6.15% (5.77%)</t>
+          <t>5.80% (5.42%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.55% (7.02%)</t>
+          <t>7.29% (6.77%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>7.04% (6.60%)</t>
+          <t>6.65% (6.21%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.51% (0.47%)</t>
+          <t>0.34% (0.31%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.88% (13.05%)</t>
+          <t>13.38% (12.56%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>7.22% (6.64%)</t>
+          <t>6.97% (6.40%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>13.21% (12.45%)</t>
+          <t>12.69% (11.94%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.89% (4.57%)</t>
+          <t>4.53% (4.22%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>4.00% (3.76%)</t>
+          <t>3.69% (3.45%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>3.13% (2.95%)</t>
+          <t>2.82% (2.65%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10.79%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-0.38%</t>
+          <t>-1.41%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.81%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>7.41%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>7.31%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-2.61%</t>
+          <t>-3.62%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>17.80%</t>
+          <t>16.59%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.95%</t>
+          <t>1.88%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>17.25%</t>
+          <t>16.04%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4.13%</t>
+          <t>3.04%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>3.60%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>1.44%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>8.09%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-2.45%</t>
+          <t>-3.47%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>3.35%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>4.67%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>4.78%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-4.73%</t>
+          <t>-5.73%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>13.48%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>0.27%</t>
+          <t>-0.78%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>12.81%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>1.12%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>0.25%</t>
+          <t>-0.80%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.65% (9.99%)</t>
+          <t>11.14% (10.48%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.99% (10.88%)</t>
+          <t>11.54% (11.43%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.74% (10.36%)</t>
+          <t>11.25% (10.88%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.07% (10.55%)</t>
+          <t>11.53% (11.01%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.61% (10.16%)</t>
+          <t>11.04% (10.61%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.32% (11.29%)</t>
+          <t>11.90% (11.87%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.50% (8.68%)</t>
+          <t>9.89% (9.07%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.48% (12.91%)</t>
+          <t>14.01% (13.44%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.33% (8.58%)</t>
+          <t>9.67% (8.92%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.76% (10.45%)</t>
+          <t>11.20% (10.90%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.46% (10.23%)</t>
+          <t>10.88% (10.65%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.44% (10.27%)</t>
+          <t>10.86% (10.69%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.97% (15.31%)</t>
+          <t>16.53% (15.87%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.85% (16.74%)</t>
+          <t>17.34% (17.23%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.28% (15.90%)</t>
+          <t>16.79% (16.41%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.55% (16.02%)</t>
+          <t>17.15% (16.63%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.04% (15.59%)</t>
+          <t>16.52% (16.08%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>17.35% (17.31%)</t>
+          <t>17.96% (17.92%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.46% (13.64%)</t>
+          <t>14.92% (14.10%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.25% (18.67%)</t>
+          <t>19.81% (19.24%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.31% (13.56%)</t>
+          <t>14.75% (14.00%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.66% (16.35%)</t>
+          <t>17.14% (16.83%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.17% (15.93%)</t>
+          <t>16.68% (16.45%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.01% (15.83%)</t>
+          <t>16.53% (16.36%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-2.76% (-3.42%)</t>
+          <t>-3.17% (-3.83%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-10.56% (-10.67%)</t>
+          <t>-10.82% (-10.93%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.27% (-6.65%)</t>
+          <t>-6.62% (-7.00%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-4.87% (-5.39%)</t>
+          <t>-5.28% (-5.80%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.06% (-5.51%)</t>
+          <t>-5.50% (-5.94%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.16% (-12.20%)</t>
+          <t>-12.37% (-12.41%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.28%)</t>
+          <t>0.00% (-0.82%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.45% (-8.02%)</t>
+          <t>-7.73% (-8.30%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-0.55% (-1.30%)</t>
+          <t>-1.14% (-1.89%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-8.88% (-9.19%)</t>
+          <t>-9.27% (-9.58%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-8.53% (-8.76%)</t>
+          <t>-8.95% (-9.18%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-8.63% (-8.80%)</t>
+          <t>-9.05% (-9.23%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.24% (-2.90%)</t>
+          <t>-2.54% (-3.19%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.05% (-9.16%)</t>
+          <t>-9.33% (-9.45%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.34% (-5.72%)</t>
+          <t>-5.65% (-6.02%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.05% (-4.57%)</t>
+          <t>-4.28% (-4.80%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.30% (-4.75%)</t>
+          <t>-4.66% (-5.10%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.37% (-10.41%)</t>
+          <t>-10.52% (-10.55%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.36%)</t>
+          <t>0.00% (-0.80%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.06% (-6.63%)</t>
+          <t>-6.27% (-6.85%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-0.56% (-1.31%)</t>
+          <t>-1.01% (-1.76%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.44% (-7.75%)</t>
+          <t>-7.75% (-8.06%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.32% (-7.55%)</t>
+          <t>-7.60% (-7.83%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-7.55% (-7.73%)</t>
+          <t>-7.83% (-8.00%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-13.42%</t>
+          <t>-14.31%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.55%</t>
+          <t>-22.36%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.01%</t>
+          <t>-17.88%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-15.94%</t>
+          <t>-16.81%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-15.67%</t>
+          <t>-16.54%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-23.48%</t>
+          <t>-24.27%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-8.96%</t>
+          <t>-9.90%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-20.93%</t>
+          <t>-21.74%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-9.88%</t>
+          <t>-10.81%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-19.64%</t>
+          <t>-20.48%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-18.98%</t>
+          <t>-19.83%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
+          <t>-19.92%</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
           <t>-19.07%</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>-18.21%</t>
-        </is>
-      </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-25.90%</t>
+          <t>-26.67%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-21.62%</t>
+          <t>-22.44%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.60%</t>
+          <t>-21.43%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-20.34%</t>
+          <t>-21.18%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-27.72%</t>
+          <t>-28.48%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.00%</t>
+          <t>-14.90%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-25.31%</t>
+          <t>-26.09%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-14.87%</t>
+          <t>-15.76%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.10%</t>
+          <t>-24.89%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.48%</t>
+          <t>-24.28%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.56%</t>
+          <t>-24.36%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.08% (0.42%)</t>
+          <t>1.71% (1.05%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2.32% (2.21%)</t>
+          <t>2.02% (1.91%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.68% (1.31%)</t>
+          <t>2.37% (2.00%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.88% (1.36%)</t>
+          <t>2.49% (1.98%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.34% (0.90%)</t>
+          <t>1.94% (1.50%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.72% (0.68%)</t>
+          <t>0.48% (0.45%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.55% (-0.28%)</t>
+          <t>0.00% (-0.82%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.37% (4.80%)</t>
+          <t>6.14% (5.58%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.55% (-1.30%)</t>
+          <t>-0.24% (-0.99%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.10% (1.80%)</t>
+          <t>2.74% (2.44%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.68% (1.45%)</t>
+          <t>2.29% (2.06%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.68% (1.50%)</t>
+          <t>2.28% (2.11%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.61% (0.95%)</t>
+          <t>2.37% (1.72%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.85% (1.74%)</t>
+          <t>1.53% (1.42%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.69% (2.31%)</t>
+          <t>3.44% (3.06%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2.74% (2.21%)</t>
+          <t>3.58% (3.06%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.14% (1.69%)</t>
+          <t>2.84% (2.40%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.51% (0.47%)</t>
+          <t>0.34% (0.31%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.46% (-0.36%)</t>
+          <t>0.02% (-0.80%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.93% (6.36%)</t>
+          <t>6.97% (6.40%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.56% (-1.31%)</t>
+          <t>-0.12% (-0.87%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.71% (3.40%)</t>
+          <t>4.46% (4.15%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.02% (2.78%)</t>
+          <t>3.69% (3.45%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.87% (2.70%)</t>
+          <t>2.82% (2.65%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 29/6/2026</t>
+          <t>As of 30/6/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.16%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8.34%</t>
+          <t>7.85%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.93%</t>
+          <t>5.41%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.73%</t>
+          <t>7.84%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7.31%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.51%</t>
+          <t>-5.94%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.55%</t>
+          <t>11.01%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.93%</t>
+          <t>8.46%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.80%</t>
+          <t>5.26%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.07%</t>
+          <t>8.19%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7.41%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.39%</t>
+          <t>-5.80%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>13.44%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.91%</t>
+          <t>7.58%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.79%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.82%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2.95%</t>
+          <t>1.88%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.02%</t>
+          <t>-8.30%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.99%</t>
+          <t>10.48%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>10.88%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.67%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.95%</t>
+          <t>5.03%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10.79%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.42%</t>
+          <t>-3.83%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.58%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.71%</t>
+          <t>15.02%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>1.05%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>17.25%</t>
+          <t>16.04%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.30%</t>
+          <t>-1.89%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.68%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>15.63%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17.80%</t>
+          <t>16.59%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.28%</t>
+          <t>-0.82%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.87%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.68%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>12.93%</t>
+          <t>13.19%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>17.62%</t>
+          <t>18.85%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-2.61%</t>
+          <t>-3.62%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.20%</t>
+          <t>-12.41%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>11.43%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2.21%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>11.30%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.72%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.38%</t>
+          <t>-1.41%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.67%</t>
+          <t>-10.93%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.27%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4.07%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.72%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>12.38%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>1.44%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.80%</t>
+          <t>-9.23%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5.13%</t>
+          <t>4.64%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.67%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.09%</t>
+          <t>12.26%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3.60%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.76%</t>
+          <t>-9.18%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.45%</t>
+          <t>10.90%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>6.03%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.19%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.99%</t>
+          <t>13.18%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4.13%</t>
+          <t>3.04%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.19%</t>
+          <t>-9.58%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.36%</t>
+          <t>10.88%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7.24%</t>
+          <t>6.84%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>6.61%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.45%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5.81%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.65%</t>
+          <t>-7.00%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 29/6/2026</t>
+          <t>As of 30/6/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.59%</t>
+          <t>16.08%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.60%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.10%</t>
+          <t>4.48%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.71%</t>
+          <t>7.84%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.78%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-4.75%</t>
+          <t>-5.10%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.02%</t>
+          <t>16.63%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.02%</t>
+          <t>6.77%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>4.16%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.06%</t>
+          <t>8.19%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.67%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.57%</t>
+          <t>-4.80%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.67%</t>
+          <t>19.24%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.64%</t>
+          <t>6.40%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.20%</t>
+          <t>6.44%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.80%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.27%</t>
+          <t>-0.78%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.63%</t>
+          <t>-6.85%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>8.85%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.12%</t>
+          <t>2.43%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.93%</t>
+          <t>5.03%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.09%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-2.90%</t>
+          <t>-3.19%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.56%</t>
+          <t>14.00%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.45%</t>
+          <t>11.94%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.15%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>12.81%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-1.76%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.64%</t>
+          <t>14.10%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>12.56%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.48%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.16%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>13.48%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>-0.80%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>17.92%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>10.86%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>17.61%</t>
+          <t>18.85%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.73%</t>
+          <t>-5.73%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.41%</t>
+          <t>-10.55%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.74%</t>
+          <t>17.23%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.74%</t>
+          <t>1.42%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.14%</t>
+          <t>9.48%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.71%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.45%</t>
+          <t>-3.47%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.16%</t>
+          <t>-9.45%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.83%</t>
+          <t>16.36%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.95%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.46%</t>
+          <t>7.78%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>12.38%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.25%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-7.73%</t>
+          <t>-8.00%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.93%</t>
+          <t>16.45%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.26%</t>
+          <t>7.58%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.09%</t>
+          <t>12.26%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.55%</t>
+          <t>-7.83%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.35%</t>
+          <t>16.83%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.57%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.49%</t>
+          <t>7.85%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.99%</t>
+          <t>13.18%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.12%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-7.75%</t>
+          <t>-8.06%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.90%</t>
+          <t>16.41%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.77%</t>
+          <t>5.42%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>5.51%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.45%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.35%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-5.72%</t>
+          <t>-6.02%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-01]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 6/30/2026 at 11:59 AM ET)</t>
+          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>290 days</t>
+          <t>289 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>52 days</t>
+          <t>51 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>171 days</t>
+          <t>170 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>234 days</t>
+          <t>233 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>199 days</t>
+          <t>198 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>17 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>352 days</t>
+          <t>351 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>262 days</t>
+          <t>261 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>325 days</t>
+          <t>324 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>143 days</t>
+          <t>142 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>108 days</t>
+          <t>107 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>80 days</t>
+          <t>79 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>290 days</t>
+          <t>289 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>52 days</t>
+          <t>51 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>171 days</t>
+          <t>170 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>234 days</t>
+          <t>233 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>199 days</t>
+          <t>198 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>17 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>352 days</t>
+          <t>351 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>262 days</t>
+          <t>261 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>325 days</t>
+          <t>324 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>143 days</t>
+          <t>142 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>108 days</t>
+          <t>107 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>80 days</t>
+          <t>79 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.67 / 3.10%</t>
+          <t>$46.76 / 3.29%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.42 / 11.30%</t>
+          <t>$56.55 / 11.56%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.38 / 6.61%</t>
+          <t>$54.52 / 6.89%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$60.96 / 5.26%</t>
+          <t>$61.11 / 5.52%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.10 / 5.41%</t>
+          <t>$55.21 / 5.62%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.54 / 13.19%</t>
+          <t>$59.61 / 13.32%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.86 / -0.03%</t>
+          <t>$60.01 / 0.22%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.24 / 8.12%</t>
+          <t>$52.37 / 8.38%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.15 / 1.05%</t>
+          <t>$56.27 / 1.27%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.39 / 9.65%</t>
+          <t>$58.54 / 9.94%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.26 / 9.17%</t>
+          <t>$52.40 / 9.45%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.06 / 9.23%</t>
+          <t>$55.17 / 9.45%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.63 / 2.43%</t>
+          <t>$41.69 / 2.58%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.40 / 9.48%</t>
+          <t>$41.47 / 9.68%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.77 / 5.51%</t>
+          <t>$39.85 / 5.72%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$43.98 / 4.16%</t>
+          <t>$44.07 / 4.37%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$44.98 / 4.48%</t>
+          <t>$45.05 / 4.63%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.49 / 10.86%</t>
+          <t>$43.50 / 10.88%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.13 / -0.05%</t>
+          <t>$41.22 / 0.16%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.21 / 6.44%</t>
+          <t>$44.27 / 6.59%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.03 / 0.92%</t>
+          <t>$43.13 / 1.14%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.76 / 7.85%</t>
+          <t>$41.83 / 8.03%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.49 / 7.58%</t>
+          <t>$41.58 / 7.82%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$40.93 / 7.78%</t>
+          <t>$41.01 / 7.97%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$745.88 / 5.03%</t>
+          <t>$748.81 / 5.45%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$745.88 / 15.92%</t>
+          <t>$748.81 / 16.38%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$745.88 / 9.59%</t>
+          <t>$748.81 / 10.02%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$745.88 / 8.19%</t>
+          <t>$748.81 / 8.61%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$745.88 / 7.84%</t>
+          <t>$748.81 / 8.26%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$745.88 / 18.85%</t>
+          <t>$748.81 / 19.32%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$745.88 / -0.12%</t>
+          <t>$748.81 / 0.28%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$745.88 / 15.00%</t>
+          <t>$748.81 / 15.46%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$745.88 / 0.91%</t>
+          <t>$748.81 / 1.30%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$745.88 / 13.18%</t>
+          <t>$748.81 / 13.62%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$745.88 / 12.26%</t>
+          <t>$748.81 / 12.71%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$745.88 / 12.38%</t>
+          <t>$748.81 / 12.82%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$745.88 / 5.03%</t>
+          <t>$748.81 / 5.45%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$745.88 / 15.92%</t>
+          <t>$748.81 / 16.38%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$745.88 / 9.59%</t>
+          <t>$748.81 / 10.02%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$745.88 / 8.19%</t>
+          <t>$748.81 / 8.61%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$745.88 / 7.84%</t>
+          <t>$748.81 / 8.26%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$745.88 / 18.85%</t>
+          <t>$748.81 / 19.32%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$745.88 / -0.12%</t>
+          <t>$748.81 / 0.28%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$745.88 / 15.00%</t>
+          <t>$748.81 / 15.46%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$745.88 / 0.91%</t>
+          <t>$748.81 / 1.30%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$745.88 / 13.18%</t>
+          <t>$748.81 / 13.62%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$745.88 / 12.26%</t>
+          <t>$748.81 / 12.71%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$745.88 / 12.38%</t>
+          <t>$748.81 / 12.82%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.53% (10.88%)</t>
+          <t>11.33% (10.68%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2.02% (1.91%)</t>
+          <t>1.78% (1.67%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.21% (6.84%)</t>
+          <t>6.93% (6.56%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.98% (8.46%)</t>
+          <t>8.71% (8.19%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.29% (7.85%)</t>
+          <t>8.07% (7.63%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.48% (0.45%)</t>
+          <t>0.37% (0.34%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.45% (15.63%)</t>
+          <t>16.16% (15.35%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.15% (7.58%)</t>
+          <t>7.89% (7.33%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.77% (15.02%)</t>
+          <t>15.51% (14.77%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.88% (5.58%)</t>
+          <t>5.61% (5.31%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.87% (4.64%)</t>
+          <t>4.60% (4.37%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.76% (3.59%)</t>
+          <t>3.55% (3.39%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.51% (8.85%)</t>
+          <t>9.35% (8.70%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.53% (1.42%)</t>
+          <t>1.34% (1.23%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.80% (5.42%)</t>
+          <t>5.59% (5.21%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.29% (6.77%)</t>
+          <t>7.07% (6.55%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.65% (6.21%)</t>
+          <t>6.49% (6.05%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.34% (0.31%)</t>
+          <t>0.32% (0.28%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.38% (12.56%)</t>
+          <t>13.14% (12.32%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.97% (6.40%)</t>
+          <t>6.83% (6.26%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.69% (11.94%)</t>
+          <t>12.44% (11.70%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.53% (4.22%)</t>
+          <t>4.36% (4.05%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.69% (3.45%)</t>
+          <t>3.46% (3.23%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.82% (2.65%)</t>
+          <t>2.63% (2.46%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.41%</t>
+          <t>-1.79%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>5.89%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>5.79%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-3.62%</t>
+          <t>-4.00%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.59%</t>
+          <t>16.13%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.88%</t>
+          <t>1.49%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.04%</t>
+          <t>15.58%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.04%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>2.12%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.44%</t>
+          <t>1.04%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>6.54%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.47%</t>
+          <t>-3.85%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.57%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.28%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-5.73%</t>
+          <t>-6.10%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.48%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.78%</t>
+          <t>-1.17%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.81%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>-0.33%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-1.19%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.14% (10.48%)</t>
+          <t>11.30% (10.65%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.54% (11.43%)</t>
+          <t>11.63% (11.53%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.25% (10.88%)</t>
+          <t>11.33% (10.96%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.53% (11.01%)</t>
+          <t>11.62% (11.10%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.04% (10.61%)</t>
+          <t>11.18% (10.74%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.90% (11.87%)</t>
+          <t>12.10% (12.07%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.89% (9.07%)</t>
+          <t>10.00% (9.18%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.01% (13.44%)</t>
+          <t>14.09% (13.53%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.67% (8.92%)</t>
+          <t>9.80% (9.05%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.20% (10.90%)</t>
+          <t>11.28% (10.98%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.88% (10.65%)</t>
+          <t>10.96% (10.73%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.86% (10.69%)</t>
+          <t>10.99% (10.82%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.53% (15.87%)</t>
+          <t>16.71% (16.05%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.34% (17.23%)</t>
+          <t>17.46% (17.35%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.79% (16.41%)</t>
+          <t>16.90% (16.53%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.15% (16.63%)</t>
+          <t>17.26% (16.74%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.52% (16.08%)</t>
+          <t>16.69% (16.25%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>17.96% (17.92%)</t>
+          <t>18.22% (18.18%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.92% (14.10%)</t>
+          <t>15.04% (14.23%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.81% (19.24%)</t>
+          <t>19.98% (19.41%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.75% (14.00%)</t>
+          <t>14.86% (14.11%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.14% (16.83%)</t>
+          <t>17.28% (16.97%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.68% (16.45%)</t>
+          <t>16.78% (16.55%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.53% (16.36%)</t>
+          <t>16.66% (16.49%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.17% (-3.83%)</t>
+          <t>-3.35% (-4.00%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-10.82% (-10.93%)</t>
+          <t>-11.03% (-11.14%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.62% (-7.00%)</t>
+          <t>-6.87% (-7.24%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.28% (-5.80%)</t>
+          <t>-5.52% (-6.03%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.50% (-5.94%)</t>
+          <t>-5.69% (-6.12%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.37% (-12.41%)</t>
+          <t>-12.47% (-12.50%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.82%)</t>
+          <t>-0.25% (-1.07%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.73% (-8.30%)</t>
+          <t>-7.96% (-8.52%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.14% (-1.89%)</t>
+          <t>-1.36% (-2.11%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.27% (-9.58%)</t>
+          <t>-9.51% (-9.81%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-8.95% (-9.18%)</t>
+          <t>-9.18% (-9.41%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.05% (-9.23%)</t>
+          <t>-9.24% (-9.41%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.54% (-3.19%)</t>
+          <t>-2.68% (-3.33%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.33% (-9.45%)</t>
+          <t>-9.50% (-9.61%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.65% (-6.02%)</t>
+          <t>-5.84% (-6.21%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.28% (-4.80%)</t>
+          <t>-4.48% (-5.00%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.66% (-5.10%)</t>
+          <t>-4.80% (-5.24%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.52% (-10.55%)</t>
+          <t>-10.54% (-10.57%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.80%)</t>
+          <t>-0.19% (-1.00%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.27% (-6.85%)</t>
+          <t>-6.40% (-6.97%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.01% (-1.76%)</t>
+          <t>-1.23% (-1.98%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.75% (-8.06%)</t>
+          <t>-7.91% (-8.22%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.60% (-7.83%)</t>
+          <t>-7.80% (-8.03%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-7.83% (-8.00%)</t>
+          <t>-8.00% (-8.17%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.31%</t>
+          <t>-14.65%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.36%</t>
+          <t>-22.66%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.88%</t>
+          <t>-18.20%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.81%</t>
+          <t>-17.14%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.54%</t>
+          <t>-16.87%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.27%</t>
+          <t>-24.57%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.90%</t>
+          <t>-10.25%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>-22.05%</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>-11.16%</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>-20.79%</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>-20.15%</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>-20.23%</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>-19.39%</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>-26.96%</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-22.74%</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
           <t>-21.74%</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>-10.81%</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>-20.48%</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>-19.83%</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>-19.92%</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>-19.07%</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>-26.67%</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>-22.44%</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>-21.43%</t>
-        </is>
-      </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.18%</t>
+          <t>-21.48%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-28.48%</t>
+          <t>-28.76%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.90%</t>
+          <t>-15.23%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.09%</t>
+          <t>-26.38%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.76%</t>
+          <t>-16.09%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.89%</t>
+          <t>-25.19%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.28%</t>
+          <t>-24.58%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.36%</t>
+          <t>-24.66%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.71% (1.05%)</t>
+          <t>1.92% (1.27%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2.02% (1.91%)</t>
+          <t>1.78% (1.67%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.37% (2.00%)</t>
+          <t>2.51% (2.14%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.49% (1.98%)</t>
+          <t>2.64% (2.13%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.94% (1.50%)</t>
+          <t>2.13% (1.70%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.48% (0.45%)</t>
+          <t>0.37% (0.34%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.00% (-0.82%)</t>
+          <t>0.02% (-0.79%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.14% (5.58%)</t>
+          <t>6.30% (5.74%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.24% (-0.99%)</t>
+          <t>-0.08% (-0.82%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.74% (2.44%)</t>
+          <t>2.88% (2.58%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.29% (2.06%)</t>
+          <t>2.42% (2.20%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.28% (2.11%)</t>
+          <t>2.48% (2.31%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.37% (1.72%)</t>
+          <t>2.63% (1.97%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.53% (1.42%)</t>
+          <t>1.34% (1.23%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.44% (3.06%)</t>
+          <t>3.64% (3.26%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.58% (3.06%)</t>
+          <t>3.77% (3.25%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.84% (2.40%)</t>
+          <t>3.10% (2.66%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.34% (0.31%)</t>
+          <t>0.32% (0.28%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.02% (-0.80%)</t>
+          <t>0.09% (-0.73%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.97% (6.40%)</t>
+          <t>6.83% (6.26%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.12% (-0.87%)</t>
+          <t>0.05% (-0.69%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>4.46% (4.15%)</t>
+          <t>4.36% (4.05%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.69% (3.45%)</t>
+          <t>3.46% (3.23%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.82% (2.65%)</t>
+          <t>2.63% (2.46%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 30/6/2026</t>
+          <t>As of 1/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.74%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.85%</t>
+          <t>7.63%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>5.62%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.84%</t>
+          <t>8.26%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>5.79%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.94%</t>
+          <t>-6.12%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.01%</t>
+          <t>11.10%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.46%</t>
+          <t>8.19%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.26%</t>
+          <t>5.52%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.19%</t>
+          <t>8.61%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>5.89%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.80%</t>
+          <t>-6.03%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.53%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.58%</t>
+          <t>7.33%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.12%</t>
+          <t>8.38%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>15.46%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.88%</t>
+          <t>1.49%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.30%</t>
+          <t>-8.52%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.48%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.03%</t>
+          <t>5.45%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.83%</t>
+          <t>-4.00%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>9.05%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.02%</t>
+          <t>14.77%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.05%</t>
+          <t>1.27%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>1.30%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.04%</t>
+          <t>15.58%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.89%</t>
+          <t>-2.11%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.63%</t>
+          <t>15.35%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>0.22%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.59%</t>
+          <t>16.13%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>-1.07%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.87%</t>
+          <t>12.07%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.19%</t>
+          <t>13.32%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.85%</t>
+          <t>19.32%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-3.62%</t>
+          <t>-4.00%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.41%</t>
+          <t>-12.50%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.43%</t>
+          <t>11.53%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.67%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.30%</t>
+          <t>11.56%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.38%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.41%</t>
+          <t>-1.79%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.93%</t>
+          <t>-11.14%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>10.82%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.38%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.44%</t>
+          <t>1.04%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.23%</t>
+          <t>-9.41%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.64%</t>
+          <t>4.37%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.26%</t>
+          <t>12.71%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>2.12%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.18%</t>
+          <t>-9.41%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.90%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.58%</t>
+          <t>5.31%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.18%</t>
+          <t>13.62%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.04%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.58%</t>
+          <t>-9.81%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.84%</t>
+          <t>6.56%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.61%</t>
+          <t>6.89%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.00%</t>
+          <t>-7.24%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 30/6/2026</t>
+          <t>As of 1/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.08%</t>
+          <t>16.25%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>6.05%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.48%</t>
+          <t>4.63%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.84%</t>
+          <t>8.26%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.28%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.10%</t>
+          <t>-5.24%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.63%</t>
+          <t>16.74%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.77%</t>
+          <t>6.55%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.16%</t>
+          <t>4.37%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.19%</t>
+          <t>8.61%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.57%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.80%</t>
+          <t>-5.00%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.24%</t>
+          <t>19.41%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.40%</t>
+          <t>6.26%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.44%</t>
+          <t>6.59%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>15.46%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.78%</t>
+          <t>-1.17%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.85%</t>
+          <t>-6.97%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.85%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.43%</t>
+          <t>2.58%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.03%</t>
+          <t>5.45%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>6.54%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.19%</t>
+          <t>-3.33%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>14.11%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.94%</t>
+          <t>11.70%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>1.14%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>1.30%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.81%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.76%</t>
+          <t>-1.98%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.10%</t>
+          <t>14.23%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.56%</t>
+          <t>12.32%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.48%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-1.00%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17.92%</t>
+          <t>18.18%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.86%</t>
+          <t>10.88%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.85%</t>
+          <t>19.32%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-5.73%</t>
+          <t>-6.10%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.55%</t>
+          <t>-10.57%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.23%</t>
+          <t>17.35%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.42%</t>
+          <t>1.23%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.48%</t>
+          <t>9.68%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.38%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.47%</t>
+          <t>-3.85%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.45%</t>
+          <t>-9.61%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.36%</t>
+          <t>16.49%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>2.46%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.78%</t>
+          <t>7.97%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.38%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-1.19%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.00%</t>
+          <t>-8.17%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.45%</t>
+          <t>16.55%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.45%</t>
+          <t>3.23%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.58%</t>
+          <t>7.82%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.26%</t>
+          <t>12.71%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.83%</t>
+          <t>-8.03%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.83%</t>
+          <t>16.97%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.22%</t>
+          <t>4.05%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.85%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.18%</t>
+          <t>13.62%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>-0.33%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.06%</t>
+          <t>-8.22%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.41%</t>
+          <t>16.53%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.42%</t>
+          <t>5.21%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.51%</t>
+          <t>5.72%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.02%</t>
+          <t>-6.21%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-02]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/1/2026 at 11:58 AM ET)</t>
+          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>289 days</t>
+          <t>288 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>51 days</t>
+          <t>50 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>170 days</t>
+          <t>169 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>233 days</t>
+          <t>232 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>198 days</t>
+          <t>197 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>15 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>351 days</t>
+          <t>350 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>261 days</t>
+          <t>260 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>324 days</t>
+          <t>323 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>142 days</t>
+          <t>141 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>107 days</t>
+          <t>106 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>79 days</t>
+          <t>78 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>289 days</t>
+          <t>288 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>51 days</t>
+          <t>50 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>170 days</t>
+          <t>169 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>233 days</t>
+          <t>232 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>198 days</t>
+          <t>197 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>15 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>351 days</t>
+          <t>350 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>261 days</t>
+          <t>260 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>324 days</t>
+          <t>323 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>142 days</t>
+          <t>141 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>107 days</t>
+          <t>106 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>79 days</t>
+          <t>78 days</t>
         </is>
       </c>
     </row>
@@ -2326,27 +2326,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.76 / 3.29%</t>
+          <t>$46.69 / 3.14%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.55 / 11.56%</t>
+          <t>$56.51 / 11.49%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.52 / 6.89%</t>
+          <t>$54.45 / 6.75%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.11 / 5.52%</t>
+          <t>$61.01 / 5.34%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.21 / 5.62%</t>
+          <t>$55.15 / 5.52%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2356,92 +2356,92 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.01 / 0.22%</t>
+          <t>$59.90 / 0.04%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.37 / 8.38%</t>
+          <t>$52.32 / 8.28%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.27 / 1.27%</t>
+          <t>$56.15 / 1.06%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.54 / 9.94%</t>
+          <t>$58.45 / 9.78%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.40 / 9.45%</t>
+          <t>$52.33 / 9.32%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.17 / 9.45%</t>
+          <t>$55.14 / 9.39%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.69 / 2.58%</t>
+          <t>$41.65 / 2.48%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.47 / 9.68%</t>
+          <t>$41.44 / 9.60%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.85 / 5.72%</t>
+          <t>$39.82 / 5.64%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.07 / 4.37%</t>
+          <t>$44.02 / 4.26%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.05 / 4.63%</t>
+          <t>$45.02 / 4.56%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.50 / 10.88%</t>
+          <t>$43.52 / 10.93%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.22 / 0.16%</t>
+          <t>$41.16 / 0.01%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.27 / 6.59%</t>
+          <t>$44.26 / 6.56%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.13 / 1.14%</t>
+          <t>$43.08 / 1.02%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.83 / 8.03%</t>
+          <t>$41.82 / 8.00%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.58 / 7.82%</t>
+          <t>$41.56 / 7.75%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.01 / 7.97%</t>
+          <t>$40.98 / 7.91%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$748.81 / 5.45%</t>
+          <t>$745.82 / 5.02%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$748.81 / 16.38%</t>
+          <t>$745.82 / 15.91%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$748.81 / 10.02%</t>
+          <t>$745.82 / 9.58%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$748.81 / 8.61%</t>
+          <t>$745.82 / 8.18%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$748.81 / 8.26%</t>
+          <t>$745.82 / 7.83%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$748.81 / 19.32%</t>
+          <t>$745.82 / 18.84%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$748.81 / 0.28%</t>
+          <t>$745.82 / -0.12%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$748.81 / 15.46%</t>
+          <t>$745.82 / 14.99%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$748.81 / 1.30%</t>
+          <t>$745.82 / 0.90%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$748.81 / 13.62%</t>
+          <t>$745.82 / 13.17%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$748.81 / 12.71%</t>
+          <t>$745.82 / 12.26%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$748.81 / 12.82%</t>
+          <t>$745.82 / 12.37%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$748.81 / 5.45%</t>
+          <t>$745.82 / 5.02%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$748.81 / 16.38%</t>
+          <t>$745.54 / 15.87%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$748.81 / 10.02%</t>
+          <t>$745.54 / 9.54%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$748.81 / 8.61%</t>
+          <t>$745.82 / 8.18%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$748.81 / 8.26%</t>
+          <t>$745.82 / 7.83%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$748.81 / 19.32%</t>
+          <t>$745.54 / 18.80%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$748.81 / 0.28%</t>
+          <t>$745.82 / -0.12%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$748.81 / 15.46%</t>
+          <t>$745.82 / 14.99%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$748.81 / 1.30%</t>
+          <t>$745.82 / 0.90%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$748.81 / 13.62%</t>
+          <t>$745.54 / 13.13%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$748.81 / 12.71%</t>
+          <t>$745.54 / 12.21%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$748.81 / 12.82%</t>
+          <t>$745.54 / 12.33%</t>
         </is>
       </c>
     </row>
@@ -2580,27 +2580,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.33% (10.68%)</t>
+          <t>11.48% (10.83%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.78% (1.67%)</t>
+          <t>1.84% (1.74%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.93% (6.56%)</t>
+          <t>7.07% (6.70%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.71% (8.19%)</t>
+          <t>8.89% (8.38%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.07% (7.63%)</t>
+          <t>8.17% (7.74%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2610,92 +2610,92 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.16% (15.35%)</t>
+          <t>16.37% (15.56%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.89% (7.33%)</t>
+          <t>7.99% (7.43%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.51% (14.77%)</t>
+          <t>15.76% (15.01%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.61% (5.31%)</t>
+          <t>5.76% (5.46%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.60% (4.37%)</t>
+          <t>4.73% (4.50%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.55% (3.39%)</t>
+          <t>3.61% (3.44%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.35% (8.70%)</t>
+          <t>9.45% (8.80%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.34% (1.23%)</t>
+          <t>1.41% (1.31%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.59% (5.21%)</t>
+          <t>5.67% (5.29%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.07% (6.55%)</t>
+          <t>7.18% (6.66%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.49% (6.05%)</t>
+          <t>6.56% (6.12%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.32% (0.28%)</t>
+          <t>0.27% (0.24%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.14% (12.32%)</t>
+          <t>13.30% (12.49%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.83% (6.26%)</t>
+          <t>6.85% (6.28%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.44% (11.70%)</t>
+          <t>12.57% (11.83%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.36% (4.05%)</t>
+          <t>4.38% (4.07%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.46% (3.23%)</t>
+          <t>3.52% (3.29%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.63% (2.46%)</t>
+          <t>2.70% (2.53%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.79%</t>
+          <t>-1.40%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.30%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.89%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.79%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-4.00%</t>
+          <t>-3.61%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.13%</t>
+          <t>16.59%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.49%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15.58%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.64%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.12%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.04%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.54%</t>
+          <t>6.97%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.85%</t>
+          <t>-3.43%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.17%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.28%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-6.10%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.33%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.19%</t>
+          <t>-0.76%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.30% (10.65%)</t>
+          <t>11.09% (10.44%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.63% (11.53%)</t>
+          <t>11.38% (11.27%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.33% (10.96%)</t>
+          <t>11.12% (10.75%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.62% (11.10%)</t>
+          <t>11.45% (10.93%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.18% (10.74%)</t>
+          <t>10.94% (10.50%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.10% (12.07%)</t>
+          <t>11.80% (11.77%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.00% (9.18%)</t>
+          <t>9.82% (9.00%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.09% (13.53%)</t>
+          <t>13.87% (13.31%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.80% (9.05%)</t>
+          <t>9.65% (8.90%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.28% (10.98%)</t>
+          <t>11.09% (10.79%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.96% (10.73%)</t>
+          <t>10.75% (10.53%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.99% (10.82%)</t>
+          <t>10.72% (10.55%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.71% (16.05%)</t>
+          <t>16.48% (15.82%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.46% (17.35%)</t>
+          <t>17.20% (17.09%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.90% (16.53%)</t>
+          <t>16.63% (16.26%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.26% (16.74%)</t>
+          <t>17.04% (16.52%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.69% (16.25%)</t>
+          <t>16.44% (16.00%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>18.22% (18.18%)</t>
+          <t>17.86% (17.83%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.04% (14.23%)</t>
+          <t>14.85% (14.03%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.98% (19.41%)</t>
+          <t>19.70% (19.13%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.86% (14.11%)</t>
+          <t>14.64% (13.89%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.28% (16.97%)</t>
+          <t>16.97% (16.67%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.78% (16.55%)</t>
+          <t>16.50% (16.27%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.66% (16.49%)</t>
+          <t>16.38% (16.22%)</t>
         </is>
       </c>
     </row>
@@ -2961,27 +2961,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.35% (-4.00%)</t>
+          <t>-3.22% (-3.87%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.03% (-11.14%)</t>
+          <t>-10.98% (-11.08%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.87% (-7.24%)</t>
+          <t>-6.75% (-7.12%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.52% (-6.03%)</t>
+          <t>-5.36% (-5.87%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.69% (-6.12%)</t>
+          <t>-5.60% (-6.03%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2991,92 +2991,92 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.25% (-1.07%)</t>
+          <t>-0.07% (-0.89%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.96% (-8.52%)</t>
+          <t>-7.87% (-8.43%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.36% (-2.11%)</t>
+          <t>-1.15% (-1.90%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.51% (-9.81%)</t>
+          <t>-9.38% (-9.68%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.18% (-9.41%)</t>
+          <t>-9.07% (-9.30%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.24% (-9.41%)</t>
+          <t>-9.19% (-9.36%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.68% (-3.33%)</t>
+          <t>-2.59% (-3.24%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.50% (-9.61%)</t>
+          <t>-9.44% (-9.54%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.84% (-6.21%)</t>
+          <t>-5.77% (-6.14%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.48% (-5.00%)</t>
+          <t>-4.38% (-4.90%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.80% (-5.24%)</t>
+          <t>-4.73% (-5.17%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.54% (-10.57%)</t>
+          <t>-10.58% (-10.62%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.19% (-1.00%)</t>
+          <t>-0.04% (-0.86%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.40% (-6.97%)</t>
+          <t>-6.38% (-6.95%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.23% (-1.98%)</t>
+          <t>-1.12% (-1.86%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.91% (-8.22%)</t>
+          <t>-7.89% (-8.19%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.80% (-8.03%)</t>
+          <t>-7.75% (-7.98%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.00% (-8.17%)</t>
+          <t>-7.94% (-8.11%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.65%</t>
+          <t>-14.30%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.66%</t>
+          <t>-22.35%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.20%</t>
+          <t>-17.87%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.14%</t>
+          <t>-16.80%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.87%</t>
+          <t>-16.54%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.57%</t>
+          <t>-24.27%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.25%</t>
+          <t>-9.89%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.05%</t>
+          <t>-21.74%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.16%</t>
+          <t>-10.80%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.79%</t>
+          <t>-20.47%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.15%</t>
+          <t>-19.83%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.23%</t>
+          <t>-19.91%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.39%</t>
+          <t>-19.06%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.96%</t>
+          <t>-26.64%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.74%</t>
+          <t>-22.40%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-21.74%</t>
+          <t>-21.42%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.48%</t>
+          <t>-21.17%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-28.76%</t>
+          <t>-28.45%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.23%</t>
+          <t>-14.89%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.38%</t>
+          <t>-26.08%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.09%</t>
+          <t>-15.76%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.19%</t>
+          <t>-24.86%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.58%</t>
+          <t>-24.25%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.66%</t>
+          <t>-24.33%</t>
         </is>
       </c>
     </row>
@@ -3215,27 +3215,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.92% (1.27%)</t>
+          <t>1.65% (1.00%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.78% (1.67%)</t>
+          <t>1.84% (1.74%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.51% (2.14%)</t>
+          <t>2.23% (1.86%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.64% (2.13%)</t>
+          <t>2.41% (1.89%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.13% (1.70%)</t>
+          <t>1.82% (1.39%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3245,92 +3245,92 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.02% (-0.79%)</t>
+          <t>-0.07% (-0.89%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.30% (5.74%)</t>
+          <t>5.98% (5.42%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.08% (-0.82%)</t>
+          <t>-0.27% (-1.01%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.88% (2.58%)</t>
+          <t>2.62% (2.32%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.42% (2.20%)</t>
+          <t>2.14% (1.91%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.48% (2.31%)</t>
+          <t>2.12% (1.95%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.63% (1.97%)</t>
+          <t>2.31% (1.66%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.34% (1.23%)</t>
+          <t>1.41% (1.31%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.64% (3.26%)</t>
+          <t>3.26% (2.89%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.77% (3.25%)</t>
+          <t>3.46% (2.94%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.10% (2.66%)</t>
+          <t>2.75% (2.31%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.32% (0.28%)</t>
+          <t>0.27% (0.24%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.09% (-0.73%)</t>
+          <t>-0.04% (-0.86%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.83% (6.26%)</t>
+          <t>6.85% (6.28%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.05% (-0.69%)</t>
+          <t>-0.23% (-0.98%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>4.36% (4.05%)</t>
+          <t>4.26% (3.96%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.46% (3.23%)</t>
+          <t>3.52% (3.29%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.63% (2.46%)</t>
+          <t>2.70% (2.53%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 1/7/2026</t>
+          <t>As of 2/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.74%</t>
+          <t>10.50%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.63%</t>
+          <t>7.74%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.62%</t>
+          <t>5.52%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.26%</t>
+          <t>7.83%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.79%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.12%</t>
+          <t>-6.03%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.10%</t>
+          <t>10.93%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.19%</t>
+          <t>8.38%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.52%</t>
+          <t>5.34%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.61%</t>
+          <t>8.18%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.89%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.03%</t>
+          <t>-5.87%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.53%</t>
+          <t>13.31%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.33%</t>
+          <t>7.43%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.38%</t>
+          <t>8.28%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.46%</t>
+          <t>14.99%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.49%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.52%</t>
+          <t>-8.43%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>10.44%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>10.83%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>3.14%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.45%</t>
+          <t>5.02%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.00%</t>
+          <t>-3.87%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.05%</t>
+          <t>8.90%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.77%</t>
+          <t>15.01%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.30%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>15.58%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.11%</t>
+          <t>-1.90%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>15.56%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.13%</t>
+          <t>16.59%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>-0.89%</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.07%</t>
+          <t>11.77%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3647,12 +3647,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.32%</t>
+          <t>18.84%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.00%</t>
+          <t>-3.61%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.53%</t>
+          <t>11.27%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.67%</t>
+          <t>1.74%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.56%</t>
+          <t>11.49%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.38%</t>
+          <t>15.91%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.79%</t>
+          <t>-1.40%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.14%</t>
+          <t>-11.08%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.82%</t>
+          <t>10.55%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>3.44%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>9.39%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.04%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.41%</t>
+          <t>-9.36%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.53%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.37%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>9.32%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>12.26%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.12%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.41%</t>
+          <t>-9.30%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>10.79%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.31%</t>
+          <t>5.46%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.94%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.62%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.64%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.81%</t>
+          <t>-9.68%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>10.75%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.56%</t>
+          <t>6.70%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.89%</t>
+          <t>6.75%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>9.58%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.30%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.24%</t>
+          <t>-7.12%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 1/7/2026</t>
+          <t>As of 2/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.25%</t>
+          <t>16.00%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.05%</t>
+          <t>6.12%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.63%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.26%</t>
+          <t>7.83%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.28%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.24%</t>
+          <t>-5.17%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.74%</t>
+          <t>16.52%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.55%</t>
+          <t>6.66%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.37%</t>
+          <t>4.26%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.61%</t>
+          <t>8.18%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.17%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.00%</t>
+          <t>-4.90%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.41%</t>
+          <t>19.13%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.26%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.59%</t>
+          <t>6.56%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.46%</t>
+          <t>14.99%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.97%</t>
+          <t>-6.95%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>15.82%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.58%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.45%</t>
+          <t>5.02%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.54%</t>
+          <t>6.97%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.33%</t>
+          <t>-3.24%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.11%</t>
+          <t>13.89%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.70%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.14%</t>
+          <t>1.02%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.30%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.98%</t>
+          <t>-1.86%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.23%</t>
+          <t>14.03%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.32%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>0.01%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.00%</t>
+          <t>-0.86%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.18%</t>
+          <t>17.83%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>10.93%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.32%</t>
+          <t>18.80%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-6.10%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.57%</t>
+          <t>-10.62%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.35%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.23%</t>
+          <t>1.31%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.68%</t>
+          <t>9.60%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.38%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.85%</t>
+          <t>-3.43%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.61%</t>
+          <t>-9.54%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.49%</t>
+          <t>16.22%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.46%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.97%</t>
+          <t>7.91%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.33%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.19%</t>
+          <t>-0.76%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.17%</t>
+          <t>-8.11%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.55%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.23%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.82%</t>
+          <t>7.75%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>12.21%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.03%</t>
+          <t>-7.98%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.97%</t>
+          <t>16.67%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>4.07%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>8.00%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.62%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.33%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.22%</t>
+          <t>-8.19%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.53%</t>
+          <t>16.26%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.21%</t>
+          <t>5.29%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.72%</t>
+          <t>5.64%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.21%</t>
+          <t>-6.14%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-03]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:43 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026 at 11:44 AM ET)</t>
+          <t>Current Values(as of 7/2/2026)</t>
         </is>
       </c>
     </row>
@@ -2326,77 +2326,77 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.69 / 3.14%</t>
+          <t>$46.66 / 3.08%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.51 / 11.49%</t>
+          <t>$56.50 / 11.48%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.45 / 6.75%</t>
+          <t>$54.43 / 6.71%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.01 / 5.34%</t>
+          <t>$60.99 / 5.32%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.15 / 5.52%</t>
+          <t>$55.11 / 5.43%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.61 / 13.32%</t>
+          <t>$59.62 / 13.35%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.90 / 0.04%</t>
+          <t>$59.81 / -0.10%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.32 / 8.28%</t>
+          <t>$52.30 / 8.26%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.15 / 1.06%</t>
+          <t>$56.10 / 0.96%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.45 / 9.78%</t>
+          <t>$58.44 / 9.76%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.33 / 9.32%</t>
+          <t>$52.32 / 9.30%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.14 / 9.39%</t>
+          <t>$55.12 / 9.35%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.65 / 2.48%</t>
+          <t>$41.66 / 2.50%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.44 / 9.60%</t>
+          <t>$41.45 / 9.63%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.82 / 5.64%</t>
+          <t>$39.82 / 5.66%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2406,42 +2406,42 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.02 / 4.56%</t>
+          <t>$45.00 / 4.53%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.52 / 10.93%</t>
+          <t>$43.55 / 11.03%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.16 / 0.01%</t>
+          <t>$41.11 / -0.09%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.26 / 6.56%</t>
+          <t>$44.27 / 6.60%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.08 / 1.02%</t>
+          <t>$43.01 / 0.88%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.82 / 8.00%</t>
+          <t>$41.81 / 7.99%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.56 / 7.75%</t>
+          <t>$41.55 / 7.74%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$40.98 / 7.91%</t>
+          <t>$40.98 / 7.90%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$745.82 / 5.02%</t>
+          <t>$744.78 / 4.88%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$745.82 / 15.91%</t>
+          <t>$744.78 / 15.75%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$745.82 / 9.58%</t>
+          <t>$744.78 / 9.43%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$745.82 / 8.18%</t>
+          <t>$744.78 / 8.03%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$745.82 / 7.83%</t>
+          <t>$744.78 / 7.68%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$745.82 / 18.84%</t>
+          <t>$744.78 / 18.67%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$745.82 / -0.12%</t>
+          <t>$744.78 / -0.26%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$745.82 / 14.99%</t>
+          <t>$744.78 / 14.83%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$745.82 / 0.90%</t>
+          <t>$744.78 / 0.76%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$745.82 / 13.17%</t>
+          <t>$744.78 / 13.01%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$745.82 / 12.26%</t>
+          <t>$744.78 / 12.10%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$745.82 / 12.37%</t>
+          <t>$744.78 / 12.22%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$745.82 / 5.02%</t>
+          <t>$744.78 / 4.88%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$745.54 / 15.87%</t>
+          <t>$744.78 / 15.75%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$745.54 / 9.54%</t>
+          <t>$744.78 / 9.43%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$745.82 / 8.18%</t>
+          <t>$744.78 / 8.03%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$745.82 / 7.83%</t>
+          <t>$744.78 / 7.68%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$745.54 / 18.80%</t>
+          <t>$744.78 / 18.67%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$745.82 / -0.12%</t>
+          <t>$744.78 / -0.26%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$745.82 / 14.99%</t>
+          <t>$744.78 / 14.83%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$745.82 / 0.90%</t>
+          <t>$744.78 / 0.76%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$745.54 / 13.13%</t>
+          <t>$744.78 / 13.01%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$745.54 / 12.21%</t>
+          <t>$744.78 / 12.10%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$745.54 / 12.33%</t>
+          <t>$744.78 / 12.22%</t>
         </is>
       </c>
     </row>
@@ -2580,77 +2580,77 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.48% (10.83%)</t>
+          <t>11.55% (10.90%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.84% (1.74%)</t>
+          <t>1.85% (1.75%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.07% (6.70%)</t>
+          <t>7.10% (6.74%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.89% (8.38%)</t>
+          <t>8.91% (8.40%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.17% (7.74%)</t>
+          <t>8.26% (7.83%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.37% (0.34%)</t>
+          <t>0.34% (0.31%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.37% (15.56%)</t>
+          <t>16.54% (15.72%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.99% (7.43%)</t>
+          <t>8.01% (7.45%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.76% (15.01%)</t>
+          <t>15.87% (15.12%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.76% (5.46%)</t>
+          <t>5.78% (5.48%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.73% (4.50%)</t>
+          <t>4.75% (4.52%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.61% (3.44%)</t>
+          <t>3.65% (3.48%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.45% (8.80%)</t>
+          <t>9.43% (8.78%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.41% (1.31%)</t>
+          <t>1.39% (1.28%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.67% (5.29%)</t>
+          <t>5.65% (5.28%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2660,37 +2660,37 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.56% (6.12%)</t>
+          <t>6.59% (6.15%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.27% (0.24%)</t>
+          <t>0.18% (0.15%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.30% (12.49%)</t>
+          <t>13.43% (12.61%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.85% (6.28%)</t>
+          <t>6.81% (6.24%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.57% (11.83%)</t>
+          <t>12.73% (11.98%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.38% (4.07%)</t>
+          <t>4.39% (4.09%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.52% (3.29%)</t>
+          <t>3.53% (3.30%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.40%</t>
+          <t>-1.26%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.86%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>6.46%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>6.36%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-3.61%</t>
+          <t>-3.48%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.59%</t>
+          <t>16.76%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>16.21%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>3.19%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.67%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.59%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.43%</t>
+          <t>-3.33%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>2.42%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-5.59%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>13.65%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.64%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.98%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.21%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.76%</t>
+          <t>-0.65%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.09% (10.44%)</t>
+          <t>11.03% (10.38%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.38% (11.27%)</t>
+          <t>11.28% (11.18%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.12% (10.75%)</t>
+          <t>11.04% (10.67%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.45% (10.93%)</t>
+          <t>11.35% (10.84%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.94% (10.50%)</t>
+          <t>10.90% (10.46%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.80% (11.77%)</t>
+          <t>11.67% (11.64%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.82% (9.00%)</t>
+          <t>9.83% (9.02%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.87% (13.31%)</t>
+          <t>13.78% (13.22%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.65% (8.90%)</t>
+          <t>9.62% (8.87%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.09% (10.79%)</t>
+          <t>11.00% (10.70%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.75% (10.53%)</t>
+          <t>10.66% (10.43%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.72% (10.55%)</t>
+          <t>10.64% (10.48%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.48% (15.82%)</t>
+          <t>16.34% (15.69%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.20% (17.09%)</t>
+          <t>17.10% (17.00%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.63% (16.26%)</t>
+          <t>16.54% (16.17%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.04% (16.52%)</t>
+          <t>16.94% (16.42%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.44% (16.00%)</t>
+          <t>16.35% (15.91%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>17.86% (17.83%)</t>
+          <t>17.71% (17.68%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.85% (14.03%)</t>
+          <t>14.84% (14.02%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.70% (19.13%)</t>
+          <t>19.56% (18.99%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.64% (13.89%)</t>
+          <t>14.66% (13.91%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.97% (16.67%)</t>
+          <t>16.91% (16.60%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.50% (16.27%)</t>
+          <t>16.43% (16.20%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.38% (16.22%)</t>
+          <t>16.31% (16.14%)</t>
         </is>
       </c>
     </row>
@@ -2961,117 +2961,117 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.22% (-3.87%)</t>
+          <t>-3.16% (-3.81%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-10.98% (-11.08%)</t>
+          <t>-10.97% (-11.07%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.75% (-7.12%)</t>
+          <t>-6.72% (-7.09%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.36% (-5.87%)</t>
+          <t>-5.34% (-5.85%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.60% (-6.03%)</t>
+          <t>-5.52% (-5.96%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.47% (-12.50%)</t>
+          <t>-12.49% (-12.53%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.07% (-0.89%)</t>
+          <t>0.00% (-0.75%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.87% (-8.43%)</t>
+          <t>-7.85% (-8.41%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.15% (-1.90%)</t>
+          <t>-1.06% (-1.81%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.38% (-9.68%)</t>
+          <t>-9.36% (-9.66%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.07% (-9.30%)</t>
+          <t>-9.06% (-9.28%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.19% (-9.36%)</t>
+          <t>-9.16% (-9.32%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.59% (-3.24%)</t>
+          <t>-2.61% (-3.26%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.44% (-9.54%)</t>
+          <t>-9.46% (-9.57%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.77% (-6.14%)</t>
+          <t>-5.78% (-6.16%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.38% (-4.90%)</t>
+          <t>-4.38% (-4.89%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.73% (-5.17%)</t>
+          <t>-4.71% (-5.15%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.58% (-10.62%)</t>
+          <t>-10.66% (-10.69%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.04% (-0.86%)</t>
+          <t>0.00% (-0.75%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.38% (-6.95%)</t>
+          <t>-6.42% (-6.99%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.12% (-1.86%)</t>
+          <t>-0.98% (-1.73%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.89% (-8.19%)</t>
+          <t>-7.88% (-8.18%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.75% (-7.98%)</t>
+          <t>-7.74% (-7.97%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.30%</t>
+          <t>-14.19%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.35%</t>
+          <t>-22.25%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.87%</t>
+          <t>-17.76%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.80%</t>
+          <t>-16.69%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.54%</t>
+          <t>-16.42%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.27%</t>
+          <t>-24.16%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.89%</t>
+          <t>-9.76%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.74%</t>
+          <t>-21.63%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.80%</t>
+          <t>-10.68%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.47%</t>
+          <t>-20.36%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.83%</t>
+          <t>-19.71%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-19.91%</t>
+          <t>-19.80%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.06%</t>
+          <t>-18.95%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.64%</t>
+          <t>-26.56%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.40%</t>
+          <t>-22.32%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-21.42%</t>
+          <t>-21.31%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.17%</t>
+          <t>-21.06%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-28.45%</t>
+          <t>-28.37%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.89%</t>
+          <t>-14.77%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.08%</t>
+          <t>-25.98%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.76%</t>
+          <t>-15.64%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.86%</t>
+          <t>-24.78%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
+          <t>-24.17%</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
           <t>-24.25%</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>-24.33%</t>
         </is>
       </c>
     </row>
@@ -3215,102 +3215,102 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.65% (1.00%)</t>
+          <t>1.58% (0.92%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.84% (1.74%)</t>
+          <t>1.85% (1.75%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.23% (1.86%)</t>
+          <t>2.12% (1.75%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.41% (1.89%)</t>
+          <t>2.28% (1.77%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.82% (1.39%)</t>
+          <t>1.76% (1.33%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.37% (0.34%)</t>
+          <t>0.34% (0.31%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.07% (-0.89%)</t>
+          <t>0.07% (-0.75%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.98% (5.42%)</t>
+          <t>5.85% (5.29%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.27% (-1.01%)</t>
+          <t>-0.31% (-1.05%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.62% (2.32%)</t>
+          <t>2.49% (2.19%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.14% (1.91%)</t>
+          <t>2.01% (1.79%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.12% (1.95%)</t>
+          <t>2.02% (1.85%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.31% (1.66%)</t>
+          <t>2.15% (1.50%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.41% (1.31%)</t>
+          <t>1.39% (1.28%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.26% (2.89%)</t>
+          <t>3.14% (2.77%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.46% (2.94%)</t>
+          <t>3.32% (2.80%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.75% (2.31%)</t>
+          <t>2.64% (2.20%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.27% (0.24%)</t>
+          <t>0.18% (0.15%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.04% (-0.86%)</t>
+          <t>0.06% (-0.75%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.85% (6.28%)</t>
+          <t>6.81% (6.24%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -3320,12 +3320,12 @@
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>4.26% (3.96%)</t>
+          <t>4.17% (3.87%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.52% (3.29%)</t>
+          <t>3.49% (3.26%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.50%</t>
+          <t>10.46%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.74%</t>
+          <t>7.83%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.52%</t>
+          <t>5.43%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.83%</t>
+          <t>7.68%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>6.36%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.03%</t>
+          <t>-5.96%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>10.84%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.38%</t>
+          <t>8.40%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.34%</t>
+          <t>5.32%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.18%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>6.46%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.87%</t>
+          <t>-5.85%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.31%</t>
+          <t>13.22%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.43%</t>
+          <t>7.45%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.28%</t>
+          <t>8.26%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.99%</t>
+          <t>14.83%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.43%</t>
+          <t>-8.41%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.44%</t>
+          <t>10.38%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.83%</t>
+          <t>10.90%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.14%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.02%</t>
+          <t>4.88%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.87%</t>
+          <t>-3.81%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.90%</t>
+          <t>8.87%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.01%</t>
+          <t>15.12%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>16.21%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.90%</t>
+          <t>-1.81%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>9.02%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.56%</t>
+          <t>15.72%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.10%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>-0.26%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.59%</t>
+          <t>16.76%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-0.75%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.77%</t>
+          <t>11.64%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.32%</t>
+          <t>13.35%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.84%</t>
+          <t>18.67%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-3.61%</t>
+          <t>-3.48%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.50%</t>
+          <t>-12.53%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.27%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.74%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.49%</t>
+          <t>11.48%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.91%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.40%</t>
+          <t>-1.26%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.08%</t>
+          <t>-11.07%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.55%</t>
+          <t>10.48%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.44%</t>
+          <t>3.48%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.39%</t>
+          <t>9.35%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>12.22%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.59%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.36%</t>
+          <t>-9.32%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.53%</t>
+          <t>10.43%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>4.52%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.32%</t>
+          <t>9.30%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.26%</t>
+          <t>12.10%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.67%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.30%</t>
+          <t>-9.28%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.79%</t>
+          <t>10.70%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.46%</t>
+          <t>5.48%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>9.76%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>13.01%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>3.19%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.68%</t>
+          <t>-9.66%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.75%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.70%</t>
+          <t>6.74%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.75%</t>
+          <t>6.71%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.86%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.12%</t>
+          <t>-7.09%</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.00%</t>
+          <t>15.91%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.12%</t>
+          <t>6.15%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.83%</t>
+          <t>7.68%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.17%</t>
+          <t>-5.15%</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.52%</t>
+          <t>16.42%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3977,17 +3977,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.18%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.90%</t>
+          <t>-4.89%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.13%</t>
+          <t>18.99%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.24%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.56%</t>
+          <t>6.60%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.99%</t>
+          <t>14.83%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.64%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.95%</t>
+          <t>-6.99%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.82%</t>
+          <t>15.69%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>8.78%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.02%</t>
+          <t>4.88%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.24%</t>
+          <t>-3.26%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.89%</t>
+          <t>13.91%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.98%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.02%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.98%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.86%</t>
+          <t>-1.73%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.03%</t>
+          <t>14.02%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>12.61%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.01%</t>
+          <t>-0.09%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>-0.26%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>13.65%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.86%</t>
+          <t>-0.75%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17.83%</t>
+          <t>17.68%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.15%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>11.03%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.80%</t>
+          <t>18.67%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-5.59%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.62%</t>
+          <t>-10.69%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>17.00%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.31%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.60%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.43%</t>
+          <t>-3.33%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.54%</t>
+          <t>-9.57%</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.22%</t>
+          <t>16.14%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4231,17 +4231,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.91%</t>
+          <t>7.90%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>12.22%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.76%</t>
+          <t>-0.65%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>16.20%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>3.30%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.75%</t>
+          <t>7.74%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.21%</t>
+          <t>12.10%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.98%</t>
+          <t>-7.97%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>16.60%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.07%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.00%</t>
+          <t>7.99%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.01%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.21%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.19%</t>
+          <t>-8.18%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.26%</t>
+          <t>16.17%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.29%</t>
+          <t>5.28%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.64%</t>
+          <t>5.66%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>2.42%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.14%</t>
+          <t>-6.16%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-06]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:31 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:31 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/2/2026)</t>
+          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>288 days</t>
+          <t>284 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>50 days</t>
+          <t>46 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>169 days</t>
+          <t>165 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>232 days</t>
+          <t>228 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>197 days</t>
+          <t>193 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>15 days</t>
+          <t>11 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>350 days</t>
+          <t>346 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>260 days</t>
+          <t>256 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>323 days</t>
+          <t>319 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>141 days</t>
+          <t>137 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>106 days</t>
+          <t>102 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>78 days</t>
+          <t>74 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>288 days</t>
+          <t>284 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>50 days</t>
+          <t>46 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>169 days</t>
+          <t>165 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>232 days</t>
+          <t>228 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>197 days</t>
+          <t>193 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>15 days</t>
+          <t>11 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>350 days</t>
+          <t>346 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>260 days</t>
+          <t>256 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>323 days</t>
+          <t>319 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>141 days</t>
+          <t>137 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>106 days</t>
+          <t>102 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>78 days</t>
+          <t>74 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.66 / 3.08%</t>
+          <t>$46.88 / 3.55%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.50 / 11.48%</t>
+          <t>$56.66 / 11.79%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.43 / 6.71%</t>
+          <t>$54.64 / 7.11%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$60.99 / 5.32%</t>
+          <t>$61.21 / 5.69%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.11 / 5.43%</t>
+          <t>$55.33 / 5.85%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.62 / 13.35%</t>
+          <t>$59.72 / 13.53%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.81 / -0.10%</t>
+          <t>$60.13 / 0.43%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.30 / 8.26%</t>
+          <t>$52.44 / 8.54%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.10 / 0.96%</t>
+          <t>$56.39 / 1.48%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.44 / 9.76%</t>
+          <t>$58.66 / 10.17%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.32 / 9.30%</t>
+          <t>$52.52 / 9.72%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.12 / 9.35%</t>
+          <t>$55.33 / 9.76%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.66 / 2.50%</t>
+          <t>$41.78 / 2.80%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.45 / 9.63%</t>
+          <t>$41.54 / 9.85%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.82 / 5.66%</t>
+          <t>$39.92 / 5.92%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.02 / 4.26%</t>
+          <t>$44.13 / 4.52%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.00 / 4.53%</t>
+          <t>$45.14 / 4.84%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.55 / 11.03%</t>
+          <t>$43.56 / 11.05%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.11 / -0.09%</t>
+          <t>$41.29 / 0.33%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.27 / 6.60%</t>
+          <t>$44.34 / 6.75%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.01 / 0.88%</t>
+          <t>$43.21 / 1.34%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.81 / 7.99%</t>
+          <t>$41.91 / 8.22%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.55 / 7.74%</t>
+          <t>$41.66 / 8.02%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$40.98 / 7.90%</t>
+          <t>$41.08 / 8.17%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$744.78 / 4.88%</t>
+          <t>$750.65 / 5.70%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$744.78 / 15.75%</t>
+          <t>$750.65 / 16.66%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$744.78 / 9.43%</t>
+          <t>$750.65 / 10.29%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$744.78 / 8.03%</t>
+          <t>$750.51 / 8.86%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$744.78 / 7.68%</t>
+          <t>$750.51 / 8.51%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$744.78 / 18.67%</t>
+          <t>$750.65 / 19.61%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$744.78 / -0.26%</t>
+          <t>$750.65 / 0.52%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$744.78 / 14.83%</t>
+          <t>$750.65 / 15.74%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$744.78 / 0.76%</t>
+          <t>$750.65 / 1.55%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$744.78 / 13.01%</t>
+          <t>$750.65 / 13.90%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$744.78 / 12.10%</t>
+          <t>$750.65 / 12.98%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$744.78 / 12.22%</t>
+          <t>$750.65 / 13.10%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$744.78 / 4.88%</t>
+          <t>$750.65 / 5.70%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$744.78 / 15.75%</t>
+          <t>$750.65 / 16.66%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$744.78 / 9.43%</t>
+          <t>$750.65 / 10.29%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$744.78 / 8.03%</t>
+          <t>$750.65 / 8.88%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$744.78 / 7.68%</t>
+          <t>$750.65 / 8.53%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$744.78 / 18.67%</t>
+          <t>$750.65 / 19.61%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$744.78 / -0.26%</t>
+          <t>$750.65 / 0.52%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$744.78 / 14.83%</t>
+          <t>$750.65 / 15.74%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$744.78 / 0.76%</t>
+          <t>$750.65 / 1.55%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$744.78 / 13.01%</t>
+          <t>$750.65 / 13.90%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$744.78 / 12.10%</t>
+          <t>$750.65 / 12.98%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$744.78 / 12.22%</t>
+          <t>$750.65 / 13.10%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.55% (10.90%)</t>
+          <t>11.03% (10.39%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.85% (1.75%)</t>
+          <t>1.56% (1.47%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.10% (6.74%)</t>
+          <t>6.70% (6.34%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.91% (8.40%)</t>
+          <t>8.52% (8.01%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.26% (7.83%)</t>
+          <t>7.82% (7.40%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.34% (0.31%)</t>
+          <t>0.18% (0.15%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.54% (15.72%)</t>
+          <t>15.91% (15.11%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.01% (7.45%)</t>
+          <t>7.72% (7.17%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.87% (15.12%)</t>
+          <t>15.26% (14.53%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.78% (5.48%)</t>
+          <t>5.37% (5.08%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.75% (4.52%)</t>
+          <t>4.34% (4.13%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.65% (3.48%)</t>
+          <t>3.24% (3.09%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.43% (8.78%)</t>
+          <t>9.11% (8.46%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.39% (1.28%)</t>
+          <t>1.17% (1.07%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.65% (5.28%)</t>
+          <t>5.38% (5.02%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.18% (6.66%)</t>
+          <t>6.90% (6.39%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.59% (6.15%)</t>
+          <t>6.27% (5.84%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.18% (0.15%)</t>
+          <t>0.16% (0.13%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.43% (12.61%)</t>
+          <t>12.94% (12.13%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.81% (6.24%)</t>
+          <t>6.65% (6.09%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.73% (11.98%)</t>
+          <t>12.21% (11.48%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.39% (4.09%)</t>
+          <t>4.16% (3.86%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.53% (3.30%)</t>
+          <t>3.25% (3.03%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.70% (2.53%)</t>
+          <t>2.44% (2.28%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-2.03%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.86%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.46%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.36%</t>
+          <t>5.55%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-3.48%</t>
+          <t>-4.23%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.76%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.21%</t>
+          <t>15.30%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.19%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.67%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.59%</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.33%</t>
+          <t>-4.09%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.42%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>3.03%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-5.59%</t>
+          <t>-6.33%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.65%</t>
+          <t>12.76%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.64%</t>
+          <t>-1.41%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.98%</t>
+          <t>12.09%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.74%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.65%</t>
+          <t>-1.43%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.03% (10.38%)</t>
+          <t>11.25% (10.61%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.28% (11.18%)</t>
+          <t>11.63% (11.54%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.04% (10.67%)</t>
+          <t>11.33% (10.97%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.35% (10.84%)</t>
+          <t>11.64% (11.14%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.90% (10.46%)</t>
+          <t>11.15% (10.73%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.67% (11.64%)</t>
+          <t>12.12% (12.09%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.83% (9.02%)</t>
+          <t>10.00% (9.19%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.78% (13.22%)</t>
+          <t>14.14% (13.59%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.62% (8.87%)</t>
+          <t>9.80% (9.07%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.00% (10.70%)</t>
+          <t>11.27% (10.98%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.66% (10.43%)</t>
+          <t>10.93% (10.71%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.64% (10.48%)</t>
+          <t>10.91% (10.76%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.34% (15.69%)</t>
+          <t>16.69% (16.04%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.10% (17.00%)</t>
+          <t>17.48% (17.39%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.54% (16.17%)</t>
+          <t>16.90% (16.54%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.94% (16.42%)</t>
+          <t>17.30% (16.79%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.35% (15.91%)</t>
+          <t>16.68% (16.25%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>17.71% (17.68%)</t>
+          <t>18.25% (18.23%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.84% (14.02%)</t>
+          <t>15.07% (14.27%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.56% (18.99%)</t>
+          <t>20.00% (19.44%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.66% (13.91%)</t>
+          <t>14.86% (14.13%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.91% (16.60%)</t>
+          <t>17.29% (16.99%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.43% (16.20%)</t>
+          <t>16.78% (16.56%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.31% (16.14%)</t>
+          <t>16.67% (16.51%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.16% (-3.81%)</t>
+          <t>-3.61% (-4.25%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-10.97% (-11.07%)</t>
+          <t>-11.22% (-11.32%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.72% (-7.09%)</t>
+          <t>-7.07% (-7.43%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.34% (-5.85%)</t>
+          <t>-5.68% (-6.19%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.52% (-5.96%)</t>
+          <t>-5.90% (-6.33%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.49% (-12.53%)</t>
+          <t>-12.64% (-12.66%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.75%)</t>
+          <t>-0.47% (-1.27%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.85% (-8.41%)</t>
+          <t>-8.10% (-8.65%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.06% (-1.81%)</t>
+          <t>-1.58% (-2.31%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.36% (-9.66%)</t>
+          <t>-9.71% (-10.00%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.06% (-9.28%)</t>
+          <t>-9.41% (-9.63%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.16% (-9.32%)</t>
+          <t>-9.51% (-9.67%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.61% (-3.26%)</t>
+          <t>-2.90% (-3.54%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.46% (-9.57%)</t>
+          <t>-9.65% (-9.75%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.78% (-6.16%)</t>
+          <t>-6.03% (-6.39%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.38% (-4.89%)</t>
+          <t>-4.63% (-5.14%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.71% (-5.15%)</t>
+          <t>-5.00% (-5.42%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.66% (-10.69%)</t>
+          <t>-10.68% (-10.71%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.75%)</t>
+          <t>-0.37% (-1.17%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.42% (-6.99%)</t>
+          <t>-6.56% (-7.12%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-0.98% (-1.73%)</t>
+          <t>-1.44% (-2.17%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.88% (-8.18%)</t>
+          <t>-8.08% (-8.38%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.74% (-7.97%)</t>
+          <t>-7.99% (-8.21%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-7.94% (-8.11%)</t>
+          <t>-8.18% (-8.34%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.19%</t>
+          <t>-14.86%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.25%</t>
+          <t>-22.85%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.76%</t>
+          <t>-18.40%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.69%</t>
+          <t>-17.32%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.42%</t>
+          <t>-17.06%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.16%</t>
+          <t>-24.76%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.76%</t>
+          <t>-10.47%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.63%</t>
+          <t>-22.24%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.68%</t>
+          <t>-11.38%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.36%</t>
+          <t>-20.98%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.71%</t>
+          <t>-20.34%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-19.80%</t>
+          <t>-20.42%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-18.95%</t>
+          <t>-19.58%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
+          <t>-27.14%</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-22.93%</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-21.93%</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-21.68%</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>-28.93%</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>-15.44%</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
           <t>-26.56%</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>-22.32%</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>-21.31%</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>-21.06%</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>-28.37%</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>-14.77%</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>-25.98%</t>
-        </is>
-      </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.64%</t>
+          <t>-16.30%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.78%</t>
+          <t>-25.37%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.17%</t>
+          <t>-24.77%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.25%</t>
+          <t>-24.84%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.58% (0.92%)</t>
+          <t>1.90% (1.26%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.85% (1.75%)</t>
+          <t>1.56% (1.47%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.12% (1.75%)</t>
+          <t>2.54% (2.18%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.28% (1.77%)</t>
+          <t>2.70% (2.20%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.76% (1.33%)</t>
+          <t>2.13% (1.71%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.34% (0.31%)</t>
+          <t>0.18% (0.15%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.07% (-0.75%)</t>
+          <t>0.05% (-0.75%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.85% (5.29%)</t>
+          <t>6.40% (5.85%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.31% (-1.05%)</t>
+          <t>-0.05% (-0.78%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.49% (2.19%)</t>
+          <t>2.91% (2.62%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.01% (1.79%)</t>
+          <t>2.42% (2.21%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.02% (1.85%)</t>
+          <t>2.42% (2.27%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.15% (1.50%)</t>
+          <t>2.65% (2.00%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.39% (1.28%)</t>
+          <t>1.17% (1.07%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.14% (2.77%)</t>
+          <t>3.69% (3.33%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.32% (2.80%)</t>
+          <t>3.87% (3.36%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.64% (2.20%)</t>
+          <t>3.14% (2.71%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.18% (0.15%)</t>
+          <t>0.16% (0.13%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.06% (-0.75%)</t>
+          <t>0.15% (-0.65%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.81% (6.24%)</t>
+          <t>6.65% (6.09%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.23% (-0.98%)</t>
+          <t>0.09% (-0.64%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>4.17% (3.87%)</t>
+          <t>4.16% (3.86%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.49% (3.26%)</t>
+          <t>3.25% (3.03%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.70% (2.53%)</t>
+          <t>2.44% (2.28%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 2/7/2026</t>
+          <t>As of 6/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.46%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.83%</t>
+          <t>7.40%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.43%</t>
+          <t>5.85%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.68%</t>
+          <t>8.51%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.36%</t>
+          <t>5.55%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.96%</t>
+          <t>-6.33%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.84%</t>
+          <t>11.14%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.40%</t>
+          <t>8.01%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.32%</t>
+          <t>5.69%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>8.86%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.46%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.85%</t>
+          <t>-6.19%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.22%</t>
+          <t>13.59%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.45%</t>
+          <t>7.17%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.26%</t>
+          <t>8.54%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.83%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.41%</t>
+          <t>-8.65%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.38%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.90%</t>
+          <t>10.39%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>3.55%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.88%</t>
+          <t>5.70%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-4.25%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.87%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.12%</t>
+          <t>14.53%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.48%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>1.55%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.21%</t>
+          <t>15.30%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.81%</t>
+          <t>-2.31%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.02%</t>
+          <t>9.19%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.72%</t>
+          <t>15.11%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.10%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.26%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.76%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-1.27%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.64%</t>
+          <t>12.09%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>0.15%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.35%</t>
+          <t>13.53%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.67%</t>
+          <t>19.61%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-3.48%</t>
+          <t>-4.23%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.53%</t>
+          <t>-12.66%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>11.54%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>1.47%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.48%</t>
+          <t>11.79%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>16.66%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-2.03%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.07%</t>
+          <t>-11.32%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.48%</t>
+          <t>10.76%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.48%</t>
+          <t>3.09%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.35%</t>
+          <t>9.76%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.22%</t>
+          <t>13.10%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.59%</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.32%</t>
+          <t>-9.67%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.43%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>4.13%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.30%</t>
+          <t>9.72%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.10%</t>
+          <t>12.98%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.67%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.28%</t>
+          <t>-9.63%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.70%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.48%</t>
+          <t>5.08%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.76%</t>
+          <t>10.17%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.01%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.19%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.66%</t>
+          <t>-10.00%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.97%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.74%</t>
+          <t>6.34%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.71%</t>
+          <t>7.11%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.43%</t>
+          <t>10.29%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.86%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.09%</t>
+          <t>-7.43%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 2/7/2026</t>
+          <t>As of 6/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.91%</t>
+          <t>16.25%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.15%</t>
+          <t>5.84%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.68%</t>
+          <t>8.53%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>3.03%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.15%</t>
+          <t>-5.42%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.42%</t>
+          <t>16.79%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.66%</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.26%</t>
+          <t>4.52%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.89%</t>
+          <t>-5.14%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.99%</t>
+          <t>19.44%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>6.09%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.60%</t>
+          <t>6.75%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.83%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.64%</t>
+          <t>-1.41%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.99%</t>
+          <t>-7.12%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.69%</t>
+          <t>16.04%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.78%</t>
+          <t>8.46%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.88%</t>
+          <t>5.70%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.26%</t>
+          <t>-3.54%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.91%</t>
+          <t>14.13%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.98%</t>
+          <t>11.48%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>1.34%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>1.55%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.98%</t>
+          <t>12.09%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.73%</t>
+          <t>-2.17%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.02%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.61%</t>
+          <t>12.13%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.26%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.65%</t>
+          <t>12.76%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-1.17%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17.68%</t>
+          <t>18.23%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.15%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.03%</t>
+          <t>11.05%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.67%</t>
+          <t>19.61%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-5.59%</t>
+          <t>-6.33%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.69%</t>
+          <t>-10.71%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.00%</t>
+          <t>17.39%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>1.07%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.85%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>16.66%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.33%</t>
+          <t>-4.09%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.57%</t>
+          <t>-9.75%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.14%</t>
+          <t>16.51%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.28%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.90%</t>
+          <t>8.17%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.22%</t>
+          <t>13.10%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.65%</t>
+          <t>-1.43%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.11%</t>
+          <t>-8.34%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.20%</t>
+          <t>16.56%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.30%</t>
+          <t>3.03%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.74%</t>
+          <t>8.02%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.10%</t>
+          <t>12.98%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.74%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.97%</t>
+          <t>-8.21%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.60%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>3.86%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.99%</t>
+          <t>8.22%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.01%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.18%</t>
+          <t>-8.38%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.17%</t>
+          <t>16.54%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.28%</t>
+          <t>5.02%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.66%</t>
+          <t>5.92%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.43%</t>
+          <t>10.29%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.42%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.16%</t>
+          <t>-6.39%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-07]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:31 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:31 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/6/2026 at 12:32 PM ET)</t>
+          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>284 days</t>
+          <t>283 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>46 days</t>
+          <t>45 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>165 days</t>
+          <t>164 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>228 days</t>
+          <t>227 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>193 days</t>
+          <t>192 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>11 days</t>
+          <t>10 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>346 days</t>
+          <t>345 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>256 days</t>
+          <t>255 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>319 days</t>
+          <t>318 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>137 days</t>
+          <t>136 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>102 days</t>
+          <t>101 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>74 days</t>
+          <t>73 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>284 days</t>
+          <t>283 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>46 days</t>
+          <t>45 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>165 days</t>
+          <t>164 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>228 days</t>
+          <t>227 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>193 days</t>
+          <t>192 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>11 days</t>
+          <t>10 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>346 days</t>
+          <t>345 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>256 days</t>
+          <t>255 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>319 days</t>
+          <t>318 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>137 days</t>
+          <t>136 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>102 days</t>
+          <t>101 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>74 days</t>
+          <t>73 days</t>
         </is>
       </c>
     </row>
@@ -2326,87 +2326,87 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.88 / 3.55%</t>
+          <t>$46.74 / 3.25%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.66 / 11.79%</t>
+          <t>$56.62 / 11.71%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.64 / 7.11%</t>
+          <t>$54.51 / 6.86%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.21 / 5.69%</t>
+          <t>$61.10 / 5.49%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.33 / 5.85%</t>
+          <t>$55.19 / 5.59%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.72 / 13.53%</t>
+          <t>$59.71 / 13.51%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.13 / 0.43%</t>
+          <t>$59.94 / 0.11%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.44 / 8.54%</t>
+          <t>$52.36 / 8.37%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.39 / 1.48%</t>
+          <t>$56.22 / 1.17%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.66 / 10.17%</t>
+          <t>$58.52 / 9.91%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.52 / 9.72%</t>
+          <t>$52.42 / 9.50%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.33 / 9.76%</t>
+          <t>$55.22 / 9.55%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.78 / 2.80%</t>
+          <t>$41.70 / 2.59%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.54 / 9.85%</t>
+          <t>$41.50 / 9.76%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.92 / 5.92%</t>
+          <t>$39.86 / 5.76%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.13 / 4.52%</t>
+          <t>$44.06 / 4.35%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.14 / 4.84%</t>
+          <t>$45.07 / 4.68%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2416,32 +2416,32 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.29 / 0.33%</t>
+          <t>$41.18 / 0.08%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.34 / 6.75%</t>
+          <t>$44.29 / 6.65%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.21 / 1.34%</t>
+          <t>$43.08 / 1.03%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.91 / 8.22%</t>
+          <t>$41.85 / 8.08%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.66 / 8.02%</t>
+          <t>$41.60 / 7.85%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.08 / 8.17%</t>
+          <t>$41.04 / 8.05%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$750.65 / 5.70%</t>
+          <t>$747.34 / 5.24%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$750.65 / 16.66%</t>
+          <t>$747.34 / 16.15%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$750.65 / 10.29%</t>
+          <t>$747.34 / 9.81%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$750.51 / 8.86%</t>
+          <t>$747.34 / 8.40%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$750.51 / 8.51%</t>
+          <t>$747.34 / 8.05%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$750.65 / 19.61%</t>
+          <t>$747.34 / 19.08%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$750.65 / 0.52%</t>
+          <t>$747.34 / 0.08%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$750.65 / 15.74%</t>
+          <t>$747.34 / 15.23%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$750.65 / 1.55%</t>
+          <t>$747.34 / 1.11%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$750.65 / 13.90%</t>
+          <t>$747.34 / 13.40%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$750.65 / 12.98%</t>
+          <t>$747.34 / 12.49%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$750.65 / 13.10%</t>
+          <t>$747.34 / 12.60%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$750.65 / 5.70%</t>
+          <t>$747.34 / 5.24%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$750.65 / 16.66%</t>
+          <t>$747.34 / 16.15%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$750.65 / 10.29%</t>
+          <t>$747.34 / 9.81%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$750.65 / 8.88%</t>
+          <t>$747.34 / 8.40%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$750.65 / 8.53%</t>
+          <t>$747.34 / 8.05%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$750.65 / 19.61%</t>
+          <t>$747.34 / 19.08%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$750.65 / 0.52%</t>
+          <t>$747.34 / 0.08%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$750.65 / 15.74%</t>
+          <t>$747.34 / 15.23%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$750.65 / 1.55%</t>
+          <t>$747.34 / 1.11%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$750.65 / 13.90%</t>
+          <t>$747.34 / 13.40%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$750.65 / 12.98%</t>
+          <t>$747.34 / 12.49%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$750.65 / 13.10%</t>
+          <t>$747.34 / 12.60%</t>
         </is>
       </c>
     </row>
@@ -2580,87 +2580,87 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.03% (10.39%)</t>
+          <t>11.35% (10.71%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.56% (1.47%)</t>
+          <t>1.63% (1.54%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.70% (6.34%)</t>
+          <t>6.95% (6.59%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.52% (8.01%)</t>
+          <t>8.72% (8.22%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.82% (7.40%)</t>
+          <t>8.08% (7.66%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.18% (0.15%)</t>
+          <t>0.19% (0.17%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.91% (15.11%)</t>
+          <t>16.28% (15.48%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.72% (7.17%)</t>
+          <t>7.88% (7.34%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.26% (14.53%)</t>
+          <t>15.61% (14.88%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.37% (5.08%)</t>
+          <t>5.62% (5.34%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.34% (4.13%)</t>
+          <t>4.55% (4.33%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.24% (3.09%)</t>
+          <t>3.45% (3.29%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.11% (8.46%)</t>
+          <t>9.33% (8.68%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.17% (1.07%)</t>
+          <t>1.25% (1.16%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.38% (5.02%)</t>
+          <t>5.53% (5.17%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.90% (6.39%)</t>
+          <t>7.08% (6.57%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.27% (5.84%)</t>
+          <t>6.43% (6.00%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2670,32 +2670,32 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.94% (12.13%)</t>
+          <t>13.22% (12.42%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.65% (6.09%)</t>
+          <t>6.75% (6.20%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.21% (11.48%)</t>
+          <t>12.55% (11.81%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.16% (3.86%)</t>
+          <t>4.29% (4.00%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.25% (3.03%)</t>
+          <t>3.41% (3.19%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.44% (2.28%)</t>
+          <t>2.55% (2.39%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.95%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-2.03%</t>
+          <t>-1.60%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.04%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>6.10%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.55%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-4.23%</t>
+          <t>-3.81%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>15.84%</t>
+          <t>16.36%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>1.68%</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>15.81%</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2.84%</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2.32%</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
           <t>1.24%</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>15.30%</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>2.39%</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>1.87%</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>0.80%</t>
-        </is>
-      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.75%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-4.09%</t>
+          <t>-3.66%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.62%</t>
+          <t>2.07%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>3.37%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.03%</t>
+          <t>3.48%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-6.33%</t>
+          <t>-5.91%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>13.26%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.41%</t>
+          <t>-0.98%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.09%</t>
+          <t>12.59%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-0.13%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.74%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>-0.99%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.25% (10.61%)</t>
+          <t>11.15% (10.51%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.63% (11.54%)</t>
+          <t>11.35% (11.26%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.33% (10.97%)</t>
+          <t>11.19% (10.83%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.64% (11.14%)</t>
+          <t>11.46% (10.96%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.15% (10.73%)</t>
+          <t>11.03% (10.61%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.12% (12.09%)</t>
+          <t>11.80% (11.77%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.00% (9.19%)</t>
+          <t>9.92% (9.12%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.14% (13.59%)</t>
+          <t>13.94% (13.39%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.80% (9.07%)</t>
+          <t>9.70% (8.97%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.27% (10.98%)</t>
+          <t>11.14% (10.85%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.93% (10.71%)</t>
+          <t>10.76% (10.54%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.91% (10.76%)</t>
+          <t>10.74% (10.58%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.69% (16.04%)</t>
+          <t>16.52% (15.88%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.48% (17.39%)</t>
+          <t>17.24% (17.14%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.90% (16.54%)</t>
+          <t>16.70% (16.34%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.30% (16.79%)</t>
+          <t>17.12% (16.61%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.68% (16.25%)</t>
+          <t>16.48% (16.05%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>18.25% (18.23%)</t>
+          <t>17.93% (17.91%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.07% (14.27%)</t>
+          <t>14.95% (14.15%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.00% (19.44%)</t>
+          <t>19.76% (19.21%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.86% (14.13%)</t>
+          <t>14.78% (14.05%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.29% (16.99%)</t>
+          <t>17.07% (16.78%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.78% (16.56%)</t>
+          <t>16.58% (16.37%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.67% (16.51%)</t>
+          <t>16.43% (16.28%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.61% (-4.25%)</t>
+          <t>-3.33% (-3.97%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.22% (-11.32%)</t>
+          <t>-11.16% (-11.25%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.07% (-7.43%)</t>
+          <t>-6.85% (-7.21%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.68% (-6.19%)</t>
+          <t>-5.51% (-6.01%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.90% (-6.33%)</t>
+          <t>-5.68% (-6.10%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.64% (-12.66%)</t>
+          <t>-12.63% (-12.65%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.47% (-1.27%)</t>
+          <t>-0.15% (-0.95%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.10% (-8.65%)</t>
+          <t>-7.96% (-8.51%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.58% (-2.31%)</t>
+          <t>-1.28% (-2.01%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.71% (-10.00%)</t>
+          <t>-9.50% (-9.79%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.41% (-9.63%)</t>
+          <t>-9.23% (-9.45%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.51% (-9.67%)</t>
+          <t>-9.33% (-9.49%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.90% (-3.54%)</t>
+          <t>-2.70% (-3.35%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.65% (-9.75%)</t>
+          <t>-9.58% (-9.67%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.03% (-6.39%)</t>
+          <t>-5.89% (-6.25%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.63% (-5.14%)</t>
+          <t>-4.47% (-4.97%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.00% (-5.42%)</t>
+          <t>-4.85% (-5.28%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.68% (-10.71%)</t>
+          <t>-10.69% (-10.71%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.37% (-1.17%)</t>
+          <t>-0.12% (-0.92%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.56% (-7.12%)</t>
+          <t>-6.47% (-7.02%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.44% (-2.17%)</t>
+          <t>-1.14% (-1.88%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.08% (-8.38%)</t>
+          <t>-7.97% (-8.26%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.99% (-8.21%)</t>
+          <t>-7.85% (-8.07%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.18% (-8.34%)</t>
+          <t>-8.08% (-8.23%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.86%</t>
+          <t>-14.48%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.85%</t>
+          <t>-22.51%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.40%</t>
+          <t>-18.04%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.32%</t>
+          <t>-16.97%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-17.06%</t>
+          <t>-16.71%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.76%</t>
+          <t>-24.42%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.47%</t>
+          <t>-10.07%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.24%</t>
+          <t>-21.89%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.38%</t>
+          <t>-10.98%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.98%</t>
+          <t>-20.63%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.34%</t>
+          <t>-19.99%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.42%</t>
+          <t>-20.07%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.58%</t>
+          <t>-19.23%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-27.14%</t>
+          <t>-26.82%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.93%</t>
+          <t>-22.59%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-21.93%</t>
+          <t>-21.58%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.68%</t>
+          <t>-21.33%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-28.93%</t>
+          <t>-28.62%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.44%</t>
+          <t>-15.07%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.56%</t>
+          <t>-26.23%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.30%</t>
+          <t>-15.93%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.37%</t>
+          <t>-25.04%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.77%</t>
+          <t>-24.43%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.84%</t>
+          <t>-24.51%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.90% (1.26%)</t>
+          <t>1.74% (1.10%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.56% (1.47%)</t>
+          <t>1.63% (1.54%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.54% (2.18%)</t>
+          <t>2.33% (1.97%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.70% (2.20%)</t>
+          <t>2.45% (1.95%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.13% (1.71%)</t>
+          <t>1.95% (1.52%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.18% (0.15%)</t>
+          <t>0.19% (0.17%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.05% (-0.75%)</t>
+          <t>-0.07% (-0.87%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.40% (5.85%)</t>
+          <t>6.09% (5.54%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
+          <t>-0.19% (-0.92%)</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2.69% (2.41%)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2.17% (1.96%)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2.17% (2.02%)</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2.40% (1.76%)</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>1.25% (1.16%)</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>3.38% (3.02%)</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>3.58% (3.07%)</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>2.84% (2.41%)</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>0.16% (0.13%)</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>-0.04% (-0.84%)</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>6.75% (6.20%)</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
           <t>-0.05% (-0.78%)</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>2.91% (2.62%)</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>2.42% (2.21%)</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>2.42% (2.27%)</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>2.65% (2.00%)</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>1.17% (1.07%)</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>3.69% (3.33%)</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>3.87% (3.36%)</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>3.14% (2.71%)</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>0.16% (0.13%)</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>0.15% (-0.65%)</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>6.65% (6.09%)</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>0.09% (-0.64%)</t>
-        </is>
-      </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>4.16% (3.86%)</t>
+          <t>4.29% (4.00%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.25% (3.03%)</t>
+          <t>3.41% (3.19%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.44% (2.28%)</t>
+          <t>2.55% (2.39%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 6/7/2026</t>
+          <t>As of 7/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.40%</t>
+          <t>7.66%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.85%</t>
+          <t>5.59%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.51%</t>
+          <t>8.05%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.55%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.33%</t>
+          <t>-6.10%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.14%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>8.22%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.69%</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.86%</t>
+          <t>8.40%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>6.10%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.19%</t>
+          <t>-6.01%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.59%</t>
+          <t>13.39%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.17%</t>
+          <t>7.34%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.54%</t>
+          <t>8.37%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>15.23%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>1.68%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.65%</t>
+          <t>-8.51%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.39%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.55%</t>
+          <t>3.25%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.70%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.95%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.25%</t>
+          <t>-3.97%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>8.97%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.53%</t>
+          <t>14.88%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.48%</t>
+          <t>1.17%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.55%</t>
+          <t>1.11%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>15.30%</t>
+          <t>15.81%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.31%</t>
+          <t>-2.01%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.19%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.11%</t>
+          <t>15.48%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.84%</t>
+          <t>16.36%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.27%</t>
+          <t>-0.95%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.09%</t>
+          <t>11.77%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.15%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.53%</t>
+          <t>13.51%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.61%</t>
+          <t>19.08%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.23%</t>
+          <t>-3.81%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.66%</t>
+          <t>-12.65%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>11.26%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.47%</t>
+          <t>1.54%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.79%</t>
+          <t>11.71%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.66%</t>
+          <t>16.15%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.03%</t>
+          <t>-1.60%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.32%</t>
+          <t>-11.25%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.76%</t>
+          <t>10.58%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.09%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.76%</t>
+          <t>9.55%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.10%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.67%</t>
+          <t>-9.49%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.54%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.13%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.72%</t>
+          <t>9.50%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.98%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.63%</t>
+          <t>-9.45%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.08%</t>
+          <t>5.34%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.17%</t>
+          <t>9.91%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>13.40%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.00%</t>
+          <t>-9.79%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.97%</t>
+          <t>10.83%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.34%</t>
+          <t>6.59%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.11%</t>
+          <t>6.86%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.29%</t>
+          <t>9.81%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.04%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.43%</t>
+          <t>-7.21%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 6/7/2026</t>
+          <t>As of 7/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.25%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.84%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.53%</t>
+          <t>8.05%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.03%</t>
+          <t>3.48%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.42%</t>
+          <t>-5.28%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.79%</t>
+          <t>16.61%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.57%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>8.40%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>3.37%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.14%</t>
+          <t>-4.97%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.44%</t>
+          <t>19.21%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.09%</t>
+          <t>6.20%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.75%</t>
+          <t>6.65%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>15.23%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.41%</t>
+          <t>-0.98%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.12%</t>
+          <t>-7.02%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.04%</t>
+          <t>15.88%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.46%</t>
+          <t>8.68%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.80%</t>
+          <t>2.59%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.70%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.75%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.54%</t>
+          <t>-3.35%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>14.05%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.48%</t>
+          <t>11.81%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.55%</t>
+          <t>1.11%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.09%</t>
+          <t>12.59%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.17%</t>
+          <t>-1.88%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.15%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.13%</t>
+          <t>12.42%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>13.26%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>-0.92%</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.23%</t>
+          <t>17.91%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4162,12 +4162,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.61%</t>
+          <t>19.08%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-6.33%</t>
+          <t>-5.91%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.39%</t>
+          <t>17.14%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.85%</t>
+          <t>9.76%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.66%</t>
+          <t>16.15%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.09%</t>
+          <t>-3.66%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.75%</t>
+          <t>-9.67%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.51%</t>
+          <t>16.28%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.28%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.17%</t>
+          <t>8.05%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.10%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>-0.99%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.34%</t>
+          <t>-8.23%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.56%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.03%</t>
+          <t>3.19%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.02%</t>
+          <t>7.85%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.98%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.74%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.21%</t>
+          <t>-8.07%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.78%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.86%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.22%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>13.40%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-0.13%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.38%</t>
+          <t>-8.26%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.54%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.02%</t>
+          <t>5.17%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.92%</t>
+          <t>5.76%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.29%</t>
+          <t>9.81%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.62%</t>
+          <t>2.07%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.39%</t>
+          <t>-6.25%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-08]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/7/2026 at 12:00 PM ET)</t>
+          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>283 days</t>
+          <t>282 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>45 days</t>
+          <t>44 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>164 days</t>
+          <t>163 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>227 days</t>
+          <t>226 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>192 days</t>
+          <t>191 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10 days</t>
+          <t>9 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>345 days</t>
+          <t>344 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>255 days</t>
+          <t>254 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>318 days</t>
+          <t>317 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>136 days</t>
+          <t>135 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>101 days</t>
+          <t>100 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>73 days</t>
+          <t>72 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>283 days</t>
+          <t>282 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>45 days</t>
+          <t>44 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>164 days</t>
+          <t>163 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>227 days</t>
+          <t>226 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>192 days</t>
+          <t>191 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>10 days</t>
+          <t>9 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>345 days</t>
+          <t>344 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>255 days</t>
+          <t>254 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>318 days</t>
+          <t>317 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>136 days</t>
+          <t>135 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>101 days</t>
+          <t>100 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>73 days</t>
+          <t>72 days</t>
         </is>
       </c>
     </row>
@@ -2326,87 +2326,87 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.74 / 3.25%</t>
+          <t>$46.53 / 2.78%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.62 / 11.71%</t>
+          <t>$56.44 / 11.34%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.51 / 6.86%</t>
+          <t>$54.29 / 6.43%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.10 / 5.49%</t>
+          <t>$60.83 / 5.03%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.19 / 5.59%</t>
+          <t>$54.95 / 5.12%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.71 / 13.51%</t>
+          <t>$59.64 / 13.38%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.94 / 0.11%</t>
+          <t>$59.63 / -0.41%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.36 / 8.37%</t>
+          <t>$52.18 / 7.99%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.22 / 1.17%</t>
+          <t>$55.90 / 0.61%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.52 / 9.91%</t>
+          <t>$58.26 / 9.42%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.42 / 9.50%</t>
+          <t>$52.17 / 8.97%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.22 / 9.55%</t>
+          <t>$55.00 / 9.11%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.70 / 2.59%</t>
+          <t>$41.56 / 2.24%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.50 / 9.76%</t>
+          <t>$41.41 / 9.51%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.86 / 5.76%</t>
+          <t>$39.74 / 5.43%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.06 / 4.35%</t>
+          <t>$43.93 / 4.05%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.07 / 4.68%</t>
+          <t>$44.92 / 4.34%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2416,32 +2416,32 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.18 / 0.08%</t>
+          <t>$41.00 / -0.36%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.29 / 6.65%</t>
+          <t>$44.18 / 6.37%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.08 / 1.03%</t>
+          <t>$42.90 / 0.60%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.85 / 8.08%</t>
+          <t>$41.74 / 7.79%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.60 / 7.85%</t>
+          <t>$41.47 / 7.53%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.04 / 8.05%</t>
+          <t>$40.90 / 7.70%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$747.34 / 5.24%</t>
+          <t>$741.11 / 4.36%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$747.34 / 16.15%</t>
+          <t>$741.11 / 15.18%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$747.34 / 9.81%</t>
+          <t>$741.11 / 8.89%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$747.34 / 8.40%</t>
+          <t>$741.11 / 7.50%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$747.34 / 8.05%</t>
+          <t>$741.11 / 7.15%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$747.34 / 19.08%</t>
+          <t>$741.11 / 18.09%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$747.34 / 0.08%</t>
+          <t>$741.11 / -0.75%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$747.34 / 15.23%</t>
+          <t>$741.11 / 14.27%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$747.34 / 1.11%</t>
+          <t>$741.11 / 0.26%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$747.34 / 13.40%</t>
+          <t>$741.11 / 12.45%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$747.34 / 12.49%</t>
+          <t>$741.11 / 11.55%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$747.34 / 12.60%</t>
+          <t>$741.11 / 11.66%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$747.34 / 5.24%</t>
+          <t>$741.11 / 4.36%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$747.34 / 16.15%</t>
+          <t>$741.11 / 15.18%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$747.34 / 9.81%</t>
+          <t>$741.11 / 8.89%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$747.34 / 8.40%</t>
+          <t>$741.11 / 7.50%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$747.34 / 8.05%</t>
+          <t>$741.11 / 7.15%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$747.34 / 19.08%</t>
+          <t>$741.11 / 18.09%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$747.34 / 0.08%</t>
+          <t>$741.11 / -0.75%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$747.34 / 15.23%</t>
+          <t>$741.11 / 14.27%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$747.34 / 1.11%</t>
+          <t>$741.11 / 0.26%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$747.34 / 13.40%</t>
+          <t>$741.11 / 12.45%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$747.34 / 12.49%</t>
+          <t>$741.11 / 11.55%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$747.34 / 12.60%</t>
+          <t>$741.11 / 11.66%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.35% (10.71%)</t>
+          <t>11.86% (11.22%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.63% (1.54%)</t>
+          <t>1.96% (1.87%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.95% (6.59%)</t>
+          <t>7.38% (7.03%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.72% (8.22%)</t>
+          <t>9.19% (8.69%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.08% (7.66%)</t>
+          <t>8.56% (8.14%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.19% (0.17%)</t>
+          <t>0.31% (0.29%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.28% (15.48%)</t>
+          <t>16.88% (16.08%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.88% (7.34%)</t>
+          <t>8.26% (7.72%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.61% (14.88%)</t>
+          <t>16.26% (15.53%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.62% (5.34%)</t>
+          <t>6.09% (5.81%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.55% (4.33%)</t>
+          <t>5.05% (4.83%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.45% (3.29%)</t>
+          <t>3.86% (3.71%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.33% (8.68%)</t>
+          <t>9.69% (9.05%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.25% (1.16%)</t>
+          <t>1.48% (1.39%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.53% (5.17%)</t>
+          <t>5.86% (5.50%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.08% (6.57%)</t>
+          <t>7.38% (6.88%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.43% (6.00%)</t>
+          <t>6.77% (6.35%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.16% (0.13%)</t>
+          <t>0.15% (0.13%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.22% (12.42%)</t>
+          <t>13.72% (12.91%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.75% (6.20%)</t>
+          <t>7.03% (6.47%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.55% (11.81%)</t>
+          <t>13.03% (12.29%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.29% (4.00%)</t>
+          <t>4.58% (4.29%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.41% (3.19%)</t>
+          <t>3.72% (3.50%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.55% (2.39%)</t>
+          <t>2.88% (2.73%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.43%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.60%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>5.38%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>6.99%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>6.89%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-3.00%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.36%</t>
+          <t>17.34%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.68%</t>
+          <t>2.54%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15.81%</t>
+          <t>16.78%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>3.70%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>3.18%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.75%</t>
+          <t>7.65%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.66%</t>
+          <t>-2.85%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.07%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.37%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.48%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-5.91%</t>
+          <t>-5.12%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.26%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>-0.14%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.59%</t>
+          <t>13.54%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>0.71%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>0.54%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.99%</t>
+          <t>-0.16%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.15% (10.51%)</t>
+          <t>10.87% (10.23%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.35% (11.26%)</t>
+          <t>10.99% (10.90%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.19% (10.83%)</t>
+          <t>10.87% (10.51%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.46% (10.96%)</t>
+          <t>11.18% (10.67%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.03% (10.61%)</t>
+          <t>10.75% (10.32%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.80% (11.77%)</t>
+          <t>11.26% (11.24%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.92% (9.12%)</t>
+          <t>9.68% (8.88%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.94% (13.39%)</t>
+          <t>13.60% (13.05%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.70% (8.97%)</t>
+          <t>9.51% (8.77%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.14% (10.85%)</t>
+          <t>10.87% (10.58%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.76% (10.54%)</t>
+          <t>10.52% (10.30%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.74% (10.58%)</t>
+          <t>10.43% (10.27%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.52% (15.88%)</t>
+          <t>16.17% (15.53%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.24% (17.14%)</t>
+          <t>16.83% (16.73%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.70% (16.34%)</t>
+          <t>16.34% (15.98%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.12% (16.61%)</t>
+          <t>16.73% (16.22%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.48% (16.05%)</t>
+          <t>16.12% (15.70%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>17.93% (17.91%)</t>
+          <t>17.33% (17.31%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.95% (14.15%)</t>
+          <t>14.67% (13.87%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.76% (19.21%)</t>
+          <t>19.39% (18.83%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.78% (14.05%)</t>
+          <t>14.50% (13.77%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.07% (16.78%)</t>
+          <t>16.70% (16.40%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.58% (16.37%)</t>
+          <t>16.22% (16.01%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.43% (16.28%)</t>
+          <t>16.10% (15.94%)</t>
         </is>
       </c>
     </row>
@@ -2961,87 +2961,87 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.33% (-3.97%)</t>
+          <t>-2.89% (-3.53%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.16% (-11.25%)</t>
+          <t>-10.87% (-10.96%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.85% (-7.21%)</t>
+          <t>-6.48% (-6.83%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.51% (-6.01%)</t>
+          <t>-5.10% (-5.60%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.68% (-6.10%)</t>
+          <t>-5.26% (-5.68%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.63% (-12.65%)</t>
+          <t>-12.53% (-12.55%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.15% (-0.95%)</t>
+          <t>0.00% (-0.44%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.96% (-8.51%)</t>
+          <t>-7.64% (-8.18%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.28% (-2.01%)</t>
+          <t>-0.73% (-1.46%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.50% (-9.79%)</t>
+          <t>-9.10% (-9.38%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.23% (-9.45%)</t>
+          <t>-8.80% (-9.01%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.33% (-9.49%)</t>
+          <t>-8.97% (-9.13%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.70% (-3.35%)</t>
+          <t>-2.38% (-3.02%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.58% (-9.67%)</t>
+          <t>-9.37% (-9.47%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.89% (-6.25%)</t>
+          <t>-5.59% (-5.95%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.47% (-4.97%)</t>
+          <t>-4.20% (-4.70%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.85% (-5.28%)</t>
+          <t>-4.55% (-4.97%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -3051,32 +3051,32 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.12% (-0.92%)</t>
+          <t>0.00% (-0.48%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.47% (-7.02%)</t>
+          <t>-6.23% (-6.78%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.14% (-1.88%)</t>
+          <t>-0.72% (-1.45%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.97% (-8.26%)</t>
+          <t>-7.71% (-8.01%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.85% (-8.07%)</t>
+          <t>-7.57% (-7.79%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.08% (-8.23%)</t>
+          <t>-7.78% (-7.93%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.48%</t>
+          <t>-13.76%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.51%</t>
+          <t>-21.86%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.04%</t>
+          <t>-17.35%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.97%</t>
+          <t>-16.28%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.71%</t>
+          <t>-16.01%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.42%</t>
+          <t>-23.79%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.07%</t>
+          <t>-9.32%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.89%</t>
+          <t>-21.24%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.98%</t>
+          <t>-10.24%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.63%</t>
+          <t>-19.97%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.99%</t>
+          <t>-19.32%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.07%</t>
+          <t>-19.40%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.23%</t>
+          <t>-18.55%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.82%</t>
+          <t>-26.20%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.59%</t>
+          <t>-21.94%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-21.58%</t>
+          <t>-20.92%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.33%</t>
+          <t>-20.67%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-28.62%</t>
+          <t>-28.02%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.07%</t>
+          <t>-14.35%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.23%</t>
+          <t>-25.61%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.93%</t>
+          <t>-15.22%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.04%</t>
+          <t>-24.41%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.43%</t>
+          <t>-23.80%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.51%</t>
+          <t>-23.87%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.74% (1.10%)</t>
+          <t>1.35% (0.72%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.63% (1.54%)</t>
+          <t>1.96% (1.87%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.33% (1.97%)</t>
+          <t>1.88% (1.52%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.45% (1.95%)</t>
+          <t>2.04% (1.54%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.95% (1.52%)</t>
+          <t>1.54% (1.12%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.19% (0.17%)</t>
+          <t>0.31% (0.29%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.07% (-0.87%)</t>
+          <t>0.37% (-0.44%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.09% (5.54%)</t>
+          <t>5.58% (5.03%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.19% (-0.92%)</t>
+          <t>-0.47% (-1.20%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.69% (2.41%)</t>
+          <t>2.29% (2.00%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.17% (1.96%)</t>
+          <t>1.80% (1.58%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.17% (2.02%)</t>
+          <t>1.72% (1.56%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.40% (1.76%)</t>
+          <t>1.88% (1.24%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.25% (1.16%)</t>
+          <t>1.48% (1.39%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.38% (3.02%)</t>
+          <t>2.84% (2.48%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.58% (3.07%)</t>
+          <t>3.00% (2.50%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.84% (2.41%)</t>
+          <t>2.30% (1.88%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.16% (0.13%)</t>
+          <t>0.15% (0.13%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.04% (-0.84%)</t>
+          <t>0.32% (-0.48%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.75% (6.20%)</t>
+          <t>7.03% (6.47%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.05% (-0.78%)</t>
+          <t>-0.46% (-1.20%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>4.29% (4.00%)</t>
+          <t>3.84% (3.55%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.41% (3.19%)</t>
+          <t>3.16% (2.95%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.55% (2.39%)</t>
+          <t>2.88% (2.73%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 7/7/2026</t>
+          <t>As of 8/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.66%</t>
+          <t>8.14%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.59%</t>
+          <t>5.12%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.05%</t>
+          <t>7.15%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>6.89%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.10%</t>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.22%</t>
+          <t>8.69%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>5.03%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.40%</t>
+          <t>7.50%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>6.99%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.01%</t>
+          <t>-5.60%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.39%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.34%</t>
+          <t>7.72%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.37%</t>
+          <t>7.99%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.23%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.68%</t>
+          <t>2.54%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.51%</t>
+          <t>-8.18%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>11.22%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>4.36%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.43%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.97%</t>
+          <t>-3.53%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.97%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.88%</t>
+          <t>15.53%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.17%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.11%</t>
+          <t>0.26%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>15.81%</t>
+          <t>16.78%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.01%</t>
+          <t>-1.46%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.48%</t>
+          <t>16.08%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>-0.41%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>-0.75%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.36%</t>
+          <t>17.34%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.95%</t>
+          <t>-0.44%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.77%</t>
+          <t>11.24%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.51%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.08%</t>
+          <t>18.09%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-3.00%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.65%</t>
+          <t>-12.55%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.26%</t>
+          <t>10.90%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.54%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.71%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.15%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.60%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.25%</t>
+          <t>-10.96%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.58%</t>
+          <t>10.27%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>3.71%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.55%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>11.66%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.49%</t>
+          <t>-9.13%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.54%</t>
+          <t>10.30%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>4.83%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.50%</t>
+          <t>8.97%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>3.18%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.45%</t>
+          <t>-9.01%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.58%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.34%</t>
+          <t>5.81%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.91%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.40%</t>
+          <t>12.45%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>3.70%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.79%</t>
+          <t>-9.38%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.83%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.59%</t>
+          <t>7.03%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.86%</t>
+          <t>6.43%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.81%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>5.38%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.21%</t>
+          <t>-6.83%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 7/7/2026</t>
+          <t>As of 8/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>15.70%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>6.35%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.34%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.05%</t>
+          <t>7.15%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.48%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.28%</t>
+          <t>-4.97%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.61%</t>
+          <t>16.22%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.57%</t>
+          <t>6.88%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.05%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.40%</t>
+          <t>7.50%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.37%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.97%</t>
+          <t>-4.70%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.21%</t>
+          <t>18.83%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.20%</t>
+          <t>6.47%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.65%</t>
+          <t>6.37%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.23%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>-0.14%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.02%</t>
+          <t>-6.78%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.88%</t>
+          <t>15.53%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.68%</t>
+          <t>9.05%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.59%</t>
+          <t>2.24%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>4.36%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.75%</t>
+          <t>7.65%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.35%</t>
+          <t>-3.02%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.05%</t>
+          <t>13.77%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.81%</t>
+          <t>12.29%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>0.60%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.11%</t>
+          <t>0.26%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.59%</t>
+          <t>13.54%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.88%</t>
+          <t>-1.45%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.15%</t>
+          <t>13.87%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.42%</t>
+          <t>12.91%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>-0.36%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>-0.75%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.26%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.92%</t>
+          <t>-0.48%</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17.91%</t>
+          <t>17.31%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4162,12 +4162,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.08%</t>
+          <t>18.09%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-5.91%</t>
+          <t>-5.12%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.14%</t>
+          <t>16.73%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.16%</t>
+          <t>1.39%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.76%</t>
+          <t>9.51%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.15%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.66%</t>
+          <t>-2.85%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.67%</t>
+          <t>-9.47%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.28%</t>
+          <t>15.94%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>2.73%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.05%</t>
+          <t>7.70%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>11.66%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.99%</t>
+          <t>-0.16%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.23%</t>
+          <t>-7.93%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.19%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.85%</t>
+          <t>7.53%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>0.54%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.07%</t>
+          <t>-7.79%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.78%</t>
+          <t>16.40%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>4.29%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.79%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.40%</t>
+          <t>12.45%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>0.71%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.26%</t>
+          <t>-8.01%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>5.50%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.76%</t>
+          <t>5.43%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.81%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.07%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.25%</t>
+          <t>-5.95%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-09]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/8/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>282 days</t>
+          <t>281 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>44 days</t>
+          <t>43 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>163 days</t>
+          <t>162 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>226 days</t>
+          <t>225 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>191 days</t>
+          <t>190 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>9 days</t>
+          <t>8 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>344 days</t>
+          <t>343 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>254 days</t>
+          <t>253 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>317 days</t>
+          <t>316 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>135 days</t>
+          <t>134 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>100 days</t>
+          <t>99 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>72 days</t>
+          <t>71 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>282 days</t>
+          <t>281 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>44 days</t>
+          <t>43 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>163 days</t>
+          <t>162 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>226 days</t>
+          <t>225 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>191 days</t>
+          <t>190 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>9 days</t>
+          <t>8 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>344 days</t>
+          <t>343 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>254 days</t>
+          <t>253 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>317 days</t>
+          <t>316 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>135 days</t>
+          <t>134 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>100 days</t>
+          <t>99 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>72 days</t>
+          <t>71 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.53 / 2.78%</t>
+          <t>$46.86 / 3.52%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.44 / 11.34%</t>
+          <t>$56.72 / 11.89%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.29 / 6.43%</t>
+          <t>$54.66 / 7.16%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$60.83 / 5.03%</t>
+          <t>$61.25 / 5.75%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$54.95 / 5.12%</t>
+          <t>$55.35 / 5.90%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.64 / 13.38%</t>
+          <t>$59.75 / 13.59%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.63 / -0.41%</t>
+          <t>$60.12 / 0.41%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.18 / 7.99%</t>
+          <t>$52.46 / 8.58%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$55.90 / 0.61%</t>
+          <t>$56.37 / 1.45%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.26 / 9.42%</t>
+          <t>$58.67 / 10.19%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.17 / 8.97%</t>
+          <t>$52.54 / 9.76%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.00 / 9.11%</t>
+          <t>$55.36 / 9.82%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.56 / 2.24%</t>
+          <t>$41.79 / 2.82%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.41 / 9.51%</t>
+          <t>$41.56 / 9.90%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.74 / 5.43%</t>
+          <t>$39.96 / 6.02%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$43.93 / 4.05%</t>
+          <t>$44.17 / 4.61%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$44.92 / 4.34%</t>
+          <t>$45.17 / 4.92%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.56 / 11.05%</t>
+          <t>$43.59 / 11.11%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.00 / -0.36%</t>
+          <t>$41.27 / 0.29%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.18 / 6.37%</t>
+          <t>$44.36 / 6.81%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$42.90 / 0.60%</t>
+          <t>$43.20 / 1.30%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.74 / 7.79%</t>
+          <t>$41.92 / 8.25%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.47 / 7.53%</t>
+          <t>$41.67 / 8.04%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$40.90 / 7.70%</t>
+          <t>$41.11 / 8.24%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$741.11 / 4.36%</t>
+          <t>$750.30 / 5.65%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$741.11 / 15.18%</t>
+          <t>$750.30 / 16.61%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$741.11 / 8.89%</t>
+          <t>$750.30 / 10.24%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$741.11 / 7.50%</t>
+          <t>$750.30 / 8.83%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$741.11 / 7.15%</t>
+          <t>$750.30 / 8.48%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$741.11 / 18.09%</t>
+          <t>$750.30 / 19.55%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$741.11 / -0.75%</t>
+          <t>$750.30 / 0.48%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$741.11 / 14.27%</t>
+          <t>$750.30 / 15.68%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$741.11 / 0.26%</t>
+          <t>$750.30 / 1.51%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$741.11 / 12.45%</t>
+          <t>$750.30 / 13.85%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$741.11 / 11.55%</t>
+          <t>$750.30 / 12.93%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$741.11 / 11.66%</t>
+          <t>$750.30 / 13.05%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$741.11 / 4.36%</t>
+          <t>$750.30 / 5.65%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$741.11 / 15.18%</t>
+          <t>$750.30 / 16.61%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$741.11 / 8.89%</t>
+          <t>$750.30 / 10.24%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$741.11 / 7.50%</t>
+          <t>$750.30 / 8.83%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$741.11 / 7.15%</t>
+          <t>$750.30 / 8.48%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$741.11 / 18.09%</t>
+          <t>$750.30 / 19.55%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$741.11 / -0.75%</t>
+          <t>$750.30 / 0.48%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$741.11 / 14.27%</t>
+          <t>$750.30 / 15.68%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$741.11 / 0.26%</t>
+          <t>$750.30 / 1.51%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$741.11 / 12.45%</t>
+          <t>$750.30 / 13.85%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$741.11 / 11.55%</t>
+          <t>$750.30 / 12.93%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$741.11 / 11.66%</t>
+          <t>$750.30 / 13.05%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.86% (11.22%)</t>
+          <t>11.06% (10.43%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.96% (1.87%)</t>
+          <t>1.46% (1.37%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.38% (7.03%)</t>
+          <t>6.64% (6.29%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>9.19% (8.69%)</t>
+          <t>8.45% (7.95%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.56% (8.14%)</t>
+          <t>7.77% (7.35%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.31% (0.29%)</t>
+          <t>0.11% (0.09%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.88% (16.08%)</t>
+          <t>15.93% (15.13%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.26% (7.72%)</t>
+          <t>7.67% (7.13%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>16.26% (15.53%)</t>
+          <t>15.29% (14.56%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>6.09% (5.81%)</t>
+          <t>5.35% (5.07%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5.05% (4.83%)</t>
+          <t>4.30% (4.09%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.86% (3.71%)</t>
+          <t>3.18% (3.03%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.69% (9.05%)</t>
+          <t>9.07% (8.44%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.48% (1.39%)</t>
+          <t>1.12% (1.03%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.86% (5.50%)</t>
+          <t>5.28% (4.92%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.38% (6.88%)</t>
+          <t>6.81% (6.31%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.77% (6.35%)</t>
+          <t>6.18% (5.76%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.15% (0.13%)</t>
+          <t>0.09% (0.08%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.72% (12.91%)</t>
+          <t>12.97% (12.18%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>7.03% (6.47%)</t>
+          <t>6.58% (6.03%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>13.03% (12.29%)</t>
+          <t>12.24% (11.52%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.58% (4.29%)</t>
+          <t>4.13% (3.84%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.72% (3.50%)</t>
+          <t>3.23% (3.02%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.88% (2.73%)</t>
+          <t>2.37% (2.22%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-1.99%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.38%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.99%</t>
+          <t>5.68%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.89%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-3.00%</t>
+          <t>-4.19%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>17.34%</t>
+          <t>15.90%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.54%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.78%</t>
+          <t>15.35%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.70%</t>
+          <t>2.43%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>3.18%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>0.84%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>7.65%</t>
+          <t>6.33%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-2.85%</t>
+          <t>-4.04%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.93%</t>
+          <t>1.67%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>4.24%</t>
+          <t>2.96%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-5.12%</t>
+          <t>-6.28%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.14%</t>
+          <t>-1.37%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>13.54%</t>
+          <t>12.15%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.71%</t>
+          <t>-0.52%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>0.54%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>-1.38%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.87% (10.23%)</t>
+          <t>11.23% (10.60%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.99% (10.90%)</t>
+          <t>11.50% (11.41%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.87% (10.51%)</t>
+          <t>11.24% (10.89%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.18% (10.67%)</t>
+          <t>11.56% (11.06%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.75% (10.32%)</t>
+          <t>11.08% (10.66%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.26% (11.24%)</t>
+          <t>12.02% (12.01%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.68% (8.88%)</t>
+          <t>9.97% (9.18%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.60% (13.05%)</t>
+          <t>14.06% (13.52%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.51% (8.77%)</t>
+          <t>9.78% (9.05%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.87% (10.58%)</t>
+          <t>11.21% (10.93%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.52% (10.30%)</t>
+          <t>10.85% (10.64%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.43% (10.27%)</t>
+          <t>10.82% (10.67%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.17% (15.53%)</t>
+          <t>16.62% (15.98%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.83% (16.73%)</t>
+          <t>17.40% (17.31%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.34% (15.98%)</t>
+          <t>16.78% (16.42%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.73% (16.22%)</t>
+          <t>17.18% (16.68%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.12% (15.70%)</t>
+          <t>16.56% (16.14%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>17.33% (17.31%)</t>
+          <t>18.16% (18.14%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.67% (13.87%)</t>
+          <t>15.06% (14.26%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.39% (18.83%)</t>
+          <t>19.90% (19.35%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.50% (13.77%)</t>
+          <t>14.85% (14.12%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.70% (16.40%)</t>
+          <t>17.22% (16.93%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.22% (16.01%)</t>
+          <t>16.72% (16.51%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.10% (15.94%)</t>
+          <t>16.57% (16.42%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-2.89% (-3.53%)</t>
+          <t>-3.59% (-4.22%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-10.87% (-10.96%)</t>
+          <t>-11.31% (-11.40%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.48% (-6.83%)</t>
+          <t>-7.12% (-7.47%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.10% (-5.60%)</t>
+          <t>-5.74% (-6.24%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.26% (-5.68%)</t>
+          <t>-5.95% (-6.37%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.53% (-12.55%)</t>
+          <t>-12.70% (-12.71%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.44%)</t>
+          <t>-0.45% (-1.25%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.64% (-8.18%)</t>
+          <t>-8.14% (-8.68%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-0.73% (-1.46%)</t>
+          <t>-1.56% (-2.28%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.10% (-9.38%)</t>
+          <t>-9.73% (-10.02%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-8.80% (-9.01%)</t>
+          <t>-9.45% (-9.66%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-8.97% (-9.13%)</t>
+          <t>-9.57% (-9.72%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.38% (-3.02%)</t>
+          <t>-2.93% (-3.57%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.37% (-9.47%)</t>
+          <t>-9.70% (-9.79%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.59% (-5.95%)</t>
+          <t>-6.12% (-6.47%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.20% (-4.70%)</t>
+          <t>-4.71% (-5.21%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.55% (-4.97%)</t>
+          <t>-5.08% (-5.50%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.69% (-10.71%)</t>
+          <t>-10.74% (-10.76%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.48%)</t>
+          <t>-0.34% (-1.14%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.23% (-6.78%)</t>
+          <t>-6.62% (-7.17%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-0.72% (-1.45%)</t>
+          <t>-1.41% (-2.14%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.71% (-8.01%)</t>
+          <t>-8.11% (-8.40%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.57% (-7.79%)</t>
+          <t>-8.01% (-8.22%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-7.78% (-7.93%)</t>
+          <t>-8.24% (-8.39%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-13.76%</t>
+          <t>-14.82%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.86%</t>
+          <t>-22.82%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.35%</t>
+          <t>-18.36%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.28%</t>
+          <t>-17.30%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.01%</t>
+          <t>-17.03%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-23.79%</t>
+          <t>-24.72%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.32%</t>
+          <t>-10.43%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.24%</t>
+          <t>-22.20%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.24%</t>
+          <t>-11.33%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-19.97%</t>
+          <t>-20.95%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.32%</t>
+          <t>-20.30%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-19.40%</t>
+          <t>-20.39%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-18.55%</t>
+          <t>-19.55%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.20%</t>
+          <t>-27.10%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-21.94%</t>
+          <t>-22.89%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.92%</t>
+          <t>-21.89%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-20.67%</t>
+          <t>-21.64%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-28.02%</t>
+          <t>-28.90%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.35%</t>
+          <t>-15.40%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-25.61%</t>
+          <t>-26.52%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.22%</t>
+          <t>-16.26%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.41%</t>
+          <t>-25.34%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.80%</t>
+          <t>-24.73%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.87%</t>
+          <t>-24.81%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.35% (0.72%)</t>
+          <t>1.88% (1.25%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.96% (1.87%)</t>
+          <t>1.46% (1.37%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.88% (1.52%)</t>
+          <t>2.44% (2.08%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.04% (1.54%)</t>
+          <t>2.60% (2.11%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.54% (1.12%)</t>
+          <t>2.05% (1.63%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.31% (0.29%)</t>
+          <t>0.11% (0.09%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.37% (-0.44%)</t>
+          <t>0.02% (-0.78%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.58% (5.03%)</t>
+          <t>6.31% (5.76%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.47% (-1.20%)</t>
+          <t>-0.07% (-0.80%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.29% (2.00%)</t>
+          <t>2.83% (2.55%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.80% (1.58%)</t>
+          <t>2.33% (2.12%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.72% (1.56%)</t>
+          <t>2.31% (2.16%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.88% (1.24%)</t>
+          <t>2.57% (1.93%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.48% (1.39%)</t>
+          <t>1.12% (1.03%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.84% (2.48%)</t>
+          <t>3.54% (3.19%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.00% (2.50%)</t>
+          <t>3.73% (3.23%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.30% (1.88%)</t>
+          <t>3.00% (2.58%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.15% (0.13%)</t>
+          <t>0.09% (0.08%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.32% (-0.48%)</t>
+          <t>0.13% (-0.66%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>7.03% (6.47%)</t>
+          <t>6.58% (6.03%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.46% (-1.20%)</t>
+          <t>0.07% (-0.65%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.84% (3.55%)</t>
+          <t>4.13% (3.84%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.16% (2.95%)</t>
+          <t>3.23% (3.02%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.88% (2.73%)</t>
+          <t>2.37% (2.22%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 8/7/2026</t>
+          <t>As of 9/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8.14%</t>
+          <t>7.35%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.12%</t>
+          <t>5.90%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.15%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.89%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-6.37%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>11.06%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.69%</t>
+          <t>7.95%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.03%</t>
+          <t>5.75%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.50%</t>
+          <t>8.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.99%</t>
+          <t>5.68%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.60%</t>
+          <t>-6.24%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>13.52%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.72%</t>
+          <t>7.13%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.99%</t>
+          <t>8.58%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>15.68%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2.54%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.18%</t>
+          <t>-8.68%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11.22%</t>
+          <t>10.43%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.36%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.53%</t>
+          <t>-4.22%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>9.05%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.53%</t>
+          <t>14.56%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.26%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.78%</t>
+          <t>15.35%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.46%</t>
+          <t>-2.28%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16.08%</t>
+          <t>15.13%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.41%</t>
+          <t>0.41%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>0.48%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17.34%</t>
+          <t>15.90%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.44%</t>
+          <t>-1.25%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.24%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>0.09%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>13.59%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.09%</t>
+          <t>19.55%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-3.00%</t>
+          <t>-4.19%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.55%</t>
+          <t>-12.71%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.90%</t>
+          <t>11.41%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>1.37%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>11.89%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>16.61%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-1.99%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.96%</t>
+          <t>-11.40%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.27%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.71%</t>
+          <t>3.03%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.82%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.66%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>0.84%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.13%</t>
+          <t>-9.72%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.30%</t>
+          <t>10.64%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.83%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.97%</t>
+          <t>9.76%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>12.93%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3.18%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.01%</t>
+          <t>-9.66%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.58%</t>
+          <t>10.93%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.81%</t>
+          <t>5.07%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>10.19%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12.45%</t>
+          <t>13.85%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.70%</t>
+          <t>2.43%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.38%</t>
+          <t>-10.02%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>10.89%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7.03%</t>
+          <t>6.29%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.43%</t>
+          <t>7.16%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5.38%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.83%</t>
+          <t>-7.47%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 8/7/2026</t>
+          <t>As of 9/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.70%</t>
+          <t>16.14%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.35%</t>
+          <t>5.76%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.34%</t>
+          <t>4.92%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.15%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-4.97%</t>
+          <t>-5.50%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.22%</t>
+          <t>16.68%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.88%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>4.61%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.50%</t>
+          <t>8.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.24%</t>
+          <t>2.96%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.70%</t>
+          <t>-5.21%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.83%</t>
+          <t>19.35%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.47%</t>
+          <t>6.03%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.37%</t>
+          <t>6.81%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>15.68%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.14%</t>
+          <t>-1.37%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.78%</t>
+          <t>-7.17%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.53%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9.05%</t>
+          <t>8.44%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.24%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.36%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.65%</t>
+          <t>6.33%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.02%</t>
+          <t>-3.57%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.77%</t>
+          <t>14.12%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.29%</t>
+          <t>11.52%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.60%</t>
+          <t>1.30%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.26%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.54%</t>
+          <t>12.15%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.45%</t>
+          <t>-2.14%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.87%</t>
+          <t>14.26%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>12.18%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>0.48%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.48%</t>
+          <t>-1.14%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>18.14%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.05%</t>
+          <t>11.11%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.09%</t>
+          <t>19.55%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-5.12%</t>
+          <t>-6.28%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.71%</t>
+          <t>-10.76%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.73%</t>
+          <t>17.31%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.51%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>16.61%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.85%</t>
+          <t>-4.04%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.47%</t>
+          <t>-9.79%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.94%</t>
+          <t>16.42%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.73%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.70%</t>
+          <t>8.24%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.66%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>-1.38%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-7.93%</t>
+          <t>-8.39%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>16.51%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.02%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.53%</t>
+          <t>8.04%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>12.93%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.54%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.79%</t>
+          <t>-8.22%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.40%</t>
+          <t>16.93%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.29%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.79%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12.45%</t>
+          <t>13.85%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.71%</t>
+          <t>-0.52%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.01%</t>
+          <t>-8.40%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>16.42%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.50%</t>
+          <t>4.92%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.43%</t>
+          <t>6.02%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.93%</t>
+          <t>1.67%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-5.95%</t>
+          <t>-6.47%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-10]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/9/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>281 days</t>
+          <t>280 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>43 days</t>
+          <t>42 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>162 days</t>
+          <t>161 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>225 days</t>
+          <t>224 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>190 days</t>
+          <t>189 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>8 days</t>
+          <t>7 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>343 days</t>
+          <t>342 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>253 days</t>
+          <t>252 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>316 days</t>
+          <t>315 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>134 days</t>
+          <t>133 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>99 days</t>
+          <t>98 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>71 days</t>
+          <t>70 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>281 days</t>
+          <t>280 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>43 days</t>
+          <t>42 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>162 days</t>
+          <t>161 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>225 days</t>
+          <t>224 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>190 days</t>
+          <t>189 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>8 days</t>
+          <t>7 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>343 days</t>
+          <t>342 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>253 days</t>
+          <t>252 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>316 days</t>
+          <t>315 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>134 days</t>
+          <t>133 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>99 days</t>
+          <t>98 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>71 days</t>
+          <t>70 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.86 / 3.52%</t>
+          <t>$46.95 / 3.72%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.72 / 11.89%</t>
+          <t>$56.79 / 12.04%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.66 / 7.16%</t>
+          <t>$54.75 / 7.33%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.25 / 5.75%</t>
+          <t>$61.34 / 5.91%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.35 / 5.90%</t>
+          <t>$55.44 / 6.06%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.75 / 13.59%</t>
+          <t>$59.80 / 13.68%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.12 / 0.41%</t>
+          <t>$60.25 / 0.62%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.46 / 8.58%</t>
+          <t>$52.56 / 8.78%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.37 / 1.45%</t>
+          <t>$56.48 / 1.64%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.67 / 10.19%</t>
+          <t>$58.79 / 10.42%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.54 / 9.76%</t>
+          <t>$52.63 / 9.95%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.36 / 9.82%</t>
+          <t>$55.45 / 10.00%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.79 / 2.82%</t>
+          <t>$41.85 / 2.96%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.56 / 9.90%</t>
+          <t>$41.61 / 10.05%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.96 / 6.02%</t>
+          <t>$40.02 / 6.18%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.17 / 4.61%</t>
+          <t>$44.21 / 4.70%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.17 / 4.92%</t>
+          <t>$45.22 / 5.04%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.59 / 11.11%</t>
+          <t>$43.61 / 11.17%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.27 / 0.29%</t>
+          <t>$41.36 / 0.50%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.36 / 6.81%</t>
+          <t>$44.43 / 6.97%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.20 / 1.30%</t>
+          <t>$43.26 / 1.44%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.92 / 8.25%</t>
+          <t>$42.00 / 8.47%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.67 / 8.04%</t>
+          <t>$41.74 / 8.22%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.11 / 8.24%</t>
+          <t>$41.17 / 8.41%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$750.30 / 5.65%</t>
+          <t>$752.74 / 6.00%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$750.30 / 16.61%</t>
+          <t>$752.74 / 16.99%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$750.30 / 10.24%</t>
+          <t>$752.74 / 10.60%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$750.30 / 8.83%</t>
+          <t>$752.74 / 9.18%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$750.30 / 8.48%</t>
+          <t>$752.74 / 8.83%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$750.30 / 19.55%</t>
+          <t>$752.74 / 19.94%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$750.30 / 0.48%</t>
+          <t>$752.74 / 0.80%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$750.30 / 15.68%</t>
+          <t>$752.74 / 16.06%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$750.30 / 1.51%</t>
+          <t>$752.74 / 1.84%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$750.30 / 13.85%</t>
+          <t>$752.74 / 14.22%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$750.30 / 12.93%</t>
+          <t>$752.74 / 13.30%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$750.30 / 13.05%</t>
+          <t>$752.74 / 13.42%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$750.30 / 5.65%</t>
+          <t>$752.74 / 6.00%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$750.30 / 16.61%</t>
+          <t>$752.74 / 16.99%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$750.30 / 10.24%</t>
+          <t>$752.74 / 10.60%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$750.30 / 8.83%</t>
+          <t>$752.74 / 9.18%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$750.30 / 8.48%</t>
+          <t>$752.74 / 8.83%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$750.30 / 19.55%</t>
+          <t>$752.74 / 19.94%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$750.30 / 0.48%</t>
+          <t>$752.74 / 0.80%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$750.30 / 15.68%</t>
+          <t>$752.74 / 16.06%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$750.30 / 1.51%</t>
+          <t>$752.74 / 1.84%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$750.30 / 13.85%</t>
+          <t>$752.74 / 14.22%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$750.30 / 12.93%</t>
+          <t>$752.74 / 13.30%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$750.30 / 13.05%</t>
+          <t>$752.74 / 13.42%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.06% (10.43%)</t>
+          <t>10.85% (10.22%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.46% (1.37%)</t>
+          <t>1.32% (1.24%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.64% (6.29%)</t>
+          <t>6.48% (6.13%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.45% (7.95%)</t>
+          <t>8.29% (7.79%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.77% (7.35%)</t>
+          <t>7.60% (7.19%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.11% (0.09%)</t>
+          <t>0.03% (0.02%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.93% (15.13%)</t>
+          <t>15.68% (14.89%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.67% (7.13%)</t>
+          <t>7.48% (6.94%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.29% (14.56%)</t>
+          <t>15.07% (14.35%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.35% (5.07%)</t>
+          <t>5.13% (4.85%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.30% (4.09%)</t>
+          <t>4.12% (3.91%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.18% (3.03%)</t>
+          <t>3.01% (2.86%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.07% (8.44%)</t>
+          <t>8.93% (8.29%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.12% (1.03%)</t>
+          <t>0.98% (0.89%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.28% (4.92%)</t>
+          <t>5.12% (4.77%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.81% (6.31%)</t>
+          <t>6.71% (6.21%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.18% (5.76%)</t>
+          <t>6.06% (5.64%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.09% (0.08%)</t>
+          <t>0.03% (0.02%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.97% (12.18%)</t>
+          <t>12.74% (11.94%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.58% (6.03%)</t>
+          <t>6.42% (5.87%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.24% (11.52%)</t>
+          <t>12.08% (11.36%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.13% (3.84%)</t>
+          <t>3.91% (3.63%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.23% (3.02%)</t>
+          <t>3.06% (2.84%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.37% (2.22%)</t>
+          <t>2.20% (2.05%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.64%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.99%</t>
+          <t>-2.30%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.68%</t>
+          <t>5.34%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.58%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-4.19%</t>
+          <t>-4.50%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>15.90%</t>
+          <t>15.52%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.43%</t>
+          <t>2.10%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.58%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.84%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.33%</t>
+          <t>5.98%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-4.04%</t>
+          <t>-4.35%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.67%</t>
+          <t>1.34%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.96%</t>
+          <t>2.63%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-6.28%</t>
+          <t>-6.59%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.45%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-1.69%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.15%</t>
+          <t>11.78%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>-0.85%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>-1.02%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.38%</t>
+          <t>-1.70%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.23% (10.60%)</t>
+          <t>11.32% (10.69%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.50% (11.41%)</t>
+          <t>11.64% (11.55%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.24% (10.89%)</t>
+          <t>11.36% (11.01%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.56% (11.06%)</t>
+          <t>11.68% (11.19%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.08% (10.66%)</t>
+          <t>11.20% (10.79%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.02% (12.01%)</t>
+          <t>12.20% (12.19%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.97% (9.18%)</t>
+          <t>10.05% (9.25%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.06% (13.52%)</t>
+          <t>14.15% (13.61%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.78% (9.05%)</t>
+          <t>9.88% (9.16%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.21% (10.93%)</t>
+          <t>11.28% (11.00%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.85% (10.64%)</t>
+          <t>10.95% (10.75%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.82% (10.67%)</t>
+          <t>10.93% (10.78%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.62% (15.98%)</t>
+          <t>16.75% (16.12%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.40% (17.31%)</t>
+          <t>17.52% (17.43%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.78% (16.42%)</t>
+          <t>16.89% (16.53%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.18% (16.68%)</t>
+          <t>17.35% (16.85%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.56% (16.14%)</t>
+          <t>16.71% (16.29%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>18.16% (18.14%)</t>
+          <t>18.34% (18.32%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.06% (14.26%)</t>
+          <t>15.13% (14.34%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.90% (19.35%)</t>
+          <t>20.00% (19.45%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.85% (14.12%)</t>
+          <t>14.98% (14.26%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.22% (16.93%)</t>
+          <t>17.28% (16.99%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.72% (16.51%)</t>
+          <t>16.81% (16.60%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.57% (16.42%)</t>
+          <t>16.67% (16.52%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.59% (-4.22%)</t>
+          <t>-3.77% (-4.40%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.31% (-11.40%)</t>
+          <t>-11.43% (-11.52%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.12% (-7.47%)</t>
+          <t>-7.27% (-7.62%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.74% (-6.24%)</t>
+          <t>-5.89% (-6.38%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.95% (-6.37%)</t>
+          <t>-6.10% (-6.51%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.70% (-12.71%)</t>
+          <t>-12.76% (-12.78%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.45% (-1.25%)</t>
+          <t>-0.67% (-1.46%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.14% (-8.68%)</t>
+          <t>-8.31% (-8.85%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.56% (-2.28%)</t>
+          <t>-1.74% (-2.46%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.73% (-10.02%)</t>
+          <t>-9.92% (-10.20%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.45% (-9.66%)</t>
+          <t>-9.61% (-9.82%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.57% (-9.72%)</t>
+          <t>-9.72% (-9.86%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.93% (-3.57%)</t>
+          <t>-3.06% (-3.69%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.70% (-9.79%)</t>
+          <t>-9.82% (-9.91%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.12% (-6.47%)</t>
+          <t>-6.26% (-6.61%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.71% (-5.21%)</t>
+          <t>-4.80% (-5.30%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.08% (-5.50%)</t>
+          <t>-5.18% (-5.60%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.74% (-10.76%)</t>
+          <t>-10.80% (-10.81%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.34% (-1.14%)</t>
+          <t>-0.55% (-1.34%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.62% (-7.17%)</t>
+          <t>-6.76% (-7.31%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.41% (-2.14%)</t>
+          <t>-1.55% (-2.27%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.11% (-8.40%)</t>
+          <t>-8.30% (-8.59%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.01% (-8.22%)</t>
+          <t>-8.16% (-8.37%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.24% (-8.39%)</t>
+          <t>-8.39% (-8.54%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.82%</t>
+          <t>-15.09%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.82%</t>
+          <t>-23.07%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.36%</t>
+          <t>-18.63%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>-17.57%</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>-17.30%</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>-17.03%</t>
-        </is>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.72%</t>
+          <t>-24.96%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.43%</t>
+          <t>-10.72%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.20%</t>
+          <t>-22.46%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.33%</t>
+          <t>-11.62%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.95%</t>
+          <t>-21.20%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.30%</t>
+          <t>-20.56%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.39%</t>
+          <t>-20.65%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.55%</t>
+          <t>-19.81%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-27.10%</t>
+          <t>-27.34%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.89%</t>
+          <t>-23.14%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
+          <t>-22.15%</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
           <t>-21.89%</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>-21.64%</t>
-        </is>
-      </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-28.90%</t>
+          <t>-29.13%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.40%</t>
+          <t>-15.67%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.52%</t>
+          <t>-26.76%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.26%</t>
+          <t>-16.53%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.34%</t>
+          <t>-25.58%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.73%</t>
+          <t>-24.97%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.81%</t>
+          <t>-25.05%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.88% (1.25%)</t>
+          <t>2.01% (1.38%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.46% (1.37%)</t>
+          <t>1.32% (1.24%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.44% (2.08%)</t>
+          <t>2.61% (2.26%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.60% (2.11%)</t>
+          <t>2.79% (2.29%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.05% (1.63%)</t>
+          <t>2.23% (1.81%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.11% (0.09%)</t>
+          <t>0.03% (0.02%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.02% (-0.78%)</t>
+          <t>0.13% (-0.66%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.31% (5.76%)</t>
+          <t>6.46% (5.92%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.07% (-0.80%)</t>
+          <t>0.06% (-0.66%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.83% (2.55%)</t>
+          <t>2.96% (2.68%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.33% (2.12%)</t>
+          <t>2.49% (2.28%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.31% (2.16%)</t>
+          <t>2.48% (2.33%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.57% (1.93%)</t>
+          <t>2.76% (2.13%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.12% (1.03%)</t>
+          <t>0.98% (0.89%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.54% (3.19%)</t>
+          <t>3.72% (3.37%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.73% (3.23%)</t>
+          <t>3.97% (3.47%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.00% (2.58%)</t>
+          <t>3.22% (2.80%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.09% (0.08%)</t>
+          <t>0.03% (0.02%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.13% (-0.66%)</t>
+          <t>0.25% (-0.54%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.58% (6.03%)</t>
+          <t>6.42% (5.87%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.07% (-0.65%)</t>
+          <t>0.26% (-0.47%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>4.13% (3.84%)</t>
+          <t>3.91% (3.63%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.23% (3.02%)</t>
+          <t>3.06% (2.84%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.37% (2.22%)</t>
+          <t>2.20% (2.05%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 9/7/2026</t>
+          <t>As of 10/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>10.79%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.35%</t>
+          <t>7.19%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.90%</t>
+          <t>6.06%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>8.83%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.58%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.37%</t>
+          <t>-6.51%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.06%</t>
+          <t>11.19%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.95%</t>
+          <t>7.79%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.75%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.83%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.68%</t>
+          <t>5.34%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.24%</t>
+          <t>-6.38%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.61%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.13%</t>
+          <t>6.94%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.58%</t>
+          <t>8.78%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.68%</t>
+          <t>16.06%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.68%</t>
+          <t>-8.85%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.43%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.72%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.64%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.22%</t>
+          <t>-4.40%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.05%</t>
+          <t>9.16%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.56%</t>
+          <t>14.35%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>1.84%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.28%</t>
+          <t>-2.46%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>9.25%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.13%</t>
+          <t>14.89%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.41%</t>
+          <t>0.62%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.48%</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.90%</t>
+          <t>15.52%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.25%</t>
+          <t>-1.46%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>12.19%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.09%</t>
+          <t>0.02%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.59%</t>
+          <t>13.68%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.55%</t>
+          <t>19.94%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.19%</t>
+          <t>-4.50%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.71%</t>
+          <t>-12.78%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.37%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.89%</t>
+          <t>12.04%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.61%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.99%</t>
+          <t>-2.30%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.40%</t>
+          <t>-11.52%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.78%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.03%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.82%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.84%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.72%</t>
+          <t>-9.86%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.64%</t>
+          <t>10.75%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.76%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.93%</t>
+          <t>13.30%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.58%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.66%</t>
+          <t>-9.82%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.07%</t>
+          <t>4.85%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.19%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.85%</t>
+          <t>14.22%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.43%</t>
+          <t>2.10%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.02%</t>
+          <t>-10.20%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.89%</t>
+          <t>11.01%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.29%</t>
+          <t>6.13%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.16%</t>
+          <t>7.33%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.47%</t>
+          <t>-7.62%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 9/7/2026</t>
+          <t>As of 10/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.14%</t>
+          <t>16.29%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.76%</t>
+          <t>5.64%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.92%</t>
+          <t>5.04%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>8.83%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.50%</t>
+          <t>-5.60%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.68%</t>
+          <t>16.85%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.61%</t>
+          <t>4.70%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.83%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.96%</t>
+          <t>2.63%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.21%</t>
+          <t>-5.30%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.35%</t>
+          <t>19.45%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.03%</t>
+          <t>5.87%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.81%</t>
+          <t>6.97%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.68%</t>
+          <t>16.06%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-1.69%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.17%</t>
+          <t>-7.31%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>16.12%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.44%</t>
+          <t>8.29%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.82%</t>
+          <t>2.96%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.33%</t>
+          <t>5.98%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.57%</t>
+          <t>-3.69%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.12%</t>
+          <t>14.26%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.52%</t>
+          <t>11.36%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.30%</t>
+          <t>1.44%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>1.84%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.15%</t>
+          <t>11.78%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.14%</t>
+          <t>-2.27%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.26%</t>
+          <t>14.34%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.18%</t>
+          <t>11.94%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.48%</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.45%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-1.34%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.14%</t>
+          <t>18.32%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>0.02%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.11%</t>
+          <t>11.17%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.55%</t>
+          <t>19.94%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-6.28%</t>
+          <t>-6.59%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.76%</t>
+          <t>-10.81%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>17.43%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>0.89%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>10.05%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.61%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.04%</t>
+          <t>-4.35%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.79%</t>
+          <t>-9.91%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.42%</t>
+          <t>16.52%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>2.05%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>8.41%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.38%</t>
+          <t>-1.70%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.39%</t>
+          <t>-8.54%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.51%</t>
+          <t>16.60%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.04%</t>
+          <t>8.22%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.93%</t>
+          <t>13.30%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>-1.02%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.22%</t>
+          <t>-8.37%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.93%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>3.63%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>8.47%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.85%</t>
+          <t>14.22%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>-0.85%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.40%</t>
+          <t>-8.59%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.42%</t>
+          <t>16.53%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.92%</t>
+          <t>4.77%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.02%</t>
+          <t>6.18%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.67%</t>
+          <t>1.34%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.47%</t>
+          <t>-6.61%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-13]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:03 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:03 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:03 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/10/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>280 days</t>
+          <t>277 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>42 days</t>
+          <t>39 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>161 days</t>
+          <t>158 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>224 days</t>
+          <t>221 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>189 days</t>
+          <t>186 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7 days</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>342 days</t>
+          <t>339 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>252 days</t>
+          <t>249 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>315 days</t>
+          <t>312 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>133 days</t>
+          <t>130 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>98 days</t>
+          <t>95 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>70 days</t>
+          <t>67 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>280 days</t>
+          <t>277 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>42 days</t>
+          <t>39 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>161 days</t>
+          <t>158 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>224 days</t>
+          <t>221 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>189 days</t>
+          <t>186 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>7 days</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>342 days</t>
+          <t>339 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>252 days</t>
+          <t>249 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>315 days</t>
+          <t>312 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>133 days</t>
+          <t>130 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>98 days</t>
+          <t>95 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>70 days</t>
+          <t>67 days</t>
         </is>
       </c>
     </row>
@@ -2326,27 +2326,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.95 / 3.72%</t>
+          <t>$46.94 / 3.69%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.79 / 12.04%</t>
+          <t>$56.78 / 12.01%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.75 / 7.33%</t>
+          <t>$54.75 / 7.34%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.34 / 5.91%</t>
+          <t>$61.28 / 5.81%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.44 / 6.06%</t>
+          <t>$55.42 / 6.03%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2356,82 +2356,82 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.25 / 0.62%</t>
+          <t>$60.19 / 0.53%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.56 / 8.78%</t>
+          <t>$52.52 / 8.69%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.48 / 1.64%</t>
+          <t>$56.41 / 1.51%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.79 / 10.42%</t>
+          <t>$58.77 / 10.37%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.63 / 9.95%</t>
+          <t>$52.60 / 9.88%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.45 / 10.00%</t>
+          <t>$55.43 / 9.96%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.85 / 2.96%</t>
+          <t>$41.82 / 2.90%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.61 / 10.05%</t>
+          <t>$41.60 / 10.02%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.02 / 6.18%</t>
+          <t>$39.99 / 6.10%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.21 / 4.70%</t>
+          <t>$44.20 / 4.68%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.22 / 5.04%</t>
+          <t>$45.20 / 4.99%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.61 / 11.17%</t>
+          <t>$43.61 / 11.16%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.36 / 0.50%</t>
+          <t>$41.32 / 0.40%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.43 / 6.97%</t>
+          <t>$44.39 / 6.89%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.26 / 1.44%</t>
+          <t>$43.23 / 1.37%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.00 / 8.47%</t>
+          <t>$41.99 / 8.44%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.17 / 8.41%</t>
+          <t>$41.16 / 8.37%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$752.74 / 6.00%</t>
+          <t>$751.33 / 5.80%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$752.74 / 16.99%</t>
+          <t>$751.33 / 16.77%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$752.74 / 10.60%</t>
+          <t>$751.33 / 10.39%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$752.74 / 9.18%</t>
+          <t>$751.17 / 8.95%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$752.74 / 8.83%</t>
+          <t>$751.17 / 8.60%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$752.74 / 19.94%</t>
+          <t>$751.33 / 19.72%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$752.74 / 0.80%</t>
+          <t>$751.33 / 0.61%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$752.74 / 16.06%</t>
+          <t>$751.17 / 15.82%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$752.74 / 1.84%</t>
+          <t>$751.33 / 1.65%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$752.74 / 14.22%</t>
+          <t>$751.33 / 14.01%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$752.74 / 13.30%</t>
+          <t>$751.33 / 13.09%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$752.74 / 13.42%</t>
+          <t>$751.33 / 13.20%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$752.74 / 6.00%</t>
+          <t>$751.33 / 5.80%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$752.74 / 16.99%</t>
+          <t>$751.33 / 16.77%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$752.74 / 10.60%</t>
+          <t>$751.33 / 10.39%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$752.74 / 9.18%</t>
+          <t>$751.33 / 8.98%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$752.74 / 8.83%</t>
+          <t>$751.33 / 8.63%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$752.74 / 19.94%</t>
+          <t>$751.33 / 19.72%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$752.74 / 0.80%</t>
+          <t>$751.33 / 0.61%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$752.74 / 16.06%</t>
+          <t>$751.33 / 15.84%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$752.74 / 1.84%</t>
+          <t>$751.33 / 1.65%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$752.74 / 14.22%</t>
+          <t>$751.33 / 14.01%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$752.74 / 13.30%</t>
+          <t>$751.33 / 13.09%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$752.74 / 13.42%</t>
+          <t>$751.33 / 13.20%</t>
         </is>
       </c>
     </row>
@@ -2580,27 +2580,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.85% (10.22%)</t>
+          <t>10.86% (10.24%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.32% (1.24%)</t>
+          <t>1.34% (1.26%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.48% (6.13%)</t>
+          <t>6.46% (6.12%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.29% (7.79%)</t>
+          <t>8.38% (7.89%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.60% (7.19%)</t>
+          <t>7.62% (7.21%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2610,92 +2610,92 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.68% (14.89%)</t>
+          <t>15.78% (14.99%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.48% (6.94%)</t>
+          <t>7.55% (7.02%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.07% (14.35%)</t>
+          <t>15.21% (14.49%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.13% (4.85%)</t>
+          <t>5.17% (4.90%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.12% (3.91%)</t>
+          <t>4.17% (3.97%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.01% (2.86%)</t>
+          <t>3.04% (2.90%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>8.93% (8.29%)</t>
+          <t>8.98% (8.36%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.98% (0.89%)</t>
+          <t>1.00% (0.92%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.12% (4.77%)</t>
+          <t>5.19% (4.84%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.71% (6.21%)</t>
+          <t>6.73% (6.24%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.06% (5.64%)</t>
+          <t>6.10% (5.69%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.03% (0.02%)</t>
+          <t>0.04% (0.03%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.74% (11.94%)</t>
+          <t>12.84% (12.05%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.42% (5.87%)</t>
+          <t>6.50% (5.96%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.08% (11.36%)</t>
+          <t>12.15% (11.44%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.91% (3.63%)</t>
+          <t>3.93% (3.65%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.06% (2.84%)</t>
+          <t>3.05% (2.84%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.20% (2.05%)</t>
+          <t>2.23% (2.09%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.64%</t>
+          <t>8.85%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-2.30%</t>
+          <t>-2.12%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>3.95%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.34%</t>
+          <t>5.56%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>5.46%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-4.50%</t>
+          <t>-4.32%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>15.52%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.17%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>15.19%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.10%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.58%</t>
+          <t>1.77%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>0.70%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>5.98%</t>
+          <t>6.18%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-4.35%</t>
+          <t>-4.17%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.63%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2.74%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-6.59%</t>
+          <t>-6.41%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.45%</t>
+          <t>12.66%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.69%</t>
+          <t>-1.50%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>11.78%</t>
+          <t>11.99%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-0.66%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-1.02%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.70%</t>
+          <t>-1.52%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.32% (10.69%)</t>
+          <t>11.18% (10.55%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.64% (11.55%)</t>
+          <t>11.51% (11.43%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.36% (11.01%)</t>
+          <t>11.19% (10.85%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.68% (11.19%)</t>
+          <t>11.59% (11.10%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.20% (10.79%)</t>
+          <t>11.05% (10.64%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.20% (12.19%)</t>
+          <t>12.05% (12.04%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.05% (9.25%)</t>
+          <t>9.96% (9.18%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.15% (13.61%)</t>
+          <t>14.05% (13.51%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.88% (9.16%)</t>
+          <t>9.83% (9.11%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.28% (11.00%)</t>
+          <t>11.17% (10.89%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.95% (10.75%)</t>
+          <t>10.85% (10.65%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.93% (10.78%)</t>
+          <t>10.81% (10.67%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.75% (16.12%)</t>
+          <t>16.65% (16.02%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.52% (17.43%)</t>
+          <t>17.39% (17.31%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.89% (16.53%)</t>
+          <t>16.81% (16.46%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.35% (16.85%)</t>
+          <t>17.22% (16.72%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.71% (16.29%)</t>
+          <t>16.60% (16.19%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>18.34% (18.32%)</t>
+          <t>18.21% (18.20%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.13% (14.34%)</t>
+          <t>15.06% (14.27%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.00% (19.45%)</t>
+          <t>19.93% (19.39%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.98% (14.26%)</t>
+          <t>14.89% (14.17%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.28% (16.99%)</t>
+          <t>17.15% (16.87%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.81% (16.60%)</t>
+          <t>16.66% (16.46%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.67% (16.52%)</t>
+          <t>16.55% (16.41%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.77% (-4.40%)</t>
+          <t>-3.76% (-4.38%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.43% (-11.52%)</t>
+          <t>-11.41% (-11.50%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.27% (-7.62%)</t>
+          <t>-7.28% (-7.63%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.89% (-6.38%)</t>
+          <t>-5.81% (-6.29%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-6.10% (-6.51%)</t>
+          <t>-6.08% (-6.49%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.76% (-12.78%)</t>
+          <t>-12.77% (-12.78%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.67% (-1.46%)</t>
+          <t>-0.59% (-1.37%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.31% (-8.85%)</t>
+          <t>-8.24% (-8.78%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.74% (-2.46%)</t>
+          <t>-1.63% (-2.34%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.92% (-10.20%)</t>
+          <t>-9.89% (-10.16%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.61% (-9.82%)</t>
+          <t>-9.56% (-9.77%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.72% (-9.86%)</t>
+          <t>-9.69% (-9.83%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-3.06% (-3.69%)</t>
+          <t>-3.01% (-3.63%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.82% (-9.91%)</t>
+          <t>-9.81% (-9.89%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.26% (-6.61%)</t>
+          <t>-6.19% (-6.54%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.80% (-5.30%)</t>
+          <t>-4.78% (-5.28%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.18% (-5.60%)</t>
+          <t>-5.15% (-5.56%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.80% (-10.81%)</t>
+          <t>-10.79% (-10.80%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.55% (-1.34%)</t>
+          <t>-0.46% (-1.24%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.76% (-7.31%)</t>
+          <t>-6.69% (-7.23%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.55% (-2.27%)</t>
+          <t>-1.49% (-2.21%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.30% (-8.59%)</t>
+          <t>-8.29% (-8.57%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.16% (-8.37%)</t>
+          <t>-8.17% (-8.37%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.39% (-8.54%)</t>
+          <t>-8.36% (-8.50%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.09%</t>
+          <t>-14.93%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-23.07%</t>
+          <t>-22.92%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.63%</t>
+          <t>-18.47%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.57%</t>
+          <t>-17.40%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-17.30%</t>
+          <t>-17.13%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.96%</t>
+          <t>-24.82%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.72%</t>
+          <t>-10.55%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.46%</t>
+          <t>-22.29%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.62%</t>
+          <t>-11.46%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.20%</t>
+          <t>-21.06%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.56%</t>
+          <t>-20.41%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.65%</t>
+          <t>-20.50%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.81%</t>
+          <t>-19.66%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-27.34%</t>
+          <t>-27.20%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.14%</t>
+          <t>-23.00%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.15%</t>
+          <t>-22.00%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.89%</t>
+          <t>-21.75%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-29.13%</t>
+          <t>-29.00%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.67%</t>
+          <t>-15.52%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.76%</t>
+          <t>-26.62%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.53%</t>
+          <t>-16.37%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.58%</t>
+          <t>-25.44%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.97%</t>
+          <t>-24.83%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.05%</t>
+          <t>-24.91%</t>
         </is>
       </c>
     </row>
@@ -3215,27 +3215,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.01% (1.38%)</t>
+          <t>1.84% (1.21%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.32% (1.24%)</t>
+          <t>1.34% (1.26%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.61% (2.26%)</t>
+          <t>2.40% (2.06%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.79% (2.29%)</t>
+          <t>2.66% (2.17%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.23% (1.81%)</t>
+          <t>2.03% (1.62%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3245,92 +3245,92 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.13% (-0.66%)</t>
+          <t>0.02% (-0.76%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.46% (5.92%)</t>
+          <t>6.31% (5.78%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.06% (-0.66%)</t>
+          <t>-0.01% (-0.72%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.96% (2.68%)</t>
+          <t>2.80% (2.53%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.49% (2.28%)</t>
+          <t>2.34% (2.14%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.48% (2.33%)</t>
+          <t>2.32% (2.18%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.76% (2.13%)</t>
+          <t>2.63% (2.00%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.98% (0.89%)</t>
+          <t>1.00% (0.92%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.72% (3.37%)</t>
+          <t>3.60% (3.25%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.97% (3.47%)</t>
+          <t>3.79% (3.30%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.22% (2.80%)</t>
+          <t>3.07% (2.65%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.03% (0.02%)</t>
+          <t>0.04% (0.03%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.25% (-0.54%)</t>
+          <t>0.15% (-0.63%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.42% (5.87%)</t>
+          <t>6.50% (5.96%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.26% (-0.47%)</t>
+          <t>0.13% (-0.59%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.91% (3.63%)</t>
+          <t>3.93% (3.65%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.06% (2.84%)</t>
+          <t>3.05% (2.84%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.20% (2.05%)</t>
+          <t>2.23% (2.09%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 10/7/2026</t>
+          <t>As of 13/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.79%</t>
+          <t>10.64%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.19%</t>
+          <t>7.21%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.06%</t>
+          <t>6.03%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.83%</t>
+          <t>8.60%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>5.46%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.51%</t>
+          <t>-6.49%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.19%</t>
+          <t>11.10%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.79%</t>
+          <t>7.89%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>5.81%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.34%</t>
+          <t>5.56%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.38%</t>
+          <t>-6.29%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.61%</t>
+          <t>13.51%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.94%</t>
+          <t>7.02%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.78%</t>
+          <t>8.69%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.06%</t>
+          <t>15.82%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.17%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.85%</t>
+          <t>-8.78%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>10.55%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.72%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>5.80%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.64%</t>
+          <t>8.85%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.40%</t>
+          <t>-4.38%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.16%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.35%</t>
+          <t>14.49%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.84%</t>
+          <t>1.65%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>15.19%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.46%</t>
+          <t>-2.34%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.25%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14.89%</t>
+          <t>14.99%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.52%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.46%</t>
+          <t>-1.37%</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.19%</t>
+          <t>12.04%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3647,12 +3647,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.94%</t>
+          <t>19.72%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.50%</t>
+          <t>-4.32%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>11.43%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>1.26%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.04%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.77%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.30%</t>
+          <t>-2.12%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.52%</t>
+          <t>-11.50%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.78%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.90%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>13.20%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>0.70%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.86%</t>
+          <t>-9.83%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.75%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>9.88%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.30%</t>
+          <t>13.09%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.58%</t>
+          <t>1.77%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.82%</t>
+          <t>-9.77%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>10.89%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.85%</t>
+          <t>4.90%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>10.37%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.22%</t>
+          <t>14.01%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.10%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.20%</t>
+          <t>-10.16%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.01%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.13%</t>
+          <t>6.12%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.33%</t>
+          <t>7.34%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.39%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>3.95%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.62%</t>
+          <t>-7.63%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 10/7/2026</t>
+          <t>As of 13/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.29%</t>
+          <t>16.19%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.64%</t>
+          <t>5.69%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.04%</t>
+          <t>4.99%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.83%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.74%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.60%</t>
+          <t>-5.56%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.85%</t>
+          <t>16.72%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>6.24%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.63%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.30%</t>
+          <t>-5.28%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.45%</t>
+          <t>19.39%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.87%</t>
+          <t>5.96%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>6.89%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.06%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.69%</t>
+          <t>-1.50%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.31%</t>
+          <t>-7.23%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.12%</t>
+          <t>16.02%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.29%</t>
+          <t>8.36%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.96%</t>
+          <t>2.90%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>5.80%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.98%</t>
+          <t>6.18%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.69%</t>
+          <t>-3.63%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.26%</t>
+          <t>14.17%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.36%</t>
+          <t>11.44%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.44%</t>
+          <t>1.37%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.84%</t>
+          <t>1.65%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.78%</t>
+          <t>11.99%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.27%</t>
+          <t>-2.21%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.34%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.94%</t>
+          <t>12.05%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.50%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.45%</t>
+          <t>12.66%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.34%</t>
+          <t>-1.24%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.32%</t>
+          <t>18.20%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.02%</t>
+          <t>0.03%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.17%</t>
+          <t>11.16%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.94%</t>
+          <t>19.72%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-6.59%</t>
+          <t>-6.41%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.81%</t>
+          <t>-10.80%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.43%</t>
+          <t>17.31%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.89%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.05%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.77%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.35%</t>
+          <t>-4.17%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.91%</t>
+          <t>-9.89%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.52%</t>
+          <t>16.41%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.05%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.41%</t>
+          <t>8.37%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>13.20%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.70%</t>
+          <t>-1.52%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.54%</t>
+          <t>-8.50%</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.60%</t>
+          <t>16.46%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.30%</t>
+          <t>13.09%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.02%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.87%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.63%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.47%</t>
+          <t>8.44%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.22%</t>
+          <t>14.01%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-0.66%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.59%</t>
+          <t>-8.57%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.53%</t>
+          <t>16.46%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.77%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.18%</t>
+          <t>6.10%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.39%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.61%</t>
+          <t>-6.54%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-14]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:03 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:03 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:03 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/13/2026 at 12:04 PM ET)</t>
+          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>277 days</t>
+          <t>276 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>39 days</t>
+          <t>38 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>158 days</t>
+          <t>157 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>221 days</t>
+          <t>220 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>186 days</t>
+          <t>185 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>3 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>339 days</t>
+          <t>338 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>249 days</t>
+          <t>248 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>312 days</t>
+          <t>311 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>130 days</t>
+          <t>129 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>95 days</t>
+          <t>94 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>67 days</t>
+          <t>66 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>277 days</t>
+          <t>276 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>39 days</t>
+          <t>38 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>158 days</t>
+          <t>157 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>221 days</t>
+          <t>220 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>186 days</t>
+          <t>185 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>3 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>339 days</t>
+          <t>338 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>249 days</t>
+          <t>248 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>312 days</t>
+          <t>311 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>130 days</t>
+          <t>129 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>95 days</t>
+          <t>94 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>67 days</t>
+          <t>66 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.94 / 3.69%</t>
+          <t>$46.94 / 3.68%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.78 / 12.01%</t>
+          <t>$56.80 / 12.05%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.75 / 7.34%</t>
+          <t>$54.77 / 7.38%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.28 / 5.81%</t>
+          <t>$61.34 / 5.92%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.42 / 6.03%</t>
+          <t>$55.44 / 6.06%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.80 / 13.68%</t>
+          <t>$59.83 / 13.74%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.19 / 0.53%</t>
+          <t>$60.23 / 0.59%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.52 / 8.69%</t>
+          <t>$52.56 / 8.79%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.41 / 1.51%</t>
+          <t>$56.45 / 1.60%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.77 / 10.37%</t>
+          <t>$58.79 / 10.42%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.60 / 9.88%</t>
+          <t>$52.65 / 9.98%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.43 / 9.96%</t>
+          <t>$55.46 / 10.02%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.82 / 2.90%</t>
+          <t>$41.85 / 2.97%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.60 / 10.02%</t>
+          <t>$41.62 / 10.06%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.99 / 6.10%</t>
+          <t>$40.03 / 6.20%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.20 / 4.68%</t>
+          <t>$44.21 / 4.71%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.20 / 4.99%</t>
+          <t>$45.24 / 5.09%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.61 / 11.16%</t>
+          <t>$43.63 / 11.21%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.32 / 0.40%</t>
+          <t>$41.37 / 0.53%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.39 / 6.89%</t>
+          <t>$44.41 / 6.94%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.23 / 1.37%</t>
+          <t>$43.26 / 1.44%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.99 / 8.44%</t>
+          <t>$42.00 / 8.46%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.74 / 8.22%</t>
+          <t>$41.73 / 8.20%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.16 / 8.37%</t>
+          <t>$41.18 / 8.43%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$751.33 / 5.80%</t>
+          <t>$751.89 / 5.88%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$751.33 / 16.77%</t>
+          <t>$751.89 / 16.85%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$751.33 / 10.39%</t>
+          <t>$751.89 / 10.48%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$751.17 / 8.95%</t>
+          <t>$751.89 / 9.06%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$751.17 / 8.60%</t>
+          <t>$751.89 / 8.71%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$751.33 / 19.72%</t>
+          <t>$751.89 / 19.81%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$751.33 / 0.61%</t>
+          <t>$751.89 / 0.69%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$751.17 / 15.82%</t>
+          <t>$751.89 / 15.93%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$751.33 / 1.65%</t>
+          <t>$751.89 / 1.72%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$751.33 / 14.01%</t>
+          <t>$751.89 / 14.09%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$751.33 / 13.09%</t>
+          <t>$751.89 / 13.17%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$751.33 / 13.20%</t>
+          <t>$751.89 / 13.29%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$751.33 / 5.80%</t>
+          <t>$751.89 / 5.88%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$751.33 / 16.77%</t>
+          <t>$751.89 / 16.85%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$751.33 / 10.39%</t>
+          <t>$751.89 / 10.48%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$751.33 / 8.98%</t>
+          <t>$751.89 / 9.06%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$751.33 / 8.63%</t>
+          <t>$751.89 / 8.71%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$751.33 / 19.72%</t>
+          <t>$751.89 / 19.81%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$751.33 / 0.61%</t>
+          <t>$751.89 / 0.69%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$751.33 / 15.84%</t>
+          <t>$751.89 / 15.93%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$751.33 / 1.65%</t>
+          <t>$751.89 / 1.72%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$751.33 / 14.01%</t>
+          <t>$751.89 / 14.09%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$751.33 / 13.09%</t>
+          <t>$751.89 / 13.17%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$751.33 / 13.20%</t>
+          <t>$751.89 / 13.29%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.86% (10.24%)</t>
+          <t>10.87% (10.25%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.34% (1.26%)</t>
+          <t>1.31% (1.23%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.46% (6.12%)</t>
+          <t>6.42% (6.08%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.38% (7.89%)</t>
+          <t>8.27% (7.79%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.62% (7.21%)</t>
+          <t>7.59% (7.19%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.03% (0.02%)</t>
+          <t>-0.02% (-0.03%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.78% (14.99%)</t>
+          <t>15.71% (14.92%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.55% (7.02%)</t>
+          <t>7.46% (6.93%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.21% (14.49%)</t>
+          <t>15.11% (14.40%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.17% (4.90%)</t>
+          <t>5.12% (4.85%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.17% (3.97%)</t>
+          <t>4.08% (3.88%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.04% (2.90%)</t>
+          <t>2.98% (2.85%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>8.98% (8.36%)</t>
+          <t>8.90% (8.28%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.00% (0.92%)</t>
+          <t>0.96% (0.88%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.19% (4.84%)</t>
+          <t>5.08% (4.74%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.73% (6.24%)</t>
+          <t>6.69% (6.20%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.10% (5.69%)</t>
+          <t>6.00% (5.59%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.04% (0.03%)</t>
+          <t>-0.01% (-0.01%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.84% (12.05%)</t>
+          <t>12.70% (11.92%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.50% (5.96%)</t>
+          <t>6.45% (5.91%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.15% (11.44%)</t>
+          <t>12.07% (11.36%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.93% (3.65%)</t>
+          <t>3.92% (3.64%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.05% (2.84%)</t>
+          <t>3.06% (2.86%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.23% (2.09%)</t>
+          <t>2.17% (2.03%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.85%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-2.12%</t>
+          <t>-2.19%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.95%</t>
+          <t>3.87%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.56%</t>
+          <t>5.46%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.46%</t>
+          <t>5.36%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>-4.39%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>15.65%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.17%</t>
+          <t>1.07%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15.19%</t>
+          <t>15.11%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.29%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.77%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.70%</t>
+          <t>0.63%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.18%</t>
+          <t>6.11%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-4.17%</t>
+          <t>-4.24%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>1.46%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.82%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2.93%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-6.41%</t>
+          <t>-6.48%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.66%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.50%</t>
+          <t>-1.58%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>11.99%</t>
+          <t>11.91%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-0.91%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.52%</t>
+          <t>-1.59%</t>
         </is>
       </c>
     </row>
@@ -2834,117 +2834,117 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.18% (10.55%)</t>
+          <t>11.25% (10.63%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.51% (11.43%)</t>
+          <t>11.53% (11.45%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.19% (10.85%)</t>
+          <t>11.22% (10.87%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.59% (11.10%)</t>
+          <t>11.57% (11.09%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.05% (10.64%)</t>
+          <t>11.10% (10.70%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.05% (12.04%)</t>
+          <t>12.06% (12.06%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.96% (9.18%)</t>
+          <t>9.97% (9.19%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.05% (13.51%)</t>
+          <t>14.04% (13.51%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.83% (9.11%)</t>
+          <t>9.81% (9.10%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.17% (10.89%)</t>
+          <t>11.19% (10.91%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.85% (10.65%)</t>
+          <t>10.83% (10.63%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.81% (10.67%)</t>
+          <t>10.82% (10.68%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.65% (16.02%)</t>
+          <t>16.64% (16.01%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.39% (17.31%)</t>
+          <t>17.41% (17.33%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.81% (16.46%)</t>
+          <t>16.77% (16.42%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.22% (16.72%)</t>
+          <t>17.24% (16.75%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.60% (16.19%)</t>
+          <t>16.57% (16.16%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>18.21% (18.20%)</t>
+          <t>18.22% (18.21%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.06% (14.27%)</t>
+          <t>15.00% (14.22%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.93% (19.39%)</t>
+          <t>19.94% (19.40%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.89% (14.17%)</t>
+          <t>14.88% (14.16%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.15% (16.87%)</t>
+          <t>17.19% (16.92%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.66% (16.46%)</t>
+          <t>16.73% (16.53%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.76% (-4.38%)</t>
+          <t>-3.75% (-4.37%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.41% (-11.50%)</t>
+          <t>-11.45% (-11.53%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.28% (-7.63%)</t>
+          <t>-7.32% (-7.66%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.81% (-6.29%)</t>
+          <t>-5.90% (-6.39%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-6.08% (-6.49%)</t>
+          <t>-6.11% (-6.51%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.77% (-12.78%)</t>
+          <t>-12.82% (-12.82%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.59% (-1.37%)</t>
+          <t>-0.65% (-1.43%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.24% (-8.78%)</t>
+          <t>-8.32% (-8.86%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.63% (-2.34%)</t>
+          <t>-1.71% (-2.42%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.89% (-10.16%)</t>
+          <t>-9.93% (-10.20%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.56% (-9.77%)</t>
+          <t>-9.64% (-9.84%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.69% (-9.83%)</t>
+          <t>-9.74% (-9.88%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-3.01% (-3.63%)</t>
+          <t>-3.08% (-3.70%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.81% (-9.89%)</t>
+          <t>-9.84% (-9.92%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.19% (-6.54%)</t>
+          <t>-6.29% (-6.64%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.78% (-5.28%)</t>
+          <t>-4.82% (-5.31%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.15% (-5.56%)</t>
+          <t>-5.23% (-5.64%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.79% (-10.80%)</t>
+          <t>-10.83% (-10.84%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.46% (-1.24%)</t>
+          <t>-0.58% (-1.36%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.69% (-7.23%)</t>
+          <t>-6.74% (-7.28%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.49% (-2.21%)</t>
+          <t>-1.56% (-2.27%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.29% (-8.57%)</t>
+          <t>-8.30% (-8.58%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.17% (-8.37%)</t>
+          <t>-8.16% (-8.36%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.36% (-8.50%)</t>
+          <t>-8.42% (-8.56%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.93%</t>
+          <t>-15.00%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.92%</t>
+          <t>-22.98%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.47%</t>
+          <t>-18.53%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.40%</t>
+          <t>-17.48%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-17.13%</t>
+          <t>-17.21%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.82%</t>
+          <t>-24.88%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.55%</t>
+          <t>-10.62%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.29%</t>
+          <t>-22.37%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.46%</t>
+          <t>-11.52%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.06%</t>
+          <t>-21.11%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.41%</t>
+          <t>-20.47%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.50%</t>
+          <t>-20.56%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.66%</t>
+          <t>-19.72%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-27.20%</t>
+          <t>-27.26%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.00%</t>
+          <t>-23.06%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.00%</t>
+          <t>-22.06%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.75%</t>
+          <t>-21.81%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-29.00%</t>
+          <t>-29.05%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.52%</t>
+          <t>-15.58%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.62%</t>
+          <t>-26.68%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.37%</t>
+          <t>-16.44%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.44%</t>
+          <t>-25.49%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.83%</t>
+          <t>-24.89%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.91%</t>
+          <t>-24.97%</t>
         </is>
       </c>
     </row>
@@ -3215,62 +3215,62 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.84% (1.21%)</t>
+          <t>1.92% (1.30%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.34% (1.26%)</t>
+          <t>1.31% (1.23%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.40% (2.06%)</t>
+          <t>2.44% (2.10%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.66% (2.17%)</t>
+          <t>2.65% (2.17%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.03% (1.62%)</t>
+          <t>2.10% (1.70%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.03% (0.02%)</t>
+          <t>-0.02% (-0.03%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.02% (-0.76%)</t>
+          <t>0.04% (-0.74%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.31% (5.78%)</t>
+          <t>6.32% (5.79%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.01% (-0.72%)</t>
+          <t>-0.01% (-0.73%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.80% (2.53%)</t>
+          <t>2.83% (2.56%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.34% (2.14%)</t>
+          <t>2.33% (2.13%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.32% (2.18%)</t>
+          <t>2.34% (2.20%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -3280,57 +3280,57 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.00% (0.92%)</t>
+          <t>0.96% (0.88%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.60% (3.25%)</t>
+          <t>3.57% (3.23%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.79% (3.30%)</t>
+          <t>3.83% (3.34%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.07% (2.65%)</t>
+          <t>3.05% (2.64%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.04% (0.03%)</t>
+          <t>-0.01% (-0.01%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.15% (-0.63%)</t>
+          <t>0.10% (-0.68%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.50% (5.96%)</t>
+          <t>6.45% (5.91%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.13% (-0.59%)</t>
+          <t>0.13% (-0.58%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.93% (3.65%)</t>
+          <t>3.92% (3.64%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.05% (2.84%)</t>
+          <t>3.06% (2.86%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.23% (2.09%)</t>
+          <t>2.17% (2.03%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 13/7/2026</t>
+          <t>As of 14/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.64%</t>
+          <t>10.70%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.21%</t>
+          <t>7.19%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.03%</t>
+          <t>6.06%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.60%</t>
+          <t>8.71%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.46%</t>
+          <t>5.36%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.49%</t>
+          <t>-6.51%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.10%</t>
+          <t>11.09%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.89%</t>
+          <t>7.79%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.81%</t>
+          <t>5.92%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.95%</t>
+          <t>9.06%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.56%</t>
+          <t>5.46%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.29%</t>
+          <t>-6.39%</t>
         </is>
       </c>
     </row>
@@ -3489,27 +3489,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.02%</t>
+          <t>6.93%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.69%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.82%</t>
+          <t>15.93%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.17%</t>
+          <t>1.07%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.78%</t>
+          <t>-8.86%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.55%</t>
+          <t>10.63%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.25%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.68%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.80%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.85%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.38%</t>
+          <t>-4.37%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.10%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.49%</t>
+          <t>14.40%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>1.60%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.65%</t>
+          <t>1.72%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>15.19%</t>
+          <t>15.11%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.34%</t>
+          <t>-2.42%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>9.19%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14.99%</t>
+          <t>14.92%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>0.59%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>15.65%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-1.43%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.04%</t>
+          <t>12.06%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.02%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.68%</t>
+          <t>13.74%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.72%</t>
+          <t>19.81%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>-4.39%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.78%</t>
+          <t>-12.82%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.43%</t>
+          <t>11.45%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.26%</t>
+          <t>1.23%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>12.05%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.77%</t>
+          <t>16.85%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.12%</t>
+          <t>-2.19%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.50%</t>
+          <t>-11.53%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.90%</t>
+          <t>2.85%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.20%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.70%</t>
+          <t>0.63%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.83%</t>
+          <t>-9.88%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>10.63%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>3.88%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.88%</t>
+          <t>9.98%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.09%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.77%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.77%</t>
+          <t>-9.84%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.89%</t>
+          <t>10.91%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.90%</t>
+          <t>4.85%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.37%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.01%</t>
+          <t>14.09%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.29%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.16%</t>
+          <t>-10.20%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.87%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.12%</t>
+          <t>6.08%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.34%</t>
+          <t>7.38%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.39%</t>
+          <t>10.48%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.95%</t>
+          <t>3.87%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.63%</t>
+          <t>-7.66%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 13/7/2026</t>
+          <t>As of 14/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.19%</t>
+          <t>16.16%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.69%</t>
+          <t>5.59%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>5.09%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.63%</t>
+          <t>8.71%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.93%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.56%</t>
+          <t>-5.64%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.72%</t>
+          <t>16.75%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>6.20%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.98%</t>
+          <t>9.06%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.82%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.28%</t>
+          <t>-5.31%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.39%</t>
+          <t>19.40%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.96%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.89%</t>
+          <t>6.94%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.84%</t>
+          <t>15.93%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.50%</t>
+          <t>-1.58%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.23%</t>
+          <t>-7.28%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.02%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.36%</t>
+          <t>8.28%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.90%</t>
+          <t>2.97%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.80%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.18%</t>
+          <t>6.11%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.63%</t>
+          <t>-3.70%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.17%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.44%</t>
+          <t>11.36%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.37%</t>
+          <t>1.44%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.65%</t>
+          <t>1.72%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.99%</t>
+          <t>11.91%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.21%</t>
+          <t>-2.27%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.22%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.05%</t>
+          <t>11.92%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.66%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.24%</t>
+          <t>-1.36%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.20%</t>
+          <t>18.21%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.03%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.16%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.72%</t>
+          <t>19.81%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-6.41%</t>
+          <t>-6.48%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.80%</t>
+          <t>-10.84%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>17.33%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.77%</t>
+          <t>16.85%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.17%</t>
+          <t>-4.24%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.89%</t>
+          <t>-9.92%</t>
         </is>
       </c>
     </row>
@@ -4226,27 +4226,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.37%</t>
+          <t>8.43%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.20%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.52%</t>
+          <t>-1.59%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.50%</t>
+          <t>-8.56%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.46%</t>
+          <t>16.53%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.22%</t>
+          <t>8.20%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.09%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-0.91%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.37%</t>
+          <t>-8.36%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.87%</t>
+          <t>16.92%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>3.64%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.44%</t>
+          <t>8.46%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.01%</t>
+          <t>14.09%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.57%</t>
+          <t>-8.58%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.46%</t>
+          <t>16.42%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>4.74%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>6.20%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.39%</t>
+          <t>10.48%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>1.46%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.54%</t>
+          <t>-6.64%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-15]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/14/2026 at 10:59 AM ET)</t>
+          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>276 days</t>
+          <t>275 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>38 days</t>
+          <t>37 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>157 days</t>
+          <t>156 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>220 days</t>
+          <t>219 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>185 days</t>
+          <t>184 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>338 days</t>
+          <t>337 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>248 days</t>
+          <t>247 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>311 days</t>
+          <t>310 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>129 days</t>
+          <t>128 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>94 days</t>
+          <t>93 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>66 days</t>
+          <t>65 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>276 days</t>
+          <t>275 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>38 days</t>
+          <t>37 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>157 days</t>
+          <t>156 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>220 days</t>
+          <t>219 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>185 days</t>
+          <t>184 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>338 days</t>
+          <t>337 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>248 days</t>
+          <t>247 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>311 days</t>
+          <t>310 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>129 days</t>
+          <t>128 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>94 days</t>
+          <t>93 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>66 days</t>
+          <t>65 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.94 / 3.68%</t>
+          <t>$47.01 / 3.85%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.80 / 12.05%</t>
+          <t>$56.84 / 12.13%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.77 / 7.38%</t>
+          <t>$54.86 / 7.55%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.34 / 5.92%</t>
+          <t>$61.41 / 6.04%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.44 / 6.06%</t>
+          <t>$55.52 / 6.22%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.83 / 13.74%</t>
+          <t>$59.82 / 13.72%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.23 / 0.59%</t>
+          <t>$60.32 / 0.74%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.56 / 8.79%</t>
+          <t>$52.59 / 8.84%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.45 / 1.60%</t>
+          <t>$56.55 / 1.77%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.79 / 10.42%</t>
+          <t>$58.86 / 10.54%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.65 / 9.98%</t>
+          <t>$52.71 / 10.10%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.46 / 10.02%</t>
+          <t>$55.53 / 10.16%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.85 / 2.97%</t>
+          <t>$41.91 / 3.10%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.62 / 10.06%</t>
+          <t>$41.63 / 10.09%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.03 / 6.20%</t>
+          <t>$40.06 / 6.28%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.21 / 4.71%</t>
+          <t>$44.27 / 4.85%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.24 / 5.09%</t>
+          <t>$45.28 / 5.18%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.63 / 11.21%</t>
+          <t>$43.60 / 11.15%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.37 / 0.53%</t>
+          <t>$41.40 / 0.61%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.41 / 6.94%</t>
+          <t>$44.47 / 7.07%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.26 / 1.44%</t>
+          <t>$43.33 / 1.61%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.00 / 8.46%</t>
+          <t>$42.03 / 8.55%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.73 / 8.20%</t>
+          <t>$41.80 / 8.39%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.18 / 8.43%</t>
+          <t>$41.21 / 8.50%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$751.89 / 5.88%</t>
+          <t>$753.46 / 6.10%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$751.89 / 16.85%</t>
+          <t>$753.46 / 17.10%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$751.89 / 10.48%</t>
+          <t>$753.46 / 10.71%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$751.89 / 9.06%</t>
+          <t>$753.46 / 9.29%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$751.89 / 8.71%</t>
+          <t>$753.46 / 8.94%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$751.89 / 19.81%</t>
+          <t>$753.46 / 20.06%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$751.89 / 0.69%</t>
+          <t>$753.46 / 0.90%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$751.89 / 15.93%</t>
+          <t>$753.46 / 16.17%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$751.89 / 1.72%</t>
+          <t>$753.46 / 1.93%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$751.89 / 14.09%</t>
+          <t>$753.46 / 14.33%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$751.89 / 13.17%</t>
+          <t>$753.46 / 13.41%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$751.89 / 13.29%</t>
+          <t>$753.46 / 13.52%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$751.89 / 5.88%</t>
+          <t>$753.46 / 6.10%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$751.89 / 16.85%</t>
+          <t>$753.46 / 17.10%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$751.89 / 10.48%</t>
+          <t>$753.46 / 10.71%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$751.89 / 9.06%</t>
+          <t>$753.46 / 9.29%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$751.89 / 8.71%</t>
+          <t>$753.46 / 8.94%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$751.89 / 19.81%</t>
+          <t>$753.46 / 20.06%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$751.89 / 0.69%</t>
+          <t>$753.46 / 0.90%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$751.89 / 15.93%</t>
+          <t>$753.46 / 16.17%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$751.89 / 1.72%</t>
+          <t>$753.46 / 1.93%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$751.89 / 14.09%</t>
+          <t>$753.46 / 14.33%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$751.89 / 13.17%</t>
+          <t>$753.46 / 13.41%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$751.89 / 13.29%</t>
+          <t>$753.46 / 13.52%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.87% (10.25%)</t>
+          <t>10.69% (10.08%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.31% (1.23%)</t>
+          <t>1.23% (1.16%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.42% (6.08%)</t>
+          <t>6.24% (5.90%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.27% (7.79%)</t>
+          <t>8.14% (7.66%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.59% (7.19%)</t>
+          <t>7.42% (7.02%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-0.02% (-0.03%)</t>
+          <t>-0.01% (-0.01%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.71% (14.92%)</t>
+          <t>15.53% (14.75%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.46% (6.93%)</t>
+          <t>7.41% (6.88%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.11% (14.40%)</t>
+          <t>14.92% (14.21%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.12% (4.85%)</t>
+          <t>5.01% (4.74%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.08% (3.88%)</t>
+          <t>3.96% (3.76%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2.98% (2.85%)</t>
+          <t>2.85% (2.72%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>8.90% (8.28%)</t>
+          <t>8.76% (8.14%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.96% (0.88%)</t>
+          <t>0.93% (0.86%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.08% (4.74%)</t>
+          <t>5.00% (4.66%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.69% (6.20%)</t>
+          <t>6.54% (6.06%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.00% (5.59%)</t>
+          <t>5.91% (5.50%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>-0.01% (-0.01%)</t>
+          <t>0.05% (0.04%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.70% (11.92%)</t>
+          <t>12.60% (11.82%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.45% (5.91%)</t>
+          <t>6.32% (5.78%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.07% (11.36%)</t>
+          <t>11.89% (11.18%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.92% (3.64%)</t>
+          <t>3.83% (3.55%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.06% (2.86%)</t>
+          <t>2.88% (2.68%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.17% (2.03%)</t>
+          <t>2.11% (1.97%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>8.54%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-2.19%</t>
+          <t>-2.40%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.87%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.46%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.36%</t>
+          <t>5.14%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-4.39%</t>
+          <t>-4.59%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>15.65%</t>
+          <t>15.41%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>0.86%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15.11%</t>
+          <t>14.87%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>2.00%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>1.49%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.63%</t>
+          <t>0.42%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.11%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-4.24%</t>
+          <t>-4.44%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.46%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-6.48%</t>
+          <t>-6.68%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.58%</t>
+          <t>12.34%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.58%</t>
+          <t>-1.78%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>11.91%</t>
+          <t>11.67%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.94%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.91%</t>
+          <t>-1.11%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.59%</t>
+          <t>-1.80%</t>
         </is>
       </c>
     </row>
@@ -2834,112 +2834,112 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.25% (10.63%)</t>
+          <t>11.27% (10.65%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.53% (11.45%)</t>
+          <t>11.63% (11.55%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.22% (10.87%)</t>
+          <t>11.23% (10.89%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.57% (11.09%)</t>
+          <t>11.64% (11.16%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.10% (10.70%)</t>
+          <t>11.13% (10.73%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.06% (12.06%)</t>
+          <t>12.23% (12.23%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.97% (9.19%)</t>
+          <t>10.00% (9.23%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.04% (13.51%)</t>
+          <t>14.16% (13.63%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.81% (9.10%)</t>
+          <t>9.83% (9.12%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.19% (10.91%)</t>
+          <t>11.25% (10.98%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.83% (10.63%)</t>
+          <t>10.89% (10.69%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.82% (10.68%)</t>
+          <t>10.87% (10.73%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.64% (16.01%)</t>
+          <t>16.68% (16.05%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.41% (17.33%)</t>
+          <t>17.54% (17.46%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.77% (16.42%)</t>
+          <t>16.86% (16.51%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.24% (16.75%)</t>
+          <t>17.27% (16.78%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.57% (16.16%)</t>
+          <t>16.65% (16.24%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>18.22% (18.21%)</t>
+          <t>18.41% (18.41%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.00% (14.22%)</t>
+          <t>15.09% (14.31%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.94% (19.40%)</t>
+          <t>19.98% (19.44%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.88% (14.16%)</t>
+          <t>14.89% (14.18%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.19% (16.92%)</t>
+          <t>17.27% (17.00%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.55% (16.41%)</t>
+          <t>16.65% (16.51%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.75% (-4.37%)</t>
+          <t>-3.91% (-4.52%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.45% (-11.53%)</t>
+          <t>-11.51% (-11.59%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.32% (-7.66%)</t>
+          <t>-7.47% (-7.81%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.90% (-6.39%)</t>
+          <t>-6.01% (-6.49%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-6.11% (-6.51%)</t>
+          <t>-6.25% (-6.66%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.82% (-12.82%)</t>
+          <t>-12.80% (-12.81%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.65% (-1.43%)</t>
+          <t>-0.80% (-1.58%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.32% (-8.86%)</t>
+          <t>-8.37% (-8.90%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.71% (-2.42%)</t>
+          <t>-1.88% (-2.58%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.93% (-10.20%)</t>
+          <t>-10.03% (-10.30%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.64% (-9.84%)</t>
+          <t>-9.75% (-9.95%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.74% (-9.88%)</t>
+          <t>-9.86% (-9.99%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-3.08% (-3.70%)</t>
+          <t>-3.21% (-3.83%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.84% (-9.92%)</t>
+          <t>-9.87% (-9.95%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.29% (-6.64%)</t>
+          <t>-6.36% (-6.71%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.82% (-5.31%)</t>
+          <t>-4.95% (-5.44%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.23% (-5.64%)</t>
+          <t>-5.32% (-5.73%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.83% (-10.84%)</t>
+          <t>-10.79% (-10.79%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.58% (-1.36%)</t>
+          <t>-0.67% (-1.45%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.74% (-7.28%)</t>
+          <t>-6.85% (-7.39%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.56% (-2.27%)</t>
+          <t>-1.72% (-2.43%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.30% (-8.58%)</t>
+          <t>-8.38% (-8.65%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.16% (-8.36%)</t>
+          <t>-8.32% (-8.52%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.42% (-8.56%)</t>
+          <t>-8.47% (-8.61%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.00%</t>
+          <t>-15.17%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.98%</t>
+          <t>-23.14%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.53%</t>
+          <t>-18.70%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.48%</t>
+          <t>-17.65%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-17.21%</t>
+          <t>-17.38%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.88%</t>
+          <t>-25.04%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.62%</t>
+          <t>-10.80%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.37%</t>
+          <t>-22.53%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.52%</t>
+          <t>-11.71%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.11%</t>
+          <t>-21.28%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.47%</t>
+          <t>-20.64%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.56%</t>
+          <t>-20.72%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.72%</t>
+          <t>-19.88%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-27.26%</t>
+          <t>-27.41%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.06%</t>
+          <t>-23.22%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.06%</t>
+          <t>-22.22%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.81%</t>
+          <t>-21.97%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-29.05%</t>
+          <t>-29.20%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.58%</t>
+          <t>-15.76%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.68%</t>
+          <t>-26.83%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.44%</t>
+          <t>-16.61%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.49%</t>
+          <t>-25.65%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.89%</t>
+          <t>-25.05%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.97%</t>
+          <t>-25.12%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.92% (1.30%)</t>
+          <t>1.97% (1.35%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.31% (1.23%)</t>
+          <t>1.23% (1.16%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.44% (2.10%)</t>
+          <t>2.48% (2.14%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.65% (2.17%)</t>
+          <t>2.75% (2.27%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.10% (1.70%)</t>
+          <t>2.16% (1.75%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.03%)</t>
+          <t>-0.01% (-0.01%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.04% (-0.74%)</t>
+          <t>0.10% (-0.68%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.32% (5.79%)</t>
+          <t>6.49% (5.96%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.01% (-0.73%)</t>
+          <t>0.02% (-0.68%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.83% (2.56%)</t>
+          <t>2.93% (2.66%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.33% (2.13%)</t>
+          <t>2.43% (2.23%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.34% (2.20%)</t>
+          <t>2.42% (2.28%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.63% (2.00%)</t>
+          <t>2.70% (2.08%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.96% (0.88%)</t>
+          <t>0.93% (0.86%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.57% (3.23%)</t>
+          <t>3.71% (3.37%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.83% (3.34%)</t>
+          <t>3.91% (3.42%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.05% (2.64%)</t>
+          <t>3.17% (2.76%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>-0.01% (-0.01%)</t>
+          <t>0.05% (0.04%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.10% (-0.68%)</t>
+          <t>0.23% (-0.55%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.45% (5.91%)</t>
+          <t>6.32% (5.78%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.13% (-0.58%)</t>
+          <t>0.18% (-0.53%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.92% (3.64%)</t>
+          <t>3.83% (3.55%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.06% (2.86%)</t>
+          <t>2.88% (2.68%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.17% (2.03%)</t>
+          <t>2.11% (1.97%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 14/7/2026</t>
+          <t>As of 15/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.70%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.19%</t>
+          <t>7.02%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.06%</t>
+          <t>6.22%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.71%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.36%</t>
+          <t>5.14%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.51%</t>
+          <t>-6.66%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.09%</t>
+          <t>11.16%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.79%</t>
+          <t>7.66%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.92%</t>
+          <t>6.04%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.06%</t>
+          <t>9.29%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.46%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.39%</t>
+          <t>-6.49%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.51%</t>
+          <t>13.63%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.93%</t>
+          <t>6.88%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>8.84%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.93%</t>
+          <t>16.17%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>0.86%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.86%</t>
+          <t>-8.90%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.63%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.25%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.68%</t>
+          <t>3.85%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>6.10%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>8.54%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.37%</t>
+          <t>-4.52%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.10%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.40%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>1.77%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.72%</t>
+          <t>1.93%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>15.11%</t>
+          <t>14.87%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.42%</t>
+          <t>-2.58%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.19%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14.92%</t>
+          <t>14.75%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.59%</t>
+          <t>0.74%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.65%</t>
+          <t>15.41%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>-1.58%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.06%</t>
+          <t>12.23%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.74%</t>
+          <t>13.72%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.81%</t>
+          <t>20.06%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.39%</t>
+          <t>-4.59%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.82%</t>
+          <t>-12.81%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.45%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.23%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.05%</t>
+          <t>12.13%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.85%</t>
+          <t>17.10%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.19%</t>
+          <t>-2.40%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.53%</t>
+          <t>-11.59%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.85%</t>
+          <t>2.72%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>10.16%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>13.52%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.63%</t>
+          <t>0.42%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.88%</t>
+          <t>-9.99%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.63%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.88%</t>
+          <t>3.76%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>10.10%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>13.41%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>1.49%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.84%</t>
+          <t>-9.95%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.91%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.85%</t>
+          <t>4.74%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>10.54%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.09%</t>
+          <t>14.33%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>2.00%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.20%</t>
+          <t>-10.30%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.87%</t>
+          <t>10.89%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.08%</t>
+          <t>5.90%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.38%</t>
+          <t>7.55%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.48%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.87%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.66%</t>
+          <t>-7.81%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 14/7/2026</t>
+          <t>As of 15/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.16%</t>
+          <t>16.24%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.59%</t>
+          <t>5.50%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.09%</t>
+          <t>5.18%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.71%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.64%</t>
+          <t>-5.73%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.75%</t>
+          <t>16.78%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.20%</t>
+          <t>6.06%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.85%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.06%</t>
+          <t>9.29%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.31%</t>
+          <t>-5.44%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.40%</t>
+          <t>19.44%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>5.78%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.94%</t>
+          <t>7.07%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.93%</t>
+          <t>16.17%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.58%</t>
+          <t>-1.78%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.28%</t>
+          <t>-7.39%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.28%</t>
+          <t>8.14%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.97%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>6.10%</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>5.88%</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>6.11%</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.70%</t>
+          <t>-3.83%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>14.18%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.36%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.44%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.72%</t>
+          <t>1.93%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.91%</t>
+          <t>11.67%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.27%</t>
+          <t>-2.43%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.22%</t>
+          <t>14.31%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.92%</t>
+          <t>11.82%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.58%</t>
+          <t>12.34%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.36%</t>
+          <t>-1.45%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.21%</t>
+          <t>18.41%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>11.15%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>19.81%</t>
+          <t>20.06%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-6.48%</t>
+          <t>-6.68%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.84%</t>
+          <t>-10.79%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.33%</t>
+          <t>17.46%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>0.86%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.06%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.85%</t>
+          <t>17.10%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.24%</t>
+          <t>-4.44%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.92%</t>
+          <t>-9.95%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.41%</t>
+          <t>16.51%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>1.97%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.43%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>13.52%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.59%</t>
+          <t>-1.80%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.56%</t>
+          <t>-8.61%</t>
         </is>
       </c>
     </row>
@@ -4263,27 +4263,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.68%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.20%</t>
+          <t>8.39%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>13.41%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.91%</t>
+          <t>-1.11%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.36%</t>
+          <t>-8.52%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.92%</t>
+          <t>17.00%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.64%</t>
+          <t>3.55%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.46%</t>
+          <t>8.55%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.09%</t>
+          <t>14.33%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.94%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.58%</t>
+          <t>-8.65%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.42%</t>
+          <t>16.51%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.74%</t>
+          <t>4.66%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.20%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.48%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.46%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.64%</t>
+          <t>-6.71%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-16]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/15/2026 at 11:01 AM ET)</t>
+          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>275 days</t>
+          <t>274 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>37 days</t>
+          <t>36 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>156 days</t>
+          <t>155 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>219 days</t>
+          <t>218 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>184 days</t>
+          <t>183 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>1 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>337 days</t>
+          <t>336 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>247 days</t>
+          <t>246 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>310 days</t>
+          <t>309 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>128 days</t>
+          <t>127 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>93 days</t>
+          <t>92 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>65 days</t>
+          <t>64 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>275 days</t>
+          <t>274 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>37 days</t>
+          <t>36 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>156 days</t>
+          <t>155 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>219 days</t>
+          <t>218 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>184 days</t>
+          <t>183 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>1 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>337 days</t>
+          <t>336 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>247 days</t>
+          <t>246 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>310 days</t>
+          <t>309 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>128 days</t>
+          <t>127 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>93 days</t>
+          <t>92 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>65 days</t>
+          <t>64 days</t>
         </is>
       </c>
     </row>
@@ -2326,62 +2326,62 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.01 / 3.85%</t>
+          <t>$47.03 / 3.88%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.84 / 12.13%</t>
+          <t>$56.87 / 12.19%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.86 / 7.55%</t>
+          <t>$54.86 / 7.54%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.41 / 6.04%</t>
+          <t>$61.44 / 6.08%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.52 / 6.22%</t>
+          <t>$55.55 / 6.28%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.82 / 13.72%</t>
+          <t>$59.82 / 13.73%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.32 / 0.74%</t>
+          <t>$60.36 / 0.82%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.59 / 8.84%</t>
+          <t>$52.62 / 8.90%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.55 / 1.77%</t>
+          <t>$56.56 / 1.78%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.86 / 10.54%</t>
+          <t>$58.90 / 10.62%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.71 / 10.10%</t>
+          <t>$52.75 / 10.20%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.53 / 10.16%</t>
+          <t>$55.55 / 10.19%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2391,12 +2391,12 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.63 / 10.09%</t>
+          <t>$41.64 / 10.11%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.06 / 6.28%</t>
+          <t>$40.07 / 6.31%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2411,12 +2411,12 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.60 / 11.15%</t>
+          <t>$43.66 / 11.29%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.40 / 0.61%</t>
+          <t>$41.42 / 0.65%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2426,17 +2426,17 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.33 / 1.61%</t>
+          <t>$43.33 / 1.62%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.03 / 8.55%</t>
+          <t>$42.04 / 8.57%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.80 / 8.39%</t>
+          <t>$41.78 / 8.32%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$753.46 / 6.10%</t>
+          <t>$753.29 / 6.08%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$753.46 / 17.10%</t>
+          <t>$753.29 / 17.07%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$753.46 / 10.71%</t>
+          <t>$753.26 / 10.68%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$753.46 / 9.29%</t>
+          <t>$753.29 / 9.26%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$753.46 / 8.94%</t>
+          <t>$753.29 / 8.91%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$753.46 / 20.06%</t>
+          <t>$753.29 / 20.03%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$753.46 / 0.90%</t>
+          <t>$753.29 / 0.88%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$753.46 / 16.17%</t>
+          <t>$753.29 / 16.15%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$753.46 / 1.93%</t>
+          <t>$753.29 / 1.91%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$753.46 / 14.33%</t>
+          <t>$753.26 / 14.30%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$753.46 / 13.41%</t>
+          <t>$753.29 / 13.38%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$753.46 / 13.52%</t>
+          <t>$753.29 / 13.50%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$753.46 / 6.10%</t>
+          <t>$753.26 / 6.07%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$753.46 / 17.10%</t>
+          <t>$753.26 / 17.07%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$753.46 / 10.71%</t>
+          <t>$753.26 / 10.68%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$753.46 / 9.29%</t>
+          <t>$753.26 / 9.26%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$753.46 / 8.94%</t>
+          <t>$753.26 / 8.91%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$753.46 / 20.06%</t>
+          <t>$753.26 / 20.03%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$753.46 / 0.90%</t>
+          <t>$753.26 / 0.87%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$753.46 / 16.17%</t>
+          <t>$753.26 / 16.14%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$753.46 / 1.93%</t>
+          <t>$753.26 / 1.91%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$753.46 / 14.33%</t>
+          <t>$753.26 / 14.30%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$753.46 / 13.41%</t>
+          <t>$753.26 / 13.38%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$753.46 / 13.52%</t>
+          <t>$753.26 / 13.49%</t>
         </is>
       </c>
     </row>
@@ -2580,62 +2580,62 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.69% (10.08%)</t>
+          <t>10.65% (10.04%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.23% (1.16%)</t>
+          <t>1.18% (1.10%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.24% (5.90%)</t>
+          <t>6.25% (5.91%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.14% (7.66%)</t>
+          <t>8.10% (7.62%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.42% (7.02%)</t>
+          <t>7.36% (6.96%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-0.01% (-0.01%)</t>
+          <t>-0.02% (-0.02%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.53% (14.75%)</t>
+          <t>15.44% (14.67%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.41% (6.88%)</t>
+          <t>7.34% (6.82%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>14.92% (14.21%)</t>
+          <t>14.90% (14.19%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.01% (4.74%)</t>
+          <t>4.92% (4.66%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>3.96% (3.76%)</t>
+          <t>3.87% (3.67%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2.85% (2.72%)</t>
+          <t>2.82% (2.69%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.93% (0.86%)</t>
+          <t>0.91% (0.83%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.00% (4.66%)</t>
+          <t>4.98% (4.64%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2665,37 +2665,37 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.05% (0.04%)</t>
+          <t>-0.08% (-0.08%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.60% (11.82%)</t>
+          <t>12.56% (11.78%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.32% (5.78%)</t>
+          <t>6.31% (5.78%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>11.89% (11.18%)</t>
+          <t>11.88% (11.17%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.83% (3.55%)</t>
+          <t>3.80% (3.53%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2.88% (2.68%)</t>
+          <t>2.94% (2.75%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.11% (1.97%)</t>
+          <t>2.10% (1.97%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.54%</t>
+          <t>8.56%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-2.40%</t>
+          <t>-2.38%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>3.68%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>5.26%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.14%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-4.59%</t>
+          <t>-4.57%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>15.41%</t>
+          <t>15.44%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.86%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>14.87%</t>
+          <t>14.90%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.00%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.49%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.44%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-4.44%</t>
+          <t>-4.42%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>1.27%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2.64%</t>
+          <t>2.67%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-6.68%</t>
+          <t>-6.65%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.34%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.78%</t>
+          <t>-1.75%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>11.67%</t>
+          <t>11.70%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.94%</t>
+          <t>-0.91%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-1.11%</t>
+          <t>-1.09%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.80%</t>
+          <t>-1.77%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.27% (10.65%)</t>
+          <t>11.22% (10.60%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.63% (11.55%)</t>
+          <t>11.56% (11.49%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.23% (10.89%)</t>
+          <t>11.22% (10.88%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.64% (11.16%)</t>
+          <t>11.58% (11.10%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.13% (10.73%)</t>
+          <t>11.06% (10.66%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.23% (12.23%)</t>
+          <t>12.21% (12.20%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.00% (9.23%)</t>
+          <t>9.91% (9.13%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.16% (13.63%)</t>
+          <t>14.09% (13.56%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.83% (9.12%)</t>
+          <t>9.79% (9.09%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.25% (10.98%)</t>
+          <t>11.16% (10.89%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.89% (10.69%)</t>
+          <t>10.79% (10.60%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.87% (10.73%)</t>
+          <t>10.82% (10.69%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.68% (16.05%)</t>
+          <t>16.65% (16.03%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.54% (17.46%)</t>
+          <t>17.50% (17.42%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.86% (16.51%)</t>
+          <t>16.81% (16.47%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.27% (16.78%)</t>
+          <t>17.25% (16.76%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.65% (16.24%)</t>
+          <t>16.63% (16.22%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>18.41% (18.41%)</t>
+          <t>18.28% (18.28%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.09% (14.31%)</t>
+          <t>15.03% (14.25%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.98% (19.44%)</t>
+          <t>19.96% (19.42%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.89% (14.18%)</t>
+          <t>14.85% (14.15%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.27% (17.00%)</t>
+          <t>17.23% (16.96%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.73% (16.53%)</t>
+          <t>16.76% (16.56%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.65% (16.51%)</t>
+          <t>16.63% (16.49%)</t>
         </is>
       </c>
     </row>
@@ -2961,62 +2961,62 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.91% (-4.52%)</t>
+          <t>-3.94% (-4.55%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.51% (-11.59%)</t>
+          <t>-11.56% (-11.64%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.47% (-7.81%)</t>
+          <t>-7.47% (-7.80%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-6.01% (-6.49%)</t>
+          <t>-6.05% (-6.53%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-6.25% (-6.66%)</t>
+          <t>-6.31% (-6.71%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.80% (-12.81%)</t>
+          <t>-12.81% (-12.82%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.80% (-1.58%)</t>
+          <t>-0.87% (-1.65%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.37% (-8.90%)</t>
+          <t>-8.43% (-8.95%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.88% (-2.58%)</t>
+          <t>-1.89% (-2.60%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-10.03% (-10.30%)</t>
+          <t>-10.10% (-10.37%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.75% (-9.95%)</t>
+          <t>-9.83% (-10.02%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.86% (-9.99%)</t>
+          <t>-9.88% (-10.02%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -3026,12 +3026,12 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.87% (-9.95%)</t>
+          <t>-9.89% (-9.97%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.36% (-6.71%)</t>
+          <t>-6.39% (-6.73%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -3046,12 +3046,12 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.79% (-10.79%)</t>
+          <t>-10.90% (-10.90%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.67% (-1.45%)</t>
+          <t>-0.70% (-1.48%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -3061,22 +3061,22 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.72% (-2.43%)</t>
+          <t>-1.73% (-2.44%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.38% (-8.65%)</t>
+          <t>-8.40% (-8.67%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.32% (-8.52%)</t>
+          <t>-8.26% (-8.46%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.47% (-8.61%)</t>
+          <t>-8.48% (-8.61%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.17%</t>
+          <t>-15.15%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-23.14%</t>
+          <t>-23.12%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.70%</t>
+          <t>-18.68%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.65%</t>
+          <t>-17.63%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-17.38%</t>
+          <t>-17.36%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-25.04%</t>
+          <t>-25.02%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.80%</t>
+          <t>-10.78%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.53%</t>
+          <t>-22.51%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.71%</t>
+          <t>-11.69%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.28%</t>
+          <t>-21.26%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.64%</t>
+          <t>-20.62%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.72%</t>
+          <t>-20.70%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.88%</t>
+          <t>-19.86%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-27.41%</t>
+          <t>-27.39%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.22%</t>
+          <t>-23.20%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.22%</t>
+          <t>-22.20%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.97%</t>
+          <t>-21.95%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-29.20%</t>
+          <t>-29.18%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.76%</t>
+          <t>-15.73%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.83%</t>
+          <t>-26.81%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.61%</t>
+          <t>-16.59%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.65%</t>
+          <t>-25.63%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-25.05%</t>
+          <t>-25.03%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.12%</t>
+          <t>-25.10%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.97% (1.35%)</t>
+          <t>1.91% (1.30%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.23% (1.16%)</t>
+          <t>1.18% (1.10%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.48% (2.14%)</t>
+          <t>2.46% (2.13%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.75% (2.27%)</t>
+          <t>2.68% (2.20%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.16% (1.75%)</t>
+          <t>2.08% (1.68%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-0.01% (-0.01%)</t>
+          <t>-0.02% (-0.02%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.10% (-0.68%)</t>
+          <t>0.00% (-0.78%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.49% (5.96%)</t>
+          <t>6.40% (5.87%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.02% (-0.68%)</t>
+          <t>-0.02% (-0.73%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.93% (2.66%)</t>
+          <t>2.82% (2.56%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.43% (2.23%)</t>
+          <t>2.31% (2.12%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.42% (2.28%)</t>
+          <t>2.37% (2.23%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.70% (2.08%)</t>
+          <t>2.67% (2.06%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.93% (0.86%)</t>
+          <t>0.91% (0.83%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.71% (3.37%)</t>
+          <t>3.65% (3.31%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.91% (3.42%)</t>
+          <t>3.87% (3.39%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.17% (2.76%)</t>
+          <t>3.14% (2.74%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.05% (0.04%)</t>
+          <t>-0.08% (-0.08%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.23% (-0.55%)</t>
+          <t>0.16% (-0.62%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.32% (5.78%)</t>
+          <t>6.31% (5.78%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.18% (-0.53%)</t>
+          <t>0.14% (-0.57%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.83% (3.55%)</t>
+          <t>3.80% (3.53%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.88% (2.68%)</t>
+          <t>2.94% (2.75%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.11% (1.97%)</t>
+          <t>2.10% (1.97%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 15/7/2026</t>
+          <t>As of 16/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.02%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.22%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.14%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.66%</t>
+          <t>-6.71%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.16%</t>
+          <t>11.10%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.66%</t>
+          <t>7.62%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.04%</t>
+          <t>6.08%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.29%</t>
+          <t>9.26%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>5.26%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.49%</t>
+          <t>-6.53%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.63%</t>
+          <t>13.56%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.88%</t>
+          <t>6.82%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.84%</t>
+          <t>8.90%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.17%</t>
+          <t>16.15%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.86%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.90%</t>
+          <t>-8.95%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>10.04%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.85%</t>
+          <t>3.88%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>6.08%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.54%</t>
+          <t>8.56%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.52%</t>
+          <t>-4.55%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>9.09%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>14.19%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.77%</t>
+          <t>1.78%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.93%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.87%</t>
+          <t>14.90%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.58%</t>
+          <t>-2.60%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14.75%</t>
+          <t>14.67%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.74%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.41%</t>
+          <t>15.44%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.58%</t>
+          <t>-1.65%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.23%</t>
+          <t>12.20%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.72%</t>
+          <t>13.73%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20.06%</t>
+          <t>20.03%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.59%</t>
+          <t>-4.57%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.81%</t>
+          <t>-12.82%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>11.49%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.16%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.13%</t>
+          <t>12.19%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>17.10%</t>
+          <t>17.07%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.40%</t>
+          <t>-2.38%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.59%</t>
+          <t>-11.64%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.72%</t>
+          <t>2.69%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.16%</t>
+          <t>10.19%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.50%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.44%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.99%</t>
+          <t>-10.02%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>3.67%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.10%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.49%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.95%</t>
+          <t>-10.02%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>10.89%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.74%</t>
+          <t>4.66%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.54%</t>
+          <t>10.62%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.33%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.00%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.30%</t>
+          <t>-10.37%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.89%</t>
+          <t>10.88%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.90%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.55%</t>
+          <t>7.54%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>3.68%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.81%</t>
+          <t>-7.80%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 15/7/2026</t>
+          <t>As of 16/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,7 +3925,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.24%</t>
+          <t>16.22%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3940,12 +3940,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.64%</t>
+          <t>2.67%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.78%</t>
+          <t>16.76%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3977,12 +3977,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.29%</t>
+          <t>9.26%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.44%</t>
+          <t>19.42%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4014,12 +4014,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.17%</t>
+          <t>16.14%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.78%</t>
+          <t>-1.75%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>16.03%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4051,12 +4051,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.18%</t>
+          <t>14.15%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>11.17%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.93%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.67%</t>
+          <t>11.70%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.43%</t>
+          <t>-2.44%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.31%</t>
+          <t>14.25%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.82%</t>
+          <t>11.78%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>0.87%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.34%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.45%</t>
+          <t>-1.48%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.41%</t>
+          <t>18.28%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.08%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.15%</t>
+          <t>11.29%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20.06%</t>
+          <t>20.03%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-6.68%</t>
+          <t>-6.65%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.79%</t>
+          <t>-10.90%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.46%</t>
+          <t>17.42%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.86%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>10.11%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>17.10%</t>
+          <t>17.07%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.44%</t>
+          <t>-4.42%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.95%</t>
+          <t>-9.97%</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.51%</t>
+          <t>16.49%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4236,12 +4236,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.80%</t>
+          <t>-1.77%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.53%</t>
+          <t>16.56%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.68%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.39%</t>
+          <t>8.32%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.11%</t>
+          <t>-1.09%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.52%</t>
+          <t>-8.46%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.00%</t>
+          <t>16.96%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.55%</t>
+          <t>3.53%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.55%</t>
+          <t>8.57%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.33%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.94%</t>
+          <t>-0.91%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.65%</t>
+          <t>-8.67%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.51%</t>
+          <t>16.47%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.66%</t>
+          <t>4.64%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>1.27%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.71%</t>
+          <t>-6.73%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-17]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:08 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/16/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>274 days</t>
+          <t>273 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>36 days</t>
+          <t>35 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>155 days</t>
+          <t>154 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>218 days</t>
+          <t>217 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>183 days</t>
+          <t>182 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1 days</t>
+          <t>0 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>336 days</t>
+          <t>335 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>246 days</t>
+          <t>245 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>309 days</t>
+          <t>308 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>127 days</t>
+          <t>126 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>92 days</t>
+          <t>91 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>64 days</t>
+          <t>63 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>274 days</t>
+          <t>273 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>36 days</t>
+          <t>35 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>155 days</t>
+          <t>154 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>218 days</t>
+          <t>217 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>183 days</t>
+          <t>182 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1 days</t>
+          <t>0 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>336 days</t>
+          <t>335 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>246 days</t>
+          <t>245 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>309 days</t>
+          <t>308 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>127 days</t>
+          <t>126 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>92 days</t>
+          <t>91 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>64 days</t>
+          <t>63 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.03 / 3.88%</t>
+          <t>$46.78 / 3.34%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.87 / 12.19%</t>
+          <t>$56.67 / 11.81%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.86 / 7.54%</t>
+          <t>$54.61 / 7.05%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.44 / 6.08%</t>
+          <t>$61.15 / 5.59%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.55 / 6.28%</t>
+          <t>$55.26 / 5.72%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.82 / 13.73%</t>
+          <t>$59.85 / 13.77%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.36 / 0.82%</t>
+          <t>$60.00 / 0.21%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.62 / 8.90%</t>
+          <t>$52.42 / 8.50%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.56 / 1.78%</t>
+          <t>$56.21 / 1.15%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.90 / 10.62%</t>
+          <t>$58.63 / 10.11%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.75 / 10.20%</t>
+          <t>$52.49 / 9.65%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.55 / 10.19%</t>
+          <t>$55.30 / 9.70%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.91 / 3.10%</t>
+          <t>$41.76 / 2.75%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.64 / 10.11%</t>
+          <t>$41.56 / 9.92%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.07 / 6.31%</t>
+          <t>$39.92 / 5.92%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.27 / 4.85%</t>
+          <t>$44.12 / 4.50%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.28 / 5.18%</t>
+          <t>$45.14 / 4.84%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.66 / 11.29%</t>
+          <t>$43.65 / 11.26%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.42 / 0.65%</t>
+          <t>$41.22 / 0.16%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.47 / 7.07%</t>
+          <t>$44.40 / 6.90%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.33 / 1.62%</t>
+          <t>$43.12 / 1.12%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.04 / 8.57%</t>
+          <t>$41.93 / 8.29%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.78 / 8.32%</t>
+          <t>$41.67 / 8.05%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.21 / 8.50%</t>
+          <t>$41.10 / 8.22%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$753.29 / 6.08%</t>
+          <t>$746.08 / 5.06%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$753.29 / 17.07%</t>
+          <t>$746.08 / 15.95%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$753.26 / 10.68%</t>
+          <t>$746.08 / 9.62%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$753.29 / 9.26%</t>
+          <t>$746.08 / 8.22%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$753.29 / 8.91%</t>
+          <t>$746.08 / 7.87%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$753.29 / 20.03%</t>
+          <t>$746.08 / 18.88%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$753.29 / 0.88%</t>
+          <t>$746.08 / -0.09%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$753.29 / 16.15%</t>
+          <t>$746.08 / 15.03%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$753.29 / 1.91%</t>
+          <t>$746.08 / 0.93%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$753.26 / 14.30%</t>
+          <t>$746.08 / 13.21%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$753.29 / 13.38%</t>
+          <t>$746.08 / 12.29%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$753.29 / 13.50%</t>
+          <t>$746.08 / 12.41%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$753.26 / 6.07%</t>
+          <t>$746.08 / 5.06%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$753.26 / 17.07%</t>
+          <t>$746.08 / 15.95%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$753.26 / 10.68%</t>
+          <t>$746.08 / 9.62%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$753.26 / 9.26%</t>
+          <t>$746.08 / 8.22%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$753.26 / 8.91%</t>
+          <t>$746.08 / 7.87%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$753.26 / 20.03%</t>
+          <t>$746.08 / 18.88%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$753.26 / 0.87%</t>
+          <t>$746.08 / -0.09%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$753.26 / 16.14%</t>
+          <t>$746.08 / 15.03%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$753.26 / 1.91%</t>
+          <t>$746.08 / 0.93%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$753.26 / 14.30%</t>
+          <t>$746.08 / 13.21%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$753.26 / 13.38%</t>
+          <t>$746.08 / 12.29%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$753.26 / 13.49%</t>
+          <t>$746.08 / 12.41%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.65% (10.04%)</t>
+          <t>11.23% (10.62%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.18% (1.10%)</t>
+          <t>1.52% (1.45%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.25% (5.91%)</t>
+          <t>6.73% (6.40%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.10% (7.62%)</t>
+          <t>8.60% (8.12%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.36% (6.96%)</t>
+          <t>7.94% (7.53%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-0.02% (-0.02%)</t>
+          <t>-0.06% (-0.06%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.44% (14.67%)</t>
+          <t>16.14% (15.36%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.34% (6.82%)</t>
+          <t>7.74% (7.21%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>14.90% (14.19%)</t>
+          <t>15.61% (14.90%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>4.92% (4.66%)</t>
+          <t>5.41% (5.15%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>3.87% (3.67%)</t>
+          <t>4.38% (4.19%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2.82% (2.69%)</t>
+          <t>3.29% (3.15%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>8.76% (8.14%)</t>
+          <t>9.13% (8.51%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.91% (0.83%)</t>
+          <t>1.09% (1.01%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>4.98% (4.64%)</t>
+          <t>5.35% (5.02%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.54% (6.06%)</t>
+          <t>6.90% (6.42%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>5.91% (5.50%)</t>
+          <t>6.24% (5.84%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>-0.08% (-0.08%)</t>
+          <t>-0.06% (-0.06%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.56% (11.78%)</t>
+          <t>13.10% (12.32%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.31% (5.78%)</t>
+          <t>6.48% (5.95%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>11.88% (11.17%)</t>
+          <t>12.43% (11.72%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.80% (3.53%)</t>
+          <t>4.07% (3.80%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2.94% (2.75%)</t>
+          <t>3.20% (3.01%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.10% (1.97%)</t>
+          <t>2.36% (2.23%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.56%</t>
+          <t>9.61%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-2.38%</t>
+          <t>-1.43%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.68%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.26%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.16%</t>
+          <t>6.18%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-4.57%</t>
+          <t>-3.64%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>15.44%</t>
+          <t>16.55%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>1.86%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>14.90%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>2.49%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>1.41%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>6.93%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-4.42%</t>
+          <t>-3.50%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>2.25%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>3.55%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2.67%</t>
+          <t>3.66%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-6.65%</t>
+          <t>-5.75%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>13.45%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-0.81%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>11.70%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.91%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-1.09%</t>
+          <t>-0.13%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.77%</t>
+          <t>-0.83%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.22% (10.60%)</t>
+          <t>10.90% (10.28%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.56% (11.49%)</t>
+          <t>11.12% (11.05%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.22% (10.88%)</t>
+          <t>10.85% (10.52%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.58% (11.10%)</t>
+          <t>11.22% (10.74%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.06% (10.66%)</t>
+          <t>10.76% (10.36%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.21% (12.20%)</t>
+          <t>11.44% (11.44%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.91% (9.13%)</t>
+          <t>9.65% (8.87%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.09% (13.56%)</t>
+          <t>13.68% (13.15%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.79% (9.09%)</t>
+          <t>9.55% (8.84%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.16% (10.89%)</t>
+          <t>10.82% (10.55%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.79% (10.60%)</t>
+          <t>10.47% (10.28%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.82% (10.69%)</t>
+          <t>10.46% (10.33%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.65% (16.03%)</t>
+          <t>16.21% (15.60%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.50% (17.42%)</t>
+          <t>16.96% (16.89%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.81% (16.47%)</t>
+          <t>16.41% (16.07%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.25% (16.76%)</t>
+          <t>16.82% (16.34%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.63% (16.22%)</t>
+          <t>16.18% (15.77%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>18.28% (18.28%)</t>
+          <t>17.62% (17.62%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.03% (14.25%)</t>
+          <t>14.70% (13.92%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.96% (19.42%)</t>
+          <t>19.40% (18.86%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.85% (14.15%)</t>
+          <t>14.54% (13.83%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.23% (16.96%)</t>
+          <t>16.75% (16.48%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.76% (16.56%)</t>
+          <t>16.27% (16.07%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.63% (16.49%)</t>
+          <t>16.14% (16.00%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.94% (-4.55%)</t>
+          <t>-3.44% (-4.05%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.56% (-11.64%)</t>
+          <t>-11.26% (-11.33%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.47% (-7.80%)</t>
+          <t>-7.05% (-7.38%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-6.05% (-6.53%)</t>
+          <t>-5.62% (-6.09%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-6.31% (-6.71%)</t>
+          <t>-5.81% (-6.21%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.81% (-12.82%)</t>
+          <t>-12.85% (-12.85%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.87% (-1.65%)</t>
+          <t>-0.27% (-1.05%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.43% (-8.95%)</t>
+          <t>-8.09% (-8.61%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.89% (-2.60%)</t>
+          <t>-1.29% (-2.00%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-10.10% (-10.37%)</t>
+          <t>-9.68% (-9.95%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.83% (-10.02%)</t>
+          <t>-9.38% (-9.58%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.88% (-10.02%)</t>
+          <t>-9.48% (-9.61%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-3.21% (-3.83%)</t>
+          <t>-2.88% (-3.50%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.89% (-9.97%)</t>
+          <t>-9.73% (-9.80%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.39% (-6.73%)</t>
+          <t>-6.05% (-6.39%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.95% (-5.44%)</t>
+          <t>-4.63% (-5.11%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.32% (-5.73%)</t>
+          <t>-5.02% (-5.42%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.90% (-10.90%)</t>
+          <t>-10.88% (-10.88%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.70% (-1.48%)</t>
+          <t>-0.22% (-1.00%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.85% (-7.39%)</t>
+          <t>-6.71% (-7.24%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.73% (-2.44%)</t>
+          <t>-1.25% (-1.96%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.40% (-8.67%)</t>
+          <t>-8.16% (-8.43%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.26% (-8.46%)</t>
+          <t>-8.03% (-8.23%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.48% (-8.61%)</t>
+          <t>-8.24% (-8.38%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.15%</t>
+          <t>-14.33%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-23.12%</t>
+          <t>-22.38%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.68%</t>
+          <t>-17.90%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.63%</t>
+          <t>-16.83%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-17.36%</t>
+          <t>-16.56%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-25.02%</t>
+          <t>-24.29%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.78%</t>
+          <t>-9.92%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.51%</t>
+          <t>-21.76%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.69%</t>
+          <t>-10.83%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.26%</t>
+          <t>-20.50%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.62%</t>
+          <t>-19.85%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.70%</t>
+          <t>-19.94%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.86%</t>
+          <t>-19.09%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-27.39%</t>
+          <t>-26.69%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.20%</t>
+          <t>-22.46%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.20%</t>
+          <t>-21.45%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.95%</t>
+          <t>-21.20%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-29.18%</t>
+          <t>-28.50%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.73%</t>
+          <t>-14.92%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.81%</t>
+          <t>-26.11%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.59%</t>
+          <t>-15.78%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.63%</t>
+          <t>-24.91%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-25.03%</t>
+          <t>-24.30%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.10%</t>
+          <t>-24.38%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.91% (1.30%)</t>
+          <t>1.46% (0.84%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.18% (1.10%)</t>
+          <t>1.52% (1.45%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.46% (2.13%)</t>
+          <t>1.94% (1.61%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.68% (2.20%)</t>
+          <t>2.17% (1.69%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.08% (1.68%)</t>
+          <t>1.63% (1.23%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.02%)</t>
+          <t>-0.06% (-0.06%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.00% (-0.78%)</t>
+          <t>-0.27% (-1.05%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.40% (5.87%)</t>
+          <t>5.77% (5.24%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.73%)</t>
+          <t>-0.36% (-1.07%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.82% (2.56%)</t>
+          <t>2.31% (2.05%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.31% (2.12%)</t>
+          <t>1.83% (1.64%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.37% (2.23%)</t>
+          <t>1.84% (1.70%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.67% (2.06%)</t>
+          <t>2.04% (1.43%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.91% (0.83%)</t>
+          <t>1.09% (1.01%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.65% (3.31%)</t>
+          <t>3.03% (2.69%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.87% (3.39%)</t>
+          <t>3.23% (2.75%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.14% (2.74%)</t>
+          <t>2.48% (2.08%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>-0.08% (-0.08%)</t>
+          <t>-0.06% (-0.06%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.16% (-0.62%)</t>
+          <t>-0.22% (-1.00%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.31% (5.78%)</t>
+          <t>6.48% (5.95%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.14% (-0.57%)</t>
+          <t>-0.33% (-1.03%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.80% (3.53%)</t>
+          <t>4.03% (3.76%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.94% (2.75%)</t>
+          <t>3.20% (3.01%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.10% (1.97%)</t>
+          <t>2.36% (2.23%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 16/7/2026</t>
+          <t>As of 17/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>10.36%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>7.53%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>5.72%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>7.87%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.16%</t>
+          <t>6.18%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.71%</t>
+          <t>-6.21%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.10%</t>
+          <t>10.74%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.62%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.08%</t>
+          <t>5.59%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.26%</t>
+          <t>8.22%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.26%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.53%</t>
+          <t>-6.09%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.56%</t>
+          <t>13.15%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.82%</t>
+          <t>7.21%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.90%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.15%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>1.86%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.95%</t>
+          <t>-8.61%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.04%</t>
+          <t>10.62%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.88%</t>
+          <t>3.34%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.08%</t>
+          <t>5.06%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.56%</t>
+          <t>9.61%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.55%</t>
+          <t>-4.05%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.09%</t>
+          <t>8.84%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.19%</t>
+          <t>14.90%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.78%</t>
+          <t>1.15%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.90%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.60%</t>
+          <t>-2.00%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>8.87%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14.67%</t>
+          <t>15.36%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>0.21%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>-0.09%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.44%</t>
+          <t>16.55%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.65%</t>
+          <t>-1.05%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12.20%</t>
+          <t>11.44%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.73%</t>
+          <t>13.77%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20.03%</t>
+          <t>18.88%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-4.57%</t>
+          <t>-3.64%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.82%</t>
+          <t>-12.85%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.49%</t>
+          <t>11.05%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.19%</t>
+          <t>11.81%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>17.07%</t>
+          <t>15.95%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.38%</t>
+          <t>-1.43%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.64%</t>
+          <t>-11.33%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>10.33%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.69%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.19%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.50%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>1.41%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-10.02%</t>
+          <t>-9.61%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.67%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>12.29%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>2.49%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.02%</t>
+          <t>-9.58%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.89%</t>
+          <t>10.55%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.66%</t>
+          <t>5.15%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.62%</t>
+          <t>10.11%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>13.21%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.37%</t>
+          <t>-9.95%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>10.52%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>6.40%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.54%</t>
+          <t>7.05%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>9.62%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.68%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.80%</t>
+          <t>-7.38%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 16/7/2026</t>
+          <t>As of 17/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.22%</t>
+          <t>15.77%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.50%</t>
+          <t>5.84%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.18%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>7.87%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.67%</t>
+          <t>3.66%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.73%</t>
+          <t>-5.42%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.76%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.06%</t>
+          <t>6.42%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.85%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.26%</t>
+          <t>8.22%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>3.55%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.44%</t>
+          <t>-5.11%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.42%</t>
+          <t>18.86%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.78%</t>
+          <t>5.95%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.07%</t>
+          <t>6.90%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.14%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-0.81%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.39%</t>
+          <t>-7.24%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.03%</t>
+          <t>15.60%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.14%</t>
+          <t>8.51%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>5.06%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>6.93%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.83%</t>
+          <t>-3.50%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.15%</t>
+          <t>13.83%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.17%</t>
+          <t>11.72%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.62%</t>
+          <t>1.12%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.70%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.44%</t>
+          <t>-1.96%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.25%</t>
+          <t>13.92%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.78%</t>
+          <t>12.32%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.87%</t>
+          <t>-0.09%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>13.45%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.48%</t>
+          <t>-1.00%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.28%</t>
+          <t>17.62%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.08%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.26%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20.03%</t>
+          <t>18.88%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-6.65%</t>
+          <t>-5.75%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.90%</t>
+          <t>-10.88%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.42%</t>
+          <t>16.89%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>9.92%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>17.07%</t>
+          <t>15.95%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.42%</t>
+          <t>-3.50%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.97%</t>
+          <t>-9.80%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.49%</t>
+          <t>16.00%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.97%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8.22%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.77%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.61%</t>
+          <t>-8.38%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.56%</t>
+          <t>16.07%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.32%</t>
+          <t>8.05%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>12.29%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.09%</t>
+          <t>-0.13%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.46%</t>
+          <t>-8.23%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.96%</t>
+          <t>16.48%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.53%</t>
+          <t>3.80%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.57%</t>
+          <t>8.29%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>13.21%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.91%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.67%</t>
+          <t>-8.43%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.47%</t>
+          <t>16.07%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.64%</t>
+          <t>5.02%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>5.92%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>9.62%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>2.25%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.73%</t>
+          <t>-6.39%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-20]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/17/2026 at 10:49 AM ET)</t>
+          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7/21/2025 - 7/17/2026</t>
+          <t>7/20/2026 - 7/16/2027</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>7/21/2025 - 7/17/2026</t>
+          <t>7/20/2026 - 7/16/2027</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>14.55% (13.70%)</t>
+          <t>16.82% (15.97%)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>12.04% (11.20%)</t>
+          <t>13.82% (12.97%)</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>$52.60</t>
+          <t>$59.84</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>$39.23</t>
+          <t>$43.65</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>$59.81</t>
+          <t>$69.40</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>$43.62</t>
+          <t>$49.31</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>$627.58</t>
+          <t>$743.29</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>$627.58</t>
+          <t>$743.29</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>$718.89</t>
+          <t>$868.31</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>$703.16</t>
+          <t>$846.03</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.00% / $627.58</t>
+          <t>0.00% / $743.29</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>0.00% / $627.60</t>
+          <t>0.00% / $743.31</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.00% / $564.82</t>
+          <t>-10.00% / $668.96</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>-15.00% / $533.46</t>
+          <t>-15.00% / $631.82</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>273 days</t>
+          <t>270 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>35 days</t>
+          <t>32 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>154 days</t>
+          <t>151 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>217 days</t>
+          <t>214 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>182 days</t>
+          <t>179 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0 days</t>
+          <t>361 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>335 days</t>
+          <t>332 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>245 days</t>
+          <t>242 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>308 days</t>
+          <t>305 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>126 days</t>
+          <t>123 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>91 days</t>
+          <t>88 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>63 days</t>
+          <t>60 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>273 days</t>
+          <t>270 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>35 days</t>
+          <t>32 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>154 days</t>
+          <t>151 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>217 days</t>
+          <t>214 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>182 days</t>
+          <t>179 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>0 days</t>
+          <t>361 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>335 days</t>
+          <t>332 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>245 days</t>
+          <t>242 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>308 days</t>
+          <t>305 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>126 days</t>
+          <t>123 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>91 days</t>
+          <t>88 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>63 days</t>
+          <t>60 days</t>
         </is>
       </c>
     </row>
@@ -2326,22 +2326,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.78 / 3.34%</t>
+          <t>$46.78 / 3.33%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.67 / 11.81%</t>
+          <t>$56.71 / 11.87%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.61 / 7.05%</t>
+          <t>$54.59 / 7.02%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.15 / 5.59%</t>
+          <t>$61.16 / 5.60%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2351,82 +2351,82 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.85 / 13.77%</t>
+          <t>$59.96 / 0.18%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.00 / 0.21%</t>
+          <t>$59.94 / 0.11%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.42 / 8.50%</t>
+          <t>$52.44 / 8.53%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.21 / 1.15%</t>
+          <t>$56.19 / 1.12%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.63 / 10.11%</t>
+          <t>$58.64 / 10.12%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.49 / 9.65%</t>
+          <t>$52.51 / 9.69%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.30 / 9.70%</t>
+          <t>$55.31 / 9.72%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.76 / 2.75%</t>
+          <t>$41.75 / 2.71%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.56 / 9.92%</t>
+          <t>$41.58 / 9.97%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.92 / 5.92%</t>
+          <t>$39.93 / 5.94%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.12 / 4.50%</t>
+          <t>$44.13 / 4.52%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.14 / 4.84%</t>
+          <t>$45.12 / 4.81%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.65 / 11.26%</t>
+          <t>$43.70 / 0.11%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.22 / 0.16%</t>
+          <t>$41.19 / 0.09%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.40 / 6.90%</t>
+          <t>$44.35 / 6.78%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.12 / 1.12%</t>
+          <t>$43.09 / 1.06%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$746.08 / 5.06%</t>
+          <t>$745.83 / 5.03%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$746.08 / 15.95%</t>
+          <t>$745.83 / 15.91%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$746.08 / 9.62%</t>
+          <t>$745.83 / 9.59%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$746.08 / 8.22%</t>
+          <t>$745.83 / 8.18%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$746.08 / 7.87%</t>
+          <t>$745.83 / 7.83%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$746.08 / 18.88%</t>
+          <t>$745.83 / 0.34%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$746.08 / -0.09%</t>
+          <t>$745.83 / -0.12%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$746.08 / 15.03%</t>
+          <t>$745.83 / 15.00%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$746.08 / 0.93%</t>
+          <t>$745.83 / 0.90%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$746.08 / 13.21%</t>
+          <t>$745.83 / 13.17%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$746.08 / 12.29%</t>
+          <t>$745.83 / 12.26%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$746.08 / 12.41%</t>
+          <t>$745.83 / 12.37%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$746.08 / 5.06%</t>
+          <t>$745.83 / 5.03%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$746.08 / 15.95%</t>
+          <t>$745.83 / 15.91%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$746.08 / 9.62%</t>
+          <t>$745.59 / 9.55%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$746.08 / 8.22%</t>
+          <t>$745.83 / 8.18%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$746.08 / 7.87%</t>
+          <t>$745.83 / 7.83%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$746.08 / 18.88%</t>
+          <t>$745.83 / 0.34%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$746.08 / -0.09%</t>
+          <t>$745.83 / -0.12%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$746.08 / 15.03%</t>
+          <t>$745.83 / 15.00%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$746.08 / 0.93%</t>
+          <t>$745.83 / 0.90%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$746.08 / 13.21%</t>
+          <t>$745.59 / 13.13%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$746.08 / 12.29%</t>
+          <t>$745.83 / 12.26%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$746.08 / 12.41%</t>
+          <t>$745.83 / 12.37%</t>
         </is>
       </c>
     </row>
@@ -2580,107 +2580,107 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.23% (10.62%)</t>
+          <t>11.24% (10.63%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.52% (1.45%)</t>
+          <t>1.45% (1.39%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.73% (6.40%)</t>
+          <t>6.76% (6.43%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.60% (8.12%)</t>
+          <t>8.58% (8.11%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.94% (7.53%)</t>
+          <t>7.93% (7.53%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-0.06% (-0.06%)</t>
+          <t>16.60% (15.76%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.14% (15.36%)</t>
+          <t>16.25% (15.48%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.74% (7.21%)</t>
+          <t>7.70% (7.18%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.61% (14.90%)</t>
+          <t>15.64% (14.94%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.41% (5.15%)</t>
+          <t>5.39% (5.13%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.38% (4.19%)</t>
+          <t>4.33% (4.15%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.29% (3.15%)</t>
+          <t>3.25% (3.12%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.13% (8.51%)</t>
+          <t>9.16% (8.55%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.09% (1.01%)</t>
+          <t>1.03% (0.96%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.35% (5.02%)</t>
+          <t>5.33% (5.00%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.90% (6.42%)</t>
+          <t>6.87% (6.39%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.24% (5.84%)</t>
+          <t>6.27% (5.88%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>-0.06% (-0.06%)</t>
+          <t>13.69% (12.85%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.10% (12.32%)</t>
+          <t>13.18% (12.41%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.48% (5.95%)</t>
+          <t>6.59% (6.07%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.43% (11.72%)</t>
+          <t>12.49% (11.79%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.20% (3.01%)</t>
+          <t>3.19% (3.01%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.61%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>-1.40%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.18%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-3.64%</t>
+          <t>16.42%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.55%</t>
+          <t>16.59%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.86%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>16.04%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.49%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.41%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.93%</t>
+          <t>6.97%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-3.47%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.25%</t>
+          <t>2.31%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.55%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.66%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>-5.75%</t>
+          <t>13.44%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.45%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.81%</t>
+          <t>-0.78%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.78%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>0.10%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>-0.10%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-0.79%</t>
         </is>
       </c>
     </row>
@@ -2834,12 +2834,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.90% (10.28%)</t>
+          <t>10.87% (10.26%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.12% (11.05%)</t>
+          <t>11.03% (10.97%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2849,27 +2849,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.22% (10.74%)</t>
+          <t>11.17% (10.70%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.76% (10.36%)</t>
+          <t>10.72% (10.33%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.44% (11.44%)</t>
+          <t>10.12% (9.28%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.65% (8.87%)</t>
+          <t>9.71% (8.94%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.68% (13.15%)</t>
+          <t>13.62% (13.10%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2879,17 +2879,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.82% (10.55%)</t>
+          <t>10.77% (10.51%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.47% (10.28%)</t>
+          <t>10.40% (10.22%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.46% (10.33%)</t>
+          <t>10.40% (10.27%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2899,57 +2899,57 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.96% (16.89%)</t>
+          <t>16.89% (16.82%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.41% (16.07%)</t>
+          <t>16.34% (16.01%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.82% (16.34%)</t>
+          <t>16.77% (16.29%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.18% (15.77%)</t>
+          <t>16.17% (15.78%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>17.62% (17.62%)</t>
+          <t>15.17% (14.33%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.70% (13.92%)</t>
+          <t>14.73% (13.96%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.40% (18.86%)</t>
+          <t>19.47% (18.94%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.54% (13.83%)</t>
+          <t>14.56% (13.86%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.75% (16.48%)</t>
+          <t>16.70% (16.43%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.27% (16.07%)</t>
+          <t>16.24% (16.05%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.14% (16.00%)</t>
+          <t>16.11% (15.98%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.44% (-4.05%)</t>
+          <t>-3.43% (-4.04%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.26% (-11.33%)</t>
+          <t>-11.32% (-11.39%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.05% (-7.38%)</t>
+          <t>-7.03% (-7.35%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.62% (-6.09%)</t>
+          <t>-5.63% (-6.10%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.81% (-6.21%)</t>
+          <t>-5.82% (-6.21%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-12.85% (-12.85%)</t>
+          <t>-0.19% (-1.03%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.27% (-1.05%)</t>
+          <t>-0.18% (-0.95%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.09% (-8.61%)</t>
+          <t>-8.12% (-8.64%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.29% (-2.00%)</t>
+          <t>-1.26% (-1.96%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.68% (-9.95%)</t>
+          <t>-9.70% (-9.96%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.38% (-9.58%)</t>
+          <t>-9.42% (-9.61%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.48% (-9.61%)</t>
+          <t>-9.51% (-9.64%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.88% (-3.50%)</t>
+          <t>-2.85% (-3.46%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.73% (-9.80%)</t>
+          <t>-9.78% (-9.85%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.05% (-6.39%)</t>
+          <t>-6.07% (-6.40%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.63% (-5.11%)</t>
+          <t>-4.66% (-5.14%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.02% (-5.42%)</t>
+          <t>-5.00% (-5.39%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-10.88% (-10.88%)</t>
+          <t>-0.12% (-0.96%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.22% (-1.00%)</t>
+          <t>-0.16% (-0.93%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.71% (-7.24%)</t>
+          <t>-6.61% (-7.14%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.25% (-1.96%)</t>
+          <t>-1.20% (-1.90%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.16% (-8.43%)</t>
+          <t>-8.17% (-8.43%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.03% (-8.23%)</t>
+          <t>-8.04% (-8.23%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.24% (-8.38%)</t>
+          <t>-8.25% (-8.38%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.33%</t>
+          <t>-14.31%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.38%</t>
+          <t>-22.35%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.90%</t>
+          <t>-17.87%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.83%</t>
+          <t>-16.80%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.56%</t>
+          <t>-16.54%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-24.29%</t>
+          <t>-10.31%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.92%</t>
+          <t>-9.89%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.76%</t>
+          <t>-21.74%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.83%</t>
+          <t>-10.80%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.50%</t>
+          <t>-20.47%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.85%</t>
+          <t>-19.83%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-19.94%</t>
+          <t>-19.91%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.09%</t>
+          <t>-19.06%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.69%</t>
+          <t>-26.67%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.46%</t>
+          <t>-22.41%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-21.45%</t>
+          <t>-21.42%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.20%</t>
+          <t>-21.17%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-28.50%</t>
+          <t>-15.29%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.92%</t>
+          <t>-14.89%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.11%</t>
+          <t>-26.08%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.78%</t>
+          <t>-15.76%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.91%</t>
+          <t>-24.86%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.30%</t>
+          <t>-24.28%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.38%</t>
+          <t>-24.36%</t>
         </is>
       </c>
     </row>
@@ -3215,62 +3215,62 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.46% (0.84%)</t>
+          <t>1.43% (0.82%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.52% (1.45%)</t>
+          <t>1.45% (1.39%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.94% (1.61%)</t>
+          <t>1.93% (1.60%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.17% (1.69%)</t>
+          <t>2.12% (1.64%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.63% (1.23%)</t>
+          <t>1.59% (1.20%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.06%)</t>
+          <t>0.15% (-0.69%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.27% (-1.05%)</t>
+          <t>-0.18% (-0.95%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.77% (5.24%)</t>
+          <t>5.70% (5.18%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.36% (-1.07%)</t>
+          <t>-0.37% (-1.07%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.31% (2.05%)</t>
+          <t>2.26% (2.00%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.83% (1.64%)</t>
+          <t>1.75% (1.56%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.84% (1.70%)</t>
+          <t>1.77% (1.64%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -3280,52 +3280,52 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.09% (1.01%)</t>
+          <t>1.03% (0.96%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.03% (2.69%)</t>
+          <t>2.94% (2.61%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.23% (2.75%)</t>
+          <t>3.16% (2.69%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.48% (2.08%)</t>
+          <t>2.47% (2.08%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.06%)</t>
+          <t>0.22% (-0.62%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.22% (-1.00%)</t>
+          <t>-0.16% (-0.93%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.48% (5.95%)</t>
+          <t>6.59% (6.07%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.33% (-1.03%)</t>
+          <t>-0.31% (-1.01%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>4.03% (3.76%)</t>
+          <t>3.96% (3.69%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.20% (3.01%)</t>
+          <t>3.19% (3.01%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 17/7/2026</t>
+          <t>As of 20/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.36%</t>
+          <t>10.33%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3425,12 +3425,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.87%</t>
+          <t>7.83%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.18%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.74%</t>
+          <t>10.70%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.12%</t>
+          <t>8.11%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.59%</t>
+          <t>5.60%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.22%</t>
+          <t>8.18%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.09%</t>
+          <t>-6.10%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.15%</t>
+          <t>13.10%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.21%</t>
+          <t>7.18%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8.53%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.86%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.61%</t>
+          <t>-8.64%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.26%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.62%</t>
+          <t>10.63%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.34%</t>
+          <t>3.33%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.06%</t>
+          <t>5.03%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.61%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.05%</t>
+          <t>-4.04%</t>
         </is>
       </c>
     </row>
@@ -3563,27 +3563,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.90%</t>
+          <t>14.94%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.15%</t>
+          <t>1.12%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>16.04%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.00%</t>
+          <t>-1.96%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.87%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.36%</t>
+          <t>15.48%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.55%</t>
+          <t>16.59%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.05%</t>
+          <t>-0.95%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.44%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13.77%</t>
+          <t>0.18%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.88%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-3.64%</t>
+          <t>16.42%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-12.85%</t>
+          <t>-1.03%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.05%</t>
+          <t>10.97%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.39%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.81%</t>
+          <t>11.87%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.95%</t>
+          <t>15.91%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>-1.40%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.33%</t>
+          <t>-11.39%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.33%</t>
+          <t>10.27%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>3.12%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.72%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.41%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.61%</t>
+          <t>-9.64%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.15%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>9.69%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.29%</t>
+          <t>12.26%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.49%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.58%</t>
+          <t>-9.61%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.55%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.15%</t>
+          <t>5.13%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.21%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.95%</t>
+          <t>-9.96%</t>
         </is>
       </c>
     </row>
@@ -3822,27 +3822,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.40%</t>
+          <t>6.43%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.05%</t>
+          <t>7.02%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.62%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.38%</t>
+          <t>-7.35%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 17/7/2026</t>
+          <t>As of 20/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.77%</t>
+          <t>15.78%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.84%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.87%</t>
+          <t>7.83%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.66%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.42%</t>
+          <t>-5.39%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>16.29%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.42%</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>4.52%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.22%</t>
+          <t>8.18%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.55%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.11%</t>
+          <t>-5.14%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.86%</t>
+          <t>18.94%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.95%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.90%</t>
+          <t>6.78%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.81%</t>
+          <t>-0.78%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.24%</t>
+          <t>-7.14%</t>
         </is>
       </c>
     </row>
@@ -4041,27 +4041,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.51%</t>
+          <t>8.55%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>2.71%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.06%</t>
+          <t>5.03%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.93%</t>
+          <t>6.97%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-3.46%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.83%</t>
+          <t>13.86%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.72%</t>
+          <t>11.79%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.12%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.78%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.96%</t>
+          <t>-1.90%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.92%</t>
+          <t>13.96%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.32%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>0.09%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.45%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.00%</t>
+          <t>-0.93%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17.62%</t>
+          <t>14.33%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>12.85%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.26%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.88%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-5.75%</t>
+          <t>13.44%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-10.88%</t>
+          <t>-0.96%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.89%</t>
+          <t>16.82%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.92%</t>
+          <t>9.97%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.95%</t>
+          <t>15.91%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-3.47%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.80%</t>
+          <t>-9.85%</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.00%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4236,12 +4236,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-0.79%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.07%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.29%</t>
+          <t>12.26%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>-0.10%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.48%</t>
+          <t>16.43%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -4310,12 +4310,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.21%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>0.10%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.07%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.02%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.92%</t>
+          <t>5.94%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.62%</t>
+          <t>9.55%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.25%</t>
+          <t>2.31%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.39%</t>
+          <t>-6.40%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-21]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/20/2026 at 11:27 AM ET)</t>
+          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>270 days</t>
+          <t>269 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>32 days</t>
+          <t>31 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>151 days</t>
+          <t>150 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>214 days</t>
+          <t>213 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>179 days</t>
+          <t>178 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>361 days</t>
+          <t>360 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>332 days</t>
+          <t>331 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>242 days</t>
+          <t>241 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>305 days</t>
+          <t>304 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>123 days</t>
+          <t>122 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>88 days</t>
+          <t>87 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>60 days</t>
+          <t>59 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>270 days</t>
+          <t>269 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>32 days</t>
+          <t>31 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>151 days</t>
+          <t>150 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>214 days</t>
+          <t>213 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>179 days</t>
+          <t>178 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>361 days</t>
+          <t>360 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>332 days</t>
+          <t>331 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>242 days</t>
+          <t>241 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>305 days</t>
+          <t>304 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>123 days</t>
+          <t>122 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>88 days</t>
+          <t>87 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>60 days</t>
+          <t>59 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.78 / 3.33%</t>
+          <t>$46.85 / 3.50%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.71 / 11.87%</t>
+          <t>$56.79 / 12.03%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.59 / 7.02%</t>
+          <t>$54.64 / 7.11%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.16 / 5.60%</t>
+          <t>$61.22 / 5.71%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.26 / 5.72%</t>
+          <t>$55.32 / 5.83%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.96 / 0.18%</t>
+          <t>$60.03 / 0.31%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.94 / 0.11%</t>
+          <t>$60.02 / 0.24%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.44 / 8.53%</t>
+          <t>$52.48 / 8.62%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.19 / 1.12%</t>
+          <t>$56.27 / 1.26%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.64 / 10.12%</t>
+          <t>$58.70 / 10.24%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.51 / 9.69%</t>
+          <t>$52.58 / 9.83%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.31 / 9.72%</t>
+          <t>$55.39 / 9.87%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.75 / 2.71%</t>
+          <t>$41.77 / 2.76%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.58 / 9.97%</t>
+          <t>$41.60 / 10.02%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.93 / 5.94%</t>
+          <t>$39.98 / 6.07%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.13 / 4.52%</t>
+          <t>$44.16 / 4.59%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.12 / 4.81%</t>
+          <t>$45.18 / 4.94%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.70 / 0.11%</t>
+          <t>$43.74 / 0.21%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.19 / 0.09%</t>
+          <t>$41.25 / 0.23%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.35 / 6.78%</t>
+          <t>$44.39 / 6.87%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.09 / 1.06%</t>
+          <t>$43.14 / 1.16%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.93 / 8.29%</t>
+          <t>$41.97 / 8.39%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.67 / 8.05%</t>
+          <t>$41.70 / 8.11%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.10 / 8.22%</t>
+          <t>$41.14 / 8.33%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$745.83 / 5.03%</t>
+          <t>$747.20 / 5.22%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$745.83 / 15.91%</t>
+          <t>$747.20 / 16.13%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$745.83 / 9.59%</t>
+          <t>$747.20 / 9.79%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$745.83 / 8.18%</t>
+          <t>$747.20 / 8.38%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$745.83 / 7.83%</t>
+          <t>$747.20 / 8.03%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$745.83 / 0.34%</t>
+          <t>$747.20 / 0.53%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$745.83 / -0.12%</t>
+          <t>$747.20 / 0.06%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$745.83 / 15.00%</t>
+          <t>$747.20 / 15.21%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$745.83 / 0.90%</t>
+          <t>$747.20 / 1.09%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$745.83 / 13.17%</t>
+          <t>$747.20 / 13.38%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$745.83 / 12.26%</t>
+          <t>$747.20 / 12.46%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$745.83 / 12.37%</t>
+          <t>$747.20 / 12.58%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$745.83 / 5.03%</t>
+          <t>$747.20 / 5.22%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$745.83 / 15.91%</t>
+          <t>$747.20 / 16.13%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$745.59 / 9.55%</t>
+          <t>$747.20 / 9.79%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$745.83 / 8.18%</t>
+          <t>$747.20 / 8.38%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$745.83 / 7.83%</t>
+          <t>$747.20 / 8.03%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$745.83 / 0.34%</t>
+          <t>$747.20 / 0.53%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$745.83 / -0.12%</t>
+          <t>$747.20 / 0.06%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$745.83 / 15.00%</t>
+          <t>$747.20 / 15.21%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$745.83 / 0.90%</t>
+          <t>$747.20 / 1.09%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$745.59 / 13.13%</t>
+          <t>$747.20 / 13.38%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$745.83 / 12.26%</t>
+          <t>$747.20 / 12.46%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$745.83 / 12.37%</t>
+          <t>$747.20 / 12.58%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.24% (10.63%)</t>
+          <t>11.06% (10.45%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.45% (1.39%)</t>
+          <t>1.31% (1.24%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.76% (6.43%)</t>
+          <t>6.67% (6.34%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.58% (8.11%)</t>
+          <t>8.47% (8.00%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.93% (7.53%)</t>
+          <t>7.81% (7.42%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>16.60% (15.76%)</t>
+          <t>16.45% (15.61%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.25% (15.48%)</t>
+          <t>16.10% (15.33%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.70% (7.18%)</t>
+          <t>7.61% (7.09%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.64% (14.94%)</t>
+          <t>15.48% (14.78%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.39% (5.13%)</t>
+          <t>5.28% (5.02%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.33% (4.15%)</t>
+          <t>4.20% (4.02%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.25% (3.12%)</t>
+          <t>3.11% (2.98%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.16% (8.55%)</t>
+          <t>9.11% (8.50%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.03% (0.96%)</t>
+          <t>0.98% (0.92%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.33% (5.00%)</t>
+          <t>5.20% (4.87%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.87% (6.39%)</t>
+          <t>6.80% (6.32%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.27% (5.88%)</t>
+          <t>6.14% (5.75%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>13.69% (12.85%)</t>
+          <t>13.57% (12.73%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.18% (12.41%)</t>
+          <t>13.01% (12.24%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.59% (6.07%)</t>
+          <t>6.50% (5.97%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.49% (11.79%)</t>
+          <t>12.37% (11.67%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.07% (3.80%)</t>
+          <t>3.96% (3.70%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.19% (3.01%)</t>
+          <t>3.13% (2.94%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.36% (2.23%)</t>
+          <t>2.25% (2.13%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.40%</t>
+          <t>-1.58%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.52%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>6.12%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>6.02%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>16.42%</t>
+          <t>16.21%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.59%</t>
+          <t>16.38%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.04%</t>
+          <t>15.83%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>2.34%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.26%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>6.77%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.47%</t>
+          <t>-3.64%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.31%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.23%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>13.28%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.78%</t>
+          <t>-0.96%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.61%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.10%</t>
+          <t>-0.29%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.79%</t>
+          <t>-0.98%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.87% (10.26%)</t>
+          <t>10.87% (10.27%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.03% (10.97%)</t>
+          <t>11.05% (10.99%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.85% (10.52%)</t>
+          <t>10.92% (10.59%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.17% (10.70%)</t>
+          <t>11.23% (10.76%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.72% (10.33%)</t>
+          <t>10.77% (10.38%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.12% (9.28%)</t>
+          <t>10.15% (9.32%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.71% (8.94%)</t>
+          <t>9.74% (8.97%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.62% (13.10%)</t>
+          <t>13.68% (13.16%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.55% (8.84%)</t>
+          <t>9.57% (8.87%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.77% (10.51%)</t>
+          <t>10.82% (10.56%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.40% (10.22%)</t>
+          <t>10.44% (10.25%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.40% (10.27%)</t>
+          <t>10.42% (10.30%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.21% (15.60%)</t>
+          <t>16.31% (15.71%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.89% (16.82%)</t>
+          <t>16.98% (16.91%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.34% (16.01%)</t>
+          <t>16.39% (16.06%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.77% (16.29%)</t>
+          <t>16.84% (16.37%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.17% (15.78%)</t>
+          <t>16.20% (15.81%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.17% (14.33%)</t>
+          <t>15.22% (14.38%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.73% (13.96%)</t>
+          <t>14.74% (13.97%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.47% (18.94%)</t>
+          <t>19.52% (18.99%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.56% (13.86%)</t>
+          <t>14.61% (13.91%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.70% (16.43%)</t>
+          <t>16.77% (16.51%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.24% (16.05%)</t>
+          <t>16.32% (16.13%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.11% (15.98%)</t>
+          <t>16.15% (16.03%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.43% (-4.04%)</t>
+          <t>-3.59% (-4.20%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.32% (-11.39%)</t>
+          <t>-11.45% (-11.51%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.03% (-7.35%)</t>
+          <t>-7.10% (-7.43%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.63% (-6.10%)</t>
+          <t>-5.73% (-6.20%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.82% (-6.21%)</t>
+          <t>-5.92% (-6.31%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-0.19% (-1.03%)</t>
+          <t>-0.32% (-1.15%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.18% (-0.95%)</t>
+          <t>-0.32% (-1.08%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.12% (-8.64%)</t>
+          <t>-8.20% (-8.72%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.26% (-1.96%)</t>
+          <t>-1.40% (-2.10%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.70% (-9.96%)</t>
+          <t>-9.80% (-10.06%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.42% (-9.61%)</t>
+          <t>-9.54% (-9.72%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.51% (-9.64%)</t>
+          <t>-9.63% (-9.76%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.85% (-3.46%)</t>
+          <t>-2.90% (-3.51%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.78% (-9.85%)</t>
+          <t>-9.83% (-9.89%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.07% (-6.40%)</t>
+          <t>-6.19% (-6.52%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.66% (-5.14%)</t>
+          <t>-4.73% (-5.20%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.00% (-5.39%)</t>
+          <t>-5.11% (-5.51%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-0.12% (-0.96%)</t>
+          <t>-0.22% (-1.06%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.16% (-0.93%)</t>
+          <t>-0.31% (-1.08%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.61% (-7.14%)</t>
+          <t>-6.70% (-7.22%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.20% (-1.90%)</t>
+          <t>-1.30% (-2.00%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.17% (-8.43%)</t>
+          <t>-8.26% (-8.52%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.04% (-8.23%)</t>
+          <t>-8.10% (-8.29%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.25% (-8.38%)</t>
+          <t>-8.34% (-8.47%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.31%</t>
+          <t>-14.46%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.35%</t>
+          <t>-22.50%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.87%</t>
+          <t>-18.02%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.80%</t>
+          <t>-16.96%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.54%</t>
+          <t>-16.69%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-10.31%</t>
+          <t>-10.47%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.89%</t>
+          <t>-10.05%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.74%</t>
+          <t>-21.88%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.80%</t>
+          <t>-10.97%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.47%</t>
+          <t>-20.62%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.83%</t>
+          <t>-19.97%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-19.91%</t>
+          <t>-20.06%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.06%</t>
+          <t>-19.21%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.67%</t>
+          <t>-26.80%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.41%</t>
+          <t>-22.57%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-21.42%</t>
+          <t>-21.57%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.17%</t>
+          <t>-21.32%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-15.29%</t>
+          <t>-15.44%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.89%</t>
+          <t>-15.05%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.08%</t>
+          <t>-26.22%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.76%</t>
+          <t>-15.91%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.86%</t>
+          <t>-25.03%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.28%</t>
+          <t>-24.42%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.36%</t>
+          <t>-24.50%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.43% (0.82%)</t>
+          <t>1.45% (0.85%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.45% (1.39%)</t>
+          <t>1.31% (1.24%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.93% (1.60%)</t>
+          <t>2.03% (1.71%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.12% (1.64%)</t>
+          <t>2.19% (1.73%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.59% (1.20%)</t>
+          <t>1.67% (1.28%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.15% (-0.69%)</t>
+          <t>0.21% (-0.63%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.18% (-0.95%)</t>
+          <t>-0.25% (-1.02%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.70% (5.18%)</t>
+          <t>5.80% (5.28%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.37% (-1.07%)</t>
+          <t>-0.33% (-1.03%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.26% (2.00%)</t>
+          <t>2.34% (2.08%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.75% (1.56%)</t>
+          <t>1.81% (1.63%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.77% (1.64%)</t>
+          <t>1.82% (1.69%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.04% (1.43%)</t>
+          <t>2.18% (1.57%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.03% (0.96%)</t>
+          <t>0.98% (0.92%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.94% (2.61%)</t>
+          <t>3.04% (2.71%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.16% (2.69%)</t>
+          <t>3.28% (2.81%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.47% (2.08%)</t>
+          <t>2.54% (2.14%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.22% (-0.62%)</t>
+          <t>0.30% (-0.53%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.16% (-0.93%)</t>
+          <t>-0.25% (-1.02%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.59% (6.07%)</t>
+          <t>6.50% (5.97%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.31% (-1.01%)</t>
+          <t>-0.23% (-0.93%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.96% (3.69%)</t>
+          <t>3.96% (3.70%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.19% (3.01%)</t>
+          <t>3.13% (2.94%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.36% (2.23%)</t>
+          <t>2.25% (2.13%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 20/7/2026</t>
+          <t>As of 21/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.33%</t>
+          <t>10.38%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.53%</t>
+          <t>7.42%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.72%</t>
+          <t>5.83%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.83%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>6.02%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.21%</t>
+          <t>-6.31%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.70%</t>
+          <t>10.76%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.11%</t>
+          <t>8.00%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.60%</t>
+          <t>5.71%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.18%</t>
+          <t>8.38%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>6.12%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.10%</t>
+          <t>-6.20%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.10%</t>
+          <t>13.16%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.18%</t>
+          <t>7.09%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.53%</t>
+          <t>8.62%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>15.21%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.64%</t>
+          <t>-8.72%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.26%</t>
+          <t>10.27%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.63%</t>
+          <t>10.45%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.03%</t>
+          <t>5.22%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.04%</t>
+          <t>-4.20%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.84%</t>
+          <t>8.87%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.94%</t>
+          <t>14.78%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.12%</t>
+          <t>1.26%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.04%</t>
+          <t>15.83%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.96%</t>
+          <t>-2.10%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>8.97%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.48%</t>
+          <t>15.33%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.59%</t>
+          <t>16.38%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.95%</t>
+          <t>-1.08%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>9.32%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.61%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.18%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>16.42%</t>
+          <t>16.21%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-1.03%</t>
+          <t>-1.15%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.97%</t>
+          <t>10.99%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.87%</t>
+          <t>12.03%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.91%</t>
+          <t>16.13%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.40%</t>
+          <t>-1.58%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.39%</t>
+          <t>-11.51%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.27%</t>
+          <t>10.30%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.12%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.72%</t>
+          <t>9.87%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.26%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.64%</t>
+          <t>-9.76%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>10.25%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.15%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>9.83%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.26%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>2.34%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.61%</t>
+          <t>-9.72%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.13%</t>
+          <t>5.02%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.96%</t>
+          <t>-10.06%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>10.59%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.43%</t>
+          <t>6.34%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.02%</t>
+          <t>7.11%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.52%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.35%</t>
+          <t>-7.43%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 20/7/2026</t>
+          <t>As of 21/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.78%</t>
+          <t>15.81%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>5.75%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.83%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.39%</t>
+          <t>-5.51%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.29%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.32%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>4.59%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.18%</t>
+          <t>8.38%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.14%</t>
+          <t>-5.20%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.94%</t>
+          <t>18.99%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>5.97%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.78%</t>
+          <t>6.87%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>15.21%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.78%</t>
+          <t>-0.96%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.14%</t>
+          <t>-7.22%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.60%</t>
+          <t>15.71%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.55%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.71%</t>
+          <t>2.76%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.03%</t>
+          <t>5.22%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>6.77%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.46%</t>
+          <t>-3.51%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.86%</t>
+          <t>13.91%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.79%</t>
+          <t>11.67%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.61%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.90%</t>
+          <t>-2.00%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.96%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>12.24%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.09%</t>
+          <t>0.23%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>13.28%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.93%</t>
+          <t>-1.08%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.33%</t>
+          <t>14.38%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.85%</t>
+          <t>12.73%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.21%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.23%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.96%</t>
+          <t>-1.06%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.82%</t>
+          <t>16.91%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.97%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.91%</t>
+          <t>16.13%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.47%</t>
+          <t>-3.64%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.85%</t>
+          <t>-9.89%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>16.03%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.23%</t>
+          <t>2.13%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.22%</t>
+          <t>8.33%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.79%</t>
+          <t>-0.98%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.38%</t>
+          <t>-8.47%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>16.13%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.05%</t>
+          <t>8.11%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.26%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.10%</t>
+          <t>-0.29%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.23%</t>
+          <t>-8.29%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.43%</t>
+          <t>16.51%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.80%</t>
+          <t>3.70%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.29%</t>
+          <t>8.39%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.43%</t>
+          <t>-8.52%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>16.06%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>4.87%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.94%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.55%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.31%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.40%</t>
+          <t>-6.52%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-22]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/21/2026 at 11:12 AM ET)</t>
+          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>269 days</t>
+          <t>268 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>31 days</t>
+          <t>30 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>150 days</t>
+          <t>149 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>213 days</t>
+          <t>212 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>178 days</t>
+          <t>177 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>360 days</t>
+          <t>359 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>331 days</t>
+          <t>330 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>241 days</t>
+          <t>240 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>304 days</t>
+          <t>303 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>122 days</t>
+          <t>121 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>87 days</t>
+          <t>86 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>59 days</t>
+          <t>58 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>269 days</t>
+          <t>268 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>31 days</t>
+          <t>30 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>150 days</t>
+          <t>149 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>213 days</t>
+          <t>212 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>178 days</t>
+          <t>177 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>360 days</t>
+          <t>359 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>331 days</t>
+          <t>330 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>241 days</t>
+          <t>240 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>304 days</t>
+          <t>303 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>122 days</t>
+          <t>121 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>87 days</t>
+          <t>86 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>59 days</t>
+          <t>58 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.85 / 3.50%</t>
+          <t>$46.89 / 3.58%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.79 / 12.03%</t>
+          <t>$56.82 / 12.10%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.64 / 7.11%</t>
+          <t>$54.75 / 7.33%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.22 / 5.71%</t>
+          <t>$61.29 / 5.82%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.32 / 5.83%</t>
+          <t>$55.39 / 5.97%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$60.03 / 0.31%</t>
+          <t>$60.11 / 0.43%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.02 / 0.24%</t>
+          <t>$60.12 / 0.41%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.48 / 8.62%</t>
+          <t>$52.52 / 8.69%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.27 / 1.26%</t>
+          <t>$56.34 / 1.39%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.70 / 10.24%</t>
+          <t>$58.76 / 10.36%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.58 / 9.83%</t>
+          <t>$52.63 / 9.95%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.39 / 9.87%</t>
+          <t>$55.45 / 10.00%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.77 / 2.76%</t>
+          <t>$41.80 / 2.85%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.60 / 10.02%</t>
+          <t>$41.66 / 10.18%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.98 / 6.07%</t>
+          <t>$40.00 / 6.14%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.16 / 4.59%</t>
+          <t>$44.19 / 4.65%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.18 / 4.94%</t>
+          <t>$45.21 / 5.02%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.74 / 0.21%</t>
+          <t>$43.82 / 0.40%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.25 / 0.23%</t>
+          <t>$41.29 / 0.33%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.39 / 6.87%</t>
+          <t>$44.41 / 6.94%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.14 / 1.16%</t>
+          <t>$43.20 / 1.32%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.97 / 8.39%</t>
+          <t>$42.00 / 8.47%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.70 / 8.11%</t>
+          <t>$41.73 / 8.20%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.14 / 8.33%</t>
+          <t>$41.18 / 8.42%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$747.20 / 5.22%</t>
+          <t>$748.65 / 5.42%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$747.20 / 16.13%</t>
+          <t>$748.65 / 16.35%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$747.20 / 9.79%</t>
+          <t>$748.65 / 10.00%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$747.20 / 8.38%</t>
+          <t>$748.65 / 8.59%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$747.20 / 8.03%</t>
+          <t>$748.65 / 8.24%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$747.20 / 0.53%</t>
+          <t>$748.65 / 0.72%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$747.20 / 0.06%</t>
+          <t>$748.65 / 0.26%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$747.20 / 15.21%</t>
+          <t>$748.65 / 15.43%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$747.20 / 1.09%</t>
+          <t>$748.65 / 1.28%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$747.20 / 13.38%</t>
+          <t>$748.65 / 13.60%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$747.20 / 12.46%</t>
+          <t>$748.65 / 12.68%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$747.20 / 12.58%</t>
+          <t>$748.65 / 12.80%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$747.20 / 5.22%</t>
+          <t>$748.65 / 5.42%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$747.20 / 16.13%</t>
+          <t>$748.65 / 16.35%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$747.20 / 9.79%</t>
+          <t>$748.65 / 10.00%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$747.20 / 8.38%</t>
+          <t>$748.65 / 8.59%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$747.20 / 8.03%</t>
+          <t>$748.65 / 8.24%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$747.20 / 0.53%</t>
+          <t>$748.65 / 0.72%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$747.20 / 0.06%</t>
+          <t>$748.65 / 0.26%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$747.20 / 15.21%</t>
+          <t>$748.65 / 15.43%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$747.20 / 1.09%</t>
+          <t>$748.65 / 1.28%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$747.20 / 13.38%</t>
+          <t>$748.65 / 13.60%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$747.20 / 12.46%</t>
+          <t>$748.65 / 12.68%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$747.20 / 12.58%</t>
+          <t>$748.65 / 12.80%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.06% (10.45%)</t>
+          <t>10.96% (10.36%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.31% (1.24%)</t>
+          <t>1.24% (1.18%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.67% (6.34%)</t>
+          <t>6.45% (6.13%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.47% (8.00%)</t>
+          <t>8.35% (7.88%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.81% (7.42%)</t>
+          <t>7.67% (7.28%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>16.45% (15.61%)</t>
+          <t>16.30% (15.47%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.10% (15.33%)</t>
+          <t>15.90% (15.13%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.61% (7.09%)</t>
+          <t>7.53% (7.02%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.48% (14.78%)</t>
+          <t>15.33% (14.63%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.28% (5.02%)</t>
+          <t>5.16% (4.91%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.20% (4.02%)</t>
+          <t>4.09% (3.91%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.11% (2.98%)</t>
+          <t>2.99% (2.86%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.11% (8.50%)</t>
+          <t>9.02% (8.41%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.98% (0.92%)</t>
+          <t>0.83% (0.77%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.20% (4.87%)</t>
+          <t>5.13% (4.81%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.80% (6.32%)</t>
+          <t>6.73% (6.26%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.14% (5.75%)</t>
+          <t>6.06% (5.66%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>13.57% (12.73%)</t>
+          <t>13.36% (12.53%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.01% (12.24%)</t>
+          <t>12.90% (12.13%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.50% (5.97%)</t>
+          <t>6.43% (5.91%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.37% (11.67%)</t>
+          <t>12.20% (11.50%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.96% (3.70%)</t>
+          <t>3.89% (3.63%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.13% (2.94%)</t>
+          <t>3.04% (2.86%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.25% (2.13%)</t>
+          <t>2.17% (2.04%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>9.24%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.58%</t>
+          <t>-1.77%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>4.32%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.12%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.02%</t>
+          <t>5.81%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>16.21%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.38%</t>
+          <t>16.15%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15.83%</t>
+          <t>15.61%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.34%</t>
+          <t>2.14%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.26%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.77%</t>
+          <t>6.56%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.64%</t>
+          <t>-3.83%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>3.19%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.30%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>13.23%</t>
+          <t>13.01%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.28%</t>
+          <t>13.06%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.96%</t>
+          <t>-1.15%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.61%</t>
+          <t>12.39%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.29%</t>
+          <t>-0.48%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>-1.17%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.87% (10.27%)</t>
+          <t>10.95% (10.35%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.05% (10.99%)</t>
+          <t>11.14% (11.08%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.92% (10.59%)</t>
+          <t>10.89% (10.57%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.23% (10.76%)</t>
+          <t>11.28% (10.82%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.77% (10.38%)</t>
+          <t>10.81% (10.42%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.15% (9.32%)</t>
+          <t>10.20% (9.37%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.74% (8.97%)</t>
+          <t>9.75% (8.98%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.68% (13.16%)</t>
+          <t>13.77% (13.25%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.57% (8.87%)</t>
+          <t>9.61% (8.92%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.82% (10.56%)</t>
+          <t>10.87% (10.62%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.44% (10.25%)</t>
+          <t>10.49% (10.31%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.42% (10.30%)</t>
+          <t>10.47% (10.35%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.31% (15.71%)</t>
+          <t>16.39% (15.78%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.98% (16.91%)</t>
+          <t>16.98% (16.92%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.39% (16.06%)</t>
+          <t>16.47% (16.15%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.84% (16.37%)</t>
+          <t>16.94% (16.47%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.20% (15.81%)</t>
+          <t>16.28% (15.89%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.22% (14.38%)</t>
+          <t>15.20% (14.37%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.74% (13.97%)</t>
+          <t>14.81% (14.04%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.52% (18.99%)</t>
+          <t>19.61% (19.09%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.61% (13.91%)</t>
+          <t>14.62% (13.93%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.77% (16.51%)</t>
+          <t>16.84% (16.58%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.32% (16.13%)</t>
+          <t>16.39% (16.20%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.15% (16.03%)</t>
+          <t>16.22% (16.09%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.59% (-4.20%)</t>
+          <t>-3.68% (-4.28%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.45% (-11.51%)</t>
+          <t>-11.50% (-11.57%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.10% (-7.43%)</t>
+          <t>-7.29% (-7.62%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.73% (-6.20%)</t>
+          <t>-5.83% (-6.30%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.92% (-6.31%)</t>
+          <t>-6.04% (-6.43%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-0.32% (-1.15%)</t>
+          <t>-0.44% (-1.28%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.32% (-1.08%)</t>
+          <t>-0.48% (-1.25%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.20% (-8.72%)</t>
+          <t>-8.26% (-8.78%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.40% (-2.10%)</t>
+          <t>-1.53% (-2.22%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.80% (-10.06%)</t>
+          <t>-9.90% (-10.15%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.54% (-9.72%)</t>
+          <t>-9.63% (-9.82%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.63% (-9.76%)</t>
+          <t>-9.74% (-9.86%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.90% (-3.51%)</t>
+          <t>-2.98% (-3.59%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.83% (-9.89%)</t>
+          <t>-9.96% (-10.02%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.19% (-6.52%)</t>
+          <t>-6.25% (-6.58%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.73% (-5.20%)</t>
+          <t>-4.78% (-5.25%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.11% (-5.51%)</t>
+          <t>-5.19% (-5.58%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-0.22% (-1.06%)</t>
+          <t>-0.40% (-1.24%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.31% (-1.08%)</t>
+          <t>-0.41% (-1.17%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.70% (-7.22%)</t>
+          <t>-6.75% (-7.28%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.30% (-2.00%)</t>
+          <t>-1.45% (-2.15%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.26% (-8.52%)</t>
+          <t>-8.33% (-8.59%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.10% (-8.29%)</t>
+          <t>-8.18% (-8.36%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.34% (-8.47%)</t>
+          <t>-8.42% (-8.55%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.46%</t>
+          <t>-14.63%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.50%</t>
+          <t>-22.65%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.02%</t>
+          <t>-18.18%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.96%</t>
+          <t>-17.12%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.69%</t>
+          <t>-16.85%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-10.47%</t>
+          <t>-10.64%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.05%</t>
+          <t>-10.23%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.88%</t>
+          <t>-22.03%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.97%</t>
+          <t>-11.14%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.62%</t>
+          <t>-20.77%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.97%</t>
+          <t>-20.13%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.06%</t>
+          <t>-20.21%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.21%</t>
+          <t>-19.37%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.80%</t>
+          <t>-26.94%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.57%</t>
+          <t>-22.72%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-21.57%</t>
+          <t>-21.72%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.32%</t>
+          <t>-21.47%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-15.44%</t>
+          <t>-15.60%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.05%</t>
+          <t>-15.21%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.22%</t>
+          <t>-26.36%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.91%</t>
+          <t>-16.07%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.03%</t>
+          <t>-25.17%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.42%</t>
+          <t>-24.56%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.50%</t>
+          <t>-24.64%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.45% (0.85%)</t>
+          <t>1.56% (0.96%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.31% (1.24%)</t>
+          <t>1.24% (1.18%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.03% (1.71%)</t>
+          <t>2.02% (1.70%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.19% (1.73%)</t>
+          <t>2.28% (1.82%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.67% (1.28%)</t>
+          <t>1.73% (1.35%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.21% (-0.63%)</t>
+          <t>0.27% (-0.56%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.25% (-1.02%)</t>
+          <t>-0.23% (-0.99%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.80% (5.28%)</t>
+          <t>5.93% (5.42%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.33% (-1.03%)</t>
+          <t>-0.26% (-0.96%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.34% (2.08%)</t>
+          <t>2.42% (2.17%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.81% (1.63%)</t>
+          <t>1.90% (1.72%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.82% (1.69%)</t>
+          <t>1.89% (1.77%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.18% (1.57%)</t>
+          <t>2.29% (1.68%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.98% (0.92%)</t>
+          <t>0.83% (0.77%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.04% (2.71%)</t>
+          <t>3.17% (2.84%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.28% (2.81%)</t>
+          <t>3.42% (2.95%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.54% (2.14%)</t>
+          <t>2.65% (2.26%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.30% (-0.53%)</t>
+          <t>0.31% (-0.52%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.25% (-1.02%)</t>
+          <t>-0.15% (-0.92%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.50% (5.97%)</t>
+          <t>6.43% (5.91%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.23% (-0.93%)</t>
+          <t>-0.19% (-0.89%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.96% (3.70%)</t>
+          <t>3.89% (3.63%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.13% (2.94%)</t>
+          <t>3.04% (2.86%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.25% (2.13%)</t>
+          <t>2.17% (2.04%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 21/7/2026</t>
+          <t>As of 22/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.38%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.42%</t>
+          <t>7.28%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.83%</t>
+          <t>5.97%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>8.24%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.02%</t>
+          <t>5.81%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.31%</t>
+          <t>-6.43%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.76%</t>
+          <t>10.82%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.00%</t>
+          <t>7.88%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.71%</t>
+          <t>5.82%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.38%</t>
+          <t>8.59%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.12%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.20%</t>
+          <t>-6.30%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.16%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.09%</t>
+          <t>7.02%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.62%</t>
+          <t>8.69%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.21%</t>
+          <t>15.43%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.72%</t>
+          <t>-8.78%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.27%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.45%</t>
+          <t>10.36%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.22%</t>
+          <t>5.42%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>9.24%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.20%</t>
+          <t>-4.28%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.87%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.78%</t>
+          <t>14.63%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.26%</t>
+          <t>1.39%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>15.83%</t>
+          <t>15.61%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.10%</t>
+          <t>-2.22%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.97%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.33%</t>
+          <t>15.13%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.41%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.06%</t>
+          <t>0.26%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.38%</t>
+          <t>16.15%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.08%</t>
+          <t>-1.25%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.32%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15.61%</t>
+          <t>15.47%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>0.72%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>16.21%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-1.28%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.99%</t>
+          <t>11.08%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>1.18%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.03%</t>
+          <t>12.10%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.13%</t>
+          <t>16.35%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.58%</t>
+          <t>-1.77%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.51%</t>
+          <t>-11.57%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.30%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.98%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.87%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.58%</t>
+          <t>12.80%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.26%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.76%</t>
+          <t>-9.86%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.25%</t>
+          <t>10.31%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.83%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>12.68%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.34%</t>
+          <t>2.14%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.72%</t>
+          <t>-9.82%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.62%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.02%</t>
+          <t>4.91%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.36%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>13.60%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.06%</t>
+          <t>-10.15%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.59%</t>
+          <t>10.57%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.34%</t>
+          <t>6.13%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.11%</t>
+          <t>7.33%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>4.32%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.43%</t>
+          <t>-7.62%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 21/7/2026</t>
+          <t>As of 22/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.81%</t>
+          <t>15.89%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.75%</t>
+          <t>5.66%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>5.02%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>8.24%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.30%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.51%</t>
+          <t>-5.58%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>16.47%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.32%</t>
+          <t>6.26%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.59%</t>
+          <t>4.65%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.38%</t>
+          <t>8.59%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>3.19%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.20%</t>
+          <t>-5.25%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.99%</t>
+          <t>19.09%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.97%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.87%</t>
+          <t>6.94%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.21%</t>
+          <t>15.43%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.96%</t>
+          <t>-1.15%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.22%</t>
+          <t>-7.28%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.71%</t>
+          <t>15.78%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8.41%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.76%</t>
+          <t>2.85%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.22%</t>
+          <t>5.42%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.77%</t>
+          <t>6.56%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.51%</t>
+          <t>-3.59%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.91%</t>
+          <t>13.93%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.67%</t>
+          <t>11.50%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.16%</t>
+          <t>1.32%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.61%</t>
+          <t>12.39%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.00%</t>
+          <t>-2.15%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>14.04%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.24%</t>
+          <t>12.13%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.06%</t>
+          <t>0.26%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.28%</t>
+          <t>13.06%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.08%</t>
+          <t>-1.17%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.38%</t>
+          <t>14.37%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.73%</t>
+          <t>12.53%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>0.72%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.23%</t>
+          <t>13.01%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-1.06%</t>
+          <t>-1.24%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.91%</t>
+          <t>16.92%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.77%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>10.18%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.13%</t>
+          <t>16.35%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.64%</t>
+          <t>-3.83%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.89%</t>
+          <t>-10.02%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.03%</t>
+          <t>16.09%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.13%</t>
+          <t>2.04%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.33%</t>
+          <t>8.42%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.58%</t>
+          <t>12.80%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>-1.17%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.47%</t>
+          <t>-8.55%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.13%</t>
+          <t>16.20%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.94%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.11%</t>
+          <t>8.20%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>12.68%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.29%</t>
+          <t>-0.48%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.29%</t>
+          <t>-8.36%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.51%</t>
+          <t>16.58%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.70%</t>
+          <t>3.63%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.39%</t>
+          <t>8.47%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>13.60%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.52%</t>
+          <t>-8.59%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.06%</t>
+          <t>16.15%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.87%</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>6.14%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.52%</t>
+          <t>-6.58%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-23]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:09 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/22/2026 at 11:10 AM ET)</t>
+          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>268 days</t>
+          <t>267 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>29 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>149 days</t>
+          <t>148 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>212 days</t>
+          <t>211 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>177 days</t>
+          <t>176 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>359 days</t>
+          <t>358 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>330 days</t>
+          <t>329 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>240 days</t>
+          <t>239 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>303 days</t>
+          <t>302 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>121 days</t>
+          <t>120 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>86 days</t>
+          <t>85 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>58 days</t>
+          <t>57 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>268 days</t>
+          <t>267 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>29 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>149 days</t>
+          <t>148 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>212 days</t>
+          <t>211 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>177 days</t>
+          <t>176 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>359 days</t>
+          <t>358 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>330 days</t>
+          <t>329 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>240 days</t>
+          <t>239 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>303 days</t>
+          <t>302 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>121 days</t>
+          <t>120 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>86 days</t>
+          <t>85 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>58 days</t>
+          <t>57 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.89 / 3.58%</t>
+          <t>$46.43 / 2.57%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.82 / 12.10%</t>
+          <t>$56.49 / 11.45%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.75 / 7.33%</t>
+          <t>$54.26 / 6.37%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.29 / 5.82%</t>
+          <t>$60.74 / 4.87%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.39 / 5.97%</t>
+          <t>$54.90 / 5.03%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$60.11 / 0.43%</t>
+          <t>$59.42 / -0.71%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.12 / 0.41%</t>
+          <t>$59.45 / -0.71%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.52 / 8.69%</t>
+          <t>$52.16 / 7.95%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.34 / 1.39%</t>
+          <t>$55.68 / 0.21%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.76 / 10.36%</t>
+          <t>$58.26 / 9.42%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.63 / 9.95%</t>
+          <t>$52.15 / 8.94%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.45 / 10.00%</t>
+          <t>$54.93 / 8.97%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.80 / 2.85%</t>
+          <t>$41.51 / 2.13%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.66 / 10.18%</t>
+          <t>$41.48 / 9.69%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.00 / 6.14%</t>
+          <t>$39.72 / 5.38%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.19 / 4.65%</t>
+          <t>$43.92 / 4.01%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.21 / 5.02%</t>
+          <t>$44.92 / 4.33%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.82 / 0.40%</t>
+          <t>$43.41 / -0.55%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.29 / 0.33%</t>
+          <t>$40.91 / -0.59%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.41 / 6.94%</t>
+          <t>$44.19 / 6.41%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.20 / 1.32%</t>
+          <t>$42.85 / 0.49%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.00 / 8.47%</t>
+          <t>$41.76 / 7.84%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.73 / 8.20%</t>
+          <t>$41.48 / 7.54%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.18 / 8.42%</t>
+          <t>$40.93 / 7.76%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$748.65 / 5.42%</t>
+          <t>$735.46 / 3.56%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$748.65 / 16.35%</t>
+          <t>$735.46 / 14.30%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$748.65 / 10.00%</t>
+          <t>$735.46 / 8.06%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$748.65 / 8.59%</t>
+          <t>$735.46 / 6.68%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$748.65 / 8.24%</t>
+          <t>$735.46 / 6.33%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$748.65 / 0.72%</t>
+          <t>$735.46 / -1.05%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$748.65 / 0.26%</t>
+          <t>$735.46 / -1.51%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$748.65 / 15.43%</t>
+          <t>$735.46 / 13.40%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$748.65 / 1.28%</t>
+          <t>$735.46 / -0.50%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$748.65 / 13.60%</t>
+          <t>$735.46 / 11.60%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$748.65 / 12.68%</t>
+          <t>$735.46 / 10.70%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$748.65 / 12.80%</t>
+          <t>$735.46 / 10.81%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$748.65 / 5.42%</t>
+          <t>$735.46 / 3.56%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$748.65 / 16.35%</t>
+          <t>$735.46 / 14.30%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$748.65 / 10.00%</t>
+          <t>$735.46 / 8.06%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$748.65 / 8.59%</t>
+          <t>$735.46 / 6.68%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$748.65 / 8.24%</t>
+          <t>$735.46 / 6.33%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$748.65 / 0.72%</t>
+          <t>$735.46 / -1.05%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$748.65 / 0.26%</t>
+          <t>$735.46 / -1.51%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$748.65 / 15.43%</t>
+          <t>$735.46 / 13.40%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$748.65 / 1.28%</t>
+          <t>$735.46 / -0.50%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$748.65 / 13.60%</t>
+          <t>$735.46 / 11.60%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$748.65 / 12.68%</t>
+          <t>$735.46 / 10.70%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$748.65 / 12.80%</t>
+          <t>$735.46 / 10.81%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.96% (10.36%)</t>
+          <t>12.06% (11.45%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.24% (1.18%)</t>
+          <t>1.83% (1.77%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.45% (6.13%)</t>
+          <t>7.41% (7.08%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.35% (7.88%)</t>
+          <t>9.33% (8.86%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.67% (7.28%)</t>
+          <t>8.63% (8.24%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>16.30% (15.47%)</t>
+          <t>17.64% (16.80%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.90% (15.13%)</t>
+          <t>17.20% (16.43%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.53% (7.02%)</t>
+          <t>8.27% (7.76%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.33% (14.63%)</t>
+          <t>16.68% (15.98%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.16% (4.91%)</t>
+          <t>6.06% (5.81%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.09% (3.91%)</t>
+          <t>5.05% (4.87%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2.99% (2.86%)</t>
+          <t>3.96% (3.84%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.02% (8.41%)</t>
+          <t>9.78% (9.17%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.83% (0.77%)</t>
+          <t>1.28% (1.22%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.13% (4.81%)</t>
+          <t>5.88% (5.56%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.73% (6.26%)</t>
+          <t>7.39% (6.91%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.06% (5.66%)</t>
+          <t>6.75% (6.36%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>13.36% (12.53%)</t>
+          <t>14.44% (13.60%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.90% (12.13%)</t>
+          <t>13.95% (13.18%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.43% (5.91%)</t>
+          <t>6.96% (6.44%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.20% (11.50%)</t>
+          <t>13.11% (12.41%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.89% (3.63%)</t>
+          <t>4.50% (4.24%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.04% (2.86%)</t>
+          <t>3.67% (3.49%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.17% (2.04%)</t>
+          <t>2.79% (2.66%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9.24%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-1.77%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.32%</t>
+          <t>6.19%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>7.81%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5.81%</t>
+          <t>7.71%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>18.06%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16.15%</t>
+          <t>18.24%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>3.33%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15.61%</t>
+          <t>17.68%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.14%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>2.88%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>6.56%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-3.83%</t>
+          <t>-2.11%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>3.72%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>3.19%</t>
+          <t>5.04%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>3.30%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>13.01%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.06%</t>
+          <t>15.09%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>0.62%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>14.41%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>1.48%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-0.48%</t>
+          <t>1.31%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>0.61%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.95% (10.35%)</t>
+          <t>10.37% (9.77%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.14% (11.08%)</t>
+          <t>10.27% (10.21%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.89% (10.57%)</t>
+          <t>10.26% (9.93%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.28% (10.82%)</t>
+          <t>10.65% (10.18%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.81% (10.42%)</t>
+          <t>10.16% (9.77%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.20% (9.37%)</t>
+          <t>9.74% (8.90%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.75% (8.98%)</t>
+          <t>9.25% (8.48%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.77% (13.25%)</t>
+          <t>13.00% (12.48%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.61% (8.92%)</t>
+          <t>9.18% (8.47%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.87% (10.62%)</t>
+          <t>10.22% (9.97%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.49% (10.31%)</t>
+          <t>9.89% (9.71%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.47% (10.35%)</t>
+          <t>9.89% (9.77%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.39% (15.78%)</t>
+          <t>15.62% (15.01%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.98% (16.92%)</t>
+          <t>16.07% (16.01%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.47% (16.15%)</t>
+          <t>15.76% (15.43%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.94% (16.47%)</t>
+          <t>16.12% (15.64%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.28% (15.89%)</t>
+          <t>15.49% (15.10%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.20% (14.37%)</t>
+          <t>14.64% (13.80%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.81% (14.04%)</t>
+          <t>14.21% (13.44%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.61% (19.09%)</t>
+          <t>18.75% (18.23%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.62% (13.93%)</t>
+          <t>13.92% (13.22%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.84% (16.58%)</t>
+          <t>16.04% (15.78%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.39% (16.20%)</t>
+          <t>15.60% (15.41%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.22% (16.09%)</t>
+          <t>15.42% (15.30%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.68% (-4.28%)</t>
+          <t>-2.72% (-3.33%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.50% (-11.57%)</t>
+          <t>-10.99% (-11.05%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.29% (-7.62%)</t>
+          <t>-6.46% (-6.78%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.83% (-6.30%)</t>
+          <t>-4.98% (-5.45%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-6.04% (-6.43%)</t>
+          <t>-5.20% (-5.59%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-0.44% (-1.28%)</t>
+          <t>0.00% (-0.14%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.48% (-1.25%)</t>
+          <t>0.00% (-0.14%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.26% (-8.78%)</t>
+          <t>-7.63% (-8.15%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.53% (-2.22%)</t>
+          <t>-0.37% (-1.07%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.90% (-10.15%)</t>
+          <t>-9.13% (-9.38%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.63% (-9.82%)</t>
+          <t>-8.81% (-8.99%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.74% (-9.86%)</t>
+          <t>-8.89% (-9.01%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.98% (-3.59%)</t>
+          <t>-2.31% (-2.92%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.96% (-10.02%)</t>
+          <t>-9.56% (-9.62%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.25% (-6.58%)</t>
+          <t>-5.58% (-5.91%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.78% (-5.25%)</t>
+          <t>-4.20% (-4.67%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.19% (-5.58%)</t>
+          <t>-4.57% (-4.96%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-0.40% (-1.24%)</t>
+          <t>0.00% (-0.29%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.41% (-1.17%)</t>
+          <t>0.00% (-0.25%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.75% (-7.28%)</t>
+          <t>-6.29% (-6.81%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.45% (-2.15%)</t>
+          <t>-0.65% (-1.35%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.33% (-8.59%)</t>
+          <t>-7.79% (-8.05%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.18% (-8.36%)</t>
+          <t>-7.62% (-7.80%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.42% (-8.55%)</t>
+          <t>-7.86% (-7.99%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-14.63%</t>
+          <t>-13.10%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-22.65%</t>
+          <t>-21.26%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.18%</t>
+          <t>-16.71%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.12%</t>
+          <t>-15.63%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.85%</t>
+          <t>-15.36%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-10.64%</t>
+          <t>-9.04%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-10.23%</t>
+          <t>-8.62%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.03%</t>
+          <t>-20.63%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-11.14%</t>
+          <t>-9.55%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.77%</t>
+          <t>-19.35%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.13%</t>
+          <t>-18.70%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.21%</t>
+          <t>-18.78%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-19.37%</t>
+          <t>-17.92%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.94%</t>
+          <t>-25.63%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.72%</t>
+          <t>-21.34%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-21.72%</t>
+          <t>-20.32%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-21.47%</t>
+          <t>-20.06%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-15.60%</t>
+          <t>-14.09%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-15.21%</t>
+          <t>-13.69%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-26.36%</t>
+          <t>-25.04%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.07%</t>
+          <t>-14.57%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.17%</t>
+          <t>-23.83%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-24.56%</t>
+          <t>-23.21%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-24.64%</t>
+          <t>-23.29%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.56% (0.96%)</t>
+          <t>0.75% (0.15%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.24% (1.18%)</t>
+          <t>1.83% (1.77%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.02% (1.70%)</t>
+          <t>1.12% (0.80%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.28% (1.82%)</t>
+          <t>1.38% (0.91%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.73% (1.35%)</t>
+          <t>0.82% (0.43%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.27% (-0.56%)</t>
+          <t>0.70% (-0.14%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.23% (-0.99%)</t>
+          <t>0.64% (-0.14%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.93% (5.42%)</t>
+          <t>4.78% (4.26%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.26% (-0.96%)</t>
+          <t>-0.37% (-1.07%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.42% (2.17%)</t>
+          <t>1.47% (1.21%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.90% (1.72%)</t>
+          <t>1.01% (0.83%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.89% (1.77%)</t>
+          <t>1.03% (0.91%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.29% (1.68%)</t>
+          <t>1.18% (0.57%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.83% (0.77%)</t>
+          <t>1.28% (1.22%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.17% (2.84%)</t>
+          <t>2.07% (1.74%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.42% (2.95%)</t>
+          <t>2.22% (1.74%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.65% (2.26%)</t>
+          <t>1.50% (1.10%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.31% (-0.52%)</t>
+          <t>0.55% (-0.29%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.15% (-0.92%)</t>
+          <t>0.52% (-0.25%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.43% (5.91%)</t>
+          <t>6.30% (5.77%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.19% (-0.89%)</t>
+          <t>-0.65% (-1.35%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.89% (3.63%)</t>
+          <t>2.96% (2.70%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>3.04% (2.86%)</t>
+          <t>2.33% (2.14%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.17% (2.04%)</t>
+          <t>2.16% (2.04%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 22/7/2026</t>
+          <t>As of 23/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.28%</t>
+          <t>8.24%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.97%</t>
+          <t>5.03%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>6.33%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.81%</t>
+          <t>7.71%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.43%</t>
+          <t>-5.59%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.82%</t>
+          <t>10.18%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.88%</t>
+          <t>8.86%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.82%</t>
+          <t>4.87%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.59%</t>
+          <t>6.68%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>7.81%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.30%</t>
+          <t>-5.45%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>12.48%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.02%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.69%</t>
+          <t>7.95%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.43%</t>
+          <t>13.40%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>3.33%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.78%</t>
+          <t>-8.15%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.36%</t>
+          <t>11.45%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>2.57%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.42%</t>
+          <t>3.56%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9.24%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.28%</t>
+          <t>-3.33%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>8.47%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.63%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>0.21%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>15.61%</t>
+          <t>17.68%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.22%</t>
+          <t>-1.07%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.98%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.13%</t>
+          <t>16.43%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.41%</t>
+          <t>-0.71%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.26%</t>
+          <t>-1.51%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.15%</t>
+          <t>18.24%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.25%</t>
+          <t>-0.14%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>8.90%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15.47%</t>
+          <t>16.80%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>-0.71%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>-1.05%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>18.06%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-1.28%</t>
+          <t>-0.14%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.08%</t>
+          <t>10.21%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.18%</t>
+          <t>1.77%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.10%</t>
+          <t>11.45%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.35%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.77%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.57%</t>
+          <t>-11.05%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>8.97%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.80%</t>
+          <t>10.81%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>2.88%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.86%</t>
+          <t>-9.01%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.31%</t>
+          <t>9.71%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>4.87%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.68%</t>
+          <t>10.70%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2.14%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.82%</t>
+          <t>-8.99%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.62%</t>
+          <t>9.97%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.91%</t>
+          <t>5.81%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.36%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.60%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.15%</t>
+          <t>-9.38%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.57%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.13%</t>
+          <t>7.08%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.33%</t>
+          <t>6.37%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>8.06%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.32%</t>
+          <t>6.19%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.62%</t>
+          <t>-6.78%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 22/7/2026</t>
+          <t>As of 23/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.89%</t>
+          <t>15.10%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.66%</t>
+          <t>6.36%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.02%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>6.33%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.30%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.58%</t>
+          <t>-4.96%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.47%</t>
+          <t>15.64%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.26%</t>
+          <t>6.91%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.65%</t>
+          <t>4.01%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8.59%</t>
+          <t>6.68%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.19%</t>
+          <t>5.04%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.25%</t>
+          <t>-4.67%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.09%</t>
+          <t>18.23%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>6.44%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.94%</t>
+          <t>6.41%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.43%</t>
+          <t>13.40%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>0.62%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.28%</t>
+          <t>-6.81%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.78%</t>
+          <t>15.01%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.41%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.85%</t>
+          <t>2.13%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.42%</t>
+          <t>3.56%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.56%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.59%</t>
+          <t>-2.92%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.93%</t>
+          <t>13.22%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.50%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.32%</t>
+          <t>0.49%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>14.41%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.15%</t>
+          <t>-1.35%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.04%</t>
+          <t>13.44%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.13%</t>
+          <t>13.18%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>-0.59%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.26%</t>
+          <t>-1.51%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.06%</t>
+          <t>15.09%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>-0.25%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.37%</t>
+          <t>13.80%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.53%</t>
+          <t>13.60%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>-0.55%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>-1.05%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.01%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-1.24%</t>
+          <t>-0.29%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.92%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.77%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>9.69%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16.35%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-3.83%</t>
+          <t>-2.11%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.02%</t>
+          <t>-9.62%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.09%</t>
+          <t>15.30%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.42%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12.80%</t>
+          <t>10.81%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.55%</t>
+          <t>-7.99%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.20%</t>
+          <t>15.41%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.20%</t>
+          <t>7.54%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12.68%</t>
+          <t>10.70%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.48%</t>
+          <t>1.31%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.36%</t>
+          <t>-7.80%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.58%</t>
+          <t>15.78%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.63%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.47%</t>
+          <t>7.84%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13.60%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>1.48%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.59%</t>
+          <t>-8.05%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.15%</t>
+          <t>15.43%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>5.56%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.14%</t>
+          <t>5.38%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>8.06%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>3.72%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.58%</t>
+          <t>-5.91%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-24]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/23/2026 at 11:31 AM ET)</t>
+          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>267 days</t>
+          <t>266 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>29 days</t>
+          <t>28 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>148 days</t>
+          <t>147 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>211 days</t>
+          <t>210 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>176 days</t>
+          <t>175 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>358 days</t>
+          <t>357 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>329 days</t>
+          <t>328 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>239 days</t>
+          <t>238 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>302 days</t>
+          <t>301 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>120 days</t>
+          <t>119 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>85 days</t>
+          <t>84 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>57 days</t>
+          <t>56 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>267 days</t>
+          <t>266 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>29 days</t>
+          <t>28 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>148 days</t>
+          <t>147 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>211 days</t>
+          <t>210 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>176 days</t>
+          <t>175 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>358 days</t>
+          <t>357 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>329 days</t>
+          <t>328 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>239 days</t>
+          <t>238 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>302 days</t>
+          <t>301 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>120 days</t>
+          <t>119 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>85 days</t>
+          <t>84 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>57 days</t>
+          <t>56 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.43 / 2.57%</t>
+          <t>$46.64 / 3.02%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.49 / 11.45%</t>
+          <t>$56.70 / 11.85%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.26 / 6.37%</t>
+          <t>$54.48 / 6.81%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$60.74 / 4.87%</t>
+          <t>$61.00 / 5.33%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$54.90 / 5.03%</t>
+          <t>$55.12 / 5.46%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.42 / -0.71%</t>
+          <t>$59.72 / -0.22%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.45 / -0.71%</t>
+          <t>$59.71 / -0.27%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.16 / 7.95%</t>
+          <t>$52.33 / 8.30%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$55.68 / 0.21%</t>
+          <t>$55.97 / 0.73%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.26 / 9.42%</t>
+          <t>$58.47 / 9.81%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.15 / 8.94%</t>
+          <t>$52.35 / 9.35%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$54.93 / 8.97%</t>
+          <t>$55.19 / 9.49%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.51 / 2.13%</t>
+          <t>$41.65 / 2.48%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.48 / 9.69%</t>
+          <t>$41.59 / 9.98%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.72 / 5.38%</t>
+          <t>$39.87 / 5.79%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$43.92 / 4.01%</t>
+          <t>$44.04 / 4.30%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$44.92 / 4.33%</t>
+          <t>$45.04 / 4.61%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.41 / -0.55%</t>
+          <t>$43.59 / -0.14%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$40.91 / -0.59%</t>
+          <t>$41.08 / -0.17%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.19 / 6.41%</t>
+          <t>$44.30 / 6.66%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$42.85 / 0.49%</t>
+          <t>$42.97 / 0.76%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.76 / 7.84%</t>
+          <t>$41.85 / 8.07%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.48 / 7.54%</t>
+          <t>$41.60 / 7.85%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$40.93 / 7.76%</t>
+          <t>$41.05 / 8.08%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$735.46 / 3.56%</t>
+          <t>$740.33 / 4.25%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$735.46 / 14.30%</t>
+          <t>$740.33 / 15.06%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$735.46 / 8.06%</t>
+          <t>$740.32 / 8.78%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$735.46 / 6.68%</t>
+          <t>$740.33 / 7.38%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$735.46 / 6.33%</t>
+          <t>$740.33 / 7.04%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$735.46 / -1.05%</t>
+          <t>$740.33 / -0.40%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$735.46 / -1.51%</t>
+          <t>$740.33 / -0.86%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$735.46 / 13.40%</t>
+          <t>$740.33 / 14.15%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$735.46 / -0.50%</t>
+          <t>$740.33 / 0.16%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$735.46 / 11.60%</t>
+          <t>$740.32 / 12.33%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$735.46 / 10.70%</t>
+          <t>$740.32 / 11.43%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$735.46 / 10.81%</t>
+          <t>$740.33 / 11.55%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$735.46 / 3.56%</t>
+          <t>$740.32 / 4.25%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$735.46 / 14.30%</t>
+          <t>$740.32 / 15.06%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$735.46 / 8.06%</t>
+          <t>$740.32 / 8.78%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$735.46 / 6.68%</t>
+          <t>$740.32 / 7.38%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$735.46 / 6.33%</t>
+          <t>$740.32 / 7.04%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$735.46 / -1.05%</t>
+          <t>$740.32 / -0.40%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$735.46 / -1.51%</t>
+          <t>$740.32 / -0.86%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$735.46 / 13.40%</t>
+          <t>$740.32 / 14.15%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$735.46 / -0.50%</t>
+          <t>$740.32 / 0.16%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$735.46 / 11.60%</t>
+          <t>$740.32 / 12.33%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$735.46 / 10.70%</t>
+          <t>$740.32 / 11.43%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$735.46 / 10.81%</t>
+          <t>$740.32 / 11.54%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>12.06% (11.45%)</t>
+          <t>11.56% (10.96%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.83% (1.77%)</t>
+          <t>1.46% (1.41%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.41% (7.08%)</t>
+          <t>6.96% (6.64%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>9.33% (8.86%)</t>
+          <t>8.85% (8.39%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.63% (8.24%)</t>
+          <t>8.18% (7.80%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>17.64% (16.80%)</t>
+          <t>17.06% (16.22%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>17.20% (16.43%)</t>
+          <t>16.68% (15.92%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.27% (7.76%)</t>
+          <t>7.92% (7.41%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>16.68% (15.98%)</t>
+          <t>16.08% (15.38%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>6.06% (5.81%)</t>
+          <t>5.68% (5.43%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5.05% (4.87%)</t>
+          <t>4.65% (4.47%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.96% (3.84%)</t>
+          <t>3.47% (3.35%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.78% (9.17%)</t>
+          <t>9.40% (8.80%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.28% (1.22%)</t>
+          <t>1.01% (0.95%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.88% (5.56%)</t>
+          <t>5.47% (5.15%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.39% (6.91%)</t>
+          <t>7.09% (6.62%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.75% (6.36%)</t>
+          <t>6.46% (6.08%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>14.44% (13.60%)</t>
+          <t>13.97% (13.13%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.95% (13.18%)</t>
+          <t>13.46% (12.69%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.96% (6.44%)</t>
+          <t>6.71% (6.19%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>13.11% (12.41%)</t>
+          <t>12.81% (12.11%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.50% (4.24%)</t>
+          <t>4.27% (4.01%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.67% (3.49%)</t>
+          <t>3.37% (3.19%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.79% (2.66%)</t>
+          <t>2.49% (2.36%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11.20%</t>
+          <t>10.46%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.67%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>6.19%</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>7.81%</t>
+          <t>7.10%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>7.71%</t>
+          <t>7.00%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>18.06%</t>
+          <t>17.29%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>18.24%</t>
+          <t>17.46%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>17.68%</t>
+          <t>16.91%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>3.81%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2.88%</t>
+          <t>2.20%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-2.11%</t>
+          <t>-2.75%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>3.72%</t>
+          <t>3.04%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>5.04%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>5.16%</t>
+          <t>4.46%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>14.28%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>15.09%</t>
+          <t>14.34%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>14.41%</t>
+          <t>13.66%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>1.48%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>1.31%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>-0.06%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.37% (9.77%)</t>
+          <t>10.52% (9.91%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.27% (10.21%)</t>
+          <t>10.47% (10.41%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.26% (9.93%)</t>
+          <t>10.41% (10.09%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.65% (10.18%)</t>
+          <t>10.79% (10.32%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.16% (9.77%)</t>
+          <t>10.32% (9.94%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.74% (8.90%)</t>
+          <t>9.84% (9.01%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.25% (8.48%)</t>
+          <t>9.41% (8.64%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.00% (12.48%)</t>
+          <t>13.22% (12.71%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.18% (8.47%)</t>
+          <t>9.25% (8.56%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.22% (9.97%)</t>
+          <t>10.43% (10.17%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.89% (9.71%)</t>
+          <t>10.08% (9.91%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.89% (9.77%)</t>
+          <t>10.00% (9.88%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.62% (15.01%)</t>
+          <t>15.83% (15.22%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.07% (16.01%)</t>
+          <t>16.32% (16.26%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.76% (15.43%)</t>
+          <t>15.91% (15.58%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.12% (15.64%)</t>
+          <t>16.38% (15.91%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.49% (15.10%)</t>
+          <t>15.76% (15.37%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.64% (13.80%)</t>
+          <t>14.78% (13.95%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.21% (13.44%)</t>
+          <t>14.35% (13.58%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.75% (18.23%)</t>
+          <t>19.02% (18.50%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>13.92% (13.22%)</t>
+          <t>14.21% (13.52%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.04% (15.78%)</t>
+          <t>16.34% (16.08%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.60% (15.41%)</t>
+          <t>15.83% (15.65%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.42% (15.30%)</t>
+          <t>15.66% (15.54%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-2.72% (-3.33%)</t>
+          <t>-3.15% (-3.76%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-10.99% (-11.05%)</t>
+          <t>-11.31% (-11.37%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.46% (-6.78%)</t>
+          <t>-6.85% (-7.17%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-4.98% (-5.45%)</t>
+          <t>-5.40% (-5.86%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.20% (-5.59%)</t>
+          <t>-5.59% (-5.98%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.00% (-0.14%)</t>
+          <t>0.00% (-0.63%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.14%)</t>
+          <t>0.00% (-0.58%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.63% (-8.15%)</t>
+          <t>-7.93% (-8.45%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-0.37% (-1.07%)</t>
+          <t>-0.89% (-1.58%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.13% (-9.38%)</t>
+          <t>-9.46% (-9.71%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-8.81% (-8.99%)</t>
+          <t>-9.15% (-9.33%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-8.89% (-9.01%)</t>
+          <t>-9.32% (-9.44%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.31% (-2.92%)</t>
+          <t>-2.64% (-3.24%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.56% (-9.62%)</t>
+          <t>-9.80% (-9.86%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.58% (-5.91%)</t>
+          <t>-5.95% (-6.27%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.20% (-4.67%)</t>
+          <t>-4.46% (-4.93%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.57% (-4.96%)</t>
+          <t>-4.83% (-5.21%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>0.00% (-0.29%)</t>
+          <t>0.00% (-0.71%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.25%)</t>
+          <t>0.00% (-0.68%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.29% (-6.81%)</t>
+          <t>-6.51% (-7.03%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-0.65% (-1.35%)</t>
+          <t>-0.92% (-1.61%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.79% (-8.05%)</t>
+          <t>-7.99% (-8.25%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.62% (-7.80%)</t>
+          <t>-7.88% (-8.07%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-7.86% (-7.99%)</t>
+          <t>-8.14% (-8.26%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-13.10%</t>
+          <t>-13.67%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.26%</t>
+          <t>-21.78%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-16.71%</t>
+          <t>-17.26%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-15.63%</t>
+          <t>-16.19%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-15.36%</t>
+          <t>-15.92%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-9.04%</t>
+          <t>-9.64%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-8.62%</t>
+          <t>-9.22%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-20.63%</t>
+          <t>-21.15%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-9.55%</t>
+          <t>-10.14%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-19.35%</t>
+          <t>-19.88%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-18.70%</t>
+          <t>-19.23%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-18.78%</t>
+          <t>-19.32%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-17.92%</t>
+          <t>-18.46%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-25.63%</t>
+          <t>-26.12%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-21.34%</t>
+          <t>-21.86%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.32%</t>
+          <t>-20.84%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-20.06%</t>
+          <t>-20.58%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-14.09%</t>
+          <t>-14.66%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-13.69%</t>
+          <t>-14.26%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-25.04%</t>
+          <t>-25.53%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-14.57%</t>
+          <t>-15.13%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-23.83%</t>
+          <t>-24.33%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.21%</t>
+          <t>-23.72%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.29%</t>
+          <t>-23.79%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.75% (0.15%)</t>
+          <t>0.97% (0.37%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.83% (1.77%)</t>
+          <t>1.46% (1.41%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.12% (0.80%)</t>
+          <t>1.37% (1.05%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.38% (0.91%)</t>
+          <t>1.61% (1.15%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.82% (0.43%)</t>
+          <t>1.08% (0.69%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.70% (-0.14%)</t>
+          <t>0.20% (-0.63%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.64% (-0.14%)</t>
+          <t>0.19% (-0.58%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.78% (4.26%)</t>
+          <t>5.13% (4.62%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.37% (-1.07%)</t>
+          <t>-0.73% (-1.43%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.47% (1.21%)</t>
+          <t>1.78% (1.52%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.01% (0.83%)</t>
+          <t>1.30% (1.13%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.03% (0.91%)</t>
+          <t>1.22% (1.11%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.18% (0.57%)</t>
+          <t>1.51% (0.90%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.28% (1.22%)</t>
+          <t>1.01% (0.95%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.07% (1.74%)</t>
+          <t>2.34% (2.02%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2.22% (1.74%)</t>
+          <t>2.61% (2.14%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.50% (1.10%)</t>
+          <t>1.90% (1.51%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.55% (-0.29%)</t>
+          <t>0.13% (-0.71%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.52% (-0.25%)</t>
+          <t>0.09% (-0.68%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.30% (5.77%)</t>
+          <t>6.71% (6.19%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.65% (-1.35%)</t>
+          <t>-0.77% (-1.46%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.96% (2.70%)</t>
+          <t>3.42% (3.16%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.33% (2.14%)</t>
+          <t>2.71% (2.53%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.16% (2.04%)</t>
+          <t>2.49% (2.36%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 23/7/2026</t>
+          <t>As of 24/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>7.80%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.03%</t>
+          <t>5.46%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.33%</t>
+          <t>7.04%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7.71%</t>
+          <t>7.00%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.59%</t>
+          <t>-5.98%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.86%</t>
+          <t>8.39%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.87%</t>
+          <t>5.33%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.68%</t>
+          <t>7.38%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7.81%</t>
+          <t>7.10%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.45%</t>
+          <t>-5.86%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.48%</t>
+          <t>12.71%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>7.41%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.95%</t>
+          <t>8.30%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.40%</t>
+          <t>14.15%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.15%</t>
+          <t>-8.45%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.91%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11.45%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.57%</t>
+          <t>3.02%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11.20%</t>
+          <t>10.46%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.33%</t>
+          <t>-3.76%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.47%</t>
+          <t>8.56%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>15.38%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>0.73%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>17.68%</t>
+          <t>16.91%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>-1.58%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>8.64%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16.43%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.71%</t>
+          <t>-0.27%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.51%</t>
+          <t>-0.86%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>18.24%</t>
+          <t>17.46%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.14%</t>
+          <t>-0.58%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8.90%</t>
+          <t>9.01%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16.80%</t>
+          <t>16.22%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.71%</t>
+          <t>-0.22%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-1.05%</t>
+          <t>-0.40%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>18.06%</t>
+          <t>17.29%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.14%</t>
+          <t>-0.63%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.21%</t>
+          <t>10.41%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.77%</t>
+          <t>1.41%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.45%</t>
+          <t>11.85%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>15.06%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.67%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.05%</t>
+          <t>-11.37%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.88%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>3.35%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.97%</t>
+          <t>9.49%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10.81%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.88%</t>
+          <t>2.20%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.01%</t>
+          <t>-9.44%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.71%</t>
+          <t>9.91%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.87%</t>
+          <t>4.47%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>9.35%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.70%</t>
+          <t>11.43%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.99%</t>
+          <t>-9.33%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.97%</t>
+          <t>10.17%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.81%</t>
+          <t>5.43%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>9.81%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>12.33%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>3.81%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.38%</t>
+          <t>-9.71%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7.08%</t>
+          <t>6.64%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.37%</t>
+          <t>6.81%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.06%</t>
+          <t>8.78%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>6.19%</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.78%</t>
+          <t>-7.17%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 23/7/2026</t>
+          <t>As of 24/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.10%</t>
+          <t>15.37%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.36%</t>
+          <t>6.08%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>4.61%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.33%</t>
+          <t>7.04%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.16%</t>
+          <t>4.46%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-4.96%</t>
+          <t>-5.21%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.64%</t>
+          <t>15.91%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.91%</t>
+          <t>6.62%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.01%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.68%</t>
+          <t>7.38%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.04%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.67%</t>
+          <t>-4.93%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.23%</t>
+          <t>18.50%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.44%</t>
+          <t>6.19%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.41%</t>
+          <t>6.66%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.40%</t>
+          <t>14.15%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.81%</t>
+          <t>-7.03%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.01%</t>
+          <t>15.22%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.13%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-2.92%</t>
+          <t>-3.24%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.22%</t>
+          <t>13.52%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.49%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.41%</t>
+          <t>13.66%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.35%</t>
+          <t>-1.61%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.58%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.18%</t>
+          <t>12.69%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.59%</t>
+          <t>-0.17%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.51%</t>
+          <t>-0.86%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.09%</t>
+          <t>14.34%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.25%</t>
+          <t>-0.68%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13.80%</t>
+          <t>13.95%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.60%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.55%</t>
+          <t>-0.14%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-1.05%</t>
+          <t>-0.40%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>14.28%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.29%</t>
+          <t>-0.71%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>16.26%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>0.95%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>9.98%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>15.06%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.11%</t>
+          <t>-2.75%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.62%</t>
+          <t>-9.86%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.30%</t>
+          <t>15.54%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>2.36%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10.81%</t>
+          <t>11.54%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-7.99%</t>
+          <t>-8.26%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.41%</t>
+          <t>15.65%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>3.19%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.54%</t>
+          <t>7.85%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.70%</t>
+          <t>11.43%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.31%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.80%</t>
+          <t>-8.07%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.78%</t>
+          <t>16.08%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.24%</t>
+          <t>4.01%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.84%</t>
+          <t>8.07%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>12.33%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.48%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.05%</t>
+          <t>-8.25%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.43%</t>
+          <t>15.58%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.56%</t>
+          <t>5.15%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.38%</t>
+          <t>5.79%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.06%</t>
+          <t>8.78%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.72%</t>
+          <t>3.04%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-5.91%</t>
+          <t>-6.27%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-27]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:03 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/24/2026 at 11:04 AM ET)</t>
+          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>266 days</t>
+          <t>263 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>28 days</t>
+          <t>25 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>147 days</t>
+          <t>144 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>210 days</t>
+          <t>207 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>175 days</t>
+          <t>172 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>357 days</t>
+          <t>354 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>328 days</t>
+          <t>325 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>238 days</t>
+          <t>235 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>301 days</t>
+          <t>298 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>119 days</t>
+          <t>116 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>84 days</t>
+          <t>81 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>56 days</t>
+          <t>53 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>266 days</t>
+          <t>263 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>28 days</t>
+          <t>25 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>147 days</t>
+          <t>144 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>210 days</t>
+          <t>207 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>175 days</t>
+          <t>172 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>357 days</t>
+          <t>354 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>328 days</t>
+          <t>325 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>238 days</t>
+          <t>235 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>301 days</t>
+          <t>298 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>119 days</t>
+          <t>116 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>84 days</t>
+          <t>81 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>56 days</t>
+          <t>53 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.64 / 3.02%</t>
+          <t>$46.53 / 2.79%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.70 / 11.85%</t>
+          <t>$56.59 / 11.64%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.48 / 6.81%</t>
+          <t>$54.33 / 6.50%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.00 / 5.33%</t>
+          <t>$60.85 / 5.07%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.12 / 5.46%</t>
+          <t>$55.00 / 5.23%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.72 / -0.22%</t>
+          <t>$59.54 / -0.51%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.71 / -0.27%</t>
+          <t>$59.54 / -0.55%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.33 / 8.30%</t>
+          <t>$52.26 / 8.15%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$55.97 / 0.73%</t>
+          <t>$55.80 / 0.42%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.47 / 9.81%</t>
+          <t>$58.40 / 9.67%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.35 / 9.35%</t>
+          <t>$52.23 / 9.11%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.19 / 9.49%</t>
+          <t>$55.04 / 9.18%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.65 / 2.48%</t>
+          <t>$41.58 / 2.30%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.59 / 9.98%</t>
+          <t>$41.56 / 9.90%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.87 / 5.79%</t>
+          <t>$39.80 / 5.59%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.04 / 4.30%</t>
+          <t>$43.99 / 4.19%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.04 / 4.61%</t>
+          <t>$44.97 / 4.45%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.59 / -0.14%</t>
+          <t>$43.51 / -0.32%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.08 / -0.17%</t>
+          <t>$40.99 / -0.40%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.30 / 6.66%</t>
+          <t>$44.27 / 6.59%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$42.97 / 0.76%</t>
+          <t>$42.89 / 0.59%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.85 / 8.07%</t>
+          <t>$41.83 / 8.03%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.60 / 7.85%</t>
+          <t>$41.56 / 7.76%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.05 / 8.08%</t>
+          <t>$41.01 / 7.99%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$740.33 / 4.25%</t>
+          <t>$736.99 / 3.78%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$740.33 / 15.06%</t>
+          <t>$736.99 / 14.54%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$740.32 / 8.78%</t>
+          <t>$736.99 / 8.29%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$740.33 / 7.38%</t>
+          <t>$736.99 / 6.90%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$740.33 / 7.04%</t>
+          <t>$736.99 / 6.55%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$740.33 / -0.40%</t>
+          <t>$736.99 / -0.85%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$740.33 / -0.86%</t>
+          <t>$736.99 / -1.31%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$740.33 / 14.15%</t>
+          <t>$736.99 / 13.63%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$740.33 / 0.16%</t>
+          <t>$736.99 / -0.30%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$740.32 / 12.33%</t>
+          <t>$736.99 / 11.83%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$740.32 / 11.43%</t>
+          <t>$736.99 / 10.93%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$740.33 / 11.55%</t>
+          <t>$736.99 / 11.04%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$740.32 / 4.25%</t>
+          <t>$736.99 / 3.78%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$740.32 / 15.06%</t>
+          <t>$736.99 / 14.54%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$740.32 / 8.78%</t>
+          <t>$736.99 / 8.29%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$740.32 / 7.38%</t>
+          <t>$736.99 / 6.90%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$740.32 / 7.04%</t>
+          <t>$736.99 / 6.55%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$740.32 / -0.40%</t>
+          <t>$736.99 / -0.85%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$740.32 / -0.86%</t>
+          <t>$736.99 / -1.31%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$740.32 / 14.15%</t>
+          <t>$736.99 / 13.63%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$740.32 / 0.16%</t>
+          <t>$736.99 / -0.30%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$740.32 / 12.33%</t>
+          <t>$736.99 / 11.83%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$740.32 / 11.43%</t>
+          <t>$736.99 / 10.93%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$740.32 / 11.54%</t>
+          <t>$736.99 / 11.04%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.56% (10.96%)</t>
+          <t>11.81% (11.21%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.46% (1.41%)</t>
+          <t>1.65% (1.60%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.96% (6.64%)</t>
+          <t>7.26% (6.95%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.85% (8.39%)</t>
+          <t>9.11% (8.65%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.18% (7.80%)</t>
+          <t>8.41% (8.03%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>17.06% (16.22%)</t>
+          <t>17.39% (16.57%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.68% (15.92%)</t>
+          <t>17.01% (16.25%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.92% (7.41%)</t>
+          <t>8.06% (7.55%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>16.08% (15.38%)</t>
+          <t>16.43% (15.74%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.68% (5.43%)</t>
+          <t>5.81% (5.56%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.65% (4.47%)</t>
+          <t>4.88% (4.70%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.47% (3.35%)</t>
+          <t>3.75% (3.64%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.40% (8.80%)</t>
+          <t>9.58% (8.98%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.01% (0.95%)</t>
+          <t>1.08% (1.03%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.47% (5.15%)</t>
+          <t>5.66% (5.35%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.09% (6.62%)</t>
+          <t>7.19% (6.73%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.46% (6.08%)</t>
+          <t>6.62% (6.24%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>13.97% (13.13%)</t>
+          <t>14.17% (13.34%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.46% (12.69%)</t>
+          <t>13.71% (12.96%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.71% (6.19%)</t>
+          <t>6.77% (6.26%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.81% (12.11%)</t>
+          <t>13.00% (12.31%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.27% (4.01%)</t>
+          <t>4.30% (4.05%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.37% (3.19%)</t>
+          <t>3.45% (3.28%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.49% (2.36%)</t>
+          <t>2.57% (2.45%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10.46%</t>
+          <t>10.97%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-0.67%</t>
+          <t>-0.22%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>5.97%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>7.10%</t>
+          <t>7.59%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>7.00%</t>
+          <t>7.49%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>17.29%</t>
+          <t>17.82%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>17.46%</t>
+          <t>17.99%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.91%</t>
+          <t>17.44%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.81%</t>
+          <t>4.28%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2.20%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-2.75%</t>
+          <t>-2.31%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>3.04%</t>
+          <t>3.51%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.82%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>4.46%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>14.28%</t>
+          <t>14.80%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>14.34%</t>
+          <t>14.85%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>0.41%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>13.66%</t>
+          <t>14.17%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>1.27%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>0.40%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.52% (9.91%)</t>
+          <t>10.34% (9.74%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.47% (10.41%)</t>
+          <t>10.28% (10.22%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.41% (10.09%)</t>
+          <t>10.30% (9.98%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.79% (10.32%)</t>
+          <t>10.63% (10.18%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.32% (9.94%)</t>
+          <t>10.14% (9.76%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.84% (9.01%)</t>
+          <t>9.72% (8.89%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.41% (8.64%)</t>
+          <t>9.27% (8.51%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.22% (12.71%)</t>
+          <t>12.98% (12.47%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.25% (8.56%)</t>
+          <t>9.15% (8.46%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.43% (10.17%)</t>
+          <t>10.17% (9.93%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.08% (9.91%)</t>
+          <t>9.91% (9.74%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.00% (9.88%)</t>
+          <t>9.88% (9.77%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.83% (15.22%)</t>
+          <t>15.61% (15.01%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.32% (16.26%)</t>
+          <t>16.05% (15.99%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.91% (15.58%)</t>
+          <t>15.72% (15.41%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.38% (15.91%)</t>
+          <t>16.11% (15.65%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.76% (15.37%)</t>
+          <t>15.54% (15.16%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.78% (13.95%)</t>
+          <t>14.57% (13.75%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.35% (13.58%)</t>
+          <t>14.18% (13.42%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.02% (18.50%)</t>
+          <t>18.74% (18.22%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.21% (13.52%)</t>
+          <t>13.99% (13.30%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.34% (16.08%)</t>
+          <t>16.02% (15.77%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.83% (15.65%)</t>
+          <t>15.56% (15.38%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.66% (15.54%)</t>
+          <t>15.38% (15.27%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.15% (-3.76%)</t>
+          <t>-2.94% (-3.54%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.31% (-11.37%)</t>
+          <t>-11.15% (-11.20%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.85% (-7.17%)</t>
+          <t>-6.59% (-6.90%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.40% (-5.86%)</t>
+          <t>-5.17% (-5.63%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.59% (-5.98%)</t>
+          <t>-5.39% (-5.77%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.00% (-0.63%)</t>
+          <t>0.00% (-0.34%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.58%)</t>
+          <t>0.00% (-0.30%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.93% (-8.45%)</t>
+          <t>-7.82% (-8.32%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-0.89% (-1.58%)</t>
+          <t>-0.58% (-1.28%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.46% (-9.71%)</t>
+          <t>-9.35% (-9.59%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.15% (-9.33%)</t>
+          <t>-8.95% (-9.13%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.32% (-9.44%)</t>
+          <t>-9.07% (-9.18%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.64% (-3.24%)</t>
+          <t>-2.48% (-3.08%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.80% (-9.86%)</t>
+          <t>-9.74% (-9.79%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.95% (-6.27%)</t>
+          <t>-5.78% (-6.10%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.46% (-4.93%)</t>
+          <t>-4.37% (-4.83%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.83% (-5.21%)</t>
+          <t>-4.68% (-5.07%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>0.00% (-0.71%)</t>
+          <t>0.00% (-0.52%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.68%)</t>
+          <t>0.00% (-0.45%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.51% (-7.03%)</t>
+          <t>-6.46% (-6.97%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-0.92% (-1.61%)</t>
+          <t>-0.75% (-1.44%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.99% (-8.25%)</t>
+          <t>-7.97% (-8.22%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.88% (-8.07%)</t>
+          <t>-7.81% (-7.99%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.14% (-8.26%)</t>
+          <t>-8.06% (-8.18%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-13.67%</t>
+          <t>-13.28%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.78%</t>
+          <t>-21.42%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.26%</t>
+          <t>-16.89%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.19%</t>
+          <t>-15.81%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-15.92%</t>
+          <t>-15.54%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-9.64%</t>
+          <t>-9.23%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.22%</t>
+          <t>-8.81%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.15%</t>
+          <t>-20.80%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.14%</t>
+          <t>-9.73%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-19.88%</t>
+          <t>-19.52%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.23%</t>
+          <t>-18.87%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-19.32%</t>
+          <t>-18.95%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-18.46%</t>
+          <t>-18.09%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.12%</t>
+          <t>-25.79%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-21.86%</t>
+          <t>-21.50%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.84%</t>
+          <t>-20.48%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-20.58%</t>
+          <t>-20.22%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-14.66%</t>
+          <t>-14.27%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.26%</t>
+          <t>-13.87%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-25.53%</t>
+          <t>-25.20%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.13%</t>
+          <t>-14.75%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.33%</t>
+          <t>-23.99%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.72%</t>
+          <t>-23.37%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.79%</t>
+          <t>-23.45%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.97% (0.37%)</t>
+          <t>0.74% (0.14%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.46% (1.41%)</t>
+          <t>1.65% (1.60%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.37% (1.05%)</t>
+          <t>1.19% (0.88%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.61% (1.15%)</t>
+          <t>1.39% (0.93%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.08% (0.69%)</t>
+          <t>0.83% (0.45%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.20% (-0.63%)</t>
+          <t>0.49% (-0.34%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.19% (-0.58%)</t>
+          <t>0.47% (-0.30%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.13% (4.62%)</t>
+          <t>4.79% (4.28%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.73% (-1.43%)</t>
+          <t>-0.58% (-1.28%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.78% (1.52%)</t>
+          <t>1.44% (1.19%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.30% (1.13%)</t>
+          <t>1.06% (0.89%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.22% (1.11%)</t>
+          <t>1.04% (0.93%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.51% (0.90%)</t>
+          <t>1.21% (0.61%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.01% (0.95%)</t>
+          <t>1.08% (1.03%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.34% (2.02%)</t>
+          <t>2.07% (1.75%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2.61% (2.14%)</t>
+          <t>2.25% (1.78%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.90% (1.51%)</t>
+          <t>1.59% (1.20%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.13% (-0.71%)</t>
+          <t>0.30% (-0.52%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.09% (-0.68%)</t>
+          <t>0.31% (-0.45%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.71% (6.19%)</t>
+          <t>6.33% (5.82%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.77% (-1.46%)</t>
+          <t>-0.75% (-1.44%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.42% (3.16%)</t>
+          <t>2.98% (2.73%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.71% (2.53%)</t>
+          <t>2.32% (2.15%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.49% (2.36%)</t>
+          <t>2.16% (2.04%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 24/7/2026</t>
+          <t>As of 27/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.94%</t>
+          <t>9.76%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.80%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.46%</t>
+          <t>5.23%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.04%</t>
+          <t>6.55%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7.00%</t>
+          <t>7.49%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.98%</t>
+          <t>-5.77%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>10.18%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.39%</t>
+          <t>8.65%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.33%</t>
+          <t>5.07%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.38%</t>
+          <t>6.90%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7.10%</t>
+          <t>7.59%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.86%</t>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>12.47%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.41%</t>
+          <t>7.55%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.30%</t>
+          <t>8.15%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.15%</t>
+          <t>13.63%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.45%</t>
+          <t>-8.32%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.91%</t>
+          <t>9.74%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>2.79%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10.46%</t>
+          <t>10.97%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.76%</t>
+          <t>-3.54%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.56%</t>
+          <t>8.46%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.38%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>0.42%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.91%</t>
+          <t>17.44%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.58%</t>
+          <t>-1.28%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.64%</t>
+          <t>8.51%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.25%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>-0.55%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.86%</t>
+          <t>-1.31%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17.46%</t>
+          <t>17.99%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.58%</t>
+          <t>-0.30%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.01%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16.22%</t>
+          <t>16.57%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.22%</t>
+          <t>-0.51%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>-0.85%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>17.29%</t>
+          <t>17.82%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.63%</t>
+          <t>-0.34%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.41%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.41%</t>
+          <t>1.60%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.85%</t>
+          <t>11.64%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.06%</t>
+          <t>14.54%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.67%</t>
+          <t>-0.22%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.37%</t>
+          <t>-11.20%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.88%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.35%</t>
+          <t>3.64%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.49%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>11.04%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.20%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.44%</t>
+          <t>-9.18%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.91%</t>
+          <t>9.74%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.47%</t>
+          <t>4.70%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.35%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.43%</t>
+          <t>10.93%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.33%</t>
+          <t>-9.13%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.17%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.43%</t>
+          <t>5.56%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.81%</t>
+          <t>9.67%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.81%</t>
+          <t>4.28%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.71%</t>
+          <t>-9.59%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>9.98%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.64%</t>
+          <t>6.95%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.81%</t>
+          <t>6.50%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.78%</t>
+          <t>8.29%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>5.97%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.17%</t>
+          <t>-6.90%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 24/7/2026</t>
+          <t>As of 27/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.37%</t>
+          <t>15.16%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.08%</t>
+          <t>6.24%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.61%</t>
+          <t>4.45%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.04%</t>
+          <t>6.55%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.46%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.21%</t>
+          <t>-5.07%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.91%</t>
+          <t>15.65%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.62%</t>
+          <t>6.73%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.30%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.38%</t>
+          <t>6.90%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.82%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.93%</t>
+          <t>-4.83%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.50%</t>
+          <t>18.22%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.19%</t>
+          <t>6.26%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.66%</t>
+          <t>6.59%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.15%</t>
+          <t>13.63%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>0.41%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.03%</t>
+          <t>-6.97%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.22%</t>
+          <t>15.01%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.24%</t>
+          <t>-3.08%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.30%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>12.31%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>0.59%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.66%</t>
+          <t>14.17%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-1.44%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.58%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.69%</t>
+          <t>12.96%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.17%</t>
+          <t>-0.40%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.86%</t>
+          <t>-1.31%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.34%</t>
+          <t>14.85%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.68%</t>
+          <t>-0.45%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13.95%</t>
+          <t>13.75%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.34%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.14%</t>
+          <t>-0.32%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>-0.85%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.28%</t>
+          <t>14.80%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.71%</t>
+          <t>-0.52%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.26%</t>
+          <t>15.99%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.06%</t>
+          <t>14.54%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.75%</t>
+          <t>-2.31%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.86%</t>
+          <t>-9.79%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.54%</t>
+          <t>15.27%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.36%</t>
+          <t>2.45%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.99%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>11.04%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.26%</t>
+          <t>-8.18%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.65%</t>
+          <t>15.38%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.19%</t>
+          <t>3.28%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.85%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.43%</t>
+          <t>10.93%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.07%</t>
+          <t>-7.99%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.08%</t>
+          <t>15.77%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.01%</t>
+          <t>4.05%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.07%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>1.27%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.25%</t>
+          <t>-8.22%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.58%</t>
+          <t>15.41%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.15%</t>
+          <t>5.35%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.79%</t>
+          <t>5.59%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.78%</t>
+          <t>8.29%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.04%</t>
+          <t>3.51%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.27%</t>
+          <t>-6.10%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-28]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/27/2026 at 11:50 AM ET)</t>
+          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>263 days</t>
+          <t>262 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>25 days</t>
+          <t>24 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>144 days</t>
+          <t>143 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>207 days</t>
+          <t>206 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>172 days</t>
+          <t>171 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>354 days</t>
+          <t>353 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>325 days</t>
+          <t>324 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>235 days</t>
+          <t>234 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>298 days</t>
+          <t>297 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>116 days</t>
+          <t>115 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>81 days</t>
+          <t>80 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>53 days</t>
+          <t>52 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>263 days</t>
+          <t>262 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>25 days</t>
+          <t>24 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>144 days</t>
+          <t>143 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>207 days</t>
+          <t>206 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>172 days</t>
+          <t>171 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>354 days</t>
+          <t>353 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>325 days</t>
+          <t>324 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>235 days</t>
+          <t>234 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>298 days</t>
+          <t>297 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>116 days</t>
+          <t>115 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>81 days</t>
+          <t>80 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>53 days</t>
+          <t>52 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.53 / 2.79%</t>
+          <t>$46.72 / 3.20%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.59 / 11.64%</t>
+          <t>$56.77 / 11.99%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.33 / 6.50%</t>
+          <t>$54.56 / 6.96%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$60.85 / 5.07%</t>
+          <t>$61.10 / 5.50%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.00 / 5.23%</t>
+          <t>$55.22 / 5.65%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.54 / -0.51%</t>
+          <t>$59.83 / -0.03%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.54 / -0.55%</t>
+          <t>$59.80 / -0.12%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.26 / 8.15%</t>
+          <t>$52.43 / 8.51%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$55.80 / 0.42%</t>
+          <t>$56.06 / 0.89%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.40 / 9.67%</t>
+          <t>$58.62 / 10.09%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.23 / 9.11%</t>
+          <t>$52.43 / 9.53%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.04 / 9.18%</t>
+          <t>$55.28 / 9.66%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.58 / 2.30%</t>
+          <t>$41.72 / 2.64%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.56 / 9.90%</t>
+          <t>$41.63 / 10.10%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.80 / 5.59%</t>
+          <t>$39.93 / 5.94%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$43.99 / 4.19%</t>
+          <t>$44.12 / 4.49%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$44.97 / 4.45%</t>
+          <t>$45.13 / 4.83%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.51 / -0.32%</t>
+          <t>$43.68 / 0.07%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$40.99 / -0.40%</t>
+          <t>$41.13 / -0.05%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.27 / 6.59%</t>
+          <t>$44.41 / 6.94%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$42.89 / 0.59%</t>
+          <t>$43.03 / 0.91%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.83 / 8.03%</t>
+          <t>$41.94 / 8.31%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.56 / 7.76%</t>
+          <t>$41.67 / 8.05%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.01 / 7.99%</t>
+          <t>$41.11 / 8.25%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$736.99 / 3.78%</t>
+          <t>$741.59 / 4.43%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$736.99 / 14.54%</t>
+          <t>$741.59 / 15.25%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$736.99 / 8.29%</t>
+          <t>$741.59 / 8.96%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$736.99 / 6.90%</t>
+          <t>$741.59 / 7.57%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$736.99 / 6.55%</t>
+          <t>$741.59 / 7.22%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$736.99 / -0.85%</t>
+          <t>$741.59 / -0.23%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$736.99 / -1.31%</t>
+          <t>$741.59 / -0.69%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$736.99 / 13.63%</t>
+          <t>$741.59 / 14.34%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$736.99 / -0.30%</t>
+          <t>$741.59 / 0.33%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$736.99 / 11.83%</t>
+          <t>$741.59 / 12.53%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$736.99 / 10.93%</t>
+          <t>$741.59 / 11.62%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$736.99 / 11.04%</t>
+          <t>$741.59 / 11.74%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$736.99 / 3.78%</t>
+          <t>$741.65 / 4.44%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$736.99 / 14.54%</t>
+          <t>$741.65 / 15.26%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$736.99 / 8.29%</t>
+          <t>$741.65 / 8.97%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$736.99 / 6.90%</t>
+          <t>$741.59 / 7.57%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$736.99 / 6.55%</t>
+          <t>$741.59 / 7.22%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$736.99 / -0.85%</t>
+          <t>$741.65 / -0.22%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$736.99 / -1.31%</t>
+          <t>$741.65 / -0.68%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$736.99 / 13.63%</t>
+          <t>$741.65 / 14.35%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$736.99 / -0.30%</t>
+          <t>$741.65 / 0.34%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$736.99 / 11.83%</t>
+          <t>$741.65 / 12.54%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$736.99 / 10.93%</t>
+          <t>$741.65 / 11.63%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$736.99 / 11.04%</t>
+          <t>$741.65 / 11.74%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.81% (11.21%)</t>
+          <t>11.36% (10.77%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.65% (1.60%)</t>
+          <t>1.33% (1.28%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.26% (6.95%)</t>
+          <t>6.81% (6.50%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>9.11% (8.65%)</t>
+          <t>8.66% (8.21%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.41% (8.03%)</t>
+          <t>7.98% (7.60%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>17.39% (16.57%)</t>
+          <t>16.83% (16.01%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>17.01% (16.25%)</t>
+          <t>16.50% (15.74%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.06% (7.55%)</t>
+          <t>7.71% (7.20%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>16.43% (15.74%)</t>
+          <t>15.88% (15.20%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.81% (5.56%)</t>
+          <t>5.41% (5.16%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.88% (4.70%)</t>
+          <t>4.48% (4.31%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.75% (3.64%)</t>
+          <t>3.30% (3.19%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.58% (8.98%)</t>
+          <t>9.23% (8.63%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.08% (1.03%)</t>
+          <t>0.89% (0.84%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.66% (5.35%)</t>
+          <t>5.32% (5.00%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.19% (6.73%)</t>
+          <t>6.89% (6.43%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.62% (6.24%)</t>
+          <t>6.23% (5.85%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>14.17% (13.34%)</t>
+          <t>13.72% (12.90%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.71% (12.96%)</t>
+          <t>13.31% (12.56%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.77% (6.26%)</t>
+          <t>6.42% (5.91%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>13.00% (12.31%)</t>
+          <t>12.64% (11.96%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.30% (4.05%)</t>
+          <t>4.02% (3.78%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.45% (3.28%)</t>
+          <t>3.18% (3.01%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.57% (2.45%)</t>
+          <t>2.31% (2.20%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10.97%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>-0.84%</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>5.31%</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>6.92%</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>6.82%</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>17.09%</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>17.26%</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2.47%</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>16.71%</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>3.64%</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>3.11%</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2.03%</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>7.57%</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>-2.92%</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2.86%</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>4.17%</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>4.29%</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>14.07%</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>14.13%</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
           <t>-0.22%</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>5.97%</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>7.59%</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>7.49%</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>17.82%</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>17.99%</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>3.11%</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>17.44%</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>4.28%</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>3.75%</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2.66%</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>8.25%</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>-2.31%</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>3.51%</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>4.82%</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>4.94%</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>14.80%</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>14.85%</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>0.41%</t>
-        </is>
-      </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>14.17%</t>
+          <t>13.45%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>0.46%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>-0.23%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.34% (9.74%)</t>
+          <t>10.49% (9.90%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.28% (10.22%)</t>
+          <t>10.48% (10.43%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.30% (9.98%)</t>
+          <t>10.42% (10.11%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.63% (10.18%)</t>
+          <t>10.77% (10.31%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.14% (9.76%)</t>
+          <t>10.29% (9.91%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.72% (8.89%)</t>
+          <t>9.80% (8.98%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.27% (8.51%)</t>
+          <t>9.40% (8.65%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>12.98% (12.47%)</t>
+          <t>13.17% (12.67%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.15% (8.46%)</t>
+          <t>9.24% (8.55%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.17% (9.93%)</t>
+          <t>10.33% (10.09%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.91% (9.74%)</t>
+          <t>10.07% (9.90%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.88% (9.77%)</t>
+          <t>9.98% (9.87%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.61% (15.01%)</t>
+          <t>15.81% (15.22%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.05% (15.99%)</t>
+          <t>16.35% (16.30%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.72% (15.41%)</t>
+          <t>15.91% (15.59%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.11% (15.65%)</t>
+          <t>16.33% (15.87%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.54% (15.16%)</t>
+          <t>15.69% (15.31%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.57% (13.75%)</t>
+          <t>14.72% (13.90%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.18% (13.42%)</t>
+          <t>14.37% (13.61%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.74% (18.22%)</t>
+          <t>18.90% (18.39%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>13.99% (13.30%)</t>
+          <t>14.22% (13.53%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.02% (15.77%)</t>
+          <t>16.26% (16.01%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.56% (15.38%)</t>
+          <t>15.79% (15.62%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.38% (15.27%)</t>
+          <t>15.64% (15.53%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-2.94% (-3.54%)</t>
+          <t>-3.33% (-3.92%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.15% (-11.20%)</t>
+          <t>-11.43% (-11.48%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.59% (-6.90%)</t>
+          <t>-6.98% (-7.30%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.17% (-5.63%)</t>
+          <t>-5.56% (-6.02%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.39% (-5.77%)</t>
+          <t>-5.77% (-6.15%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.00% (-0.34%)</t>
+          <t>0.00% (-0.81%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.30%)</t>
+          <t>0.00% (-0.73%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.82% (-8.32%)</t>
+          <t>-8.12% (-8.62%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-0.58% (-1.28%)</t>
+          <t>-1.06% (-1.74%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.35% (-9.59%)</t>
+          <t>-9.69% (-9.93%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-8.95% (-9.13%)</t>
+          <t>-9.30% (-9.47%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.07% (-9.18%)</t>
+          <t>-9.47% (-9.58%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.48% (-3.08%)</t>
+          <t>-2.80% (-3.39%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.74% (-9.79%)</t>
+          <t>-9.91% (-9.96%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.78% (-6.10%)</t>
+          <t>-6.09% (-6.40%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.37% (-4.83%)</t>
+          <t>-4.64% (-5.10%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.68% (-5.07%)</t>
+          <t>-5.03% (-5.41%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>0.00% (-0.52%)</t>
+          <t>-0.09% (-0.91%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.45%)</t>
+          <t>-0.04% (-0.80%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.46% (-6.97%)</t>
+          <t>-6.77% (-7.28%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-0.75% (-1.44%)</t>
+          <t>-1.07% (-1.75%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.97% (-8.22%)</t>
+          <t>-8.21% (-8.46%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.81% (-7.99%)</t>
+          <t>-8.06% (-8.23%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.06% (-8.18%)</t>
+          <t>-8.29% (-8.40%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-13.28%</t>
+          <t>-13.82%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.42%</t>
+          <t>-21.91%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-16.89%</t>
+          <t>-17.40%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-15.81%</t>
+          <t>-16.33%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-15.54%</t>
+          <t>-16.06%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-9.23%</t>
+          <t>-9.79%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-8.81%</t>
+          <t>-9.37%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-20.80%</t>
+          <t>-21.29%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-9.73%</t>
+          <t>-10.29%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-19.52%</t>
+          <t>-20.02%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-18.87%</t>
+          <t>-19.37%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-18.95%</t>
+          <t>-19.45%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-18.09%</t>
+          <t>-18.61%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-25.79%</t>
+          <t>-26.25%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-21.50%</t>
+          <t>-22.00%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.48%</t>
+          <t>-20.98%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-20.22%</t>
+          <t>-20.72%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-14.27%</t>
+          <t>-14.81%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-13.87%</t>
+          <t>-14.41%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-25.20%</t>
+          <t>-25.67%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-14.75%</t>
+          <t>-15.28%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-23.99%</t>
+          <t>-24.47%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.37%</t>
+          <t>-23.85%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.45%</t>
+          <t>-23.93%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.74% (0.14%)</t>
+          <t>0.96% (0.37%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.65% (1.60%)</t>
+          <t>1.33% (1.28%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.19% (0.88%)</t>
+          <t>1.40% (1.08%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.39% (0.93%)</t>
+          <t>1.61% (1.15%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.83% (0.45%)</t>
+          <t>1.06% (0.68%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.49% (-0.34%)</t>
+          <t>0.01% (-0.81%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.47% (-0.30%)</t>
+          <t>0.03% (-0.73%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.79% (4.28%)</t>
+          <t>5.10% (4.60%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.58% (-1.28%)</t>
+          <t>-0.73% (-1.42%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.44% (1.19%)</t>
+          <t>1.69% (1.45%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.06% (0.89%)</t>
+          <t>1.31% (1.14%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.04% (0.93%)</t>
+          <t>1.23% (1.12%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.21% (0.61%)</t>
+          <t>1.52% (0.93%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.08% (1.03%)</t>
+          <t>0.89% (0.84%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.07% (1.75%)</t>
+          <t>2.38% (2.06%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2.25% (1.78%)</t>
+          <t>2.59% (2.13%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.59% (1.20%)</t>
+          <t>1.85% (1.47%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.30% (-0.52%)</t>
+          <t>-0.09% (-0.91%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.31% (-0.45%)</t>
+          <t>-0.04% (-0.80%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.33% (5.82%)</t>
+          <t>6.42% (5.91%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.75% (-1.44%)</t>
+          <t>-0.74% (-1.42%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.98% (2.73%)</t>
+          <t>3.36% (3.12%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.32% (2.15%)</t>
+          <t>2.70% (2.53%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.16% (2.04%)</t>
+          <t>2.31% (2.20%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 27/7/2026</t>
+          <t>As of 28/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.76%</t>
+          <t>9.91%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.23%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.55%</t>
+          <t>7.22%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7.49%</t>
+          <t>6.82%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.77%</t>
+          <t>-6.15%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>10.31%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.65%</t>
+          <t>8.21%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.07%</t>
+          <t>5.50%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.90%</t>
+          <t>7.57%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7.59%</t>
+          <t>6.92%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-6.02%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.47%</t>
+          <t>12.67%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.55%</t>
+          <t>7.20%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.15%</t>
+          <t>8.51%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.63%</t>
+          <t>14.34%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>2.47%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.32%</t>
+          <t>-8.62%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.74%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.79%</t>
+          <t>3.20%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>4.43%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10.97%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.54%</t>
+          <t>-3.92%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.46%</t>
+          <t>8.55%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>15.20%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.89%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>17.44%</t>
+          <t>16.71%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.28%</t>
+          <t>-1.74%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.51%</t>
+          <t>8.65%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16.25%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.55%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-0.69%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17.99%</t>
+          <t>17.26%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>-0.73%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16.57%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.51%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-0.23%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>17.82%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.34%</t>
+          <t>-0.81%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>10.43%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.64%</t>
+          <t>11.99%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.54%</t>
+          <t>15.25%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.22%</t>
+          <t>-0.84%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.20%</t>
+          <t>-11.48%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.87%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.64%</t>
+          <t>3.19%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>9.66%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.04%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.18%</t>
+          <t>-9.58%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.74%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.53%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.13%</t>
+          <t>-9.47%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.56%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.67%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>12.53%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4.28%</t>
+          <t>3.64%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.59%</t>
+          <t>-9.93%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>10.11%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.95%</t>
+          <t>6.50%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.50%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.29%</t>
+          <t>8.96%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5.97%</t>
+          <t>5.31%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.90%</t>
+          <t>-7.30%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 27/7/2026</t>
+          <t>As of 28/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.16%</t>
+          <t>15.31%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>5.85%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.45%</t>
+          <t>4.83%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.55%</t>
+          <t>7.22%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>4.29%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.07%</t>
+          <t>-5.41%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.65%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.73%</t>
+          <t>6.43%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.49%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.90%</t>
+          <t>7.57%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.82%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.83%</t>
+          <t>-5.10%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.22%</t>
+          <t>18.39%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.26%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.59%</t>
+          <t>6.94%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.63%</t>
+          <t>14.35%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.41%</t>
+          <t>-0.22%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.97%</t>
+          <t>-7.28%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.01%</t>
+          <t>15.22%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.98%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>4.44%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>7.57%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.08%</t>
+          <t>-3.39%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.30%</t>
+          <t>13.53%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.31%</t>
+          <t>11.96%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.59%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.17%</t>
+          <t>13.45%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-1.75%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>13.61%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.96%</t>
+          <t>12.56%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-0.68%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.85%</t>
+          <t>14.13%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.45%</t>
+          <t>-0.80%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13.75%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.34%</t>
+          <t>12.90%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-0.22%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.80%</t>
+          <t>14.07%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>-0.91%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>15.99%</t>
+          <t>16.30%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>0.84%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>10.10%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.54%</t>
+          <t>15.26%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.31%</t>
+          <t>-2.92%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.79%</t>
+          <t>-9.96%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.27%</t>
+          <t>15.53%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.45%</t>
+          <t>2.20%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.99%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.04%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>-0.23%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.18%</t>
+          <t>-8.40%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.38%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.28%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>8.05%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>11.63%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>0.46%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.99%</t>
+          <t>-8.23%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.77%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>8.31%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>12.54%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.22%</t>
+          <t>-8.46%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.41%</t>
+          <t>15.59%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.35%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.59%</t>
+          <t>5.94%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.29%</t>
+          <t>8.97%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.51%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.10%</t>
+          <t>-6.40%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-29]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:41 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/28/2026 at 11:42 AM ET)</t>
+          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>262 days</t>
+          <t>261 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>24 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>143 days</t>
+          <t>142 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>206 days</t>
+          <t>205 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>171 days</t>
+          <t>170 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>353 days</t>
+          <t>352 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>324 days</t>
+          <t>323 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>234 days</t>
+          <t>233 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>297 days</t>
+          <t>296 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>115 days</t>
+          <t>114 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>80 days</t>
+          <t>79 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>52 days</t>
+          <t>51 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>262 days</t>
+          <t>261 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>24 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>143 days</t>
+          <t>142 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>206 days</t>
+          <t>205 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>171 days</t>
+          <t>170 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>353 days</t>
+          <t>352 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>324 days</t>
+          <t>323 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>234 days</t>
+          <t>233 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>297 days</t>
+          <t>296 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>115 days</t>
+          <t>114 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>80 days</t>
+          <t>79 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>52 days</t>
+          <t>51 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.72 / 3.20%</t>
+          <t>$46.46 / 2.62%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.77 / 11.99%</t>
+          <t>$56.53 / 11.53%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.56 / 6.96%</t>
+          <t>$54.25 / 6.35%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.10 / 5.50%</t>
+          <t>$60.79 / 4.96%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.22 / 5.65%</t>
+          <t>$54.89 / 5.02%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.83 / -0.03%</t>
+          <t>$59.44 / -0.69%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.80 / -0.12%</t>
+          <t>$59.42 / -0.76%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.43 / 8.51%</t>
+          <t>$52.23 / 8.10%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.06 / 0.89%</t>
+          <t>$55.69 / 0.23%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.62 / 10.09%</t>
+          <t>$58.29 / 9.47%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.43 / 9.53%</t>
+          <t>$52.14 / 8.91%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.28 / 9.66%</t>
+          <t>$54.95 / 9.00%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.72 / 2.64%</t>
+          <t>$41.53 / 2.18%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.63 / 10.10%</t>
+          <t>$41.56 / 9.90%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.93 / 5.94%</t>
+          <t>$39.79 / 5.57%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.12 / 4.49%</t>
+          <t>$43.96 / 4.11%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.13 / 4.83%</t>
+          <t>$44.94 / 4.39%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.68 / 0.07%</t>
+          <t>$43.44 / -0.48%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.13 / -0.05%</t>
+          <t>$40.92 / -0.56%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.41 / 6.94%</t>
+          <t>$44.26 / 6.56%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.03 / 0.91%</t>
+          <t>$42.83 / 0.44%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.94 / 8.31%</t>
+          <t>$41.80 / 7.94%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.67 / 8.05%</t>
+          <t>$41.52 / 7.66%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.11 / 8.25%</t>
+          <t>$40.97 / 7.88%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$741.59 / 4.43%</t>
+          <t>$734.54 / 3.44%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$741.59 / 15.25%</t>
+          <t>$734.54 / 14.16%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$741.59 / 8.96%</t>
+          <t>$734.54 / 7.93%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$741.59 / 7.57%</t>
+          <t>$734.54 / 6.54%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$741.59 / 7.22%</t>
+          <t>$734.54 / 6.20%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$741.59 / -0.23%</t>
+          <t>$734.54 / -1.18%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$741.59 / -0.69%</t>
+          <t>$734.54 / -1.63%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$741.59 / 14.34%</t>
+          <t>$734.54 / 13.25%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$741.59 / 0.33%</t>
+          <t>$734.54 / -0.63%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$741.59 / 12.53%</t>
+          <t>$734.54 / 11.46%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$741.59 / 11.62%</t>
+          <t>$734.54 / 10.56%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$741.59 / 11.74%</t>
+          <t>$734.54 / 10.67%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$741.65 / 4.44%</t>
+          <t>$734.54 / 3.44%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$741.65 / 15.26%</t>
+          <t>$734.54 / 14.16%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$741.65 / 8.97%</t>
+          <t>$734.54 / 7.93%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$741.59 / 7.57%</t>
+          <t>$734.54 / 6.54%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$741.59 / 7.22%</t>
+          <t>$734.54 / 6.20%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$741.65 / -0.22%</t>
+          <t>$734.54 / -1.18%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$741.65 / -0.68%</t>
+          <t>$734.54 / -1.63%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$741.65 / 14.35%</t>
+          <t>$734.54 / 13.25%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$741.65 / 0.34%</t>
+          <t>$734.54 / -0.63%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$741.65 / 12.54%</t>
+          <t>$734.54 / 11.46%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$741.65 / 11.63%</t>
+          <t>$734.54 / 10.56%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$741.65 / 11.74%</t>
+          <t>$734.54 / 10.67%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.36% (10.77%)</t>
+          <t>11.98% (11.39%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.33% (1.28%)</t>
+          <t>1.75% (1.70%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.81% (6.50%)</t>
+          <t>7.42% (7.10%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.66% (8.21%)</t>
+          <t>9.22% (8.77%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>7.98% (7.60%)</t>
+          <t>8.63% (8.25%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>16.83% (16.01%)</t>
+          <t>17.60% (16.77%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.50% (15.74%)</t>
+          <t>17.25% (16.49%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.71% (7.20%)</t>
+          <t>8.11% (7.60%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.88% (15.20%)</t>
+          <t>16.65% (15.96%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.41% (5.16%)</t>
+          <t>6.00% (5.76%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.48% (4.31%)</t>
+          <t>5.06% (4.90%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.30% (3.19%)</t>
+          <t>3.92% (3.81%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.23% (8.63%)</t>
+          <t>9.71% (9.11%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.89% (0.84%)</t>
+          <t>1.07% (1.03%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.32% (5.00%)</t>
+          <t>5.69% (5.37%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.89% (6.43%)</t>
+          <t>7.28% (6.82%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.23% (5.85%)</t>
+          <t>6.68% (6.30%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>13.72% (12.90%)</t>
+          <t>14.35% (13.52%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.31% (12.56%)</t>
+          <t>13.89% (13.13%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.42% (5.91%)</t>
+          <t>6.79% (6.28%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.64% (11.96%)</t>
+          <t>13.16% (12.48%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.02% (3.78%)</t>
+          <t>4.38% (4.14%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.18% (3.01%)</t>
+          <t>3.55% (3.38%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.31% (2.20%)</t>
+          <t>2.66% (2.55%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-0.84%</t>
+          <t>0.12%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.31%</t>
+          <t>6.32%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.92%</t>
+          <t>7.95%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.82%</t>
+          <t>7.85%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>18.21%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>17.26%</t>
+          <t>18.39%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.47%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.71%</t>
+          <t>17.83%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.64%</t>
+          <t>4.63%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>4.10%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>7.57%</t>
+          <t>8.61%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-2.92%</t>
+          <t>-1.98%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>3.85%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>4.17%</t>
+          <t>5.17%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>4.29%</t>
+          <t>5.29%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>14.07%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>15.24%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.22%</t>
+          <t>0.75%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>13.45%</t>
+          <t>14.55%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>1.43%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.23%</t>
+          <t>0.73%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.49% (9.90%)</t>
+          <t>10.20% (9.61%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.48% (10.43%)</t>
+          <t>10.10% (10.05%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.42% (10.11%)</t>
+          <t>10.16% (9.84%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.77% (10.31%)</t>
+          <t>10.45% (10.00%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.29% (9.91%)</t>
+          <t>10.04% (9.67%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.80% (8.98%)</t>
+          <t>9.59% (8.76%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.40% (8.65%)</t>
+          <t>9.18% (8.42%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.17% (12.67%)</t>
+          <t>12.76% (12.25%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.24% (8.55%)</t>
+          <t>9.03% (8.34%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.33% (10.09%)</t>
+          <t>10.07% (9.83%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.07% (9.90%)</t>
+          <t>9.80% (9.63%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.98% (9.87%)</t>
+          <t>9.75% (9.64%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.81% (15.22%)</t>
+          <t>15.45% (14.86%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.35% (16.30%)</t>
+          <t>15.79% (15.75%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.91% (15.59%)</t>
+          <t>15.48% (15.17%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.33% (15.87%)</t>
+          <t>15.92% (15.46%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.69% (15.31%)</t>
+          <t>15.32% (14.94%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.72% (13.90%)</t>
+          <t>14.45% (13.62%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.37% (13.61%)</t>
+          <t>14.05% (13.29%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.90% (18.39%)</t>
+          <t>18.50% (18.00%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.22% (13.53%)</t>
+          <t>13.86% (13.17%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.26% (16.01%)</t>
+          <t>15.84% (15.60%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.79% (15.62%)</t>
+          <t>15.39% (15.22%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.64% (15.53%)</t>
+          <t>15.21% (15.10%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.33% (-3.92%)</t>
+          <t>-2.79% (-3.38%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.43% (-11.48%)</t>
+          <t>-11.06% (-11.11%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.98% (-7.30%)</t>
+          <t>-6.45% (-6.77%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.56% (-6.02%)</t>
+          <t>-5.08% (-5.53%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.77% (-6.15%)</t>
+          <t>-5.21% (-5.59%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.00% (-0.81%)</t>
+          <t>0.00% (-0.16%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.73%)</t>
+          <t>0.00% (-0.09%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.12% (-8.62%)</t>
+          <t>-7.78% (-8.28%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.06% (-1.74%)</t>
+          <t>-0.40% (-1.09%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.69% (-9.93%)</t>
+          <t>-9.18% (-9.42%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.30% (-9.47%)</t>
+          <t>-8.79% (-8.96%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.47% (-9.58%)</t>
+          <t>-8.93% (-9.04%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.80% (-3.39%)</t>
+          <t>-2.37% (-2.96%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.91% (-9.96%)</t>
+          <t>-9.75% (-9.79%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.09% (-6.40%)</t>
+          <t>-5.76% (-6.07%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.64% (-5.10%)</t>
+          <t>-4.30% (-4.76%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.03% (-5.41%)</t>
+          <t>-4.64% (-5.01%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-0.09% (-0.91%)</t>
+          <t>0.00% (-0.36%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.04% (-0.80%)</t>
+          <t>0.00% (-0.29%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.77% (-7.28%)</t>
+          <t>-6.44% (-6.95%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.07% (-1.75%)</t>
+          <t>-0.61% (-1.29%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.21% (-8.46%)</t>
+          <t>-7.89% (-8.14%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.06% (-8.23%)</t>
+          <t>-7.73% (-7.90%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.29% (-8.40%)</t>
+          <t>-7.98% (-8.09%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-13.82%</t>
+          <t>-12.99%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.91%</t>
+          <t>-21.16%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.40%</t>
+          <t>-16.61%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.33%</t>
+          <t>-15.53%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.06%</t>
+          <t>-15.25%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-9.79%</t>
+          <t>-8.93%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.37%</t>
+          <t>-8.50%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.29%</t>
+          <t>-20.53%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.29%</t>
+          <t>-9.43%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-20.02%</t>
+          <t>-19.25%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.37%</t>
+          <t>-18.59%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-19.45%</t>
+          <t>-18.68%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-18.61%</t>
+          <t>-17.82%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.25%</t>
+          <t>-25.54%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-22.00%</t>
+          <t>-21.24%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.98%</t>
+          <t>-20.22%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-20.72%</t>
+          <t>-19.96%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-14.81%</t>
+          <t>-13.98%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.41%</t>
+          <t>-13.58%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-25.67%</t>
+          <t>-24.95%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.28%</t>
+          <t>-14.46%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.47%</t>
+          <t>-23.73%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.85%</t>
+          <t>-23.11%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.93%</t>
+          <t>-23.19%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.96% (0.37%)</t>
+          <t>0.56% (-0.03%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.33% (1.28%)</t>
+          <t>1.63% (1.58%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.40% (1.08%)</t>
+          <t>1.00% (0.69%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.61% (1.15%)</t>
+          <t>1.16% (0.70%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.06% (0.68%)</t>
+          <t>0.69% (0.32%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.01% (-0.81%)</t>
+          <t>0.66% (-0.16%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.03% (-0.73%)</t>
+          <t>0.67% (-0.09%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.10% (4.60%)</t>
+          <t>4.48% (3.98%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.73% (-1.42%)</t>
+          <t>-0.40% (-1.09%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.69% (1.45%)</t>
+          <t>1.29% (1.04%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.31% (1.14%)</t>
+          <t>0.90% (0.73%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.23% (1.12%)</t>
+          <t>0.87% (0.76%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.52% (0.93%)</t>
+          <t>0.99% (0.40%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.89% (0.84%)</t>
+          <t>1.07% (1.03%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.38% (2.06%)</t>
+          <t>1.75% (1.43%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2.59% (2.13%)</t>
+          <t>1.98% (1.52%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.85% (1.47%)</t>
+          <t>1.30% (0.92%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>-0.09% (-0.91%)</t>
+          <t>0.46% (-0.36%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.04% (-0.80%)</t>
+          <t>0.47% (-0.29%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.42% (5.91%)</t>
+          <t>5.99% (5.48%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.74% (-1.42%)</t>
+          <t>-0.61% (-1.29%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.36% (3.12%)</t>
+          <t>2.72% (2.47%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.70% (2.53%)</t>
+          <t>2.08% (1.90%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.31% (2.20%)</t>
+          <t>1.91% (1.80%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 28/7/2026</t>
+          <t>As of 29/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.91%</t>
+          <t>9.67%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>5.02%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.22%</t>
+          <t>6.20%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.82%</t>
+          <t>7.85%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.15%</t>
+          <t>-5.59%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.31%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.21%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.50%</t>
+          <t>4.96%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.57%</t>
+          <t>6.54%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.92%</t>
+          <t>7.95%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.02%</t>
+          <t>-5.53%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.67%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.20%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.51%</t>
+          <t>8.10%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.34%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2.47%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.62%</t>
+          <t>-8.28%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>9.61%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>11.39%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.20%</t>
+          <t>2.62%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.43%</t>
+          <t>3.44%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.92%</t>
+          <t>-3.38%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.55%</t>
+          <t>8.34%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.20%</t>
+          <t>15.96%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.89%</t>
+          <t>0.23%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>-0.63%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.71%</t>
+          <t>17.83%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.74%</t>
+          <t>-1.09%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.65%</t>
+          <t>8.42%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>16.49%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>-0.76%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.69%</t>
+          <t>-1.63%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17.26%</t>
+          <t>18.39%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.09%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8.98%</t>
+          <t>8.76%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>16.77%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.69%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.23%</t>
+          <t>-1.18%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>18.21%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.81%</t>
+          <t>-0.16%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.43%</t>
+          <t>10.05%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.99%</t>
+          <t>11.53%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.25%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.84%</t>
+          <t>0.12%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.48%</t>
+          <t>-11.11%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.87%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.19%</t>
+          <t>3.81%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.66%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.74%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.58%</t>
+          <t>-9.04%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>4.90%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.53%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>4.10%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.47%</t>
+          <t>-8.96%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>9.83%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.16%</t>
+          <t>5.76%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>9.47%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12.53%</t>
+          <t>11.46%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.64%</t>
+          <t>4.63%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.93%</t>
+          <t>-9.42%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>9.84%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.50%</t>
+          <t>7.10%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>6.35%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.96%</t>
+          <t>7.93%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5.31%</t>
+          <t>6.32%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.30%</t>
+          <t>-6.77%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 28/7/2026</t>
+          <t>As of 29/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>14.94%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.85%</t>
+          <t>6.30%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.83%</t>
+          <t>4.39%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.22%</t>
+          <t>6.20%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.29%</t>
+          <t>5.29%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.41%</t>
+          <t>-5.01%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>15.46%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.43%</t>
+          <t>6.82%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.49%</t>
+          <t>4.11%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.57%</t>
+          <t>6.54%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.17%</t>
+          <t>5.17%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.10%</t>
+          <t>-4.76%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.39%</t>
+          <t>18.00%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.94%</t>
+          <t>6.56%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.35%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.22%</t>
+          <t>0.75%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.28%</t>
+          <t>-6.95%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.22%</t>
+          <t>14.86%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.63%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.64%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.44%</t>
+          <t>3.44%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.57%</t>
+          <t>8.61%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.39%</t>
+          <t>-2.96%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.53%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.96%</t>
+          <t>12.48%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>0.44%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>-0.63%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.45%</t>
+          <t>14.55%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-1.29%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.61%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.56%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>-0.56%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.68%</t>
+          <t>-1.63%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>15.24%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-0.29%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>13.62%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.90%</t>
+          <t>13.52%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>-0.48%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.22%</t>
+          <t>-1.18%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.07%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.91%</t>
+          <t>-0.36%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.30%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.84%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.10%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.26%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.92%</t>
+          <t>-1.98%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.96%</t>
+          <t>-9.79%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.53%</t>
+          <t>15.10%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.20%</t>
+          <t>2.55%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>7.88%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.74%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.23%</t>
+          <t>0.73%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.40%</t>
+          <t>-8.09%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>15.22%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.05%</t>
+          <t>7.66%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.63%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>1.43%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.23%</t>
+          <t>-7.90%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>15.60%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>4.14%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.31%</t>
+          <t>7.94%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12.54%</t>
+          <t>11.46%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.46%</t>
+          <t>-8.14%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.59%</t>
+          <t>15.17%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>5.37%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.94%</t>
+          <t>5.57%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.97%</t>
+          <t>7.93%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>3.85%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.40%</t>
+          <t>-6.07%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-30]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/29/2026 at 11:28 AM ET)</t>
+          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>261 days</t>
+          <t>260 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>22 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>142 days</t>
+          <t>141 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>205 days</t>
+          <t>204 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>170 days</t>
+          <t>169 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>352 days</t>
+          <t>351 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>323 days</t>
+          <t>322 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>233 days</t>
+          <t>232 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>296 days</t>
+          <t>295 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>114 days</t>
+          <t>113 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>79 days</t>
+          <t>78 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>51 days</t>
+          <t>50 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>261 days</t>
+          <t>260 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>22 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>142 days</t>
+          <t>141 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>205 days</t>
+          <t>204 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>170 days</t>
+          <t>169 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>352 days</t>
+          <t>351 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>323 days</t>
+          <t>322 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>233 days</t>
+          <t>232 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>296 days</t>
+          <t>295 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>114 days</t>
+          <t>113 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>79 days</t>
+          <t>78 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>51 days</t>
+          <t>50 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.46 / 2.62%</t>
+          <t>$46.49 / 2.69%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.53 / 11.53%</t>
+          <t>$56.61 / 11.69%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.25 / 6.35%</t>
+          <t>$54.31 / 6.46%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$60.79 / 4.96%</t>
+          <t>$60.83 / 5.03%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$54.89 / 5.02%</t>
+          <t>$54.95 / 5.13%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.44 / -0.69%</t>
+          <t>$59.51 / -0.57%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.42 / -0.76%</t>
+          <t>$59.48 / -0.65%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.23 / 8.10%</t>
+          <t>$52.28 / 8.20%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$55.69 / 0.23%</t>
+          <t>$55.72 / 0.28%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.29 / 9.47%</t>
+          <t>$58.35 / 9.58%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.14 / 8.91%</t>
+          <t>$52.18 / 8.99%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$54.95 / 9.00%</t>
+          <t>$55.00 / 9.10%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.53 / 2.18%</t>
+          <t>$41.57 / 2.27%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.56 / 9.90%</t>
+          <t>$41.60 / 10.02%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.79 / 5.57%</t>
+          <t>$39.81 / 5.63%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$43.96 / 4.11%</t>
+          <t>$44.00 / 4.20%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$44.94 / 4.39%</t>
+          <t>$44.98 / 4.48%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.44 / -0.48%</t>
+          <t>$43.47 / -0.42%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$40.92 / -0.56%</t>
+          <t>$40.96 / -0.47%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.26 / 6.56%</t>
+          <t>$44.30 / 6.66%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$42.83 / 0.44%</t>
+          <t>$42.85 / 0.49%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.80 / 7.94%</t>
+          <t>$41.83 / 8.03%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.52 / 7.66%</t>
+          <t>$41.56 / 7.75%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$40.97 / 7.88%</t>
+          <t>$40.99 / 7.92%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$734.54 / 3.44%</t>
+          <t>$735.13 / 3.52%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$734.54 / 14.16%</t>
+          <t>$735.13 / 14.25%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$734.54 / 7.93%</t>
+          <t>$735.13 / 8.01%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$734.54 / 6.54%</t>
+          <t>$735.13 / 6.63%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$734.54 / 6.20%</t>
+          <t>$735.13 / 6.28%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$734.54 / -1.18%</t>
+          <t>$735.13 / -1.10%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$734.54 / -1.63%</t>
+          <t>$735.13 / -1.56%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$734.54 / 13.25%</t>
+          <t>$735.13 / 13.35%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$734.54 / -0.63%</t>
+          <t>$735.13 / -0.55%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$734.54 / 11.46%</t>
+          <t>$735.13 / 11.55%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$734.54 / 10.56%</t>
+          <t>$735.13 / 10.65%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$734.54 / 10.67%</t>
+          <t>$735.13 / 10.76%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$734.54 / 3.44%</t>
+          <t>$735.13 / 3.52%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$734.54 / 14.16%</t>
+          <t>$735.13 / 14.25%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$734.54 / 7.93%</t>
+          <t>$735.13 / 8.01%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$734.54 / 6.54%</t>
+          <t>$735.13 / 6.63%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$734.54 / 6.20%</t>
+          <t>$735.13 / 6.28%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$734.54 / -1.18%</t>
+          <t>$735.13 / -1.10%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$734.54 / -1.63%</t>
+          <t>$735.13 / -1.56%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$734.54 / 13.25%</t>
+          <t>$735.13 / 13.35%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$734.54 / -0.63%</t>
+          <t>$735.13 / -0.55%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$734.54 / 11.46%</t>
+          <t>$735.13 / 11.55%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$734.54 / 10.56%</t>
+          <t>$735.13 / 10.65%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$734.54 / 10.67%</t>
+          <t>$735.13 / 10.76%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.98% (11.39%)</t>
+          <t>11.91% (11.32%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.75% (1.70%)</t>
+          <t>1.60% (1.56%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.42% (7.10%)</t>
+          <t>7.29% (6.99%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>9.22% (8.77%)</t>
+          <t>9.15% (8.70%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.63% (8.25%)</t>
+          <t>8.51% (8.13%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>17.60% (16.77%)</t>
+          <t>17.46% (16.63%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>17.25% (16.49%)</t>
+          <t>17.12% (16.36%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.11% (7.60%)</t>
+          <t>8.01% (7.51%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>16.65% (15.96%)</t>
+          <t>16.58% (15.90%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>6.00% (5.76%)</t>
+          <t>5.89% (5.65%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5.06% (4.90%)</t>
+          <t>4.98% (4.81%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.92% (3.81%)</t>
+          <t>3.82% (3.71%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.71% (9.11%)</t>
+          <t>9.61% (9.02%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.07% (1.03%)</t>
+          <t>0.96% (0.92%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.69% (5.37%)</t>
+          <t>5.62% (5.31%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.28% (6.82%)</t>
+          <t>7.18% (6.72%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.68% (6.30%)</t>
+          <t>6.58% (6.21%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>14.35% (13.52%)</t>
+          <t>14.27% (13.45%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.89% (13.13%)</t>
+          <t>13.79% (13.04%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.79% (6.28%)</t>
+          <t>6.69% (6.19%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>13.16% (12.48%)</t>
+          <t>13.10% (12.41%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.38% (4.14%)</t>
+          <t>4.29% (4.05%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.55% (3.38%)</t>
+          <t>3.46% (3.29%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.66% (2.55%)</t>
+          <t>2.62% (2.51%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>11.25%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>6.32%</t>
+          <t>6.24%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>7.95%</t>
+          <t>7.86%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>7.85%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>18.21%</t>
+          <t>18.12%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>18.39%</t>
+          <t>18.29%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.37%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>17.83%</t>
+          <t>17.73%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4.63%</t>
+          <t>4.55%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>4.10%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.92%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>8.61%</t>
+          <t>8.52%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-1.98%</t>
+          <t>-2.06%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>3.85%</t>
+          <t>3.77%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>5.09%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>5.29%</t>
+          <t>5.20%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>15.09%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>15.24%</t>
+          <t>15.14%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>0.75%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>14.55%</t>
+          <t>14.46%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>1.43%</t>
+          <t>1.35%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>0.65%</t>
         </is>
       </c>
     </row>
@@ -2839,12 +2839,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.10% (10.05%)</t>
+          <t>10.03% (9.99%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.16% (9.84%)</t>
+          <t>10.12% (9.81%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2854,32 +2854,32 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.04% (9.67%)</t>
+          <t>10.01% (9.63%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.59% (8.76%)</t>
+          <t>9.54% (8.72%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.18% (8.42%)</t>
+          <t>9.14% (8.38%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>12.76% (12.25%)</t>
+          <t>12.74% (12.24%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.03% (8.34%)</t>
+          <t>9.05% (8.36%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.07% (9.83%)</t>
+          <t>10.04% (9.80%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2889,17 +2889,17 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.75% (9.64%)</t>
+          <t>9.73% (9.63%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.45% (14.86%)</t>
+          <t>15.43% (14.84%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>15.79% (15.75%)</t>
+          <t>15.75% (15.71%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2909,47 +2909,47 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>15.92% (15.46%)</t>
+          <t>15.89% (15.44%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.32% (14.94%)</t>
+          <t>15.30% (14.92%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.45% (13.62%)</t>
+          <t>14.44% (13.62%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.05% (13.29%)</t>
+          <t>14.03% (13.28%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.50% (18.00%)</t>
+          <t>18.48% (17.97%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>13.86% (13.17%)</t>
+          <t>13.86% (13.18%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>15.84% (15.60%)</t>
+          <t>15.82% (15.58%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.39% (15.22%)</t>
+          <t>15.37% (15.20%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.21% (15.10%)</t>
+          <t>15.24% (15.13%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-2.79% (-3.38%)</t>
+          <t>-2.85% (-3.44%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.06% (-11.11%)</t>
+          <t>-11.19% (-11.24%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.45% (-6.77%)</t>
+          <t>-6.56% (-6.87%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.08% (-5.53%)</t>
+          <t>-5.14% (-5.59%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.21% (-5.59%)</t>
+          <t>-5.31% (-5.69%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.00% (-0.16%)</t>
+          <t>0.00% (-0.28%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.09%)</t>
+          <t>0.00% (-0.20%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.78% (-8.28%)</t>
+          <t>-7.86% (-8.36%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-0.40% (-1.09%)</t>
+          <t>-0.46% (-1.14%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.18% (-9.42%)</t>
+          <t>-9.28% (-9.52%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-8.79% (-8.96%)</t>
+          <t>-8.86% (-9.03%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-8.93% (-9.04%)</t>
+          <t>-9.01% (-9.12%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.37% (-2.96%)</t>
+          <t>-2.45% (-3.04%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.75% (-9.79%)</t>
+          <t>-9.85% (-9.89%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.76% (-6.07%)</t>
+          <t>-5.82% (-6.13%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.30% (-4.76%)</t>
+          <t>-4.39% (-4.84%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.64% (-5.01%)</t>
+          <t>-4.72% (-5.10%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>0.00% (-0.36%)</t>
+          <t>0.00% (-0.43%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.29%)</t>
+          <t>0.00% (-0.38%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.44% (-6.95%)</t>
+          <t>-6.53% (-7.03%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-0.61% (-1.29%)</t>
+          <t>-0.67% (-1.35%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.89% (-8.14%)</t>
+          <t>-7.97% (-8.22%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.73% (-7.90%)</t>
+          <t>-7.81% (-7.98%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-7.98% (-8.09%)</t>
+          <t>-8.01% (-8.12%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-12.99%</t>
+          <t>-13.06%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.16%</t>
+          <t>-21.22%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-16.61%</t>
+          <t>-16.68%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-15.53%</t>
+          <t>-15.59%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-15.25%</t>
+          <t>-15.32%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-8.93%</t>
+          <t>-9.00%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-8.50%</t>
+          <t>-8.58%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-20.53%</t>
+          <t>-20.60%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-9.43%</t>
+          <t>-9.51%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-19.25%</t>
+          <t>-19.32%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-18.59%</t>
+          <t>-18.66%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-18.68%</t>
+          <t>-18.74%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-17.82%</t>
+          <t>-17.89%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-25.54%</t>
+          <t>-25.60%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-21.24%</t>
+          <t>-21.30%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.22%</t>
+          <t>-20.28%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-19.96%</t>
+          <t>-20.02%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-13.98%</t>
+          <t>-14.05%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-13.58%</t>
+          <t>-13.65%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-24.95%</t>
+          <t>-25.01%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-14.46%</t>
+          <t>-14.53%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-23.73%</t>
+          <t>-23.80%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.11%</t>
+          <t>-23.18%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.19%</t>
+          <t>-23.26%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.56% (-0.03%)</t>
+          <t>0.57% (-0.02%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.63% (1.58%)</t>
+          <t>1.57% (1.52%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.00% (0.69%)</t>
+          <t>0.97% (0.66%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.16% (0.70%)</t>
+          <t>1.17% (0.72%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.69% (0.32%)</t>
+          <t>0.66% (0.29%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.66% (-0.16%)</t>
+          <t>0.54% (-0.28%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.67% (-0.09%)</t>
+          <t>0.56% (-0.20%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.48% (3.98%)</t>
+          <t>4.47% (3.98%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.40% (-1.09%)</t>
+          <t>-0.46% (-1.14%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.29% (1.04%)</t>
+          <t>1.26% (1.02%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.90% (0.73%)</t>
+          <t>0.90% (0.74%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.87% (0.76%)</t>
+          <t>0.85% (0.75%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.99% (0.40%)</t>
+          <t>0.99% (0.39%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1.07% (1.03%)</t>
+          <t>0.96% (0.92%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>1.75% (1.43%)</t>
+          <t>1.76% (1.45%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1.98% (1.52%)</t>
+          <t>1.97% (1.51%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.30% (0.92%)</t>
+          <t>1.29% (0.91%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.46% (-0.36%)</t>
+          <t>0.39% (-0.43%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.47% (-0.29%)</t>
+          <t>0.38% (-0.38%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.99% (5.48%)</t>
+          <t>5.98% (5.48%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.61% (-1.29%)</t>
+          <t>-0.67% (-1.35%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.72% (2.47%)</t>
+          <t>2.71% (2.47%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.08% (1.90%)</t>
+          <t>2.07% (1.90%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>1.91% (1.80%)</t>
+          <t>1.95% (1.85%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 29/7/2026</t>
+          <t>As of 30/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.67%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>8.13%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.02%</t>
+          <t>5.13%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.20%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7.85%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.59%</t>
+          <t>-5.69%</t>
         </is>
       </c>
     </row>
@@ -3452,27 +3452,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.96%</t>
+          <t>5.03%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.54%</t>
+          <t>6.63%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7.95%</t>
+          <t>7.86%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.53%</t>
+          <t>-5.59%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>12.24%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.51%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.10%</t>
+          <t>8.20%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>13.35%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.37%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.28%</t>
+          <t>-8.36%</t>
         </is>
       </c>
     </row>
@@ -3526,27 +3526,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11.39%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.62%</t>
+          <t>2.69%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.44%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>11.25%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.38%</t>
+          <t>-3.44%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.34%</t>
+          <t>8.36%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.96%</t>
+          <t>15.90%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.63%</t>
+          <t>-0.55%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>17.83%</t>
+          <t>17.73%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.09%</t>
+          <t>-1.14%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.42%</t>
+          <t>8.38%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16.49%</t>
+          <t>16.36%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.76%</t>
+          <t>-0.65%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.63%</t>
+          <t>-1.56%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>18.39%</t>
+          <t>18.29%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>-0.20%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8.76%</t>
+          <t>8.72%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16.77%</t>
+          <t>16.63%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.69%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-1.10%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>18.21%</t>
+          <t>18.12%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>-0.28%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.05%</t>
+          <t>9.99%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.53%</t>
+          <t>11.69%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>14.25%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.11%</t>
+          <t>-11.24%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.81%</t>
+          <t>3.71%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>9.10%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.76%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.92%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.04%</t>
+          <t>-9.12%</t>
         </is>
       </c>
     </row>
@@ -3748,27 +3748,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.90%</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>8.99%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>4.10%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.96%</t>
+          <t>-9.03%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.83%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.76%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.47%</t>
+          <t>9.58%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.46%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4.63%</t>
+          <t>4.55%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.42%</t>
+          <t>-9.52%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.84%</t>
+          <t>9.81%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7.10%</t>
+          <t>6.99%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.35%</t>
+          <t>6.46%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7.93%</t>
+          <t>8.01%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>6.32%</t>
+          <t>6.24%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.77%</t>
+          <t>-6.87%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 29/7/2026</t>
+          <t>As of 30/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14.94%</t>
+          <t>14.92%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.30%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>4.48%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.20%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.29%</t>
+          <t>5.20%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.01%</t>
+          <t>-5.10%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.46%</t>
+          <t>15.44%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.82%</t>
+          <t>6.72%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.11%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.54%</t>
+          <t>6.63%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>5.09%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.76%</t>
+          <t>-4.84%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.00%</t>
+          <t>17.97%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.19%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.56%</t>
+          <t>6.66%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>13.35%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.75%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-6.95%</t>
+          <t>-7.03%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>14.86%</t>
+          <t>14.84%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.02%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.44%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.61%</t>
+          <t>8.52%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-2.96%</t>
+          <t>-3.04%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>13.18%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.48%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>0.49%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.63%</t>
+          <t>-0.55%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.55%</t>
+          <t>14.46%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.29%</t>
+          <t>-1.35%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>13.28%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.56%</t>
+          <t>-0.47%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.63%</t>
+          <t>-1.56%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.24%</t>
+          <t>15.14%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.29%</t>
+          <t>-0.38%</t>
         </is>
       </c>
     </row>
@@ -4152,27 +4152,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.45%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.48%</t>
+          <t>-0.42%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-1.10%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>15.09%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>-0.43%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>15.71%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>14.25%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-1.98%</t>
+          <t>-2.06%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.79%</t>
+          <t>-9.89%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.10%</t>
+          <t>15.13%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.55%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.88%</t>
+          <t>7.92%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.76%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.09%</t>
+          <t>-8.12%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.22%</t>
+          <t>15.20%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.66%</t>
+          <t>7.75%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.43%</t>
+          <t>1.35%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.90%</t>
+          <t>-7.98%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.60%</t>
+          <t>15.58%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.14%</t>
+          <t>4.05%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.94%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.46%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.14%</t>
+          <t>-8.22%</t>
         </is>
       </c>
     </row>
@@ -4337,27 +4337,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.37%</t>
+          <t>5.31%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.57%</t>
+          <t>5.63%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7.93%</t>
+          <t>8.01%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.85%</t>
+          <t>3.77%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.07%</t>
+          <t>-6.13%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-07-31]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/30/2026 at 11:29 AM ET)</t>
+          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>260 days</t>
+          <t>259 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>22 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>141 days</t>
+          <t>140 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>204 days</t>
+          <t>203 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>169 days</t>
+          <t>168 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>351 days</t>
+          <t>350 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>322 days</t>
+          <t>321 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>232 days</t>
+          <t>231 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>295 days</t>
+          <t>294 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>113 days</t>
+          <t>112 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>78 days</t>
+          <t>77 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>50 days</t>
+          <t>49 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>260 days</t>
+          <t>259 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>22 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>141 days</t>
+          <t>140 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>204 days</t>
+          <t>203 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>169 days</t>
+          <t>168 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>351 days</t>
+          <t>350 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>322 days</t>
+          <t>321 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>232 days</t>
+          <t>231 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>295 days</t>
+          <t>294 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>113 days</t>
+          <t>112 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>78 days</t>
+          <t>77 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>50 days</t>
+          <t>49 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.49 / 2.69%</t>
+          <t>$46.73 / 3.22%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.61 / 11.69%</t>
+          <t>$56.90 / 12.25%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.31 / 6.46%</t>
+          <t>$54.57 / 6.97%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$60.83 / 5.03%</t>
+          <t>$61.13 / 5.55%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$54.95 / 5.13%</t>
+          <t>$55.21 / 5.62%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.51 / -0.57%</t>
+          <t>$59.82 / -0.05%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.48 / -0.65%</t>
+          <t>$59.76 / -0.19%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.28 / 8.20%</t>
+          <t>$52.48 / 8.62%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$55.72 / 0.28%</t>
+          <t>$56.07 / 0.90%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.35 / 9.58%</t>
+          <t>$58.61 / 10.08%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.18 / 8.99%</t>
+          <t>$52.48 / 9.62%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.00 / 9.10%</t>
+          <t>$55.30 / 9.70%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.57 / 2.27%</t>
+          <t>$41.74 / 2.70%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.60 / 10.02%</t>
+          <t>$41.71 / 10.31%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.81 / 5.63%</t>
+          <t>$39.95 / 6.00%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.00 / 4.20%</t>
+          <t>$44.13 / 4.51%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$44.98 / 4.48%</t>
+          <t>$45.15 / 4.87%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.47 / -0.42%</t>
+          <t>$43.63 / -0.05%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$40.96 / -0.47%</t>
+          <t>$41.12 / -0.07%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.30 / 6.66%</t>
+          <t>$44.41 / 6.94%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$42.85 / 0.49%</t>
+          <t>$43.04 / 0.93%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.83 / 8.03%</t>
+          <t>$41.97 / 8.38%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.56 / 7.75%</t>
+          <t>$41.69 / 8.09%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$40.99 / 7.92%</t>
+          <t>$41.14 / 8.33%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$735.13 / 3.52%</t>
+          <t>$741.29 / 4.39%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$735.13 / 14.25%</t>
+          <t>$741.29 / 15.21%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$735.13 / 8.01%</t>
+          <t>$741.29 / 8.92%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$735.13 / 6.63%</t>
+          <t>$741.29 / 7.52%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$735.13 / 6.28%</t>
+          <t>$741.29 / 7.17%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$735.13 / -1.10%</t>
+          <t>$741.29 / -0.27%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$735.13 / -1.56%</t>
+          <t>$741.29 / -0.73%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$735.13 / 13.35%</t>
+          <t>$741.29 / 14.30%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$735.13 / -0.55%</t>
+          <t>$741.29 / 0.29%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$735.13 / 11.55%</t>
+          <t>$741.29 / 12.48%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$735.13 / 10.65%</t>
+          <t>$741.29 / 11.57%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$735.13 / 10.76%</t>
+          <t>$741.29 / 11.69%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$735.13 / 3.52%</t>
+          <t>$741.29 / 4.39%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$735.13 / 14.25%</t>
+          <t>$741.29 / 15.21%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$735.13 / 8.01%</t>
+          <t>$741.29 / 8.92%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$735.13 / 6.63%</t>
+          <t>$741.29 / 7.52%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$735.13 / 6.28%</t>
+          <t>$741.29 / 7.17%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$735.13 / -1.10%</t>
+          <t>$741.29 / -0.27%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$735.13 / -1.56%</t>
+          <t>$741.29 / -0.73%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$735.13 / 13.35%</t>
+          <t>$741.29 / 14.30%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$735.13 / -0.55%</t>
+          <t>$741.29 / 0.29%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$735.13 / 11.55%</t>
+          <t>$741.29 / 12.48%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$735.13 / 10.65%</t>
+          <t>$741.29 / 11.57%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$735.13 / 10.76%</t>
+          <t>$741.29 / 11.69%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.91% (11.32%)</t>
+          <t>11.33% (10.75%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.60% (1.56%)</t>
+          <t>1.09% (1.05%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.29% (6.99%)</t>
+          <t>6.78% (6.48%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>9.15% (8.70%)</t>
+          <t>8.60% (8.16%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.51% (8.13%)</t>
+          <t>8.00% (7.63%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>17.46% (16.63%)</t>
+          <t>16.85% (16.03%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>17.12% (16.36%)</t>
+          <t>16.57% (15.82%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.01% (7.51%)</t>
+          <t>7.59% (7.09%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>16.58% (15.90%)</t>
+          <t>15.86% (15.19%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.89% (5.65%)</t>
+          <t>5.41% (5.17%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.98% (4.81%)</t>
+          <t>4.38% (4.22%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.82% (3.71%)</t>
+          <t>3.26% (3.15%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.61% (9.02%)</t>
+          <t>9.15% (8.57%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.96% (0.92%)</t>
+          <t>0.69% (0.65%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.62% (5.31%)</t>
+          <t>5.24% (4.94%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>7.18% (6.72%)</t>
+          <t>6.86% (6.41%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.58% (6.21%)</t>
+          <t>6.19% (5.82%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>14.27% (13.45%)</t>
+          <t>13.85% (13.03%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.79% (13.04%)</t>
+          <t>13.33% (12.58%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.69% (6.19%)</t>
+          <t>6.41% (5.91%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>13.10% (12.41%)</t>
+          <t>12.61% (11.93%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>4.29% (4.05%)</t>
+          <t>3.96% (3.71%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.46% (3.29%)</t>
+          <t>3.13% (2.97%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.62% (2.51%)</t>
+          <t>2.23% (2.13%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11.25%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>5.35%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>7.86%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>6.86%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>18.12%</t>
+          <t>17.14%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>18.29%</t>
+          <t>17.31%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>3.37%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>17.73%</t>
+          <t>16.76%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4.55%</t>
+          <t>3.68%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2.92%</t>
+          <t>2.07%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>8.52%</t>
+          <t>7.62%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-2.06%</t>
+          <t>-2.88%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>3.77%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>5.09%</t>
+          <t>4.21%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>5.20%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>15.09%</t>
+          <t>14.13%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>15.14%</t>
+          <t>14.19%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>0.67%</t>
+          <t>-0.17%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>14.46%</t>
+          <t>13.51%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>1.35%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>-0.19%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.20% (9.61%)</t>
+          <t>10.42% (9.84%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.03% (9.99%)</t>
+          <t>10.24% (10.20%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.12% (9.81%)</t>
+          <t>10.36% (10.06%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.45% (10.00%)</t>
+          <t>10.68% (10.23%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.01% (9.63%)</t>
+          <t>10.27% (9.90%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.54% (8.72%)</t>
+          <t>9.77% (8.96%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.14% (8.38%)</t>
+          <t>9.42% (8.67%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>12.74% (12.24%)</t>
+          <t>13.04% (12.54%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.05% (8.36%)</t>
+          <t>9.19% (8.51%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.04% (9.80%)</t>
+          <t>10.30% (10.06%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.80% (9.63%)</t>
+          <t>9.95% (9.79%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.73% (9.63%)</t>
+          <t>9.91% (9.81%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.43% (14.84%)</t>
+          <t>15.71% (15.12%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>15.75% (15.71%)</t>
+          <t>16.13% (16.09%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.48% (15.17%)</t>
+          <t>15.80% (15.50%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>15.89% (15.44%)</t>
+          <t>16.27% (15.82%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.30% (14.92%)</t>
+          <t>15.62% (15.24%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.44% (13.62%)</t>
+          <t>14.79% (13.97%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.03% (13.28%)</t>
+          <t>14.34% (13.60%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.48% (17.97%)</t>
+          <t>18.86% (18.35%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>13.86% (13.18%)</t>
+          <t>14.15% (13.47%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>15.82% (15.58%)</t>
+          <t>16.16% (15.92%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.37% (15.20%)</t>
+          <t>15.72% (15.55%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.24% (15.13%)</t>
+          <t>15.53% (15.42%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-2.85% (-3.44%)</t>
+          <t>-3.36% (-3.94%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.19% (-11.24%)</t>
+          <t>-11.64% (-11.68%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-6.56% (-6.87%)</t>
+          <t>-7.01% (-7.31%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.14% (-5.59%)</t>
+          <t>-5.62% (-6.06%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.31% (-5.69%)</t>
+          <t>-5.75% (-6.12%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.00% (-0.28%)</t>
+          <t>0.00% (-0.80%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.20%)</t>
+          <t>0.00% (-0.66%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-7.86% (-8.36%)</t>
+          <t>-8.22% (-8.72%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-0.46% (-1.14%)</t>
+          <t>-1.07% (-1.75%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.28% (-9.52%)</t>
+          <t>-9.69% (-9.92%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-8.86% (-9.03%)</t>
+          <t>-9.39% (-9.55%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.01% (-9.12%)</t>
+          <t>-9.51% (-9.61%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.45% (-3.04%)</t>
+          <t>-2.86% (-3.45%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-9.85% (-9.89%)</t>
+          <t>-10.08% (-10.13%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-5.82% (-6.13%)</t>
+          <t>-6.15% (-6.46%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.39% (-4.84%)</t>
+          <t>-4.67% (-5.12%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-4.72% (-5.10%)</t>
+          <t>-5.07% (-5.45%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>0.00% (-0.43%)</t>
+          <t>0.00% (-0.80%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.00% (-0.38%)</t>
+          <t>-0.03% (-0.78%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.53% (-7.03%)</t>
+          <t>-6.77% (-7.28%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-0.67% (-1.35%)</t>
+          <t>-1.10% (-1.77%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-7.97% (-8.22%)</t>
+          <t>-8.27% (-8.51%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-7.81% (-7.98%)</t>
+          <t>-8.10% (-8.26%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.01% (-8.12%)</t>
+          <t>-8.36% (-8.47%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-13.06%</t>
+          <t>-13.78%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.22%</t>
+          <t>-21.88%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-16.68%</t>
+          <t>-17.37%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-15.59%</t>
+          <t>-16.30%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-15.32%</t>
+          <t>-16.03%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-9.00%</t>
+          <t>-9.76%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-8.58%</t>
+          <t>-9.34%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-20.60%</t>
+          <t>-21.26%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-9.51%</t>
+          <t>-10.26%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-19.32%</t>
+          <t>-19.99%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-18.66%</t>
+          <t>-19.34%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-18.74%</t>
+          <t>-19.42%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-17.89%</t>
+          <t>-18.57%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-25.60%</t>
+          <t>-26.22%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-21.30%</t>
+          <t>-21.96%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.28%</t>
+          <t>-20.94%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-20.02%</t>
+          <t>-20.69%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-14.05%</t>
+          <t>-14.77%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-13.65%</t>
+          <t>-14.37%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-25.01%</t>
+          <t>-25.63%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-14.53%</t>
+          <t>-15.24%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-23.80%</t>
+          <t>-24.43%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.18%</t>
+          <t>-23.81%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.26%</t>
+          <t>-23.89%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.57% (-0.02%)</t>
+          <t>0.89% (0.31%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.57% (1.52%)</t>
+          <t>1.09% (1.05%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.97% (0.66%)</t>
+          <t>1.33% (1.02%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.17% (0.72%)</t>
+          <t>1.51% (1.06%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.66% (0.29%)</t>
+          <t>1.04% (0.67%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.54% (-0.28%)</t>
+          <t>0.02% (-0.80%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.56% (-0.20%)</t>
+          <t>0.09% (-0.66%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.47% (3.98%)</t>
+          <t>4.94% (4.44%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.46% (-1.14%)</t>
+          <t>-0.79% (-1.47%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.26% (1.02%)</t>
+          <t>1.65% (1.41%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.90% (0.74%)</t>
+          <t>1.17% (1.01%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.85% (0.75%)</t>
+          <t>1.15% (1.05%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.99% (0.39%)</t>
+          <t>1.41% (0.82%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.96% (0.92%)</t>
+          <t>0.69% (0.65%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>1.76% (1.45%)</t>
+          <t>2.26% (1.95%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1.97% (1.51%)</t>
+          <t>2.52% (2.07%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.29% (0.91%)</t>
+          <t>1.77% (1.39%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.39% (-0.43%)</t>
+          <t>0.02% (-0.80%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.38% (-0.38%)</t>
+          <t>-0.03% (-0.78%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.98% (5.48%)</t>
+          <t>6.41% (5.91%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.67% (-1.35%)</t>
+          <t>-0.81% (-1.49%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.71% (2.47%)</t>
+          <t>3.24% (3.00%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.07% (1.90%)</t>
+          <t>2.61% (2.44%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>1.95% (1.85%)</t>
+          <t>2.23% (2.13%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 30/7/2026</t>
+          <t>As of 31/7/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8.13%</t>
+          <t>7.63%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.13%</t>
+          <t>5.62%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>7.17%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>6.86%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.69%</t>
+          <t>-6.12%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>8.16%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.03%</t>
+          <t>5.55%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.63%</t>
+          <t>7.52%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7.86%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.59%</t>
+          <t>-6.06%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.24%</t>
+          <t>12.54%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.51%</t>
+          <t>7.09%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.20%</t>
+          <t>8.62%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.35%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3.37%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.36%</t>
+          <t>-8.72%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.61%</t>
+          <t>9.84%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11.32%</t>
+          <t>10.75%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.69%</t>
+          <t>3.22%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>4.39%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11.25%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.44%</t>
+          <t>-3.94%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.36%</t>
+          <t>8.51%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.90%</t>
+          <t>15.19%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.55%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>17.73%</t>
+          <t>16.76%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-1.75%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.38%</t>
+          <t>8.67%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16.36%</t>
+          <t>15.82%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.65%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.56%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>18.29%</t>
+          <t>17.31%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.66%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8.72%</t>
+          <t>8.96%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16.63%</t>
+          <t>16.03%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-1.10%</t>
+          <t>-0.27%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>18.12%</t>
+          <t>17.14%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.28%</t>
+          <t>-0.80%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.99%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>1.05%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.69%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.25%</t>
+          <t>15.21%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.24%</t>
+          <t>-11.68%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.81%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.71%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.10%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10.76%</t>
+          <t>11.69%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.92%</t>
+          <t>2.07%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.12%</t>
+          <t>-9.61%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.99%</t>
+          <t>9.62%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.03%</t>
+          <t>-9.55%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>5.17%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>12.48%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4.55%</t>
+          <t>3.68%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.52%</t>
+          <t>-9.92%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.81%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.99%</t>
+          <t>6.48%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.46%</t>
+          <t>6.97%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>5.35%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.87%</t>
+          <t>-7.31%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 30/7/2026</t>
+          <t>As of 31/7/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14.92%</t>
+          <t>15.24%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>5.82%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.48%</t>
+          <t>4.87%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>7.17%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.20%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.10%</t>
+          <t>-5.45%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.44%</t>
+          <t>15.82%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.72%</t>
+          <t>6.41%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>4.51%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.63%</t>
+          <t>7.52%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5.09%</t>
+          <t>4.21%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-4.84%</t>
+          <t>-5.12%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>17.97%</t>
+          <t>18.35%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.19%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.66%</t>
+          <t>6.94%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.35%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.67%</t>
+          <t>-0.17%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.03%</t>
+          <t>-7.28%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>14.84%</t>
+          <t>15.12%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9.02%</t>
+          <t>8.57%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>2.70%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>4.39%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.52%</t>
+          <t>7.62%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.04%</t>
+          <t>-3.45%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.18%</t>
+          <t>13.47%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.49%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-0.55%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.46%</t>
+          <t>13.51%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.35%</t>
+          <t>-1.77%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.28%</t>
+          <t>13.60%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.47%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-1.56%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.14%</t>
+          <t>14.19%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.38%</t>
+          <t>-0.78%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13.62%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.45%</t>
+          <t>13.03%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.42%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-1.10%</t>
+          <t>-0.27%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>15.09%</t>
+          <t>14.13%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.43%</t>
+          <t>-0.80%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>15.71%</t>
+          <t>16.09%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>10.31%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14.25%</t>
+          <t>15.21%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.06%</t>
+          <t>-2.88%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-9.89%</t>
+          <t>-10.13%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.13%</t>
+          <t>15.42%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.13%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.92%</t>
+          <t>8.33%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10.76%</t>
+          <t>11.69%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.12%</t>
+          <t>-8.47%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.20%</t>
+          <t>15.55%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>2.97%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.75%</t>
+          <t>8.09%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.35%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-7.98%</t>
+          <t>-8.26%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.58%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>3.71%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>8.38%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>12.48%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.22%</t>
+          <t>-8.51%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.17%</t>
+          <t>15.50%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.31%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.63%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.77%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.13%</t>
+          <t>-6.46%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-03]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 7/31/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>259 days</t>
+          <t>256 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>21 days</t>
+          <t>18 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>140 days</t>
+          <t>137 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>203 days</t>
+          <t>200 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>168 days</t>
+          <t>165 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>350 days</t>
+          <t>347 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>321 days</t>
+          <t>318 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>231 days</t>
+          <t>228 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>294 days</t>
+          <t>291 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>112 days</t>
+          <t>109 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>77 days</t>
+          <t>74 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>49 days</t>
+          <t>46 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>259 days</t>
+          <t>256 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>21 days</t>
+          <t>18 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>140 days</t>
+          <t>137 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>203 days</t>
+          <t>200 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>168 days</t>
+          <t>165 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>350 days</t>
+          <t>347 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>321 days</t>
+          <t>318 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>231 days</t>
+          <t>228 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>294 days</t>
+          <t>291 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>112 days</t>
+          <t>109 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>77 days</t>
+          <t>74 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>49 days</t>
+          <t>46 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$46.73 / 3.22%</t>
+          <t>$47.23 / 4.32%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$56.90 / 12.25%</t>
+          <t>$57.25 / 12.95%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$54.57 / 6.97%</t>
+          <t>$55.15 / 8.11%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.13 / 5.55%</t>
+          <t>$61.72 / 6.57%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.21 / 5.62%</t>
+          <t>$55.79 / 6.73%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$59.82 / -0.05%</t>
+          <t>$60.58 / 1.22%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$59.76 / -0.19%</t>
+          <t>$60.54 / 1.12%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.48 / 8.62%</t>
+          <t>$52.88 / 9.45%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.07 / 0.90%</t>
+          <t>$56.77 / 2.17%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$58.61 / 10.08%</t>
+          <t>$59.19 / 11.17%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$52.48 / 9.62%</t>
+          <t>$53.03 / 10.77%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.30 / 9.70%</t>
+          <t>$55.88 / 10.86%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$41.74 / 2.70%</t>
+          <t>$42.08 / 3.52%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.71 / 10.31%</t>
+          <t>$41.86 / 10.71%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$39.95 / 6.00%</t>
+          <t>$40.24 / 6.76%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.13 / 4.51%</t>
+          <t>$44.45 / 5.27%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.15 / 4.87%</t>
+          <t>$45.48 / 5.64%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$43.63 / -0.05%</t>
+          <t>$44.11 / 1.05%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.12 / -0.07%</t>
+          <t>$41.54 / 0.95%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.41 / 6.94%</t>
+          <t>$44.67 / 7.55%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.04 / 0.93%</t>
+          <t>$43.47 / 1.94%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$41.97 / 8.38%</t>
+          <t>$42.25 / 9.12%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$41.69 / 8.09%</t>
+          <t>$42.00 / 8.90%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.14 / 8.33%</t>
+          <t>$41.43 / 9.08%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$741.29 / 4.39%</t>
+          <t>$755.99 / 6.46%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$741.29 / 15.21%</t>
+          <t>$755.99 / 17.49%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$741.29 / 8.92%</t>
+          <t>$755.99 / 11.08%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$741.29 / 7.52%</t>
+          <t>$755.99 / 9.65%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$741.29 / 7.17%</t>
+          <t>$755.99 / 9.30%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$741.29 / -0.27%</t>
+          <t>$755.99 / 1.71%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$741.29 / -0.73%</t>
+          <t>$755.99 / 1.24%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$741.29 / 14.30%</t>
+          <t>$755.99 / 16.56%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$741.29 / 0.29%</t>
+          <t>$755.99 / 2.27%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$741.29 / 12.48%</t>
+          <t>$755.99 / 14.71%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$741.29 / 11.57%</t>
+          <t>$755.99 / 13.79%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$741.29 / 11.69%</t>
+          <t>$755.99 / 13.90%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$741.29 / 4.39%</t>
+          <t>$755.99 / 6.46%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$741.29 / 15.21%</t>
+          <t>$755.99 / 17.49%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$741.29 / 8.92%</t>
+          <t>$755.99 / 11.08%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$741.29 / 7.52%</t>
+          <t>$755.99 / 9.65%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$741.29 / 7.17%</t>
+          <t>$755.99 / 9.30%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$741.29 / -0.27%</t>
+          <t>$755.99 / 1.71%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$741.29 / -0.73%</t>
+          <t>$755.99 / 1.24%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$741.29 / 14.30%</t>
+          <t>$755.99 / 16.56%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$741.29 / 0.29%</t>
+          <t>$755.99 / 2.27%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$741.29 / 12.48%</t>
+          <t>$755.99 / 14.71%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$741.29 / 11.57%</t>
+          <t>$755.99 / 13.79%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$741.29 / 11.69%</t>
+          <t>$755.99 / 13.90%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.33% (10.75%)</t>
+          <t>10.15% (9.57%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.09% (1.05%)</t>
+          <t>0.46% (0.42%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.78% (6.48%)</t>
+          <t>5.65% (5.36%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.60% (8.16%)</t>
+          <t>7.56% (7.12%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.00% (7.63%)</t>
+          <t>6.87% (6.51%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>16.85% (16.03%)</t>
+          <t>15.37% (14.57%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.57% (15.82%)</t>
+          <t>15.06% (14.33%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>7.59% (7.09%)</t>
+          <t>6.77% (6.28%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.86% (15.19%)</t>
+          <t>14.42% (13.76%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.41% (5.17%)</t>
+          <t>4.37% (4.14%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4.38% (4.22%)</t>
+          <t>3.29% (3.13%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3.26% (3.15%)</t>
+          <t>2.17% (2.07%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>9.15% (8.57%)</t>
+          <t>8.28% (7.70%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.69% (0.65%)</t>
+          <t>0.33% (0.29%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>5.24% (4.94%)</t>
+          <t>4.49% (4.19%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.86% (6.41%)</t>
+          <t>6.08% (5.64%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6.19% (5.82%)</t>
+          <t>5.40% (5.04%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>13.85% (13.03%)</t>
+          <t>12.60% (11.80%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.33% (12.58%)</t>
+          <t>12.18% (11.45%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>6.41% (5.91%)</t>
+          <t>5.80% (5.31%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>12.61% (11.93%)</t>
+          <t>11.49% (10.82%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.96% (3.71%)</t>
+          <t>3.25% (3.02%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>3.13% (2.97%)</t>
+          <t>2.35% (2.20%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2.23% (2.13%)</t>
+          <t>1.52% (1.43%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>8.18%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-2.72%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.35%</t>
+          <t>3.31%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>4.88%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6.86%</t>
+          <t>4.79%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>17.14%</t>
+          <t>14.86%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.76%</t>
+          <t>14.49%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.68%</t>
+          <t>1.66%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>1.15%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2.07%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>7.62%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>4.21%</t>
+          <t>2.19%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>11.91%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>14.19%</t>
+          <t>11.97%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-0.17%</t>
+          <t>-2.11%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>13.51%</t>
+          <t>11.30%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-1.27%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-0.19%</t>
+          <t>-2.13%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.42% (9.84%)</t>
+          <t>11.07% (10.50%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.24% (10.20%)</t>
+          <t>11.21% (11.17%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.36% (10.06%)</t>
+          <t>10.98% (10.69%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.68% (10.23%)</t>
+          <t>11.40% (10.96%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.27% (9.90%)</t>
+          <t>10.92% (10.56%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.77% (8.96%)</t>
+          <t>10.27% (9.47%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.42% (8.67%)</t>
+          <t>9.89% (9.16%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.04% (12.54%)</t>
+          <t>13.87% (13.38%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.19% (8.51%)</t>
+          <t>9.69% (9.03%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.30% (10.06%)</t>
+          <t>10.96% (10.73%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.95% (9.79%)</t>
+          <t>10.57% (10.42%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.91% (9.81%)</t>
+          <t>10.53% (10.43%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.71% (15.12%)</t>
+          <t>16.51% (15.93%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>16.13% (16.09%)</t>
+          <t>17.24% (17.20%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.80% (15.50%)</t>
+          <t>16.65% (16.35%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.27% (15.82%)</t>
+          <t>17.11% (16.67%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.62% (15.24%)</t>
+          <t>16.45% (16.09%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.79% (13.97%)</t>
+          <t>15.35% (14.55%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.34% (13.60%)</t>
+          <t>14.99% (14.26%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.86% (18.35%)</t>
+          <t>19.76% (19.27%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.15% (13.47%)</t>
+          <t>14.81% (14.14%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.16% (15.92%)</t>
+          <t>17.00% (16.77%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.72% (15.55%)</t>
+          <t>16.50% (16.34%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.53% (15.42%)</t>
+          <t>16.37% (16.27%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3.36% (-3.94%)</t>
+          <t>-4.39% (-4.96%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-11.64% (-11.68%)</t>
+          <t>-12.19% (-12.23%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.01% (-7.31%)</t>
+          <t>-7.99% (-8.29%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-5.62% (-6.06%)</t>
+          <t>-6.52% (-6.96%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-5.75% (-6.12%)</t>
+          <t>-6.74% (-7.10%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.00% (-0.80%)</t>
+          <t>-1.24% (-2.04%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.00% (-0.66%)</t>
+          <t>-1.21% (-1.94%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.22% (-8.72%)</t>
+          <t>-8.92% (-9.41%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.07% (-1.75%)</t>
+          <t>-2.31% (-2.97%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-9.69% (-9.92%)</t>
+          <t>-10.58% (-10.81%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-9.39% (-9.55%)</t>
+          <t>-10.33% (-10.49%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-9.51% (-9.61%)</t>
+          <t>-10.46% (-10.56%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-2.86% (-3.45%)</t>
+          <t>-3.64% (-4.22%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.08% (-10.13%)</t>
+          <t>-10.41% (-10.45%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.15% (-6.46%)</t>
+          <t>-6.82% (-7.12%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-4.67% (-5.12%)</t>
+          <t>-5.37% (-5.81%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.07% (-5.45%)</t>
+          <t>-5.78% (-6.14%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>0.00% (-0.80%)</t>
+          <t>-1.08% (-1.88%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-0.03% (-0.78%)</t>
+          <t>-1.04% (-1.78%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-6.77% (-7.28%)</t>
+          <t>-7.31% (-7.80%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-1.10% (-1.77%)</t>
+          <t>-2.08% (-2.75%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.27% (-8.51%)</t>
+          <t>-8.90% (-9.13%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.10% (-8.26%)</t>
+          <t>-8.79% (-8.95%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-8.36% (-8.47%)</t>
+          <t>-9.00% (-9.10%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-13.78%</t>
+          <t>-15.46%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-21.88%</t>
+          <t>-23.40%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-17.37%</t>
+          <t>-18.98%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-16.30%</t>
+          <t>-17.92%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-16.03%</t>
+          <t>-17.66%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-9.76%</t>
+          <t>-11.51%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-9.34%</t>
+          <t>-11.10%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-21.26%</t>
+          <t>-22.79%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-10.26%</t>
+          <t>-12.00%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-19.99%</t>
+          <t>-21.54%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-19.34%</t>
+          <t>-20.90%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-19.42%</t>
+          <t>-20.99%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-18.57%</t>
+          <t>-20.15%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-26.22%</t>
+          <t>-27.65%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-21.96%</t>
+          <t>-23.47%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-20.94%</t>
+          <t>-22.48%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-20.69%</t>
+          <t>-22.23%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-14.77%</t>
+          <t>-16.42%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-14.37%</t>
+          <t>-16.04%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-25.63%</t>
+          <t>-27.08%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-15.24%</t>
+          <t>-16.89%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-24.43%</t>
+          <t>-25.90%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-23.81%</t>
+          <t>-25.30%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-23.89%</t>
+          <t>-25.37%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.89% (0.31%)</t>
+          <t>1.80% (1.23%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.09% (1.05%)</t>
+          <t>0.46% (0.42%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.33% (1.02%)</t>
+          <t>2.25% (1.96%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.51% (1.06%)</t>
+          <t>2.53% (2.10%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.04% (0.67%)</t>
+          <t>1.97% (1.61%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.02% (-0.80%)</t>
+          <t>0.44% (-0.36%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.09% (-0.66%)</t>
+          <t>0.01% (-0.72%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.94% (4.44%)</t>
+          <t>6.21% (5.72%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.79% (-1.47%)</t>
+          <t>-0.08% (-0.74%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.65% (1.41%)</t>
+          <t>2.65% (2.43%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.17% (1.01%)</t>
+          <t>2.11% (1.96%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.15% (1.05%)</t>
+          <t>2.08% (1.99%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.41% (0.82%)</t>
+          <t>2.59% (2.01%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.69% (0.65%)</t>
+          <t>0.33% (0.29%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.26% (1.95%)</t>
+          <t>3.55% (3.25%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2.52% (2.07%)</t>
+          <t>3.80% (3.36%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.77% (1.39%)</t>
+          <t>3.02% (2.66%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.02% (-0.80%)</t>
+          <t>0.61% (-0.19%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.03% (-0.78%)</t>
+          <t>0.18% (-0.55%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>6.41% (5.91%)</t>
+          <t>5.80% (5.31%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.81% (-1.49%)</t>
+          <t>0.15% (-0.52%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.24% (3.00%)</t>
+          <t>3.25% (3.02%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.61% (2.44%)</t>
+          <t>2.35% (2.20%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2.23% (2.13%)</t>
+          <t>1.52% (1.43%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 31/7/2026</t>
+          <t>As of 3/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.63%</t>
+          <t>6.51%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.62%</t>
+          <t>6.73%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.17%</t>
+          <t>9.30%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.86%</t>
+          <t>4.79%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.12%</t>
+          <t>-7.10%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.16%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.55%</t>
+          <t>6.57%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.52%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>4.88%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.06%</t>
+          <t>-6.96%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.54%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7.09%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.62%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>16.56%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.72%</t>
+          <t>-9.41%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.84%</t>
+          <t>10.50%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.75%</t>
+          <t>9.57%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.22%</t>
+          <t>4.32%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>6.46%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>8.18%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.94%</t>
+          <t>-4.96%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.51%</t>
+          <t>9.03%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15.19%</t>
+          <t>13.76%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.76%</t>
+          <t>14.49%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-2.97%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.67%</t>
+          <t>9.16%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15.82%</t>
+          <t>14.33%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.19%</t>
+          <t>1.12%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>-1.94%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8.96%</t>
+          <t>9.47%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16.03%</t>
+          <t>14.57%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>1.71%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>17.14%</t>
+          <t>14.86%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-2.04%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>11.17%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.05%</t>
+          <t>0.42%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>12.95%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.21%</t>
+          <t>17.49%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-2.72%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-11.68%</t>
+          <t>-12.23%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.81%</t>
+          <t>10.43%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>2.07%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>10.86%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.69%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2.07%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.61%</t>
+          <t>-10.56%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.22%</t>
+          <t>3.13%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.62%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>13.79%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>1.15%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.55%</t>
+          <t>-10.49%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.06%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>4.14%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>11.17%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12.48%</t>
+          <t>14.71%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3.68%</t>
+          <t>1.66%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.92%</t>
+          <t>-10.81%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.06%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6.48%</t>
+          <t>5.36%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>8.11%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>11.08%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5.35%</t>
+          <t>3.31%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.31%</t>
+          <t>-8.29%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 31/7/2026</t>
+          <t>As of 3/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.24%</t>
+          <t>16.09%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.82%</t>
+          <t>5.04%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.87%</t>
+          <t>5.64%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7.17%</t>
+          <t>9.30%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-5.45%</t>
+          <t>-6.14%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.82%</t>
+          <t>16.67%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.41%</t>
+          <t>5.64%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.51%</t>
+          <t>5.27%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.52%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.21%</t>
+          <t>2.19%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.12%</t>
+          <t>-5.81%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.35%</t>
+          <t>19.27%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>5.31%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.94%</t>
+          <t>7.55%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>16.56%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.17%</t>
+          <t>-2.11%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.28%</t>
+          <t>-7.80%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.12%</t>
+          <t>15.93%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.57%</t>
+          <t>7.70%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.70%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>6.46%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.62%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-3.45%</t>
+          <t>-4.22%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.47%</t>
+          <t>14.14%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>10.82%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>1.94%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.51%</t>
+          <t>11.30%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-1.77%</t>
+          <t>-2.75%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.60%</t>
+          <t>14.26%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.58%</t>
+          <t>11.45%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>0.95%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.19%</t>
+          <t>11.97%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.78%</t>
+          <t>-1.78%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>14.55%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.03%</t>
+          <t>11.80%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>1.05%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>1.71%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>11.91%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-1.88%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.09%</t>
+          <t>17.20%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.31%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.21%</t>
+          <t>17.49%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.13%</t>
+          <t>-10.45%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.42%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.13%</t>
+          <t>1.43%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.33%</t>
+          <t>9.08%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11.69%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.19%</t>
+          <t>-2.13%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.47%</t>
+          <t>-9.10%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.55%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.97%</t>
+          <t>2.20%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.09%</t>
+          <t>8.90%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>13.79%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.26%</t>
+          <t>-8.95%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.77%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.71%</t>
+          <t>3.02%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.38%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12.48%</t>
+          <t>14.71%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-1.27%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-8.51%</t>
+          <t>-9.13%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.50%</t>
+          <t>16.35%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>6.76%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>11.08%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-6.46%</t>
+          <t>-7.12%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-04]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/3/2026 at 11:57 AM ET)</t>
+          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>256 days</t>
+          <t>255 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>18 days</t>
+          <t>17 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>137 days</t>
+          <t>136 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>200 days</t>
+          <t>199 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>165 days</t>
+          <t>164 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>347 days</t>
+          <t>346 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>318 days</t>
+          <t>317 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>228 days</t>
+          <t>227 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>291 days</t>
+          <t>290 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>109 days</t>
+          <t>108 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>74 days</t>
+          <t>73 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>46 days</t>
+          <t>45 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>256 days</t>
+          <t>255 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>18 days</t>
+          <t>17 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>137 days</t>
+          <t>136 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>200 days</t>
+          <t>199 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>165 days</t>
+          <t>164 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>347 days</t>
+          <t>346 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>318 days</t>
+          <t>317 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>228 days</t>
+          <t>227 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>291 days</t>
+          <t>290 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>109 days</t>
+          <t>108 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>74 days</t>
+          <t>73 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>46 days</t>
+          <t>45 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.23 / 4.32%</t>
+          <t>$47.53 / 4.99%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.25 / 12.95%</t>
+          <t>$57.34 / 13.12%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.15 / 8.11%</t>
+          <t>$55.47 / 8.74%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$61.72 / 6.57%</t>
+          <t>$62.07 / 7.18%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$55.79 / 6.73%</t>
+          <t>$56.14 / 7.40%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$60.58 / 1.22%</t>
+          <t>$61.06 / 2.02%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.54 / 1.12%</t>
+          <t>$61.04 / 1.95%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$52.88 / 9.45%</t>
+          <t>$53.07 / 9.84%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.77 / 2.17%</t>
+          <t>$57.29 / 3.10%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.19 / 11.17%</t>
+          <t>$59.50 / 11.74%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.03 / 10.77%</t>
+          <t>$53.28 / 11.29%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$55.88 / 10.86%</t>
+          <t>$56.16 / 11.40%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.08 / 3.52%</t>
+          <t>$42.27 / 3.99%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.86 / 10.71%</t>
+          <t>$41.89 / 10.78%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.24 / 6.76%</t>
+          <t>$40.42 / 7.24%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.45 / 5.27%</t>
+          <t>$44.63 / 5.71%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.48 / 5.64%</t>
+          <t>$45.70 / 6.16%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.11 / 1.05%</t>
+          <t>$44.39 / 1.70%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.54 / 0.95%</t>
+          <t>$41.80 / 1.58%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.67 / 7.55%</t>
+          <t>$44.82 / 7.92%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.47 / 1.94%</t>
+          <t>$43.76 / 2.62%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.25 / 9.12%</t>
+          <t>$42.37 / 9.41%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.00 / 8.90%</t>
+          <t>$42.13 / 9.24%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.43 / 9.08%</t>
+          <t>$41.55 / 9.40%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$755.99 / 6.46%</t>
+          <t>$768.63 / 8.24%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$755.99 / 17.49%</t>
+          <t>$768.63 / 19.46%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$755.99 / 11.08%</t>
+          <t>$768.63 / 12.94%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$755.99 / 9.65%</t>
+          <t>$768.63 / 11.49%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$755.99 / 9.30%</t>
+          <t>$768.63 / 11.13%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$755.99 / 1.71%</t>
+          <t>$768.63 / 3.41%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$755.99 / 1.24%</t>
+          <t>$768.63 / 2.93%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$755.99 / 16.56%</t>
+          <t>$768.63 / 18.51%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$755.99 / 2.27%</t>
+          <t>$768.63 / 3.99%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$755.99 / 14.71%</t>
+          <t>$768.63 / 16.63%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$755.99 / 13.79%</t>
+          <t>$768.63 / 15.69%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$755.99 / 13.90%</t>
+          <t>$768.63 / 15.81%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$755.99 / 6.46%</t>
+          <t>$768.63 / 8.24%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$755.99 / 17.49%</t>
+          <t>$768.63 / 19.46%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$755.99 / 11.08%</t>
+          <t>$768.63 / 12.94%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$755.99 / 9.65%</t>
+          <t>$768.63 / 11.49%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$755.99 / 9.30%</t>
+          <t>$768.63 / 11.13%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$755.99 / 1.71%</t>
+          <t>$768.63 / 3.41%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$755.99 / 1.24%</t>
+          <t>$768.63 / 2.93%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$755.99 / 16.56%</t>
+          <t>$768.63 / 18.51%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$755.99 / 2.27%</t>
+          <t>$768.63 / 3.99%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$755.99 / 14.71%</t>
+          <t>$768.63 / 16.63%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$755.99 / 13.79%</t>
+          <t>$768.63 / 15.69%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$755.99 / 13.90%</t>
+          <t>$768.63 / 15.81%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.15% (9.57%)</t>
+          <t>9.45% (8.88%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.46% (0.42%)</t>
+          <t>0.31% (0.27%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5.65% (5.36%)</t>
+          <t>5.04% (4.75%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>7.56% (7.12%)</t>
+          <t>6.95% (6.52%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>6.87% (6.51%)</t>
+          <t>6.20% (5.85%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>15.37% (14.57%)</t>
+          <t>14.46% (13.67%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.06% (14.33%)</t>
+          <t>14.11% (13.39%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.77% (6.28%)</t>
+          <t>6.38% (5.90%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>14.42% (13.76%)</t>
+          <t>13.39% (12.73%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>4.37% (4.14%)</t>
+          <t>3.83% (3.61%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>3.29% (3.13%)</t>
+          <t>2.80% (2.65%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2.17% (2.07%)</t>
+          <t>1.67% (1.57%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>8.28% (7.70%)</t>
+          <t>7.79% (7.22%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.33% (0.29%)</t>
+          <t>0.27% (0.23%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>4.49% (4.19%)</t>
+          <t>4.02% (3.73%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>6.08% (5.64%)</t>
+          <t>5.64% (5.20%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>5.40% (5.04%)</t>
+          <t>4.89% (4.53%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>12.60% (11.80%)</t>
+          <t>11.87% (11.08%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.18% (11.45%)</t>
+          <t>11.48% (10.75%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.80% (5.31%)</t>
+          <t>5.43% (4.94%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>11.49% (10.82%)</t>
+          <t>10.75% (10.09%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>3.25% (3.02%)</t>
+          <t>2.97% (2.74%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2.35% (2.20%)</t>
+          <t>2.04% (1.88%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>1.52% (1.43%)</t>
+          <t>1.23% (1.13%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.18%</t>
+          <t>6.40%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-2.72%</t>
+          <t>-4.32%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.31%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.88%</t>
+          <t>3.16%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4.79%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>14.86%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>-1.13%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>14.49%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.66%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.15%</t>
+          <t>-0.52%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>-1.56%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>3.79%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-4.76%</t>
+          <t>-6.33%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>-0.75%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.19%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>0.62%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>11.91%</t>
+          <t>10.07%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.97%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-2.11%</t>
+          <t>-3.72%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>11.30%</t>
+          <t>9.47%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-1.27%</t>
+          <t>-2.90%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-3.07%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-2.13%</t>
+          <t>-3.74%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.07% (10.50%)</t>
+          <t>11.86% (11.29%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11.21% (11.17%)</t>
+          <t>12.33% (12.30%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.98% (10.69%)</t>
+          <t>11.78% (11.49%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.40% (10.96%)</t>
+          <t>12.22% (11.79%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.92% (10.56%)</t>
+          <t>11.69% (11.33%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.27% (9.47%)</t>
+          <t>10.94% (10.15%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.89% (9.16%)</t>
+          <t>10.54% (9.82%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.87% (13.38%)</t>
+          <t>14.81% (14.33%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.69% (9.03%)</t>
+          <t>10.26% (9.61%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.96% (10.73%)</t>
+          <t>11.79% (11.57%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.57% (10.42%)</t>
+          <t>11.45% (11.30%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.53% (10.43%)</t>
+          <t>11.39% (11.29%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.51% (15.93%)</t>
+          <t>17.39% (16.82%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>17.24% (17.20%)</t>
+          <t>18.37% (18.34%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.65% (16.35%)</t>
+          <t>17.49% (17.20%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.11% (16.67%)</t>
+          <t>18.00% (17.56%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.45% (16.09%)</t>
+          <t>17.28% (16.92%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.35% (14.55%)</t>
+          <t>16.09% (15.29%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.99% (14.26%)</t>
+          <t>15.76% (15.03%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.76% (19.27%)</t>
+          <t>20.64% (20.15%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.81% (14.14%)</t>
+          <t>15.52% (14.87%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.00% (16.77%)</t>
+          <t>17.97% (17.74%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.50% (16.34%)</t>
+          <t>17.45% (17.29%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.37% (16.27%)</t>
+          <t>17.34% (17.24%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-4.39% (-4.96%)</t>
+          <t>-4.99% (-5.56%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.19% (-12.23%)</t>
+          <t>-12.33% (-12.36%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-7.99% (-8.29%)</t>
+          <t>-8.53% (-8.82%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-6.52% (-6.96%)</t>
+          <t>-7.05% (-7.49%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-6.74% (-7.10%)</t>
+          <t>-7.32% (-7.68%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-1.24% (-2.04%)</t>
+          <t>-2.02% (-2.81%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-1.21% (-1.94%)</t>
+          <t>-2.02% (-2.75%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.92% (-9.41%)</t>
+          <t>-9.25% (-9.73%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-2.31% (-2.97%)</t>
+          <t>-3.19% (-3.84%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-10.58% (-10.81%)</t>
+          <t>-11.04% (-11.26%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-10.33% (-10.49%)</t>
+          <t>-10.76% (-10.91%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-10.46% (-10.56%)</t>
+          <t>-10.90% (-11.00%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-3.64% (-4.22%)</t>
+          <t>-4.08% (-4.65%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.41% (-10.45%)</t>
+          <t>-10.47% (-10.50%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-6.82% (-7.12%)</t>
+          <t>-7.24% (-7.54%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-5.37% (-5.81%)</t>
+          <t>-5.76% (-6.20%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-5.78% (-6.14%)</t>
+          <t>-6.23% (-6.59%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.08% (-1.88%)</t>
+          <t>-1.71% (-2.51%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.04% (-1.78%)</t>
+          <t>-1.66% (-2.39%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.31% (-7.80%)</t>
+          <t>-7.63% (-8.12%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.08% (-2.75%)</t>
+          <t>-2.73% (-3.39%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-8.90% (-9.13%)</t>
+          <t>-9.14% (-9.37%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-8.79% (-8.95%)</t>
+          <t>-9.08% (-9.23%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.00% (-9.10%)</t>
+          <t>-9.27% (-9.36%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.46%</t>
+          <t>-16.85%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-23.40%</t>
+          <t>-24.66%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-18.98%</t>
+          <t>-20.31%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-17.92%</t>
+          <t>-19.27%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-17.66%</t>
+          <t>-19.01%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-11.51%</t>
+          <t>-12.97%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-11.10%</t>
+          <t>-12.56%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.79%</t>
+          <t>-24.06%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.00%</t>
+          <t>-13.45%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.54%</t>
+          <t>-22.83%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-20.90%</t>
+          <t>-22.21%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-20.99%</t>
+          <t>-22.29%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-20.15%</t>
+          <t>-21.47%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-27.65%</t>
+          <t>-28.84%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.47%</t>
+          <t>-24.73%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.48%</t>
+          <t>-23.76%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-22.23%</t>
+          <t>-23.51%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-16.42%</t>
+          <t>-17.80%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.04%</t>
+          <t>-17.42%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.08%</t>
+          <t>-28.27%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-16.89%</t>
+          <t>-18.26%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-25.90%</t>
+          <t>-27.12%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-25.30%</t>
+          <t>-26.53%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.37%</t>
+          <t>-26.60%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.80% (1.23%)</t>
+          <t>2.85% (2.29%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.46% (0.42%)</t>
+          <t>0.31% (0.27%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.25% (1.96%)</t>
+          <t>3.37% (3.08%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.53% (2.10%)</t>
+          <t>3.66% (3.23%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.97% (1.61%)</t>
+          <t>3.04% (2.68%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.44% (-0.36%)</t>
+          <t>1.32% (0.53%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.01% (-0.72%)</t>
+          <t>0.85% (0.13%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.21% (5.72%)</t>
+          <t>6.38% (5.90%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.08% (-0.74%)</t>
+          <t>0.68% (0.02%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.65% (2.43%)</t>
+          <t>3.83% (3.61%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.11% (1.96%)</t>
+          <t>2.80% (2.65%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2.08% (1.99%)</t>
+          <t>1.67% (1.57%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.59% (2.01%)</t>
+          <t>3.84% (3.27%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.33% (0.29%)</t>
+          <t>0.27% (0.23%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.55% (3.25%)</t>
+          <t>4.02% (3.73%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.80% (3.36%)</t>
+          <t>5.10% (4.67%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.02% (2.66%)</t>
+          <t>4.25% (3.89%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.61% (-0.19%)</t>
+          <t>1.64% (0.84%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.18% (-0.55%)</t>
+          <t>1.22% (0.49%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.80% (5.31%)</t>
+          <t>5.43% (4.94%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.15% (-0.52%)</t>
+          <t>1.15% (0.49%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>3.25% (3.02%)</t>
+          <t>2.97% (2.74%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.35% (2.20%)</t>
+          <t>2.04% (1.88%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>1.52% (1.43%)</t>
+          <t>1.23% (1.13%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 3/8/2026</t>
+          <t>As of 4/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>11.33%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.51%</t>
+          <t>5.85%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.73%</t>
+          <t>7.40%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.30%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.79%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.10%</t>
+          <t>-7.68%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>11.79%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>6.52%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.57%</t>
+          <t>7.18%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>11.49%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.88%</t>
+          <t>3.16%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.96%</t>
+          <t>-7.49%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>14.33%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>5.90%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>9.84%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.56%</t>
+          <t>18.51%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>-1.13%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.41%</t>
+          <t>-9.73%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.50%</t>
+          <t>11.29%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9.57%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.32%</t>
+          <t>4.99%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.46%</t>
+          <t>8.24%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.18%</t>
+          <t>6.40%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.96%</t>
+          <t>-5.56%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.03%</t>
+          <t>9.61%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13.76%</t>
+          <t>12.73%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.49%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.97%</t>
+          <t>-3.84%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.16%</t>
+          <t>9.82%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14.33%</t>
+          <t>13.39%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.12%</t>
+          <t>1.95%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.94%</t>
+          <t>-2.75%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.47%</t>
+          <t>10.15%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14.57%</t>
+          <t>13.67%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>2.02%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.71%</t>
+          <t>3.41%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.86%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.04%</t>
+          <t>-2.81%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.17%</t>
+          <t>12.30%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.27%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.95%</t>
+          <t>13.12%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>17.49%</t>
+          <t>19.46%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-2.72%</t>
+          <t>-4.32%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.23%</t>
+          <t>-12.36%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.43%</t>
+          <t>11.29%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.07%</t>
+          <t>1.57%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.86%</t>
+          <t>11.40%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>15.81%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>-1.56%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-10.56%</t>
+          <t>-11.00%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>11.30%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.13%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>11.29%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.79%</t>
+          <t>15.69%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.15%</t>
+          <t>-0.52%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.49%</t>
+          <t>-10.91%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.14%</t>
+          <t>3.61%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.17%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.71%</t>
+          <t>16.63%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.66%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.81%</t>
+          <t>-11.26%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>11.49%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.36%</t>
+          <t>4.75%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.11%</t>
+          <t>8.74%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.08%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.31%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.29%</t>
+          <t>-8.82%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 3/8/2026</t>
+          <t>As of 4/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.09%</t>
+          <t>16.92%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.04%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.64%</t>
+          <t>6.16%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.30%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>0.62%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.14%</t>
+          <t>-6.59%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>17.56%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.64%</t>
+          <t>5.20%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.27%</t>
+          <t>5.71%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>11.49%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.19%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-5.81%</t>
+          <t>-6.20%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.27%</t>
+          <t>20.15%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.31%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.55%</t>
+          <t>7.92%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.56%</t>
+          <t>18.51%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.11%</t>
+          <t>-3.72%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-7.80%</t>
+          <t>-8.12%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.93%</t>
+          <t>16.82%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.70%</t>
+          <t>7.22%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.46%</t>
+          <t>8.24%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>3.79%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.22%</t>
+          <t>-4.65%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.14%</t>
+          <t>14.87%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.82%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.94%</t>
+          <t>2.62%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.30%</t>
+          <t>9.47%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-2.75%</t>
+          <t>-3.39%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.26%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.45%</t>
+          <t>10.75%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>1.58%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.97%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-1.78%</t>
+          <t>-2.39%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.55%</t>
+          <t>15.29%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.80%</t>
+          <t>11.08%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.05%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.71%</t>
+          <t>3.41%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.91%</t>
+          <t>10.07%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-1.88%</t>
+          <t>-2.51%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17.20%</t>
+          <t>18.34%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>0.23%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.78%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>17.49%</t>
+          <t>19.46%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.76%</t>
+          <t>-6.33%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.45%</t>
+          <t>-10.50%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.43%</t>
+          <t>1.13%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.08%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>15.81%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.13%</t>
+          <t>-3.74%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.10%</t>
+          <t>-9.36%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>17.29%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.20%</t>
+          <t>1.88%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.90%</t>
+          <t>9.24%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.79%</t>
+          <t>15.69%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-3.07%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-8.95%</t>
+          <t>-9.23%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.77%</t>
+          <t>17.74%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>9.41%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.71%</t>
+          <t>16.63%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.27%</t>
+          <t>-2.90%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.13%</t>
+          <t>-9.37%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.35%</t>
+          <t>17.20%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.76%</t>
+          <t>7.24%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.08%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>-0.75%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.12%</t>
+          <t>-7.54%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-05]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/4/2026 at 11:49 AM ET)</t>
+          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>255 days</t>
+          <t>254 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>136 days</t>
+          <t>135 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>199 days</t>
+          <t>198 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>164 days</t>
+          <t>163 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>346 days</t>
+          <t>345 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>317 days</t>
+          <t>316 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>227 days</t>
+          <t>226 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>290 days</t>
+          <t>289 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>108 days</t>
+          <t>107 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>73 days</t>
+          <t>72 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>45 days</t>
+          <t>44 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>255 days</t>
+          <t>254 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>17 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>136 days</t>
+          <t>135 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>199 days</t>
+          <t>198 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>164 days</t>
+          <t>163 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>346 days</t>
+          <t>345 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>317 days</t>
+          <t>316 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>227 days</t>
+          <t>226 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>290 days</t>
+          <t>289 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>108 days</t>
+          <t>107 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>73 days</t>
+          <t>72 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>45 days</t>
+          <t>44 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.53 / 4.99%</t>
+          <t>$47.64 / 5.23%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.34 / 13.12%</t>
+          <t>$57.36 / 13.16%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.47 / 8.74%</t>
+          <t>$55.57 / 8.94%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.07 / 7.18%</t>
+          <t>$62.20 / 7.40%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.14 / 7.40%</t>
+          <t>$56.25 / 7.62%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.06 / 2.02%</t>
+          <t>$61.23 / 2.31%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.04 / 1.95%</t>
+          <t>$61.24 / 2.29%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.07 / 9.84%</t>
+          <t>$53.15 / 10.01%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.29 / 3.10%</t>
+          <t>$57.44 / 3.38%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.50 / 11.74%</t>
+          <t>$59.60 / 11.94%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.28 / 11.29%</t>
+          <t>$53.36 / 11.47%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.16 / 11.40%</t>
+          <t>$56.21 / 11.51%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.27 / 3.99%</t>
+          <t>$42.34 / 4.17%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.89 / 10.78%</t>
+          <t>$41.91 / 10.84%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.42 / 7.24%</t>
+          <t>$40.46 / 7.36%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.63 / 5.71%</t>
+          <t>$44.70 / 5.86%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.70 / 6.16%</t>
+          <t>$45.76 / 6.28%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.39 / 1.70%</t>
+          <t>$44.47 / 1.89%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.80 / 1.58%</t>
+          <t>$41.92 / 1.87%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.82 / 7.92%</t>
+          <t>$44.85 / 7.98%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.76 / 2.62%</t>
+          <t>$43.88 / 2.91%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.37 / 9.41%</t>
+          <t>$42.44 / 9.59%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.13 / 9.24%</t>
+          <t>$42.18 / 9.36%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.55 / 9.40%</t>
+          <t>$41.59 / 9.51%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$768.63 / 8.24%</t>
+          <t>$772.02 / 8.71%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$768.63 / 19.46%</t>
+          <t>$772.02 / 19.98%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$768.63 / 12.94%</t>
+          <t>$772.02 / 13.43%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$768.63 / 11.49%</t>
+          <t>$772.02 / 11.98%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$768.63 / 11.13%</t>
+          <t>$772.02 / 11.62%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$768.63 / 3.41%</t>
+          <t>$772.02 / 3.87%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$768.63 / 2.93%</t>
+          <t>$772.02 / 3.39%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$768.63 / 18.51%</t>
+          <t>$772.02 / 19.03%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$768.63 / 3.99%</t>
+          <t>$772.02 / 4.44%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$768.63 / 16.63%</t>
+          <t>$772.02 / 17.14%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$768.63 / 15.69%</t>
+          <t>$772.02 / 16.20%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$768.63 / 15.81%</t>
+          <t>$772.02 / 16.32%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$768.63 / 8.24%</t>
+          <t>$772.02 / 8.71%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$768.63 / 19.46%</t>
+          <t>$772.02 / 19.98%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$768.63 / 12.94%</t>
+          <t>$772.02 / 13.43%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$768.63 / 11.49%</t>
+          <t>$772.02 / 11.98%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$768.63 / 11.13%</t>
+          <t>$772.02 / 11.62%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$768.63 / 3.41%</t>
+          <t>$772.02 / 3.87%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$768.63 / 2.93%</t>
+          <t>$772.02 / 3.39%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$768.63 / 18.51%</t>
+          <t>$772.02 / 19.03%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$768.63 / 3.99%</t>
+          <t>$772.02 / 4.44%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$768.63 / 16.63%</t>
+          <t>$772.02 / 17.14%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$768.63 / 15.69%</t>
+          <t>$772.02 / 16.20%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$768.63 / 15.81%</t>
+          <t>$772.02 / 16.32%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.45% (8.88%)</t>
+          <t>9.19% (8.63%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.31% (0.27%)</t>
+          <t>0.27% (0.24%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5.04% (4.75%)</t>
+          <t>4.85% (4.56%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.95% (6.52%)</t>
+          <t>6.72% (6.30%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>6.20% (5.85%)</t>
+          <t>5.99% (5.63%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.46% (13.67%)</t>
+          <t>14.14% (13.36%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>14.11% (13.39%)</t>
+          <t>13.74% (13.02%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.38% (5.90%)</t>
+          <t>6.22% (5.74%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.39% (12.73%)</t>
+          <t>13.08% (12.43%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.83% (3.61%)</t>
+          <t>3.65% (3.43%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.80% (2.65%)</t>
+          <t>2.64% (2.49%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>1.67% (1.57%)</t>
+          <t>1.56% (1.47%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.79% (7.22%)</t>
+          <t>7.59% (7.03%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.27% (0.23%)</t>
+          <t>0.20% (0.17%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>4.02% (3.73%)</t>
+          <t>3.91% (3.61%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.64% (5.20%)</t>
+          <t>5.48% (5.05%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.89% (4.53%)</t>
+          <t>4.76% (4.41%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.87% (11.08%)</t>
+          <t>11.67% (10.88%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.48% (10.75%)</t>
+          <t>11.16% (10.44%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.43% (4.94%)</t>
+          <t>5.37% (4.88%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.75% (10.09%)</t>
+          <t>10.43% (9.77%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.97% (2.74%)</t>
+          <t>2.79% (2.57%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2.04% (1.88%)</t>
+          <t>1.93% (1.77%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>1.23% (1.13%)</t>
+          <t>1.12% (1.02%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.40%</t>
+          <t>5.93%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>-4.74%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.16%</t>
+          <t>2.71%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>2.61%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>12.47%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>12.64%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.13%</t>
+          <t>-1.57%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.45%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>-0.95%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-1.56%</t>
+          <t>-1.99%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.79%</t>
+          <t>3.34%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-6.33%</t>
+          <t>-6.74%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-1.19%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.07%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.72%</t>
+          <t>-4.14%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.47%</t>
+          <t>8.99%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.90%</t>
+          <t>-3.32%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.07%</t>
+          <t>-3.49%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-3.74%</t>
+          <t>-4.16%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.86% (11.29%)</t>
+          <t>12.00% (11.44%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.33% (12.30%)</t>
+          <t>12.63% (12.60%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.78% (11.49%)</t>
+          <t>11.97% (11.68%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.22% (11.79%)</t>
+          <t>12.38% (11.95%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.69% (11.33%)</t>
+          <t>11.85% (11.50%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.94% (10.15%)</t>
+          <t>11.05% (10.27%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.54% (9.82%)</t>
+          <t>10.60% (9.88%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.81% (14.33%)</t>
+          <t>15.00% (14.52%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.26% (9.61%)</t>
+          <t>10.38% (9.73%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.79% (11.57%)</t>
+          <t>11.97% (11.75%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.45% (11.30%)</t>
+          <t>11.65% (11.50%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.39% (11.29%)</t>
+          <t>11.64% (11.55%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.39% (16.82%)</t>
+          <t>17.56% (16.99%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.37% (18.34%)</t>
+          <t>18.63% (18.60%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.49% (17.20%)</t>
+          <t>17.72% (17.43%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.00% (17.56%)</t>
+          <t>18.19% (17.76%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.28% (16.92%)</t>
+          <t>17.50% (17.14%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.09% (15.29%)</t>
+          <t>16.27% (15.48%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.76% (15.03%)</t>
+          <t>15.83% (15.11%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.64% (20.15%)</t>
+          <t>20.90% (20.42%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.52% (14.87%)</t>
+          <t>15.60% (14.95%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.97% (17.74%)</t>
+          <t>18.14% (17.91%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.45% (17.29%)</t>
+          <t>17.67% (17.52%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.34% (17.24%)</t>
+          <t>17.56% (17.46%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-4.99% (-5.56%)</t>
+          <t>-5.21% (-5.78%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.33% (-12.36%)</t>
+          <t>-12.36% (-12.39%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.53% (-8.82%)</t>
+          <t>-8.69% (-8.98%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.05% (-7.49%)</t>
+          <t>-7.25% (-7.68%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.32% (-7.68%)</t>
+          <t>-7.52% (-7.87%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.02% (-2.81%)</t>
+          <t>-2.30% (-3.08%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.02% (-2.75%)</t>
+          <t>-2.34% (-3.06%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.25% (-9.73%)</t>
+          <t>-9.39% (-9.87%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.19% (-3.84%)</t>
+          <t>-3.45% (-4.10%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.04% (-11.26%)</t>
+          <t>-11.20% (-11.42%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-10.76% (-10.91%)</t>
+          <t>-10.90% (-11.05%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-10.90% (-11.00%)</t>
+          <t>-10.99% (-11.08%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.08% (-4.65%)</t>
+          <t>-4.25% (-4.82%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.47% (-10.50%)</t>
+          <t>-10.52% (-10.56%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.24% (-7.54%)</t>
+          <t>-7.35% (-7.64%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-5.76% (-6.20%)</t>
+          <t>-5.90% (-6.33%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.23% (-6.59%)</t>
+          <t>-6.35% (-6.71%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.71% (-2.51%)</t>
+          <t>-1.89% (-2.68%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.66% (-2.39%)</t>
+          <t>-1.95% (-2.67%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.63% (-8.12%)</t>
+          <t>-7.69% (-8.17%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.73% (-3.39%)</t>
+          <t>-3.01% (-3.67%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.14% (-9.37%)</t>
+          <t>-9.30% (-9.52%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.08% (-9.23%)</t>
+          <t>-9.18% (-9.33%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.27% (-9.36%)</t>
+          <t>-9.37% (-9.46%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.85%</t>
+          <t>-17.21%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-24.66%</t>
+          <t>-24.99%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.31%</t>
+          <t>-20.66%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.27%</t>
+          <t>-19.63%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.01%</t>
+          <t>-19.37%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.97%</t>
+          <t>-13.35%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.56%</t>
+          <t>-12.95%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.06%</t>
+          <t>-24.39%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.45%</t>
+          <t>-13.83%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.83%</t>
+          <t>-23.17%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.21%</t>
+          <t>-22.55%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.29%</t>
+          <t>-22.63%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.47%</t>
+          <t>-21.81%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-28.84%</t>
+          <t>-29.15%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.73%</t>
+          <t>-25.06%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.76%</t>
+          <t>-24.09%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.51%</t>
+          <t>-23.85%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.80%</t>
+          <t>-18.16%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.42%</t>
+          <t>-17.78%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.27%</t>
+          <t>-28.59%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.26%</t>
+          <t>-18.61%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.12%</t>
+          <t>-27.44%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.53%</t>
+          <t>-26.85%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-26.60%</t>
+          <t>-26.92%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.85% (2.29%)</t>
+          <t>3.07% (2.51%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.31% (0.27%)</t>
+          <t>0.27% (0.24%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.37% (3.08%)</t>
+          <t>3.64% (3.35%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.66% (3.23%)</t>
+          <t>3.90% (3.47%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3.04% (2.68%)</t>
+          <t>3.28% (2.93%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.32% (0.53%)</t>
+          <t>1.48% (0.70%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.85% (0.13%)</t>
+          <t>0.97% (0.25%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.38% (5.90%)</t>
+          <t>6.22% (5.74%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.68% (0.02%)</t>
+          <t>0.85% (0.20%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.83% (3.61%)</t>
+          <t>3.65% (3.43%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.80% (2.65%)</t>
+          <t>2.64% (2.49%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.67% (1.57%)</t>
+          <t>1.56% (1.47%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.84% (3.27%)</t>
+          <t>4.11% (3.54%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.27% (0.23%)</t>
+          <t>0.20% (0.17%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>4.02% (3.73%)</t>
+          <t>3.91% (3.61%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.10% (4.67%)</t>
+          <t>5.41% (4.98%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.25% (3.89%)</t>
+          <t>4.58% (4.22%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.64% (0.84%)</t>
+          <t>1.90% (1.11%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.22% (0.49%)</t>
+          <t>1.37% (0.65%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.43% (4.94%)</t>
+          <t>5.37% (4.88%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.15% (0.49%)</t>
+          <t>1.30% (0.65%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.97% (2.74%)</t>
+          <t>2.79% (2.57%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2.04% (1.88%)</t>
+          <t>1.93% (1.77%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>1.23% (1.13%)</t>
+          <t>1.12% (1.02%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 4/8/2026</t>
+          <t>As of 5/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.33%</t>
+          <t>11.50%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.85%</t>
+          <t>5.63%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.40%</t>
+          <t>7.62%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>2.61%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.68%</t>
+          <t>-7.87%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.79%</t>
+          <t>11.95%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.52%</t>
+          <t>6.30%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.18%</t>
+          <t>7.40%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.49%</t>
+          <t>11.98%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.16%</t>
+          <t>2.71%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.49%</t>
+          <t>-7.68%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.33%</t>
+          <t>14.52%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.90%</t>
+          <t>5.74%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.84%</t>
+          <t>10.01%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.51%</t>
+          <t>19.03%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.13%</t>
+          <t>-1.57%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.73%</t>
+          <t>-9.87%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.44%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>5.23%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>8.71%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.40%</t>
+          <t>5.93%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.56%</t>
+          <t>-5.78%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.61%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.73%</t>
+          <t>12.43%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>4.44%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.84%</t>
+          <t>-4.10%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.82%</t>
+          <t>9.88%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.39%</t>
+          <t>13.02%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.95%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.93%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>12.64%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.75%</t>
+          <t>-3.06%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.15%</t>
+          <t>10.27%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.67%</t>
+          <t>13.36%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.02%</t>
+          <t>2.31%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.41%</t>
+          <t>3.87%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>12.47%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.81%</t>
+          <t>-3.08%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.30%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.27%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.12%</t>
+          <t>13.16%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>19.46%</t>
+          <t>19.98%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>-4.74%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.36%</t>
+          <t>-12.39%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.57%</t>
+          <t>1.47%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.40%</t>
+          <t>11.51%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15.81%</t>
+          <t>16.32%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.56%</t>
+          <t>-1.99%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.00%</t>
+          <t>-11.08%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.30%</t>
+          <t>11.50%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>2.49%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.69%</t>
+          <t>16.20%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>-0.95%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.91%</t>
+          <t>-11.05%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>11.75%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.61%</t>
+          <t>3.43%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.74%</t>
+          <t>11.94%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.63%</t>
+          <t>17.14%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.45%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.26%</t>
+          <t>-11.42%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.49%</t>
+          <t>11.68%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.75%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.74%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.94%</t>
+          <t>13.43%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.82%</t>
+          <t>-8.98%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 4/8/2026</t>
+          <t>As of 5/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.92%</t>
+          <t>17.14%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.16%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.59%</t>
+          <t>-6.71%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.56%</t>
+          <t>17.76%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.20%</t>
+          <t>5.05%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.71%</t>
+          <t>5.86%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.49%</t>
+          <t>11.98%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.20%</t>
+          <t>-6.33%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.15%</t>
+          <t>20.42%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>4.88%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.92%</t>
+          <t>7.98%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.51%</t>
+          <t>19.03%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.72%</t>
+          <t>-4.14%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.12%</t>
+          <t>-8.17%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.82%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.22%</t>
+          <t>7.03%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>8.71%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.79%</t>
+          <t>3.34%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.65%</t>
+          <t>-4.82%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.87%</t>
+          <t>14.95%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.62%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>4.44%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.47%</t>
+          <t>8.99%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.39%</t>
+          <t>-3.67%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>15.11%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.75%</t>
+          <t>10.44%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.58%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.93%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.39%</t>
+          <t>-2.67%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.29%</t>
+          <t>15.48%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.08%</t>
+          <t>10.88%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.41%</t>
+          <t>3.87%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.07%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.51%</t>
+          <t>-2.68%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.34%</t>
+          <t>18.60%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.78%</t>
+          <t>10.84%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>19.46%</t>
+          <t>19.98%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-6.33%</t>
+          <t>-6.74%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.50%</t>
+          <t>-10.56%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>17.46%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.13%</t>
+          <t>1.02%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>9.51%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15.81%</t>
+          <t>16.32%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-3.74%</t>
+          <t>-4.16%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.36%</t>
+          <t>-9.46%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.29%</t>
+          <t>17.52%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.88%</t>
+          <t>1.77%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.24%</t>
+          <t>9.36%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.69%</t>
+          <t>16.20%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.07%</t>
+          <t>-3.49%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.23%</t>
+          <t>-9.33%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.74%</t>
+          <t>17.91%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.74%</t>
+          <t>2.57%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.41%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.63%</t>
+          <t>17.14%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.90%</t>
+          <t>-3.32%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.37%</t>
+          <t>-9.52%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.20%</t>
+          <t>17.43%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>3.61%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.24%</t>
+          <t>7.36%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.94%</t>
+          <t>13.43%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-1.19%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.54%</t>
+          <t>-7.64%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-06]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/5/2026 at 11:37 AM ET)</t>
+          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>254 days</t>
+          <t>253 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>15 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>135 days</t>
+          <t>134 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>198 days</t>
+          <t>197 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>163 days</t>
+          <t>162 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>345 days</t>
+          <t>344 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>316 days</t>
+          <t>315 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>226 days</t>
+          <t>225 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>289 days</t>
+          <t>288 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>107 days</t>
+          <t>106 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>72 days</t>
+          <t>71 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>44 days</t>
+          <t>43 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>254 days</t>
+          <t>253 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>15 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>135 days</t>
+          <t>134 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>198 days</t>
+          <t>197 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>163 days</t>
+          <t>162 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>345 days</t>
+          <t>344 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>316 days</t>
+          <t>315 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>226 days</t>
+          <t>225 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>289 days</t>
+          <t>288 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>107 days</t>
+          <t>106 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>72 days</t>
+          <t>71 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>44 days</t>
+          <t>43 days</t>
         </is>
       </c>
     </row>
@@ -2326,57 +2326,57 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.64 / 5.23%</t>
+          <t>$47.56 / 5.06%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.36 / 13.16%</t>
+          <t>$57.38 / 13.21%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.57 / 8.94%</t>
+          <t>$55.50 / 8.81%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.20 / 7.40%</t>
+          <t>$62.15 / 7.31%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.25 / 7.62%</t>
+          <t>$56.21 / 7.54%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.23 / 2.31%</t>
+          <t>$61.10 / 2.09%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.24 / 2.29%</t>
+          <t>$61.11 / 2.07%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.15 / 10.01%</t>
+          <t>$53.12 / 9.93%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.44 / 3.38%</t>
+          <t>$57.32 / 3.15%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.60 / 11.94%</t>
+          <t>$59.57 / 11.88%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.36 / 11.47%</t>
+          <t>$53.35 / 11.44%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2386,17 +2386,17 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.34 / 4.17%</t>
+          <t>$42.31 / 4.10%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.91 / 10.84%</t>
+          <t>$41.89 / 10.79%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.46 / 7.36%</t>
+          <t>$40.44 / 7.30%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2406,32 +2406,32 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.76 / 6.28%</t>
+          <t>$45.73 / 6.22%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.47 / 1.89%</t>
+          <t>$44.41 / 1.74%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.92 / 1.87%</t>
+          <t>$41.84 / 1.67%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.85 / 7.98%</t>
+          <t>$44.84 / 7.96%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.88 / 2.91%</t>
+          <t>$43.81 / 2.73%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.44 / 9.59%</t>
+          <t>$42.43 / 9.57%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.59 / 9.51%</t>
+          <t>$41.60 / 9.54%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$772.02 / 8.71%</t>
+          <t>$768.48 / 8.22%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$772.02 / 19.98%</t>
+          <t>$768.48 / 19.43%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$772.02 / 13.43%</t>
+          <t>$768.48 / 12.91%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$772.02 / 11.98%</t>
+          <t>$768.48 / 11.47%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$772.02 / 11.62%</t>
+          <t>$768.48 / 11.11%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$772.02 / 3.87%</t>
+          <t>$768.48 / 3.39%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$772.02 / 3.39%</t>
+          <t>$768.48 / 2.91%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$772.02 / 19.03%</t>
+          <t>$768.48 / 18.49%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$772.02 / 4.44%</t>
+          <t>$768.48 / 3.97%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$772.02 / 17.14%</t>
+          <t>$768.48 / 16.61%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$772.02 / 16.20%</t>
+          <t>$768.48 / 15.67%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$772.02 / 16.32%</t>
+          <t>$768.48 / 15.79%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$772.02 / 8.71%</t>
+          <t>$768.48 / 8.22%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$772.02 / 19.98%</t>
+          <t>$768.48 / 19.43%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$772.02 / 13.43%</t>
+          <t>$768.48 / 12.91%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$772.02 / 11.98%</t>
+          <t>$768.48 / 11.47%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$772.02 / 11.62%</t>
+          <t>$768.48 / 11.11%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$772.02 / 3.87%</t>
+          <t>$768.48 / 3.39%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$772.02 / 3.39%</t>
+          <t>$768.48 / 2.91%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$772.02 / 19.03%</t>
+          <t>$768.48 / 18.49%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$772.02 / 4.44%</t>
+          <t>$768.48 / 3.97%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$772.02 / 17.14%</t>
+          <t>$768.48 / 16.61%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$772.02 / 16.20%</t>
+          <t>$768.48 / 15.67%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$772.02 / 16.32%</t>
+          <t>$768.48 / 15.79%</t>
         </is>
       </c>
     </row>
@@ -2580,57 +2580,57 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.19% (8.63%)</t>
+          <t>9.36% (8.80%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.27% (0.24%)</t>
+          <t>0.23% (0.19%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.85% (4.56%)</t>
+          <t>4.97% (4.68%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.72% (6.30%)</t>
+          <t>6.82% (6.39%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.99% (5.63%)</t>
+          <t>6.06% (5.71%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.14% (13.36%)</t>
+          <t>14.38% (13.60%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.74% (13.02%)</t>
+          <t>13.98% (13.26%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.22% (5.74%)</t>
+          <t>6.29% (5.81%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.08% (12.43%)</t>
+          <t>13.32% (12.67%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.65% (3.43%)</t>
+          <t>3.70% (3.48%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.64% (2.49%)</t>
+          <t>2.66% (2.52%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2640,17 +2640,17 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.59% (7.03%)</t>
+          <t>7.67% (7.10%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.20% (0.17%)</t>
+          <t>0.25% (0.22%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.91% (3.61%)</t>
+          <t>3.96% (3.67%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2660,42 +2660,42 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.76% (4.41%)</t>
+          <t>4.82% (4.46%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.67% (10.88%)</t>
+          <t>11.83% (11.04%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.16% (10.44%)</t>
+          <t>11.38% (10.66%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.37% (4.88%)</t>
+          <t>5.39% (4.91%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.43% (9.77%)</t>
+          <t>10.61% (9.96%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.79% (2.57%)</t>
+          <t>2.82% (2.59%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.93% (1.77%)</t>
+          <t>1.92% (1.77%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>1.12% (1.02%)</t>
+          <t>1.09% (1.00%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.93%</t>
+          <t>6.42%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-4.74%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.16%</t>
+          <t>1.63%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.71%</t>
+          <t>3.18%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.47%</t>
+          <t>12.99%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.64%</t>
+          <t>13.16%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.57%</t>
+          <t>-1.11%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.45%</t>
+          <t>0.01%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.95%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-1.99%</t>
+          <t>-1.54%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.34%</t>
+          <t>3.81%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-6.74%</t>
+          <t>-6.31%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.19%</t>
+          <t>-0.74%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>10.15%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.14%</t>
+          <t>-3.70%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.99%</t>
+          <t>9.49%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.32%</t>
+          <t>-2.88%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.49%</t>
+          <t>-3.05%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-4.16%</t>
+          <t>-3.72%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12.00% (11.44%)</t>
+          <t>11.77% (11.20%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.63% (12.60%)</t>
+          <t>12.25% (12.21%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.97% (11.68%)</t>
+          <t>11.71% (11.42%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.38% (11.95%)</t>
+          <t>12.09% (11.66%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.85% (11.50%)</t>
+          <t>11.54% (11.19%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.05% (10.27%)</t>
+          <t>10.86% (10.07%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.60% (9.88%)</t>
+          <t>10.41% (9.69%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>15.00% (14.52%)</t>
+          <t>14.71% (14.24%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.38% (9.73%)</t>
+          <t>10.19% (9.54%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.97% (11.75%)</t>
+          <t>11.66% (11.44%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.65% (11.50%)</t>
+          <t>11.31% (11.16%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.64% (11.55%)</t>
+          <t>11.28% (11.19%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.56% (16.99%)</t>
+          <t>17.27% (16.70%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.63% (18.60%)</t>
+          <t>18.34% (18.31%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.72% (17.43%)</t>
+          <t>17.42% (17.13%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.19% (17.76%)</t>
+          <t>17.84% (17.41%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.50% (17.14%)</t>
+          <t>17.19% (16.84%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.27% (15.48%)</t>
+          <t>16.03% (15.24%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.83% (15.11%)</t>
+          <t>15.65% (14.93%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.90% (20.42%)</t>
+          <t>20.59% (20.11%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.60% (14.95%)</t>
+          <t>15.39% (14.74%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>18.14% (17.91%)</t>
+          <t>17.83% (17.60%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.67% (17.52%)</t>
+          <t>17.33% (17.18%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.56% (17.46%)</t>
+          <t>17.20% (17.11%)</t>
         </is>
       </c>
     </row>
@@ -2961,57 +2961,57 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.21% (-5.78%)</t>
+          <t>-5.07% (-5.63%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.36% (-12.39%)</t>
+          <t>-12.40% (-12.43%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.69% (-8.98%)</t>
+          <t>-8.59% (-8.87%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.25% (-7.68%)</t>
+          <t>-7.17% (-7.60%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.52% (-7.87%)</t>
+          <t>-7.45% (-7.80%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.30% (-3.08%)</t>
+          <t>-2.09% (-2.88%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.34% (-3.06%)</t>
+          <t>-2.14% (-2.86%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.39% (-9.87%)</t>
+          <t>-9.33% (-9.81%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.45% (-4.10%)</t>
+          <t>-3.24% (-3.89%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.20% (-11.42%)</t>
+          <t>-11.16% (-11.38%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-10.90% (-11.05%)</t>
+          <t>-10.88% (-11.03%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -3021,17 +3021,17 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.25% (-4.82%)</t>
+          <t>-4.18% (-4.75%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.52% (-10.56%)</t>
+          <t>-10.48% (-10.52%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.35% (-7.64%)</t>
+          <t>-7.30% (-7.59%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -3041,32 +3041,32 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.35% (-6.71%)</t>
+          <t>-6.30% (-6.66%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.89% (-2.68%)</t>
+          <t>-1.75% (-2.54%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.95% (-2.67%)</t>
+          <t>-1.75% (-2.47%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.69% (-8.17%)</t>
+          <t>-7.67% (-8.15%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.01% (-3.67%)</t>
+          <t>-2.85% (-3.50%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.30% (-9.52%)</t>
+          <t>-9.28% (-9.50%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.37% (-9.46%)</t>
+          <t>-9.39% (-9.48%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.21%</t>
+          <t>-16.83%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-24.99%</t>
+          <t>-24.64%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.66%</t>
+          <t>-20.29%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.63%</t>
+          <t>-19.26%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.37%</t>
+          <t>-19.00%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.35%</t>
+          <t>-12.95%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.95%</t>
+          <t>-12.55%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.39%</t>
+          <t>-24.04%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.83%</t>
+          <t>-13.43%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.17%</t>
+          <t>-22.82%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.55%</t>
+          <t>-22.19%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.63%</t>
+          <t>-22.27%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.81%</t>
+          <t>-21.45%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-29.15%</t>
+          <t>-28.83%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.06%</t>
+          <t>-24.72%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.09%</t>
+          <t>-23.74%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.85%</t>
+          <t>-23.49%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.16%</t>
+          <t>-17.78%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.78%</t>
+          <t>-17.40%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.59%</t>
+          <t>-28.26%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.61%</t>
+          <t>-18.24%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.44%</t>
+          <t>-27.10%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.85%</t>
+          <t>-26.51%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-26.92%</t>
+          <t>-26.59%</t>
         </is>
       </c>
     </row>
@@ -3215,57 +3215,57 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3.07% (2.51%)</t>
+          <t>2.75% (2.19%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.27% (0.24%)</t>
+          <t>0.23% (0.19%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.64% (3.35%)</t>
+          <t>3.28% (2.99%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.90% (3.47%)</t>
+          <t>3.52% (3.09%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3.28% (2.93%)</t>
+          <t>2.88% (2.52%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.48% (0.70%)</t>
+          <t>1.23% (0.44%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.97% (0.25%)</t>
+          <t>0.71% (0.00%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.22% (5.74%)</t>
+          <t>6.29% (5.81%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.85% (0.20%)</t>
+          <t>0.60% (-0.05%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.65% (3.43%)</t>
+          <t>3.69% (3.47%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.64% (2.49%)</t>
+          <t>2.66% (2.52%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3275,62 +3275,62 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>4.11% (3.54%)</t>
+          <t>3.70% (3.14%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.20% (0.17%)</t>
+          <t>0.25% (0.22%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.91% (3.61%)</t>
+          <t>3.96% (3.67%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.41% (4.98%)</t>
+          <t>4.93% (4.49%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.58% (4.22%)</t>
+          <t>4.15% (3.80%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.90% (1.11%)</t>
+          <t>1.58% (0.79%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.37% (0.65%)</t>
+          <t>1.11% (0.39%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.37% (4.88%)</t>
+          <t>5.39% (4.91%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.30% (0.65%)</t>
+          <t>1.01% (0.36%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.79% (2.57%)</t>
+          <t>2.82% (2.59%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.93% (1.77%)</t>
+          <t>1.92% (1.77%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>1.12% (1.02%)</t>
+          <t>1.09% (1.00%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 5/8/2026</t>
+          <t>As of 6/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.50%</t>
+          <t>11.19%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.63%</t>
+          <t>5.71%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.62%</t>
+          <t>7.54%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>11.11%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.87%</t>
+          <t>-7.80%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.95%</t>
+          <t>11.66%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.30%</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.40%</t>
+          <t>7.31%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.98%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.71%</t>
+          <t>3.18%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.68%</t>
+          <t>-7.60%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.52%</t>
+          <t>14.24%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.74%</t>
+          <t>5.81%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.01%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.03%</t>
+          <t>18.49%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.57%</t>
+          <t>-1.11%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.87%</t>
+          <t>-9.81%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.44%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.63%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.23%</t>
+          <t>5.06%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.71%</t>
+          <t>8.22%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.93%</t>
+          <t>6.42%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.78%</t>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.43%</t>
+          <t>12.67%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.44%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.10%</t>
+          <t>-3.89%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.88%</t>
+          <t>9.69%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.02%</t>
+          <t>13.26%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.29%</t>
+          <t>2.07%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.64%</t>
+          <t>13.16%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.06%</t>
+          <t>-2.86%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.27%</t>
+          <t>10.07%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.36%</t>
+          <t>13.60%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.31%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.87%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.47%</t>
+          <t>12.99%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.08%</t>
+          <t>-2.88%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>12.21%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.19%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.16%</t>
+          <t>13.21%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>19.98%</t>
+          <t>19.43%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.74%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.39%</t>
+          <t>-12.43%</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>11.19%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3721,12 +3721,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.32%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.99%</t>
+          <t>-1.54%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.50%</t>
+          <t>11.16%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.49%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>11.44%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.20%</t>
+          <t>15.67%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.95%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.05%</t>
+          <t>-11.03%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.75%</t>
+          <t>11.44%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.43%</t>
+          <t>3.48%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.94%</t>
+          <t>11.88%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.14%</t>
+          <t>16.61%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.45%</t>
+          <t>0.01%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.42%</t>
+          <t>-11.38%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.68%</t>
+          <t>11.42%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>8.81%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.43%</t>
+          <t>12.91%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.16%</t>
+          <t>1.63%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.98%</t>
+          <t>-8.87%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 5/8/2026</t>
+          <t>As of 6/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17.14%</t>
+          <t>16.84%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.41%</t>
+          <t>4.46%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.22%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>11.11%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.71%</t>
+          <t>-6.66%</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.76%</t>
+          <t>17.41%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3977,12 +3977,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.98%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.42%</t>
+          <t>20.11%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.88%</t>
+          <t>4.91%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.98%</t>
+          <t>7.96%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.03%</t>
+          <t>18.49%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.14%</t>
+          <t>-3.70%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.17%</t>
+          <t>-8.15%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.70%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.03%</t>
+          <t>7.10%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.17%</t>
+          <t>4.10%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.71%</t>
+          <t>8.22%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.34%</t>
+          <t>3.81%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.82%</t>
+          <t>-4.75%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.95%</t>
+          <t>14.74%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>2.73%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.44%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.99%</t>
+          <t>9.49%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.67%</t>
+          <t>-3.50%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.11%</t>
+          <t>14.93%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.44%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>1.67%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>10.15%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.67%</t>
+          <t>-2.47%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.48%</t>
+          <t>15.24%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>11.04%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>1.74%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.87%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.68%</t>
+          <t>-2.54%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.60%</t>
+          <t>18.31%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>0.22%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.84%</t>
+          <t>10.79%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>19.98%</t>
+          <t>19.43%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-6.74%</t>
+          <t>-6.31%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.56%</t>
+          <t>-10.52%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.46%</t>
+          <t>17.11%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.02%</t>
+          <t>1.00%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.51%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.32%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-4.16%</t>
+          <t>-3.72%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.46%</t>
+          <t>-9.48%</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.52%</t>
+          <t>17.18%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.20%</t>
+          <t>15.67%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.49%</t>
+          <t>-3.05%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.91%</t>
+          <t>17.60%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.57%</t>
+          <t>2.59%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>9.57%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.14%</t>
+          <t>16.61%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.32%</t>
+          <t>-2.88%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.52%</t>
+          <t>-9.50%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.43%</t>
+          <t>17.13%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.61%</t>
+          <t>3.67%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.36%</t>
+          <t>7.30%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.43%</t>
+          <t>12.91%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.19%</t>
+          <t>-0.74%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.64%</t>
+          <t>-7.59%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-07]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/6/2026 at 11:46 AM ET)</t>
+          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>253 days</t>
+          <t>252 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>15 days</t>
+          <t>14 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>134 days</t>
+          <t>133 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>197 days</t>
+          <t>196 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>162 days</t>
+          <t>161 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>344 days</t>
+          <t>343 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>315 days</t>
+          <t>314 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>225 days</t>
+          <t>224 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>288 days</t>
+          <t>287 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>106 days</t>
+          <t>105 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>71 days</t>
+          <t>70 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>43 days</t>
+          <t>42 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>253 days</t>
+          <t>252 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>15 days</t>
+          <t>14 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>134 days</t>
+          <t>133 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>197 days</t>
+          <t>196 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>162 days</t>
+          <t>161 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>344 days</t>
+          <t>343 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>315 days</t>
+          <t>314 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>225 days</t>
+          <t>224 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>288 days</t>
+          <t>287 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>106 days</t>
+          <t>105 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>71 days</t>
+          <t>70 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>43 days</t>
+          <t>42 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.56 / 5.06%</t>
+          <t>$47.68 / 5.33%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.38 / 13.21%</t>
+          <t>$57.43 / 13.30%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.50 / 8.81%</t>
+          <t>$55.64 / 9.07%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.15 / 7.31%</t>
+          <t>$62.25 / 7.48%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.21 / 7.54%</t>
+          <t>$56.31 / 7.73%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.10 / 2.09%</t>
+          <t>$61.28 / 2.40%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.11 / 2.07%</t>
+          <t>$61.25 / 2.30%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.12 / 9.93%</t>
+          <t>$53.19 / 10.09%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.32 / 3.15%</t>
+          <t>$57.49 / 3.47%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.57 / 11.88%</t>
+          <t>$59.64 / 12.01%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.35 / 11.44%</t>
+          <t>$53.44 / 11.64%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.21 / 11.51%</t>
+          <t>$56.32 / 11.73%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.31 / 4.10%</t>
+          <t>$42.37 / 4.24%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.89 / 10.79%</t>
+          <t>$41.92 / 10.86%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.44 / 7.30%</t>
+          <t>$40.50 / 7.45%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.70 / 5.86%</t>
+          <t>$44.73 / 5.93%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.73 / 6.22%</t>
+          <t>$45.80 / 6.39%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.41 / 1.74%</t>
+          <t>$44.50 / 1.96%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.84 / 1.67%</t>
+          <t>$41.93 / 1.89%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.84 / 7.96%</t>
+          <t>$44.89 / 8.08%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.81 / 2.73%</t>
+          <t>$43.90 / 2.96%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.43 / 9.57%</t>
+          <t>$42.47 / 9.67%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.18 / 9.36%</t>
+          <t>$42.22 / 9.47%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.60 / 9.54%</t>
+          <t>$41.64 / 9.63%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$768.48 / 8.22%</t>
+          <t>$772.76 / 8.82%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$768.48 / 19.43%</t>
+          <t>$772.76 / 20.10%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$768.48 / 12.91%</t>
+          <t>$772.76 / 13.54%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$768.48 / 11.47%</t>
+          <t>$772.76 / 12.09%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$768.48 / 11.11%</t>
+          <t>$772.76 / 11.73%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$768.48 / 3.39%</t>
+          <t>$772.76 / 3.96%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$768.48 / 2.91%</t>
+          <t>$772.76 / 3.48%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$768.48 / 18.49%</t>
+          <t>$772.76 / 19.15%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$768.48 / 3.97%</t>
+          <t>$772.76 / 4.54%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$768.48 / 16.61%</t>
+          <t>$772.76 / 17.26%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$768.48 / 15.67%</t>
+          <t>$772.76 / 16.31%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$768.48 / 15.79%</t>
+          <t>$772.76 / 16.43%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$768.48 / 8.22%</t>
+          <t>$772.76 / 8.82%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$768.48 / 19.43%</t>
+          <t>$772.96 / 20.13%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$768.48 / 12.91%</t>
+          <t>$772.96 / 13.57%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$768.48 / 11.47%</t>
+          <t>$772.76 / 12.09%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$768.48 / 11.11%</t>
+          <t>$772.76 / 11.73%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$768.48 / 3.39%</t>
+          <t>$772.76 / 3.96%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$768.48 / 2.91%</t>
+          <t>$772.76 / 3.48%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$768.48 / 18.49%</t>
+          <t>$772.76 / 19.15%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$768.48 / 3.97%</t>
+          <t>$772.76 / 4.54%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$768.48 / 16.61%</t>
+          <t>$772.96 / 17.29%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$768.48 / 15.67%</t>
+          <t>$772.96 / 16.34%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$768.48 / 15.79%</t>
+          <t>$772.96 / 16.46%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.36% (8.80%)</t>
+          <t>9.09% (8.53%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.23% (0.19%)</t>
+          <t>0.14% (0.12%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.97% (4.68%)</t>
+          <t>4.71% (4.43%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.82% (6.39%)</t>
+          <t>6.64% (6.22%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>6.06% (5.71%)</t>
+          <t>5.88% (5.53%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.38% (13.60%)</t>
+          <t>14.04% (13.26%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.98% (13.26%)</t>
+          <t>13.72% (13.00%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.29% (5.81%)</t>
+          <t>6.13% (5.66%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.32% (12.67%)</t>
+          <t>12.98% (12.33%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.70% (3.48%)</t>
+          <t>3.58% (3.36%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.66% (2.52%)</t>
+          <t>2.48% (2.33%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>1.56% (1.47%)</t>
+          <t>1.36% (1.27%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.67% (7.10%)</t>
+          <t>7.53% (6.96%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.25% (0.22%)</t>
+          <t>0.19% (0.16%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.96% (3.67%)</t>
+          <t>3.81% (3.52%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.48% (5.05%)</t>
+          <t>5.41% (4.98%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.82% (4.46%)</t>
+          <t>4.66% (4.30%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.83% (11.04%)</t>
+          <t>11.59% (10.81%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.38% (10.66%)</t>
+          <t>11.14% (10.42%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.39% (4.91%)</t>
+          <t>5.27% (4.79%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.61% (9.96%)</t>
+          <t>10.37% (9.72%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.82% (2.59%)</t>
+          <t>2.72% (2.49%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.92% (1.77%)</t>
+          <t>1.81% (1.66%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>1.09% (1.00%)</t>
+          <t>1.00% (0.91%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.42%</t>
+          <t>5.83%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-4.84%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.18%</t>
+          <t>2.61%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.99%</t>
+          <t>12.36%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.16%</t>
+          <t>12.53%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.11%</t>
+          <t>-1.66%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>12.00%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.01%</t>
+          <t>-0.54%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>-1.05%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-1.54%</t>
+          <t>-2.09%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.81%</t>
+          <t>3.24%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-6.31%</t>
+          <t>-6.86%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.74%</t>
+          <t>-1.31%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>9.48%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.15%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.70%</t>
+          <t>-4.23%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.49%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-3.44%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.05%</t>
+          <t>-3.61%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-3.72%</t>
+          <t>-4.28%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.77% (11.20%)</t>
+          <t>11.99% (11.43%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.25% (12.21%)</t>
+          <t>12.59% (12.56%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.71% (11.42%)</t>
+          <t>11.92% (11.64%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.09% (11.66%)</t>
+          <t>12.38% (11.96%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.54% (11.19%)</t>
+          <t>11.84% (11.49%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.86% (10.07%)</t>
+          <t>11.04% (10.26%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.41% (9.69%)</t>
+          <t>10.67% (9.95%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.71% (14.24%)</t>
+          <t>15.00% (14.53%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.19% (9.54%)</t>
+          <t>10.37% (9.73%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.66% (11.44%)</t>
+          <t>11.98% (11.76%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.31% (11.16%)</t>
+          <t>11.58% (11.44%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.28% (11.19%)</t>
+          <t>11.53% (11.45%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.27% (16.70%)</t>
+          <t>17.57% (17.01%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.34% (18.31%)</t>
+          <t>18.70% (18.67%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.42% (17.13%)</t>
+          <t>17.72% (17.44%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.84% (17.41%)</t>
+          <t>18.20% (17.77%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.19% (16.84%)</t>
+          <t>17.47% (17.12%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.03% (15.24%)</t>
+          <t>16.28% (15.49%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.65% (14.93%)</t>
+          <t>15.90% (15.18%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.59% (20.11%)</t>
+          <t>20.88% (20.40%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.39% (14.74%)</t>
+          <t>15.63% (14.98%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.83% (17.60%)</t>
+          <t>18.16% (17.94%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.33% (17.18%)</t>
+          <t>17.66% (17.51%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.20% (17.11%)</t>
+          <t>17.54% (17.45%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.07% (-5.63%)</t>
+          <t>-5.31% (-5.86%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.40% (-12.43%)</t>
+          <t>-12.47% (-12.50%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.59% (-8.87%)</t>
+          <t>-8.81% (-9.09%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.17% (-7.60%)</t>
+          <t>-7.32% (-7.75%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.45% (-7.80%)</t>
+          <t>-7.61% (-7.96%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.09% (-2.88%)</t>
+          <t>-2.39% (-3.17%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.14% (-2.86%)</t>
+          <t>-2.36% (-3.08%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.33% (-9.81%)</t>
+          <t>-9.46% (-9.94%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.24% (-3.89%)</t>
+          <t>-3.54% (-4.19%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.16% (-11.38%)</t>
+          <t>-11.26% (-11.48%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-10.88% (-11.03%)</t>
+          <t>-11.04% (-11.18%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-10.99% (-11.08%)</t>
+          <t>-11.17% (-11.26%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.18% (-4.75%)</t>
+          <t>-4.31% (-4.87%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.48% (-10.52%)</t>
+          <t>-10.54% (-10.57%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.30% (-7.59%)</t>
+          <t>-7.43% (-7.72%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-5.90% (-6.33%)</t>
+          <t>-5.97% (-6.40%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.30% (-6.66%)</t>
+          <t>-6.45% (-6.80%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.75% (-2.54%)</t>
+          <t>-1.96% (-2.75%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.75% (-2.47%)</t>
+          <t>-1.96% (-2.68%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.67% (-8.15%)</t>
+          <t>-7.77% (-8.26%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.85% (-3.50%)</t>
+          <t>-3.06% (-3.71%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.28% (-9.50%)</t>
+          <t>-9.36% (-9.59%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.18% (-9.33%)</t>
+          <t>-9.28% (-9.43%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.39% (-9.48%)</t>
+          <t>-9.47% (-9.56%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.83%</t>
+          <t>-17.29%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-24.64%</t>
+          <t>-25.06%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.29%</t>
+          <t>-20.73%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.26%</t>
+          <t>-19.70%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.00%</t>
+          <t>-19.45%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.95%</t>
+          <t>-13.43%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.55%</t>
+          <t>-13.03%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.04%</t>
+          <t>-24.46%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.43%</t>
+          <t>-13.91%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.82%</t>
+          <t>-23.25%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.19%</t>
+          <t>-22.62%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.27%</t>
+          <t>-22.70%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.45%</t>
+          <t>-21.89%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-28.83%</t>
+          <t>-29.24%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.72%</t>
+          <t>-25.16%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.74%</t>
+          <t>-24.16%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.49%</t>
+          <t>-23.92%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.78%</t>
+          <t>-18.24%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.40%</t>
+          <t>-17.86%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.26%</t>
+          <t>-28.66%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.24%</t>
+          <t>-18.69%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.10%</t>
+          <t>-27.53%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.51%</t>
+          <t>-26.94%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-26.59%</t>
+          <t>-27.01%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.75% (2.19%)</t>
+          <t>3.06% (2.51%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.23% (0.19%)</t>
+          <t>0.14% (0.12%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.28% (2.99%)</t>
+          <t>3.61% (3.32%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.52% (3.09%)</t>
+          <t>3.92% (3.50%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.88% (2.52%)</t>
+          <t>3.27% (2.93%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.23% (0.44%)</t>
+          <t>1.48% (0.70%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.71% (0.00%)</t>
+          <t>1.04% (0.33%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.29% (5.81%)</t>
+          <t>6.13% (5.66%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.60% (-0.05%)</t>
+          <t>0.85% (0.21%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.69% (3.47%)</t>
+          <t>3.58% (3.36%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.66% (2.52%)</t>
+          <t>2.48% (2.33%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.56% (1.47%)</t>
+          <t>1.36% (1.27%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.70% (3.14%)</t>
+          <t>4.15% (3.58%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.25% (0.22%)</t>
+          <t>0.19% (0.16%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.96% (3.67%)</t>
+          <t>3.81% (3.52%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.93% (4.49%)</t>
+          <t>5.41% (4.98%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.15% (3.80%)</t>
+          <t>4.57% (4.22%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.58% (0.79%)</t>
+          <t>1.92% (1.14%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.11% (0.39%)</t>
+          <t>1.45% (0.74%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.39% (4.91%)</t>
+          <t>5.27% (4.79%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.01% (0.36%)</t>
+          <t>1.35% (0.70%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.82% (2.59%)</t>
+          <t>2.72% (2.49%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.92% (1.77%)</t>
+          <t>1.81% (1.66%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>1.09% (1.00%)</t>
+          <t>1.00% (0.91%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 6/8/2026</t>
+          <t>As of 7/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.19%</t>
+          <t>11.49%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.71%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.54%</t>
+          <t>7.73%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.11%</t>
+          <t>11.73%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.80%</t>
+          <t>-7.96%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.66%</t>
+          <t>11.96%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.22%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.31%</t>
+          <t>7.48%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>12.09%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.18%</t>
+          <t>2.61%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.60%</t>
+          <t>-7.75%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.24%</t>
+          <t>14.53%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.81%</t>
+          <t>5.66%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.49%</t>
+          <t>19.15%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.11%</t>
+          <t>-1.66%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.81%</t>
+          <t>-9.94%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.20%</t>
+          <t>11.43%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>8.53%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.06%</t>
+          <t>5.33%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.22%</t>
+          <t>8.82%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.42%</t>
+          <t>5.83%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.86%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.67%</t>
+          <t>12.33%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>4.54%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>12.00%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.89%</t>
+          <t>-4.19%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.26%</t>
+          <t>13.00%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.07%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>3.48%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.16%</t>
+          <t>12.53%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.86%</t>
+          <t>-3.08%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.07%</t>
+          <t>10.26%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.60%</t>
+          <t>13.26%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>3.96%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.99%</t>
+          <t>12.36%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-3.17%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.21%</t>
+          <t>12.56%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.19%</t>
+          <t>0.12%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.21%</t>
+          <t>13.30%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>19.43%</t>
+          <t>20.10%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-4.84%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.43%</t>
+          <t>-12.50%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.19%</t>
+          <t>11.45%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.47%</t>
+          <t>1.27%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.51%</t>
+          <t>11.73%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>16.43%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.54%</t>
+          <t>-2.09%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.08%</t>
+          <t>-11.26%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.16%</t>
+          <t>11.44%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>2.33%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.44%</t>
+          <t>11.64%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.67%</t>
+          <t>16.31%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>-1.05%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.03%</t>
+          <t>-11.18%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.44%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.48%</t>
+          <t>3.36%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.88%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.61%</t>
+          <t>17.26%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.01%</t>
+          <t>-0.54%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.38%</t>
+          <t>-11.48%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.42%</t>
+          <t>11.64%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.43%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.81%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>13.54%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.87%</t>
+          <t>-9.09%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 6/8/2026</t>
+          <t>As of 7/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.84%</t>
+          <t>17.12%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.46%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.22%</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.11%</t>
+          <t>11.73%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.66%</t>
+          <t>-6.80%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.41%</t>
+          <t>17.77%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.05%</t>
+          <t>4.98%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.86%</t>
+          <t>5.93%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>12.09%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.33%</t>
+          <t>-6.40%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.11%</t>
+          <t>20.40%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.91%</t>
+          <t>4.79%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.96%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.49%</t>
+          <t>19.15%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.70%</t>
+          <t>-4.23%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.15%</t>
+          <t>-8.26%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.70%</t>
+          <t>17.01%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.10%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.10%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.22%</t>
+          <t>8.82%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.81%</t>
+          <t>3.24%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.75%</t>
+          <t>-4.87%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.74%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>9.72%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.73%</t>
+          <t>2.96%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>4.54%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.49%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-3.71%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.93%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.67%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>3.48%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.15%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.47%</t>
+          <t>-2.68%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.24%</t>
+          <t>15.49%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.04%</t>
+          <t>10.81%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.74%</t>
+          <t>1.96%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>3.96%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>9.48%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.54%</t>
+          <t>-2.75%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.31%</t>
+          <t>18.67%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.79%</t>
+          <t>10.86%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>19.43%</t>
+          <t>20.13%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-6.31%</t>
+          <t>-6.86%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.52%</t>
+          <t>-10.57%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.11%</t>
+          <t>17.45%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.00%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>16.46%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-3.72%</t>
+          <t>-4.28%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.48%</t>
+          <t>-9.56%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.18%</t>
+          <t>17.51%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.77%</t>
+          <t>1.66%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.36%</t>
+          <t>9.47%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.67%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.05%</t>
+          <t>-3.61%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.33%</t>
+          <t>-9.43%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.60%</t>
+          <t>17.94%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.59%</t>
+          <t>2.49%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.57%</t>
+          <t>9.67%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.61%</t>
+          <t>17.29%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-3.44%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.50%</t>
+          <t>-9.59%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.13%</t>
+          <t>17.44%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.67%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.30%</t>
+          <t>7.45%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>13.57%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.74%</t>
+          <t>-1.31%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.59%</t>
+          <t>-7.72%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-10]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/7/2026 at 10:29 AM ET)</t>
+          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>252 days</t>
+          <t>249 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14 days</t>
+          <t>11 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>133 days</t>
+          <t>130 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>196 days</t>
+          <t>193 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>161 days</t>
+          <t>158 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>343 days</t>
+          <t>340 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>314 days</t>
+          <t>311 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>224 days</t>
+          <t>221 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>287 days</t>
+          <t>284 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>105 days</t>
+          <t>102 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>70 days</t>
+          <t>67 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>42 days</t>
+          <t>39 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>252 days</t>
+          <t>249 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>14 days</t>
+          <t>11 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>133 days</t>
+          <t>130 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>196 days</t>
+          <t>193 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>161 days</t>
+          <t>158 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>343 days</t>
+          <t>340 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>314 days</t>
+          <t>311 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>224 days</t>
+          <t>221 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>287 days</t>
+          <t>284 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>105 days</t>
+          <t>102 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>70 days</t>
+          <t>67 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>42 days</t>
+          <t>39 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.68 / 5.33%</t>
+          <t>$47.73 / 5.43%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.43 / 13.30%</t>
+          <t>$57.45 / 13.34%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.64 / 9.07%</t>
+          <t>$55.65 / 9.10%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.25 / 7.48%</t>
+          <t>$62.31 / 7.58%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.31 / 7.73%</t>
+          <t>$56.36 / 7.82%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.28 / 2.40%</t>
+          <t>$61.35 / 2.51%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.25 / 2.30%</t>
+          <t>$61.35 / 2.47%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.19 / 10.09%</t>
+          <t>$53.24 / 10.18%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.49 / 3.47%</t>
+          <t>$57.58 / 3.62%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.64 / 12.01%</t>
+          <t>$59.72 / 12.15%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.44 / 11.64%</t>
+          <t>$53.50 / 11.76%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.32 / 11.73%</t>
+          <t>$56.36 / 11.81%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.37 / 4.24%</t>
+          <t>$42.41 / 4.35%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.92 / 10.86%</t>
+          <t>$41.93 / 10.89%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.50 / 7.45%</t>
+          <t>$40.53 / 7.53%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.73 / 5.93%</t>
+          <t>$44.76 / 6.00%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.80 / 6.39%</t>
+          <t>$45.85 / 6.50%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.50 / 1.96%</t>
+          <t>$44.56 / 2.09%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.93 / 1.89%</t>
+          <t>$41.98 / 2.02%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.89 / 8.08%</t>
+          <t>$44.90 / 8.12%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.90 / 2.96%</t>
+          <t>$43.94 / 3.05%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.47 / 9.67%</t>
+          <t>$42.51 / 9.79%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.22 / 9.47%</t>
+          <t>$42.25 / 9.55%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.64 / 9.63%</t>
+          <t>$41.68 / 9.75%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$772.76 / 8.82%</t>
+          <t>$774.58 / 9.07%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$772.76 / 20.10%</t>
+          <t>$774.55 / 20.38%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$772.76 / 13.54%</t>
+          <t>$774.55 / 13.80%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$772.76 / 12.09%</t>
+          <t>$774.58 / 12.35%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$772.76 / 11.73%</t>
+          <t>$774.58 / 11.99%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$772.76 / 3.96%</t>
+          <t>$774.55 / 4.20%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$772.76 / 3.48%</t>
+          <t>$774.58 / 3.73%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$772.76 / 19.15%</t>
+          <t>$774.58 / 19.43%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$772.76 / 4.54%</t>
+          <t>$774.58 / 4.79%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$772.76 / 17.26%</t>
+          <t>$774.55 / 17.53%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$772.76 / 16.31%</t>
+          <t>$774.55 / 16.58%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$772.76 / 16.43%</t>
+          <t>$774.55 / 16.70%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$772.76 / 8.82%</t>
+          <t>$774.55 / 9.07%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$772.96 / 20.13%</t>
+          <t>$774.55 / 20.38%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$772.96 / 13.57%</t>
+          <t>$774.55 / 13.80%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$772.76 / 12.09%</t>
+          <t>$774.55 / 12.35%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$772.76 / 11.73%</t>
+          <t>$774.55 / 11.98%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$772.76 / 3.96%</t>
+          <t>$774.55 / 4.20%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$772.76 / 3.48%</t>
+          <t>$774.55 / 3.72%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$772.76 / 19.15%</t>
+          <t>$774.55 / 19.42%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$772.76 / 4.54%</t>
+          <t>$774.55 / 4.79%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$772.96 / 17.29%</t>
+          <t>$774.55 / 17.53%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$772.96 / 16.34%</t>
+          <t>$774.55 / 16.58%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$772.96 / 16.46%</t>
+          <t>$774.55 / 16.70%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.09% (8.53%)</t>
+          <t>8.98% (8.43%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>0.09% (0.07%)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4.68% (4.40%)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>6.53% (6.12%)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>5.78% (5.44%)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>13.90% (13.13%)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>13.52% (12.82%)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>6.04% (5.57%)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>12.80% (12.17%)</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>3.44% (3.23%)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2.36% (2.22%)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>1.28% (1.20%)</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>7.41% (6.85%)</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
           <t>0.14% (0.12%)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>4.71% (4.43%)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>6.64% (6.22%)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>5.88% (5.53%)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>14.04% (13.26%)</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>13.72% (13.00%)</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>6.13% (5.66%)</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>12.98% (12.33%)</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>3.58% (3.36%)</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>2.48% (2.33%)</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>1.36% (1.27%)</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>7.53% (6.96%)</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>0.19% (0.16%)</t>
-        </is>
-      </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.81% (3.52%)</t>
+          <t>3.73% (3.45%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.41% (4.98%)</t>
+          <t>5.33% (4.91%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.66% (4.30%)</t>
+          <t>4.54% (4.19%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.59% (10.81%)</t>
+          <t>11.43% (10.66%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.14% (10.42%)</t>
+          <t>10.99% (10.28%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.27% (4.79%)</t>
+          <t>5.23% (4.75%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.37% (9.72%)</t>
+          <t>10.27% (9.62%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.72% (2.49%)</t>
+          <t>2.60% (2.39%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.81% (1.66%)</t>
+          <t>1.73% (1.59%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>1.00% (0.91%)</t>
+          <t>0.89% (0.80%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.83%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-4.84%</t>
+          <t>-5.06%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>2.37%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.36%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.53%</t>
+          <t>12.27%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.66%</t>
+          <t>-1.89%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.00%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.54%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.05%</t>
+          <t>-1.28%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-2.09%</t>
+          <t>-2.31%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.24%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-6.86%</t>
+          <t>-7.05%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-1.51%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.26%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>-0.15%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.48%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.23%</t>
+          <t>-4.45%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.44%</t>
+          <t>-3.64%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.61%</t>
+          <t>-3.81%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-4.28%</t>
+          <t>-4.47%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.99% (11.43%)</t>
+          <t>12.08% (11.53%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.59% (12.56%)</t>
+          <t>12.72% (12.70%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.92% (11.64%)</t>
+          <t>12.08% (11.80%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.38% (11.96%)</t>
+          <t>12.48% (12.06%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.84% (11.49%)</t>
+          <t>11.94% (11.59%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.04% (10.26%)</t>
+          <t>11.12% (10.35%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.67% (9.95%)</t>
+          <t>10.70% (10.00%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>15.00% (14.53%)</t>
+          <t>15.10% (14.63%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.37% (9.73%)</t>
+          <t>10.43% (9.79%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.98% (11.76%)</t>
+          <t>12.04% (11.83%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.58% (11.44%)</t>
+          <t>11.66% (11.52%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.53% (11.45%)</t>
+          <t>11.64% (11.56%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.57% (17.01%)</t>
+          <t>17.65% (17.09%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.70% (18.67%)</t>
+          <t>18.81% (18.78%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.72% (17.44%)</t>
+          <t>17.80% (17.52%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.20% (17.77%)</t>
+          <t>18.30% (17.88%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.47% (17.12%)</t>
+          <t>17.54% (17.19%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.28% (15.49%)</t>
+          <t>16.32% (15.55%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.90% (15.18%)</t>
+          <t>15.95% (15.24%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.88% (20.40%)</t>
+          <t>21.01% (20.54%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.63% (14.98%)</t>
+          <t>15.73% (15.08%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>18.16% (17.94%)</t>
+          <t>18.21% (17.99%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.66% (17.51%)</t>
+          <t>17.74% (17.60%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.54% (17.45%)</t>
+          <t>17.59% (17.51%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.31% (-5.86%)</t>
+          <t>-5.40% (-5.95%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.47% (-12.50%)</t>
+          <t>-12.51% (-12.54%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.81% (-9.09%)</t>
+          <t>-8.84% (-9.12%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.32% (-7.75%)</t>
+          <t>-7.42% (-7.84%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.61% (-7.96%)</t>
+          <t>-7.70% (-8.04%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.39% (-3.17%)</t>
+          <t>-2.51% (-3.28%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.36% (-3.08%)</t>
+          <t>-2.53% (-3.24%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.46% (-9.94%)</t>
+          <t>-9.54% (-10.01%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.54% (-4.19%)</t>
+          <t>-3.69% (-4.33%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.26% (-11.48%)</t>
+          <t>-11.38% (-11.59%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.04% (-11.18%)</t>
+          <t>-11.14% (-11.28%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.17% (-11.26%)</t>
+          <t>-11.24% (-11.32%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.31% (-4.87%)</t>
+          <t>-4.42% (-4.98%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.54% (-10.57%)</t>
+          <t>-10.58% (-10.60%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.43% (-7.72%)</t>
+          <t>-7.51% (-7.79%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-5.97% (-6.40%)</t>
+          <t>-6.04% (-6.46%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.45% (-6.80%)</t>
+          <t>-6.55% (-6.90%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.96% (-2.75%)</t>
+          <t>-2.10% (-2.88%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.96% (-2.68%)</t>
+          <t>-2.10% (-2.81%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.77% (-8.26%)</t>
+          <t>-7.81% (-8.29%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.06% (-3.71%)</t>
+          <t>-3.15% (-3.80%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.36% (-9.59%)</t>
+          <t>-9.47% (-9.68%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.28% (-9.43%)</t>
+          <t>-9.35% (-9.49%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.47% (-9.56%)</t>
+          <t>-9.57% (-9.65%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.29%</t>
+          <t>-17.49%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-25.06%</t>
+          <t>-25.23%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.73%</t>
+          <t>-20.92%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.70%</t>
+          <t>-19.89%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.45%</t>
+          <t>-19.63%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.43%</t>
+          <t>-13.63%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.03%</t>
+          <t>-13.23%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.46%</t>
+          <t>-24.64%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.91%</t>
+          <t>-14.11%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.25%</t>
+          <t>-23.42%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.62%</t>
+          <t>-22.80%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.70%</t>
+          <t>-22.88%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.89%</t>
+          <t>-22.07%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-29.24%</t>
+          <t>-29.39%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.16%</t>
+          <t>-25.31%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.16%</t>
+          <t>-24.34%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.92%</t>
+          <t>-24.09%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.24%</t>
+          <t>-18.43%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.86%</t>
+          <t>-18.05%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.66%</t>
+          <t>-28.82%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.69%</t>
+          <t>-18.88%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.53%</t>
+          <t>-27.67%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.94%</t>
+          <t>-27.09%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-27.01%</t>
+          <t>-27.16%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3.06% (2.51%)</t>
+          <t>3.20% (2.65%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>0.09% (0.07%)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>3.81% (3.53%)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>4.06% (3.64%)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>3.42% (3.08%)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1.59% (0.82%)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1.11% (0.40%)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>6.04% (5.57%)</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>0.93% (0.30%)</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>3.44% (3.23%)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2.36% (2.22%)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>1.28% (1.20%)</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>4.27% (3.71%)</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
           <t>0.14% (0.12%)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>3.61% (3.32%)</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>3.92% (3.50%)</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>3.27% (2.93%)</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>1.48% (0.70%)</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>1.04% (0.33%)</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>6.13% (5.66%)</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>0.85% (0.21%)</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>3.58% (3.36%)</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>2.48% (2.33%)</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>1.36% (1.27%)</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>4.15% (3.58%)</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>0.19% (0.16%)</t>
-        </is>
-      </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.81% (3.52%)</t>
+          <t>3.73% (3.45%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.41% (4.98%)</t>
+          <t>5.33% (4.91%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.57% (4.22%)</t>
+          <t>4.54% (4.19%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.92% (1.14%)</t>
+          <t>2.01% (1.24%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.45% (0.74%)</t>
+          <t>1.55% (0.84%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.27% (4.79%)</t>
+          <t>5.23% (4.75%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.35% (0.70%)</t>
+          <t>1.49% (0.84%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.72% (2.49%)</t>
+          <t>2.60% (2.39%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.81% (1.66%)</t>
+          <t>1.73% (1.59%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>1.00% (0.91%)</t>
+          <t>0.89% (0.80%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 7/8/2026</t>
+          <t>As of 10/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.49%</t>
+          <t>11.59%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.73%</t>
+          <t>7.82%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.73%</t>
+          <t>11.99%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.96%</t>
+          <t>-8.04%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.96%</t>
+          <t>12.06%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.22%</t>
+          <t>6.12%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.48%</t>
+          <t>7.58%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.09%</t>
+          <t>12.35%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>2.37%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.75%</t>
+          <t>-7.84%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.53%</t>
+          <t>14.63%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.66%</t>
+          <t>5.57%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>10.18%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.15%</t>
+          <t>19.43%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.66%</t>
+          <t>-1.89%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.94%</t>
+          <t>-10.01%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.43%</t>
+          <t>11.53%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.53%</t>
+          <t>8.43%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.33%</t>
+          <t>5.43%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.82%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.83%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.86%</t>
+          <t>-5.95%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>12.17%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.54%</t>
+          <t>4.79%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.00%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.19%</t>
+          <t>-4.33%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.00%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>2.47%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.48%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.53%</t>
+          <t>12.27%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.08%</t>
+          <t>-3.24%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.26%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.26%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.96%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.36%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.17%</t>
+          <t>-3.28%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.56%</t>
+          <t>12.70%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.30%</t>
+          <t>13.34%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.10%</t>
+          <t>20.38%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.84%</t>
+          <t>-5.06%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.50%</t>
+          <t>-12.54%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.45%</t>
+          <t>11.56%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>1.20%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.73%</t>
+          <t>11.81%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.43%</t>
+          <t>16.70%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.09%</t>
+          <t>-2.31%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.26%</t>
+          <t>-11.32%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.44%</t>
+          <t>11.52%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.33%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.64%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.31%</t>
+          <t>16.58%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.05%</t>
+          <t>-1.28%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.18%</t>
+          <t>-11.28%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.36%</t>
+          <t>3.23%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>12.15%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.26%</t>
+          <t>17.53%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.54%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.48%</t>
+          <t>-11.59%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.64%</t>
+          <t>11.80%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.43%</t>
+          <t>4.40%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>9.10%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.54%</t>
+          <t>13.80%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.09%</t>
+          <t>-9.12%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 7/8/2026</t>
+          <t>As of 10/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17.12%</t>
+          <t>17.19%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.30%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.50%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.73%</t>
+          <t>11.98%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>-0.15%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.80%</t>
+          <t>-6.90%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.77%</t>
+          <t>17.88%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.98%</t>
+          <t>4.91%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.93%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.09%</t>
+          <t>12.35%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.26%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.40%</t>
+          <t>-6.46%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.40%</t>
+          <t>20.54%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.79%</t>
+          <t>4.75%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.15%</t>
+          <t>19.42%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.23%</t>
+          <t>-4.45%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.26%</t>
+          <t>-8.29%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17.01%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>6.85%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.24%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.82%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.24%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.87%</t>
+          <t>-4.98%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>15.08%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.72%</t>
+          <t>9.62%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.96%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.54%</t>
+          <t>4.79%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.71%</t>
+          <t>-3.80%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>15.24%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>2.02%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.48%</t>
+          <t>3.72%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.68%</t>
+          <t>-2.81%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.49%</t>
+          <t>15.55%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.81%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.96%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.96%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.48%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.75%</t>
+          <t>-2.88%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.67%</t>
+          <t>18.78%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>0.12%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.86%</t>
+          <t>10.89%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.13%</t>
+          <t>20.38%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-6.86%</t>
+          <t>-7.05%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.57%</t>
+          <t>-10.60%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.45%</t>
+          <t>17.51%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.75%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.46%</t>
+          <t>16.70%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-4.28%</t>
+          <t>-4.47%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.56%</t>
+          <t>-9.65%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.51%</t>
+          <t>17.60%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.66%</t>
+          <t>1.59%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.47%</t>
+          <t>9.55%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>16.58%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.61%</t>
+          <t>-3.81%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.43%</t>
+          <t>-9.49%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.94%</t>
+          <t>17.99%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.49%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.67%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.29%</t>
+          <t>17.53%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.44%</t>
+          <t>-3.64%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.59%</t>
+          <t>-9.68%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.44%</t>
+          <t>17.52%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.45%</t>
+          <t>7.53%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.57%</t>
+          <t>13.80%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-1.51%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.72%</t>
+          <t>-7.79%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-11]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/10/2026 at 10:33 AM ET)</t>
+          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>249 days</t>
+          <t>248 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11 days</t>
+          <t>10 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>130 days</t>
+          <t>129 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>193 days</t>
+          <t>192 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>158 days</t>
+          <t>157 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>340 days</t>
+          <t>339 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>311 days</t>
+          <t>310 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>221 days</t>
+          <t>220 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>284 days</t>
+          <t>283 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>102 days</t>
+          <t>101 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>67 days</t>
+          <t>66 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>39 days</t>
+          <t>38 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>249 days</t>
+          <t>248 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>11 days</t>
+          <t>10 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>130 days</t>
+          <t>129 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>193 days</t>
+          <t>192 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>158 days</t>
+          <t>157 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>340 days</t>
+          <t>339 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>311 days</t>
+          <t>310 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>221 days</t>
+          <t>220 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>284 days</t>
+          <t>283 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>102 days</t>
+          <t>101 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>67 days</t>
+          <t>66 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>39 days</t>
+          <t>38 days</t>
         </is>
       </c>
     </row>
@@ -2326,12 +2326,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.73 / 5.43%</t>
+          <t>$47.72 / 5.41%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.45 / 13.34%</t>
+          <t>$57.45 / 13.33%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2341,37 +2341,37 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.31 / 7.58%</t>
+          <t>$62.28 / 7.54%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.36 / 7.82%</t>
+          <t>$56.37 / 7.84%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.35 / 2.51%</t>
+          <t>$61.33 / 2.48%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.35 / 2.47%</t>
+          <t>$61.33 / 2.44%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.24 / 10.18%</t>
+          <t>$53.22 / 10.14%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.58 / 3.62%</t>
+          <t>$57.53 / 3.54%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.72 / 12.15%</t>
+          <t>$59.70 / 12.12%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2381,67 +2381,67 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.36 / 11.81%</t>
+          <t>$56.37 / 11.82%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.41 / 4.35%</t>
+          <t>$42.41 / 4.33%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.93 / 10.89%</t>
+          <t>$41.94 / 10.91%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.53 / 7.53%</t>
+          <t>$40.52 / 7.52%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.76 / 6.00%</t>
+          <t>$44.77 / 6.03%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.85 / 6.50%</t>
+          <t>$45.82 / 6.43%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.56 / 2.09%</t>
+          <t>$44.54 / 2.04%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.98 / 2.02%</t>
+          <t>$41.96 / 1.97%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.90 / 8.12%</t>
+          <t>$44.91 / 8.13%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.94 / 3.05%</t>
+          <t>$43.93 / 3.02%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.51 / 9.79%</t>
+          <t>$42.50 / 9.76%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.25 / 9.55%</t>
+          <t>$42.25 / 9.54%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.68 / 9.75%</t>
+          <t>$41.68 / 9.74%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$774.58 / 9.07%</t>
+          <t>$773.58 / 8.93%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$774.55 / 20.38%</t>
+          <t>$773.58 / 20.22%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$774.55 / 13.80%</t>
+          <t>$773.58 / 13.66%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$774.58 / 12.35%</t>
+          <t>$773.58 / 12.21%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$774.58 / 11.99%</t>
+          <t>$773.58 / 11.84%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$774.55 / 4.20%</t>
+          <t>$773.58 / 4.07%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$774.58 / 3.73%</t>
+          <t>$773.58 / 3.59%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$774.58 / 19.43%</t>
+          <t>$773.58 / 19.27%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$774.58 / 4.79%</t>
+          <t>$773.58 / 4.65%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$774.55 / 17.53%</t>
+          <t>$773.58 / 17.38%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$774.55 / 16.58%</t>
+          <t>$773.58 / 16.43%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$774.55 / 16.70%</t>
+          <t>$773.58 / 16.55%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$774.55 / 9.07%</t>
+          <t>$773.58 / 8.93%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$774.55 / 20.38%</t>
+          <t>$773.58 / 20.22%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$774.55 / 13.80%</t>
+          <t>$773.58 / 13.66%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$774.55 / 12.35%</t>
+          <t>$773.58 / 12.21%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$774.55 / 11.98%</t>
+          <t>$773.58 / 11.84%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$774.55 / 4.20%</t>
+          <t>$773.58 / 4.07%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$774.55 / 3.72%</t>
+          <t>$773.58 / 3.59%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$774.55 / 19.42%</t>
+          <t>$773.58 / 19.27%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$774.55 / 4.79%</t>
+          <t>$773.58 / 4.65%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$774.55 / 17.53%</t>
+          <t>$773.58 / 17.38%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$774.55 / 16.58%</t>
+          <t>$773.58 / 16.43%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$774.55 / 16.70%</t>
+          <t>$773.58 / 16.55%</t>
         </is>
       </c>
     </row>
@@ -2580,12 +2580,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.98% (8.43%)</t>
+          <t>9.00% (8.45%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.09% (0.07%)</t>
+          <t>0.10% (0.08%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2595,37 +2595,37 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.53% (6.12%)</t>
+          <t>6.57% (6.16%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.78% (5.44%)</t>
+          <t>5.76% (5.42%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.90% (13.13%)</t>
+          <t>13.93% (13.16%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.52% (12.82%)</t>
+          <t>13.56% (12.85%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.04% (5.57%)</t>
+          <t>6.08% (5.61%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.80% (12.17%)</t>
+          <t>12.89% (12.25%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.44% (3.23%)</t>
+          <t>3.47% (3.26%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2635,67 +2635,67 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>1.28% (1.20%)</t>
+          <t>1.27% (1.19%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.41% (6.85%)</t>
+          <t>7.42% (6.86%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.14% (0.12%)</t>
+          <t>0.13% (0.11%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.73% (3.45%)</t>
+          <t>3.74% (3.46%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.33% (4.91%)</t>
+          <t>5.31% (4.88%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.54% (4.19%)</t>
+          <t>4.60% (4.26%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.43% (10.66%)</t>
+          <t>11.49% (10.72%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.99% (10.28%)</t>
+          <t>11.04% (10.33%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.23% (4.75%)</t>
+          <t>5.22% (4.74%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.27% (9.62%)</t>
+          <t>10.30% (9.66%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.60% (2.39%)</t>
+          <t>2.62% (2.41%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.73% (1.59%)</t>
+          <t>1.74% (1.60%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.89% (0.80%)</t>
+          <t>0.90% (0.82%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.58%</t>
+          <t>5.72%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-5.06%</t>
+          <t>-4.94%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.37%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.27%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.89%</t>
+          <t>-1.76%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.74%</t>
+          <t>11.88%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.65%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.28%</t>
+          <t>-1.15%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-2.31%</t>
+          <t>-2.19%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.13%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-7.05%</t>
+          <t>-6.93%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.51%</t>
+          <t>-1.39%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.26%</t>
+          <t>-0.14%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.15%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.45%</t>
+          <t>-4.34%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.63%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.64%</t>
+          <t>-3.52%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-3.68%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-4.47%</t>
+          <t>-4.35%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12.08% (11.53%)</t>
+          <t>11.99% (11.45%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.72% (12.70%)</t>
+          <t>12.63% (12.61%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>12.08% (11.80%)</t>
+          <t>11.97% (11.70%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.48% (12.06%)</t>
+          <t>12.41% (11.99%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.94% (11.59%)</t>
+          <t>11.81% (11.47%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.12% (10.35%)</t>
+          <t>11.05% (10.28%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.70% (10.00%)</t>
+          <t>10.62% (9.92%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>15.10% (14.63%)</t>
+          <t>15.03% (14.57%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.43% (9.79%)</t>
+          <t>10.39% (9.75%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>12.04% (11.83%)</t>
+          <t>11.97% (11.76%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.66% (11.52%)</t>
+          <t>11.56% (11.42%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.64% (11.56%)</t>
+          <t>11.54% (11.46%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.65% (17.09%)</t>
+          <t>17.56% (17.00%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.81% (18.78%)</t>
+          <t>18.71% (18.69%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.80% (17.52%)</t>
+          <t>17.72% (17.44%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.30% (17.88%)</t>
+          <t>18.18% (17.76%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.54% (17.19%)</t>
+          <t>17.50% (17.16%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.32% (15.55%)</t>
+          <t>16.28% (15.50%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.95% (15.24%)</t>
+          <t>15.89% (15.18%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>21.01% (20.54%)</t>
+          <t>20.91% (20.44%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.73% (15.08%)</t>
+          <t>15.65% (15.01%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>18.21% (17.99%)</t>
+          <t>18.13% (17.92%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.74% (17.60%)</t>
+          <t>17.66% (17.51%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.59% (17.51%)</t>
+          <t>17.51% (17.43%)</t>
         </is>
       </c>
     </row>
@@ -2961,12 +2961,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.40% (-5.95%)</t>
+          <t>-5.39% (-5.93%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.51% (-12.54%)</t>
+          <t>-12.51% (-12.53%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2976,107 +2976,107 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.42% (-7.84%)</t>
+          <t>-7.38% (-7.80%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.70% (-8.04%)</t>
+          <t>-7.72% (-8.06%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.51% (-3.28%)</t>
+          <t>-2.48% (-3.25%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.53% (-3.24%)</t>
+          <t>-2.50% (-3.21%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.54% (-10.01%)</t>
+          <t>-9.51% (-9.98%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.69% (-4.33%)</t>
+          <t>-3.62% (-4.25%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.38% (-11.59%)</t>
+          <t>-11.35% (-11.56%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.14% (-11.28%)</t>
+          <t>-11.15% (-11.28%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.24% (-11.32%)</t>
+          <t>-11.25% (-11.33%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.42% (-4.98%)</t>
+          <t>-4.41% (-4.96%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.58% (-10.60%)</t>
+          <t>-10.59% (-10.61%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.51% (-7.79%)</t>
+          <t>-7.50% (-7.78%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.04% (-6.46%)</t>
+          <t>-6.06% (-6.48%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.55% (-6.90%)</t>
+          <t>-6.50% (-6.84%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.10% (-2.88%)</t>
+          <t>-2.05% (-2.82%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.10% (-2.81%)</t>
+          <t>-2.05% (-2.76%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.81% (-8.29%)</t>
+          <t>-7.82% (-8.30%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.15% (-3.80%)</t>
+          <t>-3.12% (-3.76%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.47% (-9.68%)</t>
+          <t>-9.45% (-9.66%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.35% (-9.49%)</t>
+          <t>-9.34% (-9.48%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.57% (-9.65%)</t>
+          <t>-9.56% (-9.64%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.49%</t>
+          <t>-17.38%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-25.23%</t>
+          <t>-25.14%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.92%</t>
+          <t>-20.82%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.89%</t>
+          <t>-19.79%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.63%</t>
+          <t>-19.53%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.63%</t>
+          <t>-13.52%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.23%</t>
+          <t>-13.12%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.64%</t>
+          <t>-24.54%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.11%</t>
+          <t>-14.00%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.42%</t>
+          <t>-23.33%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.80%</t>
+          <t>-22.70%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.88%</t>
+          <t>-22.78%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.07%</t>
+          <t>-21.97%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-29.39%</t>
+          <t>-29.30%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.31%</t>
+          <t>-25.21%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.34%</t>
+          <t>-24.24%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.09%</t>
+          <t>-24.00%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.43%</t>
+          <t>-18.32%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.05%</t>
+          <t>-17.95%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.82%</t>
+          <t>-28.73%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.88%</t>
+          <t>-18.78%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.67%</t>
+          <t>-27.58%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.09%</t>
+          <t>-26.99%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-27.16%</t>
+          <t>-27.07%</t>
         </is>
       </c>
     </row>
@@ -3215,52 +3215,52 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3.20% (2.65%)</t>
+          <t>3.09% (2.54%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.09% (0.07%)</t>
+          <t>0.10% (0.08%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.81% (3.53%)</t>
+          <t>3.68% (3.40%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4.06% (3.64%)</t>
+          <t>3.97% (3.55%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3.42% (3.08%)</t>
+          <t>3.26% (2.93%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.59% (0.82%)</t>
+          <t>1.50% (0.73%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.11% (0.40%)</t>
+          <t>1.01% (0.30%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.04% (5.57%)</t>
+          <t>6.08% (5.61%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.93% (0.30%)</t>
+          <t>0.88% (0.24%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.44% (3.23%)</t>
+          <t>3.47% (3.26%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -3270,67 +3270,67 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.28% (1.20%)</t>
+          <t>1.27% (1.19%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>4.27% (3.71%)</t>
+          <t>4.15% (3.59%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.14% (0.12%)</t>
+          <t>0.13% (0.11%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.73% (3.45%)</t>
+          <t>3.74% (3.46%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.33% (4.91%)</t>
+          <t>5.31% (4.88%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.54% (4.19%)</t>
+          <t>4.60% (4.26%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>2.01% (1.24%)</t>
+          <t>1.94% (1.17%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.55% (0.84%)</t>
+          <t>1.47% (0.76%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.23% (4.75%)</t>
+          <t>5.22% (4.74%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.49% (0.84%)</t>
+          <t>1.39% (0.75%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.60% (2.39%)</t>
+          <t>2.62% (2.41%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.73% (1.59%)</t>
+          <t>1.74% (1.60%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.89% (0.80%)</t>
+          <t>0.90% (0.82%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 10/8/2026</t>
+          <t>As of 11/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.59%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.44%</t>
+          <t>5.42%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.82%</t>
+          <t>7.84%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.99%</t>
+          <t>11.84%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.04%</t>
+          <t>-8.06%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>12.06%</t>
+          <t>11.99%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.12%</t>
+          <t>6.16%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.58%</t>
+          <t>7.54%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.35%</t>
+          <t>12.21%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.37%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.84%</t>
+          <t>-7.80%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.63%</t>
+          <t>14.57%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.57%</t>
+          <t>5.61%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>10.14%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.43%</t>
+          <t>19.27%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.89%</t>
+          <t>-1.76%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.01%</t>
+          <t>-9.98%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.53%</t>
+          <t>11.45%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.43%</t>
+          <t>8.45%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.43%</t>
+          <t>5.41%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>8.93%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.58%</t>
+          <t>5.72%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.95%</t>
+          <t>-5.93%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>9.75%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.17%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.62%</t>
+          <t>3.54%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.79%</t>
+          <t>4.65%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.74%</t>
+          <t>11.88%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.33%</t>
+          <t>-4.25%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>9.92%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.85%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.47%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.27%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.24%</t>
+          <t>-3.21%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.16%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>4.07%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.28%</t>
+          <t>-3.25%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.70%</t>
+          <t>12.61%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.34%</t>
+          <t>13.33%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.38%</t>
+          <t>20.22%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-5.06%</t>
+          <t>-4.94%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.54%</t>
+          <t>-12.53%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.56%</t>
+          <t>11.46%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.20%</t>
+          <t>1.19%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.81%</t>
+          <t>11.82%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.70%</t>
+          <t>16.55%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.31%</t>
+          <t>-2.19%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.32%</t>
+          <t>-11.33%</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.52%</t>
+          <t>11.42%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3758,12 +3758,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.58%</t>
+          <t>16.43%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.28%</t>
+          <t>-1.15%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.23%</t>
+          <t>3.26%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.15%</t>
+          <t>12.12%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.53%</t>
+          <t>17.38%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.65%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.59%</t>
+          <t>-11.56%</t>
         </is>
       </c>
     </row>
@@ -3817,7 +3817,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.80%</t>
+          <t>11.70%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3832,12 +3832,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.80%</t>
+          <t>13.66%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 10/8/2026</t>
+          <t>As of 11/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17.19%</t>
+          <t>17.16%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.26%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.50%</t>
+          <t>6.43%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.98%</t>
+          <t>11.84%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.15%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.90%</t>
+          <t>-6.84%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.88%</t>
+          <t>17.76%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.91%</t>
+          <t>4.88%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>6.03%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.35%</t>
+          <t>12.21%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.26%</t>
+          <t>-0.14%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.46%</t>
+          <t>-6.48%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.54%</t>
+          <t>20.44%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.75%</t>
+          <t>4.74%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.12%</t>
+          <t>8.13%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.42%</t>
+          <t>19.27%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.45%</t>
+          <t>-4.34%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.29%</t>
+          <t>-8.30%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>17.00%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.85%</t>
+          <t>6.86%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>8.93%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.13%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.98%</t>
+          <t>-4.96%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.08%</t>
+          <t>15.01%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.62%</t>
+          <t>9.66%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>3.02%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.79%</t>
+          <t>4.65%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.63%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.80%</t>
+          <t>-3.76%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.24%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.33%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.02%</t>
+          <t>1.97%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.72%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.81%</t>
+          <t>-2.76%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.55%</t>
+          <t>15.50%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>10.72%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>2.04%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>4.07%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-2.82%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.78%</t>
+          <t>18.69%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.89%</t>
+          <t>10.91%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.38%</t>
+          <t>20.22%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-7.05%</t>
+          <t>-6.93%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.60%</t>
+          <t>-10.61%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.51%</t>
+          <t>17.43%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.75%</t>
+          <t>9.74%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.70%</t>
+          <t>16.55%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-4.47%</t>
+          <t>-4.35%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.65%</t>
+          <t>-9.64%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.60%</t>
+          <t>17.51%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.59%</t>
+          <t>1.60%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.55%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.58%</t>
+          <t>16.43%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-3.68%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.49%</t>
+          <t>-9.48%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.99%</t>
+          <t>17.92%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>9.76%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.53%</t>
+          <t>17.38%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.64%</t>
+          <t>-3.52%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.68%</t>
+          <t>-9.66%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.52%</t>
+          <t>17.44%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.45%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.53%</t>
+          <t>7.52%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.80%</t>
+          <t>13.66%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.51%</t>
+          <t>-1.39%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.79%</t>
+          <t>-7.78%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-12]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/11/2026 at 10:32 AM ET)</t>
+          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>248 days</t>
+          <t>247 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>10 days</t>
+          <t>9 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>129 days</t>
+          <t>128 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>192 days</t>
+          <t>191 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>157 days</t>
+          <t>156 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>339 days</t>
+          <t>338 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>310 days</t>
+          <t>309 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>220 days</t>
+          <t>219 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>283 days</t>
+          <t>282 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>101 days</t>
+          <t>100 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>66 days</t>
+          <t>65 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>38 days</t>
+          <t>37 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>248 days</t>
+          <t>247 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>10 days</t>
+          <t>9 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>129 days</t>
+          <t>128 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>192 days</t>
+          <t>191 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>157 days</t>
+          <t>156 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>339 days</t>
+          <t>338 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>310 days</t>
+          <t>309 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>220 days</t>
+          <t>219 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>283 days</t>
+          <t>282 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>101 days</t>
+          <t>100 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>66 days</t>
+          <t>65 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>38 days</t>
+          <t>37 days</t>
         </is>
       </c>
     </row>
@@ -2326,57 +2326,57 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.72 / 5.41%</t>
+          <t>$47.70 / 5.37%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.45 / 13.33%</t>
+          <t>$57.47 / 13.38%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.65 / 9.10%</t>
+          <t>$55.66 / 9.11%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.28 / 7.54%</t>
+          <t>$62.29 / 7.56%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.37 / 7.84%</t>
+          <t>$56.34 / 7.79%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.33 / 2.48%</t>
+          <t>$61.29 / 2.41%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.33 / 2.44%</t>
+          <t>$61.31 / 2.40%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.22 / 10.14%</t>
+          <t>$53.23 / 10.17%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.53 / 3.54%</t>
+          <t>$57.51 / 3.49%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.70 / 12.12%</t>
+          <t>$59.71 / 12.13%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.50 / 11.76%</t>
+          <t>$53.51 / 11.77%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2386,27 +2386,27 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.41 / 4.33%</t>
+          <t>$42.40 / 4.32%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.94 / 10.91%</t>
+          <t>$41.94 / 10.92%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.52 / 7.52%</t>
+          <t>$40.54 / 7.57%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.77 / 6.03%</t>
+          <t>$44.78 / 6.06%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.82 / 6.43%</t>
+          <t>$45.85 / 6.49%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2416,32 +2416,32 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.96 / 1.97%</t>
+          <t>$41.97 / 2.00%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.91 / 8.13%</t>
+          <t>$44.92 / 8.16%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.93 / 3.02%</t>
+          <t>$43.92 / 3.00%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.50 / 9.76%</t>
+          <t>$42.51 / 9.77%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.25 / 9.54%</t>
+          <t>$42.27 / 9.59%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.68 / 9.74%</t>
+          <t>$41.70 / 9.79%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$773.58 / 8.93%</t>
+          <t>$772.37 / 8.76%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$773.58 / 20.22%</t>
+          <t>$772.37 / 20.04%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$773.58 / 13.66%</t>
+          <t>$772.37 / 13.49%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$773.58 / 12.21%</t>
+          <t>$772.37 / 12.03%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$773.58 / 11.84%</t>
+          <t>$772.37 / 11.67%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$773.58 / 4.07%</t>
+          <t>$772.37 / 3.91%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$773.58 / 3.59%</t>
+          <t>$772.37 / 3.43%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$773.58 / 19.27%</t>
+          <t>$772.37 / 19.09%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$773.58 / 4.65%</t>
+          <t>$772.37 / 4.49%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$773.58 / 17.38%</t>
+          <t>$772.37 / 17.20%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$773.58 / 16.43%</t>
+          <t>$772.37 / 16.25%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$773.58 / 16.55%</t>
+          <t>$772.37 / 16.37%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$773.58 / 8.93%</t>
+          <t>$772.37 / 8.76%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$773.58 / 20.22%</t>
+          <t>$772.37 / 20.04%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$773.58 / 13.66%</t>
+          <t>$772.37 / 13.49%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$773.58 / 12.21%</t>
+          <t>$772.37 / 12.03%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$773.58 / 11.84%</t>
+          <t>$772.37 / 11.67%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$773.58 / 4.07%</t>
+          <t>$772.37 / 3.91%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$773.58 / 3.59%</t>
+          <t>$772.37 / 3.43%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$773.58 / 19.27%</t>
+          <t>$772.37 / 19.09%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$773.58 / 4.65%</t>
+          <t>$772.37 / 4.49%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$773.58 / 17.38%</t>
+          <t>$772.37 / 17.20%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$773.58 / 16.43%</t>
+          <t>$772.37 / 16.25%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$773.58 / 16.55%</t>
+          <t>$772.37 / 16.37%</t>
         </is>
       </c>
     </row>
@@ -2580,57 +2580,57 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.00% (8.45%)</t>
+          <t>9.03% (8.48%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.10% (0.08%)</t>
+          <t>0.06% (0.04%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.68% (4.40%)</t>
+          <t>4.66% (4.39%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.57% (6.16%)</t>
+          <t>6.56% (6.14%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.76% (5.42%)</t>
+          <t>5.80% (5.46%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.93% (13.16%)</t>
+          <t>14.01% (13.24%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.56% (12.85%)</t>
+          <t>13.59% (12.89%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.08% (5.61%)</t>
+          <t>6.04% (5.58%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.89% (12.25%)</t>
+          <t>12.94% (12.30%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.47% (3.26%)</t>
+          <t>3.45% (3.24%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.36% (2.22%)</t>
+          <t>2.34% (2.21%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2640,27 +2640,27 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.42% (6.86%)</t>
+          <t>7.43% (6.88%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.13% (0.11%)</t>
+          <t>0.12% (0.10%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.74% (3.46%)</t>
+          <t>3.69% (3.41%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.31% (4.88%)</t>
+          <t>5.27% (4.85%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.60% (4.26%)</t>
+          <t>4.54% (4.20%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2670,32 +2670,32 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.04% (10.33%)</t>
+          <t>11.01% (10.30%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.22% (4.74%)</t>
+          <t>5.18% (4.71%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.30% (9.66%)</t>
+          <t>10.31% (9.67%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.62% (2.41%)</t>
+          <t>2.61% (2.40%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.74% (1.60%)</t>
+          <t>1.69% (1.56%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.90% (0.82%)</t>
+          <t>0.85% (0.77%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.72%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-4.94%</t>
+          <t>-4.79%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.11%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>12.42%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>12.59%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.76%</t>
+          <t>-1.61%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.88%</t>
+          <t>12.06%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.65%</t>
+          <t>-0.49%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-1.00%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-2.19%</t>
+          <t>-2.04%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.13%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-6.93%</t>
+          <t>-6.78%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.39%</t>
+          <t>-1.24%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.14%</t>
+          <t>0.02%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.34%</t>
+          <t>-4.19%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.52%</t>
+          <t>-3.37%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.68%</t>
+          <t>-3.53%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-4.35%</t>
+          <t>-4.20%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.99% (11.45%)</t>
+          <t>11.89% (11.35%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.63% (12.61%)</t>
+          <t>12.48% (12.46%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.97% (11.70%)</t>
+          <t>11.84% (11.57%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.41% (11.99%)</t>
+          <t>12.26% (11.85%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.81% (11.47%)</t>
+          <t>11.73% (11.39%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.05% (10.28%)</t>
+          <t>10.97% (10.20%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.62% (9.92%)</t>
+          <t>10.51% (9.81%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>15.03% (14.57%)</t>
+          <t>14.89% (14.42%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.39% (9.75%)</t>
+          <t>10.29% (9.66%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.97% (11.76%)</t>
+          <t>11.84% (11.63%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.56% (11.42%)</t>
+          <t>11.43% (11.29%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.54% (11.46%)</t>
+          <t>11.41% (11.34%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.56% (17.00%)</t>
+          <t>17.44% (16.89%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.71% (18.69%)</t>
+          <t>18.58% (18.56%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.72% (17.44%)</t>
+          <t>17.55% (17.28%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.18% (17.76%)</t>
+          <t>18.03% (17.61%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.50% (17.16%)</t>
+          <t>17.33% (16.99%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.28% (15.50%)</t>
+          <t>16.15% (15.37%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.89% (15.18%)</t>
+          <t>15.74% (15.03%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.91% (20.44%)</t>
+          <t>20.77% (20.29%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.65% (15.01%)</t>
+          <t>15.54% (14.90%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>18.13% (17.92%)</t>
+          <t>18.01% (17.80%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.66% (17.51%)</t>
+          <t>17.50% (17.36%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.51% (17.43%)</t>
+          <t>17.35% (17.27%)</t>
         </is>
       </c>
     </row>
@@ -2961,57 +2961,57 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.39% (-5.93%)</t>
+          <t>-5.36% (-5.90%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.51% (-12.53%)</t>
+          <t>-12.55% (-12.57%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.84% (-9.12%)</t>
+          <t>-8.85% (-9.13%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.38% (-7.80%)</t>
+          <t>-7.40% (-7.81%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.72% (-8.06%)</t>
+          <t>-7.68% (-8.02%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.48% (-3.25%)</t>
+          <t>-2.42% (-3.19%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.50% (-3.21%)</t>
+          <t>-2.47% (-3.17%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.51% (-9.98%)</t>
+          <t>-9.54% (-10.00%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.62% (-4.25%)</t>
+          <t>-3.58% (-4.21%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.35% (-11.56%)</t>
+          <t>-11.37% (-11.58%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.15% (-11.28%)</t>
+          <t>-11.16% (-11.29%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -3021,27 +3021,27 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.41% (-4.96%)</t>
+          <t>-4.40% (-4.95%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.59% (-10.61%)</t>
+          <t>-10.60% (-10.62%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.50% (-7.78%)</t>
+          <t>-7.54% (-7.82%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.06% (-6.48%)</t>
+          <t>-6.09% (-6.51%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.50% (-6.84%)</t>
+          <t>-6.55% (-6.89%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -3051,32 +3051,32 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.05% (-2.76%)</t>
+          <t>-2.08% (-2.78%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.82% (-8.30%)</t>
+          <t>-7.86% (-8.33%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.12% (-3.76%)</t>
+          <t>-3.12% (-3.75%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.45% (-9.66%)</t>
+          <t>-9.46% (-9.67%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.34% (-9.48%)</t>
+          <t>-9.38% (-9.52%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.56% (-9.64%)</t>
+          <t>-9.61% (-9.69%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.38%</t>
+          <t>-17.25%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-25.14%</t>
+          <t>-25.02%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.82%</t>
+          <t>-20.69%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.79%</t>
+          <t>-19.66%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.53%</t>
+          <t>-19.41%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.52%</t>
+          <t>-13.39%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.12%</t>
+          <t>-12.99%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.54%</t>
+          <t>-24.43%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.00%</t>
+          <t>-13.87%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.33%</t>
+          <t>-23.21%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.70%</t>
+          <t>-22.58%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.78%</t>
+          <t>-22.66%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.97%</t>
+          <t>-21.85%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-29.30%</t>
+          <t>-29.19%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.21%</t>
+          <t>-25.10%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.24%</t>
+          <t>-24.12%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.00%</t>
+          <t>-23.88%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.32%</t>
+          <t>-18.20%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.95%</t>
+          <t>-17.82%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.73%</t>
+          <t>-28.62%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.78%</t>
+          <t>-18.65%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.58%</t>
+          <t>-27.47%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.99%</t>
+          <t>-26.88%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-27.07%</t>
+          <t>-26.96%</t>
         </is>
       </c>
     </row>
@@ -3215,57 +3215,57 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3.09% (2.54%)</t>
+          <t>2.96% (2.41%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.10% (0.08%)</t>
+          <t>0.06% (0.04%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.68% (3.40%)</t>
+          <t>3.50% (3.23%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.97% (3.55%)</t>
+          <t>3.79% (3.37%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3.26% (2.93%)</t>
+          <t>3.15% (2.81%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.50% (0.73%)</t>
+          <t>1.40% (0.63%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.01% (0.30%)</t>
+          <t>0.88% (0.18%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.08% (5.61%)</t>
+          <t>6.04% (5.58%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.88% (0.24%)</t>
+          <t>0.76% (0.13%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.47% (3.26%)</t>
+          <t>3.45% (3.24%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.36% (2.22%)</t>
+          <t>2.34% (2.21%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3275,62 +3275,62 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>4.15% (3.59%)</t>
+          <t>4.00% (3.44%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.13% (0.11%)</t>
+          <t>0.12% (0.10%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.74% (3.46%)</t>
+          <t>3.69% (3.41%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.31% (4.88%)</t>
+          <t>5.25% (4.83%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.60% (4.26%)</t>
+          <t>4.41% (4.07%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.94% (1.17%)</t>
+          <t>1.78% (1.01%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.47% (0.76%)</t>
+          <t>1.28% (0.58%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.22% (4.74%)</t>
+          <t>5.18% (4.71%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.39% (0.75%)</t>
+          <t>1.24% (0.61%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.62% (2.41%)</t>
+          <t>2.61% (2.40%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.74% (1.60%)</t>
+          <t>1.69% (1.56%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.90% (0.82%)</t>
+          <t>0.85% (0.77%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 11/8/2026</t>
+          <t>As of 12/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>11.39%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.42%</t>
+          <t>5.46%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.84%</t>
+          <t>7.79%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.84%</t>
+          <t>11.67%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.06%</t>
+          <t>-8.02%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.99%</t>
+          <t>11.85%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.16%</t>
+          <t>6.14%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.54%</t>
+          <t>7.56%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.21%</t>
+          <t>12.03%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.80%</t>
+          <t>-7.81%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.57%</t>
+          <t>14.42%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.61%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.14%</t>
+          <t>10.17%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.27%</t>
+          <t>19.09%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.76%</t>
+          <t>-1.61%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.98%</t>
+          <t>-10.00%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.45%</t>
+          <t>11.35%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.45%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>5.37%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.93%</t>
+          <t>8.76%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.72%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.93%</t>
+          <t>-5.90%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.75%</t>
+          <t>9.66%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>12.30%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.54%</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.65%</t>
+          <t>4.49%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.88%</t>
+          <t>12.06%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.25%</t>
+          <t>-4.21%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.92%</t>
+          <t>9.81%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.85%</t>
+          <t>12.89%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.43%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>12.59%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.21%</t>
+          <t>-3.17%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.16%</t>
+          <t>13.24%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.07%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>12.42%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.25%</t>
+          <t>-3.19%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.61%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.33%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.22%</t>
+          <t>20.04%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.94%</t>
+          <t>-4.79%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.53%</t>
+          <t>-12.57%</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.46%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3721,12 +3721,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.55%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.19%</t>
+          <t>-2.04%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.42%</t>
+          <t>11.29%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>2.21%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.77%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.43%</t>
+          <t>16.25%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-1.00%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.28%</t>
+          <t>-11.29%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.63%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.26%</t>
+          <t>3.24%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.12%</t>
+          <t>12.13%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.38%</t>
+          <t>17.20%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.65%</t>
+          <t>-0.49%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.56%</t>
+          <t>-11.58%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.70%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.40%</t>
+          <t>4.39%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.10%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.66%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.11%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.12%</t>
+          <t>-9.13%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 11/8/2026</t>
+          <t>As of 12/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17.16%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.26%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.43%</t>
+          <t>6.49%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.84%</t>
+          <t>11.67%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.84%</t>
+          <t>-6.89%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.76%</t>
+          <t>17.61%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.88%</t>
+          <t>4.85%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.03%</t>
+          <t>6.06%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.21%</t>
+          <t>12.03%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.14%</t>
+          <t>0.02%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.48%</t>
+          <t>-6.51%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.44%</t>
+          <t>20.29%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.74%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.13%</t>
+          <t>8.16%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.27%</t>
+          <t>19.09%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.34%</t>
+          <t>-4.19%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.30%</t>
+          <t>-8.33%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17.00%</t>
+          <t>16.89%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.86%</t>
+          <t>6.88%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>4.32%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.93%</t>
+          <t>8.76%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.13%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.96%</t>
+          <t>-4.95%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.01%</t>
+          <t>14.90%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.66%</t>
+          <t>9.67%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.65%</t>
+          <t>4.49%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.76%</t>
+          <t>-3.75%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.33%</t>
+          <t>10.30%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.97%</t>
+          <t>2.00%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.43%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-2.78%</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.50%</t>
+          <t>15.37%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4162,12 +4162,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.07%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.69%</t>
+          <t>18.56%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.10%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.91%</t>
+          <t>10.92%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.22%</t>
+          <t>20.04%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-6.93%</t>
+          <t>-6.78%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.61%</t>
+          <t>-10.62%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.43%</t>
+          <t>17.27%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>0.77%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.74%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.55%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-4.35%</t>
+          <t>-4.20%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.64%</t>
+          <t>-9.69%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.51%</t>
+          <t>17.36%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.43%</t>
+          <t>16.25%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.68%</t>
+          <t>-3.53%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.48%</t>
+          <t>-9.52%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.92%</t>
+          <t>17.80%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.41%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.76%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.38%</t>
+          <t>17.20%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.52%</t>
+          <t>-3.37%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.66%</t>
+          <t>-9.67%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.44%</t>
+          <t>17.28%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.41%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.52%</t>
+          <t>7.57%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.66%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.39%</t>
+          <t>-1.24%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.78%</t>
+          <t>-7.82%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-13]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/12/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>247 days</t>
+          <t>246 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>9 days</t>
+          <t>8 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>128 days</t>
+          <t>127 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>191 days</t>
+          <t>190 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>156 days</t>
+          <t>155 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>338 days</t>
+          <t>337 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>309 days</t>
+          <t>308 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>219 days</t>
+          <t>218 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>282 days</t>
+          <t>281 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>100 days</t>
+          <t>99 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>65 days</t>
+          <t>64 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>37 days</t>
+          <t>36 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>247 days</t>
+          <t>246 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>9 days</t>
+          <t>8 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>128 days</t>
+          <t>127 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>191 days</t>
+          <t>190 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>156 days</t>
+          <t>155 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>338 days</t>
+          <t>337 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>309 days</t>
+          <t>308 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>219 days</t>
+          <t>218 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>282 days</t>
+          <t>281 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>100 days</t>
+          <t>99 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>65 days</t>
+          <t>64 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>37 days</t>
+          <t>36 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.70 / 5.37%</t>
+          <t>$47.86 / 5.73%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.47 / 13.38%</t>
+          <t>$57.49 / 13.41%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.66 / 9.11%</t>
+          <t>$55.80 / 9.40%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.29 / 7.56%</t>
+          <t>$62.46 / 7.85%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.34 / 7.79%</t>
+          <t>$56.53 / 8.16%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.29 / 2.41%</t>
+          <t>$61.55 / 2.85%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.31 / 2.40%</t>
+          <t>$61.55 / 2.80%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.23 / 10.17%</t>
+          <t>$53.34 / 10.39%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.51 / 3.49%</t>
+          <t>$57.76 / 3.95%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.71 / 12.13%</t>
+          <t>$59.88 / 12.46%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.51 / 11.77%</t>
+          <t>$53.65 / 12.08%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.37 / 11.82%</t>
+          <t>$56.49 / 12.07%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.40 / 4.32%</t>
+          <t>$42.51 / 4.59%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.94 / 10.92%</t>
+          <t>$41.96 / 10.96%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.54 / 7.57%</t>
+          <t>$40.61 / 7.74%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.78 / 6.06%</t>
+          <t>$44.85 / 6.23%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.85 / 6.49%</t>
+          <t>$45.93 / 6.69%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.54 / 2.04%</t>
+          <t>$44.70 / 2.40%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.97 / 2.00%</t>
+          <t>$42.09 / 2.29%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.92 / 8.16%</t>
+          <t>$44.99 / 8.32%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.92 / 3.00%</t>
+          <t>$44.06 / 3.32%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.51 / 9.77%</t>
+          <t>$42.59 / 9.98%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.27 / 9.59%</t>
+          <t>$42.34 / 9.77%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.70 / 9.79%</t>
+          <t>$41.75 / 9.92%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$772.37 / 8.76%</t>
+          <t>$779.05 / 9.70%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$772.37 / 20.04%</t>
+          <t>$779.05 / 21.08%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$772.37 / 13.49%</t>
+          <t>$779.05 / 14.47%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$772.37 / 12.03%</t>
+          <t>$779.05 / 13.00%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$772.37 / 11.67%</t>
+          <t>$779.05 / 12.63%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$772.37 / 3.91%</t>
+          <t>$779.05 / 4.81%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$772.37 / 3.43%</t>
+          <t>$779.05 / 4.33%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$772.37 / 19.09%</t>
+          <t>$779.05 / 20.12%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$772.37 / 4.49%</t>
+          <t>$779.05 / 5.40%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$772.37 / 17.20%</t>
+          <t>$779.05 / 18.21%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$772.37 / 16.25%</t>
+          <t>$779.05 / 17.26%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$772.37 / 16.37%</t>
+          <t>$779.05 / 17.38%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$772.37 / 8.76%</t>
+          <t>$779.05 / 9.70%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$772.37 / 20.04%</t>
+          <t>$779.05 / 21.08%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$772.37 / 13.49%</t>
+          <t>$779.05 / 14.47%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$772.37 / 12.03%</t>
+          <t>$779.05 / 13.00%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$772.37 / 11.67%</t>
+          <t>$779.05 / 12.63%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$772.37 / 3.91%</t>
+          <t>$779.05 / 4.81%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$772.37 / 3.43%</t>
+          <t>$779.05 / 4.33%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$772.37 / 19.09%</t>
+          <t>$779.05 / 20.12%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$772.37 / 4.49%</t>
+          <t>$779.05 / 5.40%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$772.37 / 17.20%</t>
+          <t>$779.05 / 18.21%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$772.37 / 16.25%</t>
+          <t>$779.05 / 17.26%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$772.37 / 16.37%</t>
+          <t>$779.05 / 17.38%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.03% (8.48%)</t>
+          <t>8.66% (8.12%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.06% (0.04%)</t>
+          <t>0.03% (0.01%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.66% (4.39%)</t>
+          <t>4.39% (4.12%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.56% (6.14%)</t>
+          <t>6.26% (5.85%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.80% (5.46%)</t>
+          <t>5.44% (5.11%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.01% (13.24%)</t>
+          <t>13.52% (12.76%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.59% (12.89%)</t>
+          <t>13.16% (12.46%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.04% (5.58%)</t>
+          <t>5.83% (5.37%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.94% (12.30%)</t>
+          <t>12.44% (11.81%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.45% (3.24%)</t>
+          <t>3.15% (2.94%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.34% (2.21%)</t>
+          <t>2.07% (1.93%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>1.27% (1.19%)</t>
+          <t>1.04% (0.97%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.43% (6.88%)</t>
+          <t>7.15% (6.60%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.12% (0.10%)</t>
+          <t>0.08% (0.06%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.69% (3.41%)</t>
+          <t>3.52% (3.24%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.27% (4.85%)</t>
+          <t>5.10% (4.69%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.54% (4.20%)</t>
+          <t>4.35% (4.01%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.49% (10.72%)</t>
+          <t>11.09% (10.32%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.01% (10.30%)</t>
+          <t>10.69% (9.99%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.18% (4.71%)</t>
+          <t>5.03% (4.56%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.31% (9.67%)</t>
+          <t>9.97% (9.34%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.61% (2.40%)</t>
+          <t>2.41% (2.20%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.69% (1.56%)</t>
+          <t>1.52% (1.39%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.85% (0.77%)</t>
+          <t>0.72% (0.65%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>4.97%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-4.79%</t>
+          <t>-5.60%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.11%</t>
+          <t>0.25%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>1.78%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>1.68%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.42%</t>
+          <t>11.46%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.59%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-2.45%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.06%</t>
+          <t>11.10%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.49%</t>
+          <t>-1.35%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.00%</t>
+          <t>-1.85%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-2.04%</t>
+          <t>-2.88%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-6.78%</t>
+          <t>-7.58%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.24%</t>
+          <t>-2.08%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.02%</t>
+          <t>-0.84%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>8.60%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>8.65%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
+          <t>-5.01%</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>8.01%</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
           <t>-4.19%</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>8.94%</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>-3.37%</t>
-        </is>
-      </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.53%</t>
+          <t>-4.36%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-4.20%</t>
+          <t>-5.02%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.89% (11.35%)</t>
+          <t>12.28% (11.74%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.48% (12.46%)</t>
+          <t>13.09% (13.08%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.84% (11.57%)</t>
+          <t>12.28% (12.01%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.26% (11.85%)</t>
+          <t>12.70% (12.29%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.73% (11.39%)</t>
+          <t>12.10% (11.77%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.97% (10.20%)</t>
+          <t>11.30% (10.54%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.51% (9.81%)</t>
+          <t>10.89% (10.19%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.89% (14.42%)</t>
+          <t>15.35% (14.89%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.29% (9.66%)</t>
+          <t>10.60% (9.97%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.84% (11.63%)</t>
+          <t>12.23% (12.03%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.43% (11.29%)</t>
+          <t>11.85% (11.71%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.41% (11.34%)</t>
+          <t>11.88% (11.80%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.44% (16.89%)</t>
+          <t>17.86% (17.32%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.58% (18.56%)</t>
+          <t>19.16% (19.14%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.55% (17.28%)</t>
+          <t>18.05% (17.77%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.03% (17.61%)</t>
+          <t>18.53% (18.12%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.33% (16.99%)</t>
+          <t>17.81% (17.47%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.15% (15.37%)</t>
+          <t>16.49% (15.73%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.74% (15.03%)</t>
+          <t>16.16% (15.46%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.77% (20.29%)</t>
+          <t>21.24% (20.77%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.54% (14.90%)</t>
+          <t>15.93% (15.30%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>18.01% (17.80%)</t>
+          <t>18.46% (18.25%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.50% (17.36%)</t>
+          <t>17.97% (17.84%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.35% (17.27%)</t>
+          <t>17.86% (17.79%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.36% (-5.90%)</t>
+          <t>-5.68% (-6.22%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.55% (-12.57%)</t>
+          <t>-12.57% (-12.59%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.85% (-9.13%)</t>
+          <t>-9.09% (-9.36%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.40% (-7.81%)</t>
+          <t>-7.65% (-8.06%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.68% (-8.02%)</t>
+          <t>-7.99% (-8.33%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.42% (-3.19%)</t>
+          <t>-2.83% (-3.59%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.47% (-3.17%)</t>
+          <t>-2.85% (-3.54%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.54% (-10.00%)</t>
+          <t>-9.72% (-10.18%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.58% (-4.21%)</t>
+          <t>-4.00% (-4.63%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.37% (-11.58%)</t>
+          <t>-11.63% (-11.84%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.16% (-11.29%)</t>
+          <t>-11.40% (-11.53%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.25% (-11.33%)</t>
+          <t>-11.45% (-11.52%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.40% (-4.95%)</t>
+          <t>-4.65% (-5.20%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.60% (-10.62%)</t>
+          <t>-10.64% (-10.65%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.54% (-7.82%)</t>
+          <t>-7.69% (-7.97%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.09% (-6.51%)</t>
+          <t>-6.24% (-6.66%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.55% (-6.89%)</t>
+          <t>-6.72% (-7.06%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.05% (-2.82%)</t>
+          <t>-2.40% (-3.17%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.08% (-2.78%)</t>
+          <t>-2.36% (-3.06%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.86% (-8.33%)</t>
+          <t>-7.99% (-8.46%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.12% (-3.75%)</t>
+          <t>-3.41% (-4.05%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.46% (-9.67%)</t>
+          <t>-9.63% (-9.84%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.38% (-9.52%)</t>
+          <t>-9.54% (-9.67%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.61% (-9.69%)</t>
+          <t>-9.72% (-9.80%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.25%</t>
+          <t>-17.96%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-25.02%</t>
+          <t>-25.67%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.69%</t>
+          <t>-21.37%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.66%</t>
+          <t>-20.35%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.41%</t>
+          <t>-20.10%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.39%</t>
+          <t>-14.13%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.99%</t>
+          <t>-13.73%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.43%</t>
+          <t>-25.07%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.87%</t>
+          <t>-14.61%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.21%</t>
+          <t>-23.86%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.58%</t>
+          <t>-23.25%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.66%</t>
+          <t>-23.33%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.85%</t>
+          <t>-22.52%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-29.19%</t>
+          <t>-29.79%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.10%</t>
+          <t>-25.74%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.12%</t>
+          <t>-24.78%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.88%</t>
+          <t>-24.53%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.20%</t>
+          <t>-18.90%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.82%</t>
+          <t>-18.52%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.62%</t>
+          <t>-29.23%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.65%</t>
+          <t>-19.35%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.47%</t>
+          <t>-28.09%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.88%</t>
+          <t>-27.51%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-26.96%</t>
+          <t>-27.58%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.96% (2.41%)</t>
+          <t>3.50% (2.96%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.06% (0.04%)</t>
+          <t>0.03% (0.01%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.50% (3.23%)</t>
+          <t>4.13% (3.86%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.79% (3.37%)</t>
+          <t>4.40% (3.99%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3.15% (2.81%)</t>
+          <t>3.69% (3.36%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.40% (0.63%)</t>
+          <t>1.85% (1.08%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.88% (0.18%)</t>
+          <t>1.36% (0.67%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.04% (5.58%)</t>
+          <t>5.83% (5.37%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.76% (0.13%)</t>
+          <t>1.19% (0.56%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.45% (3.24%)</t>
+          <t>3.15% (2.94%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.34% (2.21%)</t>
+          <t>2.07% (1.93%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.27% (1.19%)</t>
+          <t>1.04% (0.97%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>4.00% (3.44%)</t>
+          <t>4.62% (4.08%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.12% (0.10%)</t>
+          <t>0.08% (0.06%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.69% (3.41%)</t>
+          <t>3.52% (3.24%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.25% (4.83%)</t>
+          <t>5.10% (4.69%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.41% (4.07%)</t>
+          <t>4.35% (4.01%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.78% (1.01%)</t>
+          <t>2.29% (1.52%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.28% (0.58%)</t>
+          <t>1.87% (1.17%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.18% (4.71%)</t>
+          <t>5.03% (4.56%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.24% (0.61%)</t>
+          <t>1.80% (1.17%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.61% (2.40%)</t>
+          <t>2.41% (2.20%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.69% (1.56%)</t>
+          <t>1.52% (1.39%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.85% (0.77%)</t>
+          <t>0.72% (0.65%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 12/8/2026</t>
+          <t>As of 13/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.39%</t>
+          <t>11.77%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.46%</t>
+          <t>5.11%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.79%</t>
+          <t>8.16%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.67%</t>
+          <t>12.63%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>1.68%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.02%</t>
+          <t>-8.33%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.85%</t>
+          <t>12.29%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.14%</t>
+          <t>5.85%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.56%</t>
+          <t>7.85%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.03%</t>
+          <t>13.00%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>1.78%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.81%</t>
+          <t>-8.06%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.42%</t>
+          <t>14.89%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.58%</t>
+          <t>5.37%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.17%</t>
+          <t>10.39%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.09%</t>
+          <t>20.12%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-2.45%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.00%</t>
+          <t>-10.18%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.35%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.37%</t>
+          <t>5.73%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.76%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>4.97%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.90%</t>
+          <t>-6.22%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.66%</t>
+          <t>9.97%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.30%</t>
+          <t>11.81%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>3.95%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.49%</t>
+          <t>5.40%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.06%</t>
+          <t>11.10%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.21%</t>
+          <t>-4.63%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.81%</t>
+          <t>10.19%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.89%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.43%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.59%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.17%</t>
+          <t>-3.54%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>10.54%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.24%</t>
+          <t>12.76%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.41%</t>
+          <t>2.85%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.42%</t>
+          <t>11.46%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.19%</t>
+          <t>-3.59%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>13.08%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>0.01%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>13.41%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.04%</t>
+          <t>21.08%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.79%</t>
+          <t>-5.60%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.57%</t>
+          <t>-12.59%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>11.80%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.19%</t>
+          <t>0.97%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.82%</t>
+          <t>12.07%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>17.38%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.04%</t>
+          <t>-2.88%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.33%</t>
+          <t>-11.52%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.71%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.21%</t>
+          <t>1.93%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.77%</t>
+          <t>12.08%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.25%</t>
+          <t>17.26%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.00%</t>
+          <t>-1.85%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.29%</t>
+          <t>-11.53%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.63%</t>
+          <t>12.03%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.24%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.13%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.20%</t>
+          <t>18.21%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.49%</t>
+          <t>-1.35%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.58%</t>
+          <t>-11.84%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>4.12%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>14.47%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.11%</t>
+          <t>0.25%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.13%</t>
+          <t>-9.36%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 12/8/2026</t>
+          <t>As of 13/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>17.47%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>4.01%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.49%</t>
+          <t>6.69%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.67%</t>
+          <t>12.63%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.89%</t>
+          <t>-7.06%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.61%</t>
+          <t>18.12%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.85%</t>
+          <t>4.69%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.06%</t>
+          <t>6.23%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.03%</t>
+          <t>13.00%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.02%</t>
+          <t>-0.84%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.51%</t>
+          <t>-6.66%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.29%</t>
+          <t>20.77%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.16%</t>
+          <t>8.32%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.09%</t>
+          <t>20.12%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.19%</t>
+          <t>-5.01%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.33%</t>
+          <t>-8.46%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.89%</t>
+          <t>17.32%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.88%</t>
+          <t>6.60%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.32%</t>
+          <t>4.59%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.76%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.95%</t>
+          <t>-5.20%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.90%</t>
+          <t>15.30%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.67%</t>
+          <t>9.34%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.32%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.49%</t>
+          <t>5.40%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>8.01%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.75%</t>
+          <t>-4.05%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>15.46%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.30%</t>
+          <t>9.99%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.00%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.43%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>8.65%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.78%</t>
+          <t>-3.06%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.37%</t>
+          <t>15.73%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.72%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>8.60%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.82%</t>
+          <t>-3.17%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.56%</t>
+          <t>19.14%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.92%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.04%</t>
+          <t>21.08%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-6.78%</t>
+          <t>-7.58%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.62%</t>
+          <t>-10.65%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.27%</t>
+          <t>17.79%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.77%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>9.92%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>17.38%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-4.20%</t>
+          <t>-5.02%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.69%</t>
+          <t>-9.80%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.36%</t>
+          <t>17.84%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>1.39%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.25%</t>
+          <t>17.26%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.53%</t>
+          <t>-4.36%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.52%</t>
+          <t>-9.67%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.80%</t>
+          <t>18.25%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.20%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.98%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.20%</t>
+          <t>18.21%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-4.19%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.67%</t>
+          <t>-9.84%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.28%</t>
+          <t>17.77%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.41%</t>
+          <t>3.24%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.57%</t>
+          <t>7.74%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>14.47%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.24%</t>
+          <t>-2.08%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.82%</t>
+          <t>-7.97%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-14]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/13/2026 at 10:34 AM ET)</t>
+          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>246 days</t>
+          <t>245 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>8 days</t>
+          <t>7 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>127 days</t>
+          <t>126 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>190 days</t>
+          <t>189 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>155 days</t>
+          <t>154 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>337 days</t>
+          <t>336 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>308 days</t>
+          <t>307 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>218 days</t>
+          <t>217 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>281 days</t>
+          <t>280 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>99 days</t>
+          <t>98 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>64 days</t>
+          <t>63 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>36 days</t>
+          <t>35 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>246 days</t>
+          <t>245 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>8 days</t>
+          <t>7 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>127 days</t>
+          <t>126 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>190 days</t>
+          <t>189 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>155 days</t>
+          <t>154 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>337 days</t>
+          <t>336 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>308 days</t>
+          <t>307 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>218 days</t>
+          <t>217 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>281 days</t>
+          <t>280 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>99 days</t>
+          <t>98 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>64 days</t>
+          <t>63 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>36 days</t>
+          <t>35 days</t>
         </is>
       </c>
     </row>
@@ -2326,52 +2326,52 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.86 / 5.73%</t>
+          <t>$47.86 / 5.72%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.49 / 13.41%</t>
+          <t>$57.47 / 13.38%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.80 / 9.40%</t>
+          <t>$55.83 / 9.45%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.46 / 7.85%</t>
+          <t>$62.47 / 7.87%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.53 / 8.16%</t>
+          <t>$56.53 / 8.15%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.55 / 2.85%</t>
+          <t>$61.47 / 2.72%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.55 / 2.80%</t>
+          <t>$61.52 / 2.75%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.34 / 10.39%</t>
+          <t>$53.35 / 10.41%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.76 / 3.95%</t>
+          <t>$57.71 / 3.85%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.88 / 12.46%</t>
+          <t>$59.89 / 12.47%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2381,67 +2381,67 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.49 / 12.07%</t>
+          <t>$56.53 / 12.14%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.51 / 4.59%</t>
+          <t>$42.50 / 4.57%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.96 / 10.96%</t>
+          <t>$41.99 / 11.04%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.61 / 7.74%</t>
+          <t>$40.62 / 7.77%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.85 / 6.23%</t>
+          <t>$44.87 / 6.26%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.93 / 6.69%</t>
+          <t>$45.96 / 6.75%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.70 / 2.40%</t>
+          <t>$44.66 / 2.31%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.09 / 2.29%</t>
+          <t>$42.08 / 2.25%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.99 / 8.32%</t>
+          <t>$45.00 / 8.34%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.06 / 3.32%</t>
+          <t>$44.04 / 3.27%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.59 / 9.98%</t>
+          <t>$42.60 / 10.01%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.34 / 9.77%</t>
+          <t>$42.34 / 9.79%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.75 / 9.92%</t>
+          <t>$41.76 / 9.95%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$779.05 / 9.70%</t>
+          <t>$777.30 / 9.46%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$779.05 / 21.08%</t>
+          <t>$777.30 / 20.80%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$779.05 / 14.47%</t>
+          <t>$777.30 / 14.21%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$779.05 / 13.00%</t>
+          <t>$777.30 / 12.74%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$779.05 / 12.63%</t>
+          <t>$777.30 / 12.38%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$779.05 / 4.81%</t>
+          <t>$777.30 / 4.57%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$779.05 / 4.33%</t>
+          <t>$777.30 / 4.09%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$779.05 / 20.12%</t>
+          <t>$777.30 / 19.85%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$779.05 / 5.40%</t>
+          <t>$777.30 / 5.16%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$779.05 / 18.21%</t>
+          <t>$777.30 / 17.95%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$779.05 / 17.26%</t>
+          <t>$777.30 / 16.99%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$779.05 / 17.38%</t>
+          <t>$777.30 / 17.12%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$779.05 / 9.70%</t>
+          <t>$777.30 / 9.46%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$779.05 / 21.08%</t>
+          <t>$777.30 / 20.80%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$779.05 / 14.47%</t>
+          <t>$777.30 / 14.21%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$779.05 / 13.00%</t>
+          <t>$777.30 / 12.74%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$779.05 / 12.63%</t>
+          <t>$777.30 / 12.38%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$779.05 / 4.81%</t>
+          <t>$777.30 / 4.57%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$779.05 / 4.33%</t>
+          <t>$777.30 / 4.09%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$779.05 / 20.12%</t>
+          <t>$777.30 / 19.85%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$779.05 / 5.40%</t>
+          <t>$777.30 / 5.16%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$779.05 / 18.21%</t>
+          <t>$777.30 / 17.95%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$779.05 / 17.26%</t>
+          <t>$777.30 / 16.99%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$779.05 / 17.38%</t>
+          <t>$777.30 / 17.12%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.66% (8.12%)</t>
+          <t>8.67% (8.13%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.03% (0.01%)</t>
+          <t>0.05% (0.04%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.39% (4.12%)</t>
+          <t>4.33% (4.06%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.26% (5.85%)</t>
+          <t>6.24% (5.84%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.44% (5.11%)</t>
+          <t>5.45% (5.12%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.52% (12.76%)</t>
+          <t>13.67% (12.91%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.16% (12.46%)</t>
+          <t>13.21% (12.51%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.83% (5.37%)</t>
+          <t>5.81% (5.35%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.44% (11.81%)</t>
+          <t>12.54% (11.91%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.15% (2.94%)</t>
+          <t>3.14% (2.93%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.07% (1.93%)</t>
+          <t>2.06% (1.93%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>1.04% (0.97%)</t>
+          <t>0.98% (0.91%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.15% (6.60%)</t>
+          <t>7.17% (6.62%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.08% (0.06%)</t>
+          <t>0.01% (-0.01%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.52% (3.24%)</t>
+          <t>3.49% (3.22%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.10% (4.69%)</t>
+          <t>5.06% (4.65%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.35% (4.01%)</t>
+          <t>4.29% (3.95%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.09% (10.32%)</t>
+          <t>11.19% (10.42%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.69% (9.99%)</t>
+          <t>10.73% (10.03%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.03% (4.56%)</t>
+          <t>5.00% (4.53%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.97% (9.34%)</t>
+          <t>10.02% (9.39%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.41% (2.20%)</t>
+          <t>2.39% (2.18%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.52% (1.39%)</t>
+          <t>1.51% (1.38%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.72% (0.65%)</t>
+          <t>0.70% (0.62%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4.97%</t>
+          <t>5.21%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-5.60%</t>
+          <t>-5.39%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.25%</t>
+          <t>0.47%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.78%</t>
+          <t>2.01%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.68%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>11.46%</t>
+          <t>11.71%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>11.87%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-2.45%</t>
+          <t>-2.23%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.10%</t>
+          <t>11.35%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-1.35%</t>
+          <t>-1.12%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.85%</t>
+          <t>-1.63%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-2.66%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.41%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-7.58%</t>
+          <t>-7.37%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-2.08%</t>
+          <t>-1.86%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.84%</t>
+          <t>-0.61%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>8.60%</t>
+          <t>8.84%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>8.65%</t>
+          <t>8.90%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-5.01%</t>
+          <t>-4.79%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-4.19%</t>
+          <t>-3.98%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-4.36%</t>
+          <t>-4.15%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-5.02%</t>
+          <t>-4.81%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12.28% (11.74%)</t>
+          <t>12.11% (11.57%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>13.09% (13.08%)</t>
+          <t>12.95% (12.93%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>12.28% (12.01%)</t>
+          <t>12.05% (11.78%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.70% (12.29%)</t>
+          <t>12.50% (12.09%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>12.10% (11.77%)</t>
+          <t>11.93% (11.60%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.30% (10.54%)</t>
+          <t>11.23% (10.47%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.89% (10.19%)</t>
+          <t>10.74% (10.04%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>15.35% (14.89%)</t>
+          <t>15.17% (14.71%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.60% (9.97%)</t>
+          <t>10.50% (9.87%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>12.23% (12.03%)</t>
+          <t>12.05% (11.85%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.85% (11.71%)</t>
+          <t>11.67% (11.54%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.88% (11.80%)</t>
+          <t>11.65% (11.57%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.86% (17.32%)</t>
+          <t>17.71% (17.16%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>19.16% (19.14%)</t>
+          <t>18.93% (18.92%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>18.05% (17.77%)</t>
+          <t>17.85% (17.58%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.53% (18.12%)</t>
+          <t>18.33% (17.92%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.81% (17.47%)</t>
+          <t>17.59% (17.25%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.49% (15.73%)</t>
+          <t>16.40% (15.63%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>16.16% (15.46%)</t>
+          <t>16.01% (15.31%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>21.24% (20.77%)</t>
+          <t>21.06% (20.59%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.93% (15.30%)</t>
+          <t>15.79% (15.16%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>18.46% (18.25%)</t>
+          <t>18.27% (18.07%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.97% (17.84%)</t>
+          <t>17.79% (17.66%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.86% (17.79%)</t>
+          <t>17.68% (17.60%)</t>
         </is>
       </c>
     </row>
@@ -2961,52 +2961,52 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.68% (-6.22%)</t>
+          <t>-5.67% (-6.21%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.57% (-12.59%)</t>
+          <t>-12.55% (-12.57%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.09% (-9.36%)</t>
+          <t>-9.14% (-9.41%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.65% (-8.06%)</t>
+          <t>-7.67% (-8.08%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.99% (-8.33%)</t>
+          <t>-7.99% (-8.32%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.83% (-3.59%)</t>
+          <t>-2.71% (-3.47%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.85% (-3.54%)</t>
+          <t>-2.80% (-3.50%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.72% (-10.18%)</t>
+          <t>-9.74% (-10.20%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.00% (-4.63%)</t>
+          <t>-3.91% (-4.54%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.63% (-11.84%)</t>
+          <t>-11.64% (-11.84%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -3016,67 +3016,67 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.45% (-11.52%)</t>
+          <t>-11.51% (-11.58%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.65% (-5.20%)</t>
+          <t>-4.63% (-5.18%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.64% (-10.65%)</t>
+          <t>-10.70% (-10.72%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.69% (-7.97%)</t>
+          <t>-7.72% (-7.99%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.24% (-6.66%)</t>
+          <t>-6.28% (-6.69%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.72% (-7.06%)</t>
+          <t>-6.78% (-7.11%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.40% (-3.17%)</t>
+          <t>-2.32% (-3.08%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.36% (-3.06%)</t>
+          <t>-2.33% (-3.03%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.99% (-8.46%)</t>
+          <t>-8.01% (-8.48%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.41% (-4.05%)</t>
+          <t>-3.37% (-4.00%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.63% (-9.84%)</t>
+          <t>-9.66% (-9.86%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.54% (-9.67%)</t>
+          <t>-9.55% (-9.68%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.72% (-9.80%)</t>
+          <t>-9.74% (-9.82%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.96%</t>
+          <t>-17.78%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-25.67%</t>
+          <t>-25.50%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-21.37%</t>
+          <t>-21.20%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-20.35%</t>
+          <t>-20.17%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-20.10%</t>
+          <t>-19.92%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-14.13%</t>
+          <t>-13.94%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.73%</t>
+          <t>-13.54%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-25.07%</t>
+          <t>-24.90%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.61%</t>
+          <t>-14.41%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.86%</t>
+          <t>-23.69%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-23.25%</t>
+          <t>-23.07%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-23.33%</t>
+          <t>-23.15%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.52%</t>
+          <t>-22.34%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-29.79%</t>
+          <t>-29.64%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.74%</t>
+          <t>-25.57%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.78%</t>
+          <t>-24.61%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.53%</t>
+          <t>-24.36%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.90%</t>
+          <t>-18.72%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.52%</t>
+          <t>-18.34%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-29.23%</t>
+          <t>-29.07%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-19.35%</t>
+          <t>-19.17%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-28.09%</t>
+          <t>-27.93%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.51%</t>
+          <t>-27.34%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-27.58%</t>
+          <t>-27.42%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3.50% (2.96%)</t>
+          <t>3.28% (2.74%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.03% (0.01%)</t>
+          <t>0.05% (0.04%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.13% (3.86%)</t>
+          <t>3.84% (3.57%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4.40% (3.99%)</t>
+          <t>4.14% (3.74%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3.69% (3.36%)</t>
+          <t>3.46% (3.13%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.85% (1.08%)</t>
+          <t>1.75% (0.99%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.36% (0.67%)</t>
+          <t>1.18% (0.49%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.83% (5.37%)</t>
+          <t>5.81% (5.35%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>1.19% (0.56%)</t>
+          <t>1.05% (0.42%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.15% (2.94%)</t>
+          <t>3.14% (2.93%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.07% (1.93%)</t>
+          <t>2.06% (1.93%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.04% (0.97%)</t>
+          <t>0.98% (0.91%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>4.62% (4.08%)</t>
+          <t>4.41% (3.86%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.08% (0.06%)</t>
+          <t>0.01% (-0.01%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.52% (3.24%)</t>
+          <t>3.49% (3.22%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.10% (4.69%)</t>
+          <t>5.06% (4.65%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.35% (4.01%)</t>
+          <t>4.29% (3.95%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>2.29% (1.52%)</t>
+          <t>2.15% (1.38%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.87% (1.17%)</t>
+          <t>1.67% (0.97%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.03% (4.56%)</t>
+          <t>5.00% (4.53%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.80% (1.17%)</t>
+          <t>1.62% (0.99%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.41% (2.20%)</t>
+          <t>2.39% (2.18%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.52% (1.39%)</t>
+          <t>1.51% (1.38%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.72% (0.65%)</t>
+          <t>0.70% (0.62%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 13/8/2026</t>
+          <t>As of 14/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.77%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.11%</t>
+          <t>5.12%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.16%</t>
+          <t>8.15%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.63%</t>
+          <t>12.38%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.68%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.33%</t>
+          <t>-8.32%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>12.29%</t>
+          <t>12.09%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.85%</t>
+          <t>5.84%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.85%</t>
+          <t>7.87%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13.00%</t>
+          <t>12.74%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.78%</t>
+          <t>2.01%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.06%</t>
+          <t>-8.08%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.89%</t>
+          <t>14.71%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.37%</t>
+          <t>5.35%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.39%</t>
+          <t>10.41%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20.12%</t>
+          <t>19.85%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.45%</t>
+          <t>-2.23%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.18%</t>
+          <t>-10.20%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.74%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.12%</t>
+          <t>8.13%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.73%</t>
+          <t>5.72%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.97%</t>
+          <t>5.21%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.22%</t>
+          <t>-6.21%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.97%</t>
+          <t>9.87%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.81%</t>
+          <t>11.91%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.95%</t>
+          <t>3.85%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.40%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.10%</t>
+          <t>11.35%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.63%</t>
+          <t>-4.54%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10.19%</t>
+          <t>10.04%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>12.51%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.80%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>11.87%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.54%</t>
+          <t>-3.50%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.54%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>12.91%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.85%</t>
+          <t>2.72%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>4.57%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.46%</t>
+          <t>11.71%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.59%</t>
+          <t>-3.47%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.08%</t>
+          <t>12.93%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.01%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>21.08%</t>
+          <t>20.80%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-5.60%</t>
+          <t>-5.39%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.59%</t>
+          <t>-12.57%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.80%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.97%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>12.07%</t>
+          <t>12.14%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>17.38%</t>
+          <t>17.12%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-2.66%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.52%</t>
+          <t>-11.58%</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.71%</t>
+          <t>11.54%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3758,12 +3758,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.26%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.85%</t>
+          <t>-1.63%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3780,27 +3780,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12.03%</t>
+          <t>11.85%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.94%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>12.47%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.21%</t>
+          <t>17.95%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.35%</t>
+          <t>-1.12%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>11.78%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.12%</t>
+          <t>4.06%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.47%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.25%</t>
+          <t>0.47%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.36%</t>
+          <t>-9.41%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 13/8/2026</t>
+          <t>As of 14/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17.47%</t>
+          <t>17.25%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.01%</t>
+          <t>3.95%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.69%</t>
+          <t>6.75%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.63%</t>
+          <t>12.38%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.06%</t>
+          <t>-7.11%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18.12%</t>
+          <t>17.92%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.69%</t>
+          <t>4.65%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.23%</t>
+          <t>6.26%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13.00%</t>
+          <t>12.74%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.84%</t>
+          <t>-0.61%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.66%</t>
+          <t>-6.69%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.77%</t>
+          <t>20.59%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.32%</t>
+          <t>8.34%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20.12%</t>
+          <t>19.85%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-5.01%</t>
+          <t>-4.79%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.46%</t>
+          <t>-8.48%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17.32%</t>
+          <t>17.16%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.60%</t>
+          <t>6.62%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.59%</t>
+          <t>4.57%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.41%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.20%</t>
+          <t>-5.18%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.30%</t>
+          <t>15.16%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.34%</t>
+          <t>9.39%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.32%</t>
+          <t>3.27%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.40%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>8.25%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.05%</t>
+          <t>-4.00%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.46%</t>
+          <t>15.31%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.99%</t>
+          <t>10.03%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.29%</t>
+          <t>2.25%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8.65%</t>
+          <t>8.90%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.06%</t>
+          <t>-3.03%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.73%</t>
+          <t>15.63%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.31%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>4.57%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8.60%</t>
+          <t>8.84%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.17%</t>
+          <t>-3.08%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>19.14%</t>
+          <t>18.92%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.06%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>11.04%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>21.08%</t>
+          <t>20.80%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-7.58%</t>
+          <t>-7.37%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.65%</t>
+          <t>-10.72%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.79%</t>
+          <t>17.60%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>0.62%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.92%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>17.38%</t>
+          <t>17.12%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-5.02%</t>
+          <t>-4.81%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.80%</t>
+          <t>-9.82%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.84%</t>
+          <t>17.66%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>1.38%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.26%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-4.36%</t>
+          <t>-4.15%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.67%</t>
+          <t>-9.68%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>18.25%</t>
+          <t>18.07%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.20%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>10.01%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.21%</t>
+          <t>17.95%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-4.19%</t>
+          <t>-3.98%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.84%</t>
+          <t>-9.86%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.77%</t>
+          <t>17.58%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.24%</t>
+          <t>3.22%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.74%</t>
+          <t>7.77%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.47%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-2.08%</t>
+          <t>-1.86%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.97%</t>
+          <t>-7.99%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-17]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/14/2026 at 10:28 AM ET)</t>
+          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>245 days</t>
+          <t>242 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7 days</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>126 days</t>
+          <t>123 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>189 days</t>
+          <t>186 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>154 days</t>
+          <t>151 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>336 days</t>
+          <t>333 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>307 days</t>
+          <t>304 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>217 days</t>
+          <t>214 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>280 days</t>
+          <t>277 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>98 days</t>
+          <t>95 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>63 days</t>
+          <t>60 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>35 days</t>
+          <t>32 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>245 days</t>
+          <t>242 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>7 days</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>126 days</t>
+          <t>123 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>189 days</t>
+          <t>186 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>154 days</t>
+          <t>151 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>336 days</t>
+          <t>333 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>307 days</t>
+          <t>304 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>217 days</t>
+          <t>214 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>280 days</t>
+          <t>277 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>98 days</t>
+          <t>95 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>63 days</t>
+          <t>60 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>35 days</t>
+          <t>32 days</t>
         </is>
       </c>
     </row>
@@ -2326,52 +2326,52 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.86 / 5.72%</t>
+          <t>$47.81 / 5.62%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.47 / 13.38%</t>
+          <t>$57.50 / 13.44%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.83 / 9.45%</t>
+          <t>$55.80 / 9.40%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.47 / 7.87%</t>
+          <t>$62.42 / 7.78%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.53 / 8.15%</t>
+          <t>$56.50 / 8.10%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.47 / 2.72%</t>
+          <t>$61.43 / 2.65%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.52 / 2.75%</t>
+          <t>$61.44 / 2.62%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.35 / 10.41%</t>
+          <t>$53.29 / 10.30%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.71 / 3.85%</t>
+          <t>$57.64 / 3.74%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.89 / 12.47%</t>
+          <t>$59.87 / 12.43%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2381,62 +2381,62 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.53 / 12.14%</t>
+          <t>$56.51 / 12.11%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.50 / 4.57%</t>
+          <t>$42.49 / 4.53%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.99 / 11.04%</t>
+          <t>$42.01 / 11.11%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.62 / 7.77%</t>
+          <t>$40.61 / 7.74%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.87 / 6.26%</t>
+          <t>$44.86 / 6.25%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.96 / 6.75%</t>
+          <t>$45.94 / 6.70%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.66 / 2.31%</t>
+          <t>$44.62 / 2.22%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.08 / 2.25%</t>
+          <t>$42.05 / 2.18%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.00 / 8.34%</t>
+          <t>$44.99 / 8.32%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.04 / 3.27%</t>
+          <t>$44.01 / 3.20%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.60 / 10.01%</t>
+          <t>$42.59 / 9.98%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.34 / 9.79%</t>
+          <t>$42.35 / 9.80%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$777.30 / 9.46%</t>
+          <t>$775.24 / 9.17%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$777.30 / 20.80%</t>
+          <t>$775.24 / 20.48%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$777.30 / 14.21%</t>
+          <t>$775.24 / 13.91%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$777.30 / 12.74%</t>
+          <t>$775.24 / 12.45%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$777.30 / 12.38%</t>
+          <t>$775.24 / 12.08%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$777.30 / 4.57%</t>
+          <t>$775.24 / 4.30%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$777.30 / 4.09%</t>
+          <t>$775.24 / 3.82%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$777.30 / 19.85%</t>
+          <t>$775.24 / 19.53%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$777.30 / 5.16%</t>
+          <t>$775.24 / 4.88%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$777.30 / 17.95%</t>
+          <t>$775.24 / 17.63%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$777.30 / 16.99%</t>
+          <t>$775.24 / 16.68%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$777.30 / 17.12%</t>
+          <t>$775.24 / 16.81%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$777.30 / 9.46%</t>
+          <t>$775.24 / 9.17%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$777.30 / 20.80%</t>
+          <t>$775.33 / 20.50%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$777.30 / 14.21%</t>
+          <t>$775.33 / 13.92%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$777.30 / 12.74%</t>
+          <t>$775.24 / 12.45%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$777.30 / 12.38%</t>
+          <t>$775.24 / 12.08%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$777.30 / 4.57%</t>
+          <t>$775.33 / 4.31%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$777.30 / 4.09%</t>
+          <t>$775.33 / 3.83%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$777.30 / 19.85%</t>
+          <t>$775.24 / 19.53%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$777.30 / 5.16%</t>
+          <t>$775.33 / 4.89%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$777.30 / 17.95%</t>
+          <t>$775.33 / 17.65%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$777.30 / 16.99%</t>
+          <t>$775.33 / 16.70%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$777.30 / 17.12%</t>
+          <t>$775.33 / 16.82%</t>
         </is>
       </c>
     </row>
@@ -2580,52 +2580,52 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.67% (8.13%)</t>
+          <t>8.77% (8.23%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.05% (0.04%)</t>
+          <t>-0.01% (-0.01%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.33% (4.06%)</t>
+          <t>4.38% (4.12%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.24% (5.84%)</t>
+          <t>6.32% (5.92%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.45% (5.12%)</t>
+          <t>5.49% (5.17%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.67% (12.91%)</t>
+          <t>13.74% (12.98%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.21% (12.51%)</t>
+          <t>13.34% (12.65%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.81% (5.35%)</t>
+          <t>5.91% (5.46%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.54% (11.91%)</t>
+          <t>12.66% (12.04%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.14% (2.93%)</t>
+          <t>3.17% (2.97%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2635,67 +2635,67 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.98% (0.91%)</t>
+          <t>1.00% (0.93%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.17% (6.62%)</t>
+          <t>7.20% (6.66%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.01% (-0.01%)</t>
+          <t>-0.06% (-0.07%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.49% (3.22%)</t>
+          <t>3.51% (3.24%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.06% (4.65%)</t>
+          <t>5.07% (4.66%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.29% (3.95%)</t>
+          <t>4.33% (4.00%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.19% (10.42%)</t>
+          <t>11.28% (10.52%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.73% (10.03%)</t>
+          <t>10.80% (10.11%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.00% (4.53%)</t>
+          <t>5.02% (4.56%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.02% (9.39%)</t>
+          <t>10.09% (9.46%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.39% (2.18%)</t>
+          <t>2.41% (2.20%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.51% (1.38%)</t>
+          <t>1.49% (1.36%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.70% (0.62%)</t>
+          <t>0.69% (0.62%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.21%</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-5.39%</t>
+          <t>-5.14%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.74%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.01%</t>
+          <t>2.28%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>11.71%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11.87%</t>
+          <t>12.17%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-2.23%</t>
+          <t>-1.97%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.35%</t>
+          <t>11.64%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-1.12%</t>
+          <t>-0.86%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.63%</t>
+          <t>-1.37%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-2.66%</t>
+          <t>-2.40%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.64%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-7.37%</t>
+          <t>-7.14%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.86%</t>
+          <t>-1.61%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.61%</t>
+          <t>-0.35%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>-0.24%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>8.84%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>8.90%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.79%</t>
+          <t>-4.54%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>8.52%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.98%</t>
+          <t>-3.73%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-4.15%</t>
+          <t>-3.90%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-4.81%</t>
+          <t>-4.57%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12.11% (11.57%)</t>
+          <t>11.97% (11.44%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.95% (12.93%)</t>
+          <t>12.70% (12.69%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>12.05% (11.78%)</t>
+          <t>11.89% (11.62%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.50% (12.09%)</t>
+          <t>12.36% (11.96%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.93% (11.60%)</t>
+          <t>11.75% (11.43%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.23% (10.47%)</t>
+          <t>11.06% (10.30%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.74% (10.04%)</t>
+          <t>10.62% (9.93%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>15.17% (14.71%)</t>
+          <t>15.05% (14.60%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.50% (9.87%)</t>
+          <t>10.37% (9.75%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>12.05% (11.85%)</t>
+          <t>11.87% (11.68%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.67% (11.54%)</t>
+          <t>11.46% (11.34%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.65% (11.57%)</t>
+          <t>11.46% (11.39%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.71% (17.16%)</t>
+          <t>17.53% (16.99%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.93% (18.92%)</t>
+          <t>18.69% (18.69%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.85% (17.58%)</t>
+          <t>17.68% (17.41%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.33% (17.92%)</t>
+          <t>18.13% (17.73%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.59% (17.25%)</t>
+          <t>17.42% (17.09%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.40% (15.63%)</t>
+          <t>16.27% (15.51%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>16.01% (15.31%)</t>
+          <t>15.87% (15.17%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>21.06% (20.59%)</t>
+          <t>20.89% (20.43%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.79% (15.16%)</t>
+          <t>15.65% (15.02%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>18.27% (18.07%)</t>
+          <t>18.10% (17.90%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.79% (17.66%)</t>
+          <t>17.59% (17.47%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.68% (17.60%)</t>
+          <t>17.49% (17.42%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.67% (-6.21%)</t>
+          <t>-5.59% (-6.12%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.55% (-12.57%)</t>
+          <t>-12.60% (-12.61%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.14% (-9.41%)</t>
+          <t>-9.10% (-9.36%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.67% (-8.08%)</t>
+          <t>-7.60% (-8.01%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.99% (-8.32%)</t>
+          <t>-7.95% (-8.28%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.71% (-3.47%)</t>
+          <t>-2.65% (-3.41%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.80% (-3.50%)</t>
+          <t>-2.69% (-3.38%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.74% (-10.20%)</t>
+          <t>-9.65% (-10.10%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.91% (-4.54%)</t>
+          <t>-3.81% (-4.44%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.64% (-11.84%)</t>
+          <t>-11.62% (-11.81%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.40% (-11.53%)</t>
+          <t>-11.41% (-11.53%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.51% (-11.58%)</t>
+          <t>-11.49% (-11.55%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.63% (-5.18%)</t>
+          <t>-4.60% (-5.14%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.70% (-10.72%)</t>
+          <t>-10.76% (-10.77%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.72% (-7.99%)</t>
+          <t>-7.70% (-7.97%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.28% (-6.69%)</t>
+          <t>-6.27% (-6.68%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.78% (-7.11%)</t>
+          <t>-6.74% (-7.07%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.32% (-3.08%)</t>
+          <t>-2.24% (-3.00%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.33% (-3.03%)</t>
+          <t>-2.27% (-2.96%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.01% (-8.48%)</t>
+          <t>-8.00% (-8.46%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.37% (-4.00%)</t>
+          <t>-3.31% (-3.94%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.66% (-9.86%)</t>
+          <t>-9.64% (-9.84%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.55% (-9.68%)</t>
+          <t>-9.57% (-9.69%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.74% (-9.82%)</t>
+          <t>-9.75% (-9.82%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.78%</t>
+          <t>-17.56%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-25.50%</t>
+          <t>-25.30%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-21.20%</t>
+          <t>-20.99%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-20.17%</t>
+          <t>-19.96%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.92%</t>
+          <t>-19.70%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.94%</t>
+          <t>-13.71%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.54%</t>
+          <t>-13.31%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.90%</t>
+          <t>-24.71%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.41%</t>
+          <t>-14.19%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.69%</t>
+          <t>-23.49%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-23.07%</t>
+          <t>-22.87%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-23.15%</t>
+          <t>-22.95%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.34%</t>
+          <t>-22.13%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-29.64%</t>
+          <t>-29.46%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.57%</t>
+          <t>-25.38%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.61%</t>
+          <t>-24.40%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.36%</t>
+          <t>-24.16%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.72%</t>
+          <t>-18.51%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.34%</t>
+          <t>-18.13%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-29.07%</t>
+          <t>-28.89%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-19.17%</t>
+          <t>-18.96%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.93%</t>
+          <t>-27.75%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.34%</t>
+          <t>-27.16%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-27.42%</t>
+          <t>-27.23%</t>
         </is>
       </c>
     </row>
@@ -3215,52 +3215,52 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3.28% (2.74%)</t>
+          <t>3.09% (2.56%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.05% (0.04%)</t>
+          <t>-0.01% (-0.01%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.84% (3.57%)</t>
+          <t>3.61% (3.35%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4.14% (3.74%)</t>
+          <t>3.94% (3.54%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3.46% (3.13%)</t>
+          <t>3.23% (2.90%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.75% (0.99%)</t>
+          <t>1.54% (0.78%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.18% (0.49%)</t>
+          <t>1.03% (0.34%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.81% (5.35%)</t>
+          <t>5.91% (5.46%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>1.05% (0.42%)</t>
+          <t>0.89% (0.27%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.14% (2.93%)</t>
+          <t>3.17% (2.97%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -3270,67 +3270,67 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.98% (0.91%)</t>
+          <t>1.00% (0.93%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>4.41% (3.86%)</t>
+          <t>4.16% (3.62%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.01% (-0.01%)</t>
+          <t>-0.06% (-0.07%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.49% (3.22%)</t>
+          <t>3.51% (3.24%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.06% (4.65%)</t>
+          <t>5.07% (4.66%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.29% (3.95%)</t>
+          <t>4.33% (4.00%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>2.15% (1.38%)</t>
+          <t>1.97% (1.22%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.67% (0.97%)</t>
+          <t>1.48% (0.79%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.00% (4.53%)</t>
+          <t>5.02% (4.56%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.62% (0.99%)</t>
+          <t>1.42% (0.80%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.39% (2.18%)</t>
+          <t>2.41% (2.20%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.51% (1.38%)</t>
+          <t>1.49% (1.36%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.70% (0.62%)</t>
+          <t>0.69% (0.62%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 14/8/2026</t>
+          <t>As of 17/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>11.43%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.12%</t>
+          <t>5.17%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.15%</t>
+          <t>8.10%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.38%</t>
+          <t>12.08%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.32%</t>
+          <t>-8.28%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>12.09%</t>
+          <t>11.96%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.84%</t>
+          <t>5.92%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.87%</t>
+          <t>7.78%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.74%</t>
+          <t>12.45%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.01%</t>
+          <t>2.28%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.08%</t>
+          <t>-8.01%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.71%</t>
+          <t>14.60%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.35%</t>
+          <t>5.46%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.41%</t>
+          <t>10.30%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.85%</t>
+          <t>19.53%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.23%</t>
+          <t>-1.97%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.20%</t>
+          <t>-10.10%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>11.44%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.13%</t>
+          <t>8.23%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.72%</t>
+          <t>5.62%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.21%</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.21%</t>
+          <t>-6.12%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.87%</t>
+          <t>9.75%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.91%</t>
+          <t>12.04%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.85%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.16%</t>
+          <t>4.88%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.35%</t>
+          <t>11.64%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.54%</t>
+          <t>-4.44%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10.04%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.51%</t>
+          <t>12.65%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>2.62%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>3.82%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.87%</t>
+          <t>12.17%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-3.38%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.47%</t>
+          <t>10.30%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>12.98%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.72%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.57%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.71%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.47%</t>
+          <t>-3.41%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.93%</t>
+          <t>12.69%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>13.44%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.80%</t>
+          <t>20.48%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-5.39%</t>
+          <t>-5.14%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.57%</t>
+          <t>-12.61%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>11.39%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>12.14%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>17.12%</t>
+          <t>16.81%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.66%</t>
+          <t>-2.40%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.58%</t>
+          <t>-11.55%</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3758,12 +3758,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.68%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.63%</t>
+          <t>-1.37%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.85%</t>
+          <t>11.68%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.93%</t>
+          <t>2.97%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.47%</t>
+          <t>12.43%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.95%</t>
+          <t>17.63%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.12%</t>
+          <t>-0.86%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.84%</t>
+          <t>-11.81%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.78%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.06%</t>
+          <t>4.12%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>13.91%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.74%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.41%</t>
+          <t>-9.36%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 14/8/2026</t>
+          <t>As of 17/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17.25%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.95%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.75%</t>
+          <t>6.70%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.38%</t>
+          <t>12.08%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>-0.24%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.11%</t>
+          <t>-7.07%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.92%</t>
+          <t>17.73%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.65%</t>
+          <t>4.66%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.26%</t>
+          <t>6.25%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.74%</t>
+          <t>12.45%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.61%</t>
+          <t>-0.35%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.69%</t>
+          <t>-6.68%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.59%</t>
+          <t>20.43%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.34%</t>
+          <t>8.32%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.85%</t>
+          <t>19.53%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.79%</t>
+          <t>-4.54%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.48%</t>
+          <t>-8.46%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17.16%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.62%</t>
+          <t>6.66%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.57%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.64%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.18%</t>
+          <t>-5.14%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.16%</t>
+          <t>15.02%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.39%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.27%</t>
+          <t>3.20%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.16%</t>
+          <t>4.89%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>8.52%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.00%</t>
+          <t>-3.94%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>15.17%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.03%</t>
+          <t>10.11%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.25%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>3.83%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8.90%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.03%</t>
+          <t>-2.96%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.63%</t>
+          <t>15.51%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>10.52%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.31%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.57%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8.84%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.08%</t>
+          <t>-3.00%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.92%</t>
+          <t>18.69%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.04%</t>
+          <t>11.11%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.80%</t>
+          <t>20.50%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-7.37%</t>
+          <t>-7.14%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.72%</t>
+          <t>-10.77%</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.60%</t>
+          <t>17.42%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4236,12 +4236,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>17.12%</t>
+          <t>16.82%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-4.81%</t>
+          <t>-4.57%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.66%</t>
+          <t>17.47%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.38%</t>
+          <t>1.36%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.70%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-4.15%</t>
+          <t>-3.90%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.68%</t>
+          <t>-9.69%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>18.07%</t>
+          <t>17.90%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>2.20%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.01%</t>
+          <t>9.98%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.95%</t>
+          <t>17.65%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.98%</t>
+          <t>-3.73%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.86%</t>
+          <t>-9.84%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.58%</t>
+          <t>17.41%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.22%</t>
+          <t>3.24%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.77%</t>
+          <t>7.74%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>13.92%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.86%</t>
+          <t>-1.61%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.99%</t>
+          <t>-7.97%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-18]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 9:59 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/17/2026 at 10:00 AM ET)</t>
+          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>242 days</t>
+          <t>241 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>3 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>123 days</t>
+          <t>122 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>186 days</t>
+          <t>185 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>151 days</t>
+          <t>150 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>333 days</t>
+          <t>332 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>304 days</t>
+          <t>303 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>214 days</t>
+          <t>213 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>277 days</t>
+          <t>276 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>95 days</t>
+          <t>94 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>60 days</t>
+          <t>59 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>32 days</t>
+          <t>31 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>242 days</t>
+          <t>241 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>3 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>123 days</t>
+          <t>122 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>186 days</t>
+          <t>185 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>151 days</t>
+          <t>150 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>333 days</t>
+          <t>332 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>304 days</t>
+          <t>303 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>214 days</t>
+          <t>213 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>277 days</t>
+          <t>276 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>95 days</t>
+          <t>94 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>60 days</t>
+          <t>59 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>32 days</t>
+          <t>31 days</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.81 / 5.62%</t>
+          <t>$47.61 / 5.17%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2336,112 +2336,112 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.80 / 9.40%</t>
+          <t>$55.60 / 9.00%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.42 / 7.78%</t>
+          <t>$62.21 / 7.42%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.50 / 8.10%</t>
+          <t>$56.28 / 7.67%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.43 / 2.65%</t>
+          <t>$61.14 / 2.16%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.44 / 2.62%</t>
+          <t>$61.12 / 2.08%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.29 / 10.30%</t>
+          <t>$53.19 / 10.09%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.64 / 3.74%</t>
+          <t>$57.37 / 3.24%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.87 / 12.43%</t>
+          <t>$59.69 / 12.11%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.65 / 12.08%</t>
+          <t>$53.51 / 11.78%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.51 / 12.11%</t>
+          <t>$56.39 / 11.87%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.49 / 4.53%</t>
+          <t>$42.37 / 4.24%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.01 / 11.11%</t>
+          <t>$41.98 / 11.03%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.61 / 7.74%</t>
+          <t>$40.52 / 7.52%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.86 / 6.25%</t>
+          <t>$44.74 / 5.96%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.94 / 6.70%</t>
+          <t>$45.80 / 6.39%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.62 / 2.22%</t>
+          <t>$44.46 / 1.85%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.05 / 2.18%</t>
+          <t>$41.87 / 1.74%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.99 / 8.32%</t>
+          <t>$44.91 / 8.14%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.01 / 3.20%</t>
+          <t>$43.84 / 2.80%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.59 / 9.98%</t>
+          <t>$42.51 / 9.77%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.35 / 9.80%</t>
+          <t>$42.28 / 9.62%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.76 / 9.95%</t>
+          <t>$41.72 / 9.84%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$775.24 / 9.17%</t>
+          <t>$769.00 / 8.29%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$775.24 / 20.48%</t>
+          <t>$769.00 / 19.51%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$775.24 / 13.91%</t>
+          <t>$769.00 / 12.99%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$775.24 / 12.45%</t>
+          <t>$769.00 / 11.54%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$775.24 / 12.08%</t>
+          <t>$769.00 / 11.18%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$775.24 / 4.30%</t>
+          <t>$769.00 / 3.46%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$775.24 / 3.82%</t>
+          <t>$769.00 / 2.98%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$775.24 / 19.53%</t>
+          <t>$769.00 / 18.57%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$775.24 / 4.88%</t>
+          <t>$769.00 / 4.04%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$775.24 / 17.63%</t>
+          <t>$769.00 / 16.69%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$775.24 / 16.68%</t>
+          <t>$769.00 / 15.75%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$775.24 / 16.81%</t>
+          <t>$769.00 / 15.87%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$775.24 / 9.17%</t>
+          <t>$769.00 / 8.29%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$775.33 / 20.50%</t>
+          <t>$769.00 / 19.51%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$775.33 / 13.92%</t>
+          <t>$769.00 / 12.99%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$775.24 / 12.45%</t>
+          <t>$769.00 / 11.54%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$775.24 / 12.08%</t>
+          <t>$769.00 / 11.18%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$775.33 / 4.31%</t>
+          <t>$769.00 / 3.46%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$775.33 / 3.83%</t>
+          <t>$769.00 / 2.98%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$775.24 / 19.53%</t>
+          <t>$769.00 / 18.57%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$775.33 / 4.89%</t>
+          <t>$769.00 / 4.04%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$775.33 / 17.65%</t>
+          <t>$769.00 / 16.69%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$775.33 / 16.70%</t>
+          <t>$769.00 / 15.75%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$775.33 / 16.82%</t>
+          <t>$769.00 / 15.87%</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.77% (8.23%)</t>
+          <t>9.22% (8.69%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2590,112 +2590,112 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.38% (4.12%)</t>
+          <t>4.76% (4.49%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.32% (5.92%)</t>
+          <t>6.68% (6.28%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.49% (5.17%)</t>
+          <t>5.91% (5.59%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.74% (12.98%)</t>
+          <t>14.27% (13.52%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.34% (12.65%)</t>
+          <t>13.94% (13.25%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.91% (5.46%)</t>
+          <t>6.11% (5.66%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.66% (12.04%)</t>
+          <t>13.20% (12.58%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.17% (2.97%)</t>
+          <t>3.47% (3.27%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.06% (1.93%)</t>
+          <t>2.32% (2.20%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>1.00% (0.93%)</t>
+          <t>1.21% (1.15%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.20% (6.66%)</t>
+          <t>7.50% (6.96%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>-0.06% (-0.07%)</t>
+          <t>0.01% (0.00%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.51% (3.24%)</t>
+          <t>3.72% (3.46%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.07% (4.66%)</t>
+          <t>5.36% (4.95%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.33% (4.00%)</t>
+          <t>4.63% (4.30%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.28% (10.52%)</t>
+          <t>11.68% (10.92%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.80% (10.11%)</t>
+          <t>11.27% (10.58%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.02% (4.56%)</t>
+          <t>5.19% (4.73%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.09% (9.46%)</t>
+          <t>10.51% (9.89%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.41% (2.20%)</t>
+          <t>2.60% (2.40%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.49% (1.36%)</t>
+          <t>1.66% (1.53%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.69% (0.62%)</t>
+          <t>0.79% (0.72%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>6.35%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-5.14%</t>
+          <t>-4.37%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.74%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.28%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>12.91%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.17%</t>
+          <t>13.08%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.97%</t>
+          <t>-1.18%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.64%</t>
+          <t>12.55%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.86%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-2.40%</t>
+          <t>-1.61%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-7.14%</t>
+          <t>-6.38%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.35%</t>
+          <t>0.46%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>0.57%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>10.07%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.54%</t>
+          <t>-3.77%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.52%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.73%</t>
+          <t>-2.94%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.90%</t>
+          <t>-3.11%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-4.57%</t>
+          <t>-3.78%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.97% (11.44%)</t>
+          <t>11.70% (11.16%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.70% (12.69%)</t>
+          <t>12.09% (12.08%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.89% (11.62%)</t>
+          <t>11.57% (11.31%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.36% (11.96%)</t>
+          <t>12.02% (11.62%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.75% (11.43%)</t>
+          <t>11.47% (11.14%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>11.06% (10.30%)</t>
+          <t>10.82% (10.06%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.62% (9.93%)</t>
+          <t>10.43% (9.74%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>15.05% (14.60%)</t>
+          <t>14.61% (14.16%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.37% (9.75%)</t>
+          <t>10.14% (9.51%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.87% (11.68%)</t>
+          <t>11.51% (11.32%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.46% (11.34%)</t>
+          <t>11.07% (10.94%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.46% (11.39%)</t>
+          <t>11.02% (10.96%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>17.53% (16.99%)</t>
+          <t>17.17% (16.63%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.69% (18.69%)</t>
+          <t>18.18% (18.17%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.68% (17.41%)</t>
+          <t>17.26% (16.99%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>18.13% (17.73%)</t>
+          <t>17.78% (17.37%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.42% (17.09%)</t>
+          <t>17.08% (16.75%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>16.27% (15.51%)</t>
+          <t>15.95% (15.19%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.87% (15.17%)</t>
+          <t>15.61% (14.92%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.89% (20.43%)</t>
+          <t>20.46% (20.00%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.65% (15.02%)</t>
+          <t>15.35% (14.73%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>18.10% (17.90%)</t>
+          <t>17.68% (17.48%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.59% (17.47%)</t>
+          <t>17.14% (17.02%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>17.49% (17.42%)</t>
+          <t>16.97% (16.91%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.59% (-6.12%)</t>
+          <t>-5.19% (-5.73%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.60% (-12.61%)</t>
+          <t>-12.61% (-12.61%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.10% (-9.36%)</t>
+          <t>-8.78% (-9.04%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.60% (-8.01%)</t>
+          <t>-7.29% (-7.69%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.95% (-8.28%)</t>
+          <t>-7.59% (-7.91%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.65% (-3.41%)</t>
+          <t>-2.19% (-2.95%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.69% (-3.38%)</t>
+          <t>-2.17% (-2.87%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.65% (-10.10%)</t>
+          <t>-9.48% (-9.94%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.81% (-4.44%)</t>
+          <t>-3.35% (-3.98%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.62% (-11.81%)</t>
+          <t>-11.36% (-11.55%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.41% (-11.53%)</t>
+          <t>-11.18% (-11.30%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.49% (-11.55%)</t>
+          <t>-11.30% (-11.37%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.60% (-5.14%)</t>
+          <t>-4.34% (-4.87%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.76% (-10.77%)</t>
+          <t>-10.70% (-10.71%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.70% (-7.97%)</t>
+          <t>-7.51% (-7.78%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.27% (-6.68%)</t>
+          <t>-6.01% (-6.42%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.74% (-7.07%)</t>
+          <t>-6.47% (-6.80%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.24% (-3.00%)</t>
+          <t>-1.89% (-2.65%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.27% (-2.96%)</t>
+          <t>-1.85% (-2.54%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.00% (-8.46%)</t>
+          <t>-7.85% (-8.31%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.31% (-3.94%)</t>
+          <t>-2.94% (-3.57%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.64% (-9.84%)</t>
+          <t>-9.47% (-9.67%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.57% (-9.69%)</t>
+          <t>-9.42% (-9.54%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.75% (-9.82%)</t>
+          <t>-9.66% (-9.73%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.56%</t>
+          <t>-16.89%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-25.30%</t>
+          <t>-24.69%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.99%</t>
+          <t>-20.35%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.96%</t>
+          <t>-19.31%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.70%</t>
+          <t>-19.05%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.71%</t>
+          <t>-13.01%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.31%</t>
+          <t>-12.60%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.71%</t>
+          <t>-24.09%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.19%</t>
+          <t>-13.49%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.49%</t>
+          <t>-22.87%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.87%</t>
+          <t>-22.24%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.95%</t>
+          <t>-22.32%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.13%</t>
+          <t>-21.50%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-29.46%</t>
+          <t>-28.88%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.38%</t>
+          <t>-24.77%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.40%</t>
+          <t>-23.79%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.16%</t>
+          <t>-23.55%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.51%</t>
+          <t>-17.84%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.13%</t>
+          <t>-17.46%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.89%</t>
+          <t>-28.31%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.96%</t>
+          <t>-18.30%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.75%</t>
+          <t>-27.15%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.16%</t>
+          <t>-26.56%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-27.23%</t>
+          <t>-26.64%</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3.09% (2.56%)</t>
+          <t>2.69% (2.15%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3225,112 +3225,112 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.61% (3.35%)</t>
+          <t>3.14% (2.88%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.94% (3.54%)</t>
+          <t>3.45% (3.05%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3.23% (2.90%)</t>
+          <t>2.80% (2.48%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.54% (0.78%)</t>
+          <t>1.19% (0.44%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.03% (0.34%)</t>
+          <t>0.75% (0.06%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.91% (5.46%)</t>
+          <t>6.11% (5.66%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.89% (0.27%)</t>
+          <t>0.55% (-0.07%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.17% (2.97%)</t>
+          <t>3.47% (3.27%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.06% (1.93%)</t>
+          <t>2.32% (2.20%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.00% (0.93%)</t>
+          <t>1.21% (1.15%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>4.16% (3.62%)</t>
+          <t>3.61% (3.07%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.07%)</t>
+          <t>0.01% (0.00%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.51% (3.24%)</t>
+          <t>3.72% (3.46%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>5.07% (4.66%)</t>
+          <t>4.88% (4.47%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>4.33% (4.00%)</t>
+          <t>4.04% (3.71%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.97% (1.22%)</t>
+          <t>1.50% (0.75%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.48% (0.79%)</t>
+          <t>1.08% (0.39%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.02% (4.56%)</t>
+          <t>5.19% (4.73%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.42% (0.80%)</t>
+          <t>0.98% (0.36%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.41% (2.20%)</t>
+          <t>2.60% (2.40%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.49% (1.36%)</t>
+          <t>1.66% (1.53%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.69% (0.62%)</t>
+          <t>0.79% (0.72%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 17/8/2026</t>
+          <t>As of 18/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.43%</t>
+          <t>11.14%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>5.59%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.10%</t>
+          <t>7.67%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.08%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.28%</t>
+          <t>-7.91%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.96%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.92%</t>
+          <t>6.28%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.78%</t>
+          <t>7.42%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.45%</t>
+          <t>11.54%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.28%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.01%</t>
+          <t>-7.69%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.60%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.46%</t>
+          <t>5.66%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.30%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.53%</t>
+          <t>18.57%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.97%</t>
+          <t>-1.18%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.10%</t>
+          <t>-9.94%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.44%</t>
+          <t>11.16%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.23%</t>
+          <t>8.69%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.62%</t>
+          <t>5.17%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>8.29%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>6.35%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.12%</t>
+          <t>-5.73%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.75%</t>
+          <t>9.51%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.04%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>3.24%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.88%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.64%</t>
+          <t>12.55%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.44%</t>
+          <t>-3.98%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>9.74%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.65%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.62%</t>
+          <t>2.08%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.82%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.17%</t>
+          <t>13.08%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.38%</t>
+          <t>-2.87%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.30%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.98%</t>
+          <t>13.52%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>2.16%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.30%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>12.91%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.41%</t>
+          <t>-2.95%</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.69%</t>
+          <t>12.08%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.48%</t>
+          <t>19.51%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-5.14%</t>
+          <t>-4.37%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.39%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>1.15%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>11.87%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.81%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.40%</t>
+          <t>-1.61%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.55%</t>
+          <t>-11.37%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>10.94%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.93%</t>
+          <t>2.20%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12.08%</t>
+          <t>11.78%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.68%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.53%</t>
+          <t>-11.30%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.68%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.97%</t>
+          <t>3.27%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.43%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.63%</t>
+          <t>16.69%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.86%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.81%</t>
+          <t>-11.55%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>11.31%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.12%</t>
+          <t>4.49%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.91%</t>
+          <t>12.99%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.74%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.36%</t>
+          <t>-9.04%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 17/8/2026</t>
+          <t>As of 18/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>16.75%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.70%</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.08%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>0.57%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.07%</t>
+          <t>-6.80%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.73%</t>
+          <t>17.37%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.66%</t>
+          <t>4.95%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.25%</t>
+          <t>5.96%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.45%</t>
+          <t>11.54%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.35%</t>
+          <t>0.46%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.68%</t>
+          <t>-6.42%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.43%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.73%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.32%</t>
+          <t>8.14%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.53%</t>
+          <t>18.57%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.54%</t>
+          <t>-3.77%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.46%</t>
+          <t>-8.31%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.63%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.66%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>8.29%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.14%</t>
+          <t>-4.87%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.02%</t>
+          <t>14.73%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.89%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.20%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.89%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.52%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.94%</t>
+          <t>-3.57%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.17%</t>
+          <t>14.92%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>10.58%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>1.74%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.83%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>10.07%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.96%</t>
+          <t>-2.54%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.51%</t>
+          <t>15.19%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>10.92%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>1.85%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.00%</t>
+          <t>-2.65%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.69%</t>
+          <t>18.17%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.11%</t>
+          <t>11.03%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20.50%</t>
+          <t>19.51%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-7.14%</t>
+          <t>-6.38%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.77%</t>
+          <t>-10.71%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.42%</t>
+          <t>16.91%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>0.72%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>9.84%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.82%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-4.57%</t>
+          <t>-3.78%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.82%</t>
+          <t>-9.73%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.47%</t>
+          <t>17.02%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.36%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>9.62%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.70%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.90%</t>
+          <t>-3.11%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.69%</t>
+          <t>-9.54%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.90%</t>
+          <t>17.48%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.20%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.65%</t>
+          <t>16.69%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.73%</t>
+          <t>-2.94%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.84%</t>
+          <t>-9.67%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17.41%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.24%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.74%</t>
+          <t>7.52%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.92%</t>
+          <t>12.99%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.97%</t>
+          <t>-7.78%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-19]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/18/2026 at 10:05 AM ET)</t>
+          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>241 days</t>
+          <t>240 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>122 days</t>
+          <t>121 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>185 days</t>
+          <t>184 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>150 days</t>
+          <t>149 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>332 days</t>
+          <t>331 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>303 days</t>
+          <t>302 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>213 days</t>
+          <t>212 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>276 days</t>
+          <t>275 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>94 days</t>
+          <t>93 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>59 days</t>
+          <t>58 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>31 days</t>
+          <t>30 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>241 days</t>
+          <t>240 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>122 days</t>
+          <t>121 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>185 days</t>
+          <t>184 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>150 days</t>
+          <t>149 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>332 days</t>
+          <t>331 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>303 days</t>
+          <t>302 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>213 days</t>
+          <t>212 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>276 days</t>
+          <t>275 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>94 days</t>
+          <t>93 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>59 days</t>
+          <t>58 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>31 days</t>
+          <t>30 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.61 / 5.17%</t>
+          <t>$47.67 / 5.31%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.50 / 13.44%</t>
+          <t>$57.52 / 13.47%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.60 / 9.00%</t>
+          <t>$55.67 / 9.13%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.21 / 7.42%</t>
+          <t>$62.29 / 7.55%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.28 / 7.67%</t>
+          <t>$56.33 / 7.76%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.14 / 2.16%</t>
+          <t>$61.21 / 2.28%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.12 / 2.08%</t>
+          <t>$61.20 / 2.22%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.19 / 10.09%</t>
+          <t>$53.25 / 10.21%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.37 / 3.24%</t>
+          <t>$57.41 / 3.31%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.69 / 12.11%</t>
+          <t>$59.75 / 12.22%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.51 / 11.78%</t>
+          <t>$53.54 / 11.85%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.39 / 11.87%</t>
+          <t>$56.43 / 11.95%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.37 / 4.24%</t>
+          <t>$42.41 / 4.33%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.98 / 11.03%</t>
+          <t>$41.99 / 11.05%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.52 / 7.52%</t>
+          <t>$40.55 / 7.59%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.74 / 5.96%</t>
+          <t>$44.77 / 6.04%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.80 / 6.39%</t>
+          <t>$45.86 / 6.52%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.46 / 1.85%</t>
+          <t>$44.51 / 1.98%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.87 / 1.74%</t>
+          <t>$41.92 / 1.86%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.91 / 8.14%</t>
+          <t>$44.94 / 8.21%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.84 / 2.80%</t>
+          <t>$43.88 / 2.91%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.51 / 9.77%</t>
+          <t>$42.54 / 9.85%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.28 / 9.62%</t>
+          <t>$42.31 / 9.70%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.72 / 9.84%</t>
+          <t>$41.75 / 9.92%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$769.00 / 8.29%</t>
+          <t>$769.94 / 8.42%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$769.00 / 19.51%</t>
+          <t>$769.94 / 19.66%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$769.00 / 12.99%</t>
+          <t>$769.94 / 13.13%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$769.00 / 11.54%</t>
+          <t>$769.94 / 11.68%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$769.00 / 11.18%</t>
+          <t>$769.94 / 11.32%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$769.00 / 3.46%</t>
+          <t>$769.94 / 3.58%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$769.00 / 2.98%</t>
+          <t>$769.94 / 3.11%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$769.00 / 18.57%</t>
+          <t>$769.94 / 18.71%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$769.00 / 4.04%</t>
+          <t>$769.94 / 4.16%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$769.00 / 16.69%</t>
+          <t>$769.94 / 16.83%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$769.00 / 15.75%</t>
+          <t>$769.94 / 15.89%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$769.00 / 15.87%</t>
+          <t>$769.94 / 16.01%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$769.00 / 8.29%</t>
+          <t>$769.94 / 8.42%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$769.00 / 19.51%</t>
+          <t>$769.94 / 19.66%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$769.00 / 12.99%</t>
+          <t>$769.94 / 13.13%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$769.00 / 11.54%</t>
+          <t>$769.94 / 11.68%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$769.00 / 11.18%</t>
+          <t>$769.94 / 11.32%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$769.00 / 3.46%</t>
+          <t>$769.94 / 3.58%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$769.00 / 2.98%</t>
+          <t>$769.94 / 3.11%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$769.00 / 18.57%</t>
+          <t>$769.94 / 18.71%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$769.00 / 4.04%</t>
+          <t>$769.94 / 4.16%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$769.00 / 16.69%</t>
+          <t>$769.94 / 16.83%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$769.00 / 15.75%</t>
+          <t>$769.94 / 15.89%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$769.00 / 15.87%</t>
+          <t>$769.94 / 16.01%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.22% (8.69%)</t>
+          <t>9.08% (8.55%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>-0.01% (-0.01%)</t>
+          <t>-0.04% (-0.04%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.76% (4.49%)</t>
+          <t>4.63% (4.37%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.68% (6.28%)</t>
+          <t>6.55% (6.15%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.91% (5.59%)</t>
+          <t>5.81% (5.49%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.27% (13.52%)</t>
+          <t>14.14% (13.39%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.94% (13.25%)</t>
+          <t>13.78% (13.09%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.11% (5.66%)</t>
+          <t>5.99% (5.54%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.20% (12.58%)</t>
+          <t>13.12% (12.50%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.47% (3.27%)</t>
+          <t>3.36% (3.17%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.32% (2.20%)</t>
+          <t>2.26% (2.14%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>1.21% (1.15%)</t>
+          <t>1.14% (1.08%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.50% (6.96%)</t>
+          <t>7.40% (6.86%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.01% (0.00%)</t>
+          <t>-0.02% (-0.02%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.72% (3.46%)</t>
+          <t>3.65% (3.38%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.36% (4.95%)</t>
+          <t>5.28% (4.87%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.63% (4.30%)</t>
+          <t>4.50% (4.18%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.68% (10.92%)</t>
+          <t>11.54% (10.78%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.27% (10.58%)</t>
+          <t>11.14% (10.45%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>5.19% (4.73%)</t>
+          <t>5.12% (4.66%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.51% (9.89%)</t>
+          <t>10.40% (9.77%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.60% (2.40%)</t>
+          <t>2.52% (2.32%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.66% (1.53%)</t>
+          <t>1.58% (1.46%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.79% (0.72%)</t>
+          <t>0.71% (0.65%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.35%</t>
+          <t>6.22%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>-4.37%</t>
+          <t>-4.49%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>1.43%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.89%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.08%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-1.30%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.55%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-0.69%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-1.73%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-6.38%</t>
+          <t>-6.49%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-0.92%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.57%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>9.88%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.07%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.77%</t>
+          <t>-3.88%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.94%</t>
+          <t>-3.06%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.11%</t>
+          <t>-3.23%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-3.78%</t>
+          <t>-3.90%</t>
         </is>
       </c>
     </row>
@@ -2834,47 +2834,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.70% (11.16%)</t>
+          <t>11.68% (11.14%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12.09% (12.08%)</t>
+          <t>12.16% (12.15%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.57% (11.31%)</t>
+          <t>11.56% (11.30%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>12.02% (11.62%)</t>
+          <t>12.00% (11.60%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.47% (11.14%)</t>
+          <t>11.48% (11.16%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.82% (10.06%)</t>
+          <t>10.81% (10.06%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.43% (9.74%)</t>
+          <t>10.40% (9.71%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.61% (14.16%)</t>
+          <t>14.60% (14.15%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.14% (9.51%)</t>
+          <t>10.17% (9.55%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2884,12 +2884,12 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>11.07% (10.94%)</t>
+          <t>11.11% (10.99%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11.02% (10.96%)</t>
+          <t>11.05% (10.99%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2899,37 +2899,37 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>18.18% (18.17%)</t>
+          <t>18.24% (18.23%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>17.26% (16.99%)</t>
+          <t>17.28% (17.02%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.78% (17.37%)</t>
+          <t>17.80% (17.39%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>17.08% (16.75%)</t>
+          <t>17.06% (16.73%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.95% (15.19%)</t>
+          <t>15.93% (15.17%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.61% (14.92%)</t>
+          <t>15.59% (14.90%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.46% (20.00%)</t>
+          <t>20.48% (20.03%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
@@ -2939,17 +2939,17 @@
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.68% (17.48%)</t>
+          <t>17.70% (17.50%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>17.14% (17.02%)</t>
+          <t>17.16% (17.04%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.97% (16.91%)</t>
+          <t>16.99% (16.93%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.19% (-5.73%)</t>
+          <t>-5.31% (-5.84%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-12.61% (-12.61%)</t>
+          <t>-12.63% (-12.63%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.78% (-9.04%)</t>
+          <t>-8.89% (-9.14%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.29% (-7.69%)</t>
+          <t>-7.41% (-7.81%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.59% (-7.91%)</t>
+          <t>-7.67% (-7.99%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.19% (-2.95%)</t>
+          <t>-2.31% (-3.06%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.17% (-2.87%)</t>
+          <t>-2.31% (-3.00%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.48% (-9.94%)</t>
+          <t>-9.59% (-10.04%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.35% (-3.98%)</t>
+          <t>-3.42% (-4.04%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.36% (-11.55%)</t>
+          <t>-11.45% (-11.64%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.18% (-11.30%)</t>
+          <t>-11.23% (-11.35%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.30% (-11.37%)</t>
+          <t>-11.37% (-11.43%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.34% (-4.87%)</t>
+          <t>-4.43% (-4.96%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-10.70% (-10.71%)</t>
+          <t>-10.72% (-10.73%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.51% (-7.78%)</t>
+          <t>-7.58% (-7.84%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.01% (-6.42%)</t>
+          <t>-6.09% (-6.49%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.47% (-6.80%)</t>
+          <t>-6.58% (-6.91%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.89% (-2.65%)</t>
+          <t>-2.01% (-2.77%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.85% (-2.54%)</t>
+          <t>-1.97% (-2.66%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-7.85% (-8.31%)</t>
+          <t>-7.91% (-8.37%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.94% (-3.57%)</t>
+          <t>-3.04% (-3.67%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.47% (-9.67%)</t>
+          <t>-9.54% (-9.74%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.42% (-9.54%)</t>
+          <t>-9.49% (-9.61%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-9.66% (-9.73%)</t>
+          <t>-9.73% (-9.80%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.89%</t>
+          <t>-16.99%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-24.69%</t>
+          <t>-24.79%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.35%</t>
+          <t>-20.44%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.31%</t>
+          <t>-19.41%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.05%</t>
+          <t>-19.15%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.01%</t>
+          <t>-13.11%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.60%</t>
+          <t>-12.71%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.09%</t>
+          <t>-24.19%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.49%</t>
+          <t>-13.60%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.87%</t>
+          <t>-22.96%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.24%</t>
+          <t>-22.34%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-22.32%</t>
+          <t>-22.42%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.50%</t>
+          <t>-21.60%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-28.88%</t>
+          <t>-28.96%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.77%</t>
+          <t>-24.86%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.79%</t>
+          <t>-23.88%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.55%</t>
+          <t>-23.64%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.84%</t>
+          <t>-17.94%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.46%</t>
+          <t>-17.56%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.31%</t>
+          <t>-28.40%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.30%</t>
+          <t>-18.39%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.15%</t>
+          <t>-27.24%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.56%</t>
+          <t>-26.65%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-26.64%</t>
+          <t>-26.72%</t>
         </is>
       </c>
     </row>
@@ -3215,17 +3215,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.69% (2.15%)</t>
+          <t>2.68% (2.15%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.01% (-0.01%)</t>
+          <t>-0.04% (-0.04%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.14% (2.88%)</t>
+          <t>3.14% (2.89%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -3235,62 +3235,62 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.80% (2.48%)</t>
+          <t>2.83% (2.51%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.19% (0.44%)</t>
+          <t>1.20% (0.45%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.75% (0.06%)</t>
+          <t>0.73% (0.04%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.11% (5.66%)</t>
+          <t>5.99% (5.54%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.55% (-0.07%)</t>
+          <t>0.60% (-0.02%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.47% (3.27%)</t>
+          <t>3.36% (3.17%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2.32% (2.20%)</t>
+          <t>2.26% (2.14%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.21% (1.15%)</t>
+          <t>1.14% (1.08%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.61% (3.07%)</t>
+          <t>3.64% (3.10%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.01% (0.00%)</t>
+          <t>-0.02% (-0.02%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.72% (3.46%)</t>
+          <t>3.65% (3.38%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.88% (4.47%)</t>
+          <t>4.92% (4.52%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -3300,7 +3300,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.50% (0.75%)</t>
+          <t>1.50% (0.74%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -3310,27 +3310,27 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>5.19% (4.73%)</t>
+          <t>5.12% (4.66%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.98% (0.36%)</t>
+          <t>1.00% (0.38%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.60% (2.40%)</t>
+          <t>2.52% (2.32%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.66% (1.53%)</t>
+          <t>1.58% (1.46%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.79% (0.72%)</t>
+          <t>0.71% (0.65%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 18/8/2026</t>
+          <t>As of 19/8/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11.14%</t>
+          <t>11.16%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.59%</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.67%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.89%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.91%</t>
+          <t>-7.99%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.28%</t>
+          <t>6.15%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.42%</t>
+          <t>7.55%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>11.68%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.69%</t>
+          <t>-7.81%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>14.15%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.66%</t>
+          <t>5.54%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>10.21%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.57%</t>
+          <t>18.71%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-1.30%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.94%</t>
+          <t>-10.04%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.16%</t>
+          <t>11.14%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.69%</t>
+          <t>8.55%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>5.31%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.29%</t>
+          <t>8.42%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.35%</t>
+          <t>6.22%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.73%</t>
+          <t>-5.84%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.51%</t>
+          <t>9.55%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.58%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.24%</t>
+          <t>3.31%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.04%</t>
+          <t>4.16%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.55%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.98%</t>
+          <t>-4.04%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.74%</t>
+          <t>9.71%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>13.09%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.08%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.98%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.08%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.87%</t>
+          <t>-3.00%</t>
         </is>
       </c>
     </row>
@@ -3637,27 +3637,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.39%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.16%</t>
+          <t>2.28%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.95%</t>
+          <t>-3.06%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12.08%</t>
+          <t>12.15%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.47%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>19.51%</t>
+          <t>19.66%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-4.37%</t>
+          <t>-4.49%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-12.61%</t>
+          <t>-12.63%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>10.99%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.15%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.87%</t>
+          <t>11.95%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-1.73%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.37%</t>
+          <t>-11.43%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.94%</t>
+          <t>10.99%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.20%</t>
+          <t>2.14%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.78%</t>
+          <t>11.85%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>15.89%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-0.69%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.30%</t>
+          <t>-11.35%</t>
         </is>
       </c>
     </row>
@@ -3785,27 +3785,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.27%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>12.22%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.69%</t>
+          <t>16.83%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.55%</t>
+          <t>-11.64%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.31%</t>
+          <t>11.30%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.49%</t>
+          <t>4.37%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.99%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>1.43%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.04%</t>
+          <t>-9.14%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 18/8/2026</t>
+          <t>As of 19/8/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.75%</t>
+          <t>16.73%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.30%</t>
+          <t>4.18%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.52%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.57%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.80%</t>
+          <t>-6.91%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.37%</t>
+          <t>17.39%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.95%</t>
+          <t>4.87%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.96%</t>
+          <t>6.04%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>11.68%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.42%</t>
+          <t>-6.49%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>20.03%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.73%</t>
+          <t>4.66%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.14%</t>
+          <t>8.21%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.57%</t>
+          <t>18.71%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.77%</t>
+          <t>-3.88%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.31%</t>
+          <t>-8.37%</t>
         </is>
       </c>
     </row>
@@ -4041,27 +4041,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>6.86%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.24%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.29%</t>
+          <t>8.42%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.87%</t>
+          <t>-4.96%</t>
         </is>
       </c>
     </row>
@@ -4078,27 +4078,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.89%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.80%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.04%</t>
+          <t>4.16%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.57%</t>
+          <t>-3.67%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.92%</t>
+          <t>14.90%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.58%</t>
+          <t>10.45%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.74%</t>
+          <t>1.86%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.98%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.07%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.54%</t>
+          <t>-2.66%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.19%</t>
+          <t>15.17%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.92%</t>
+          <t>10.78%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.85%</t>
+          <t>1.98%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>9.88%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.65%</t>
+          <t>-2.77%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18.17%</t>
+          <t>18.23%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.03%</t>
+          <t>11.05%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>19.51%</t>
+          <t>19.66%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-6.38%</t>
+          <t>-6.49%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-10.71%</t>
+          <t>-10.73%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.91%</t>
+          <t>16.93%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.84%</t>
+          <t>9.92%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-3.78%</t>
+          <t>-3.90%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-9.73%</t>
+          <t>-9.80%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17.02%</t>
+          <t>17.04%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>1.46%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.62%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>15.89%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.11%</t>
+          <t>-3.23%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.54%</t>
+          <t>-9.61%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.48%</t>
+          <t>17.50%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.85%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.69%</t>
+          <t>16.83%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.94%</t>
+          <t>-3.06%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.67%</t>
+          <t>-9.74%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>17.02%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.52%</t>
+          <t>7.59%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.99%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-0.92%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.78%</t>
+          <t>-7.84%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-08-20]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:07 AM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:07 AM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 8/19/2026 at 10:06 AM ET)</t>
+          <t>Current Values(as of 8/20/2026 at 10:08 AM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>240 days</t>
+          <t>239 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>1 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>121 days</t>
+          <t>120 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>184 days</t>
+          <t>183 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>149 days</t>
+          <t>148 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>331 days</t>
+          <t>330 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>302 days</t>
+          <t>301 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>212 days</t>
+          <t>211 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>275 days</t>
+          <t>274 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>93 days</t>
+          <t>92 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>58 days</t>
+          <t>57 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>29 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>240 days</t>
+          <t>239 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>1 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>121 days</t>
+          <t>120 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>184 days</t>
+          <t>183 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>149 days</t>
+          <t>148 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>331 days</t>
+          <t>330 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>302 days</t>
+          <t>301 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>212 days</t>
+          <t>211 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>275 days</t>
+          <t>274 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>93 days</t>
+          <t>92 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>58 days</t>
+          <t>57 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>29 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.67 / 5.31%</t>
+          <t>$47.60 / 5.15%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.52 / 13.47%</t>
+          <t>$57.51 / 13.45%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.67 / 9.13%</t>
+          <t>$55.58 / 8.96%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.29 / 7.55%</t>
+          <t>$62.20 / 7.40%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.33 / 7.76%</t>
+          <t>$56.28 / 7.68%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.21 / 2.28%</t>
+          <t>$61.06 / 2.02%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.20 / 2.22%</t>
+          <t>$61.07 / 1.99%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.25 / 10.21%</t>
+          <t>$53.22 / 10.15%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.41 / 3.31%</t>
+          <t>$57.28 / 3.08%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.75 / 12.22%</t>
+          <t>$59.69 / 12.10%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.54 / 11.85%</t>
+          <t>$53.51 / 11.78%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.43 / 11.95%</t>
+          <t>$56.36 / 11.80%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.41 / 4.33%</t>
+          <t>$42.36 / 4.21%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.99 / 11.05%</t>
+          <t>$42.01 / 11.11%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.55 / 7.59%</t>
+          <t>$40.52 / 7.50%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.77 / 6.04%</t>
+          <t>$44.75 / 5.99%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.86 / 6.52%</t>
+          <t>$45.82 / 6.43%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.51 / 1.98%</t>
+          <t>$44.43 / 1.78%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.92 / 1.86%</t>
+          <t>$41.85 / 1.69%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$44.94 / 8.21%</t>
+          <t>$44.93 / 8.19%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.88 / 2.91%</t>
+          <t>$43.80 / 2.72%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.54 / 9.85%</t>
+          <t>$42.53 / 9.83%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.31 / 9.70%</t>
+          <t>$42.30